<commit_message>
Expand and refresh conference catalog
</commit_message>
<xml_diff>
--- a/data/core_conferences_normalized_tags.xlsx
+++ b/data/core_conferences_normalized_tags.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Conferences" sheetId="1" r:id="R9df255e54181423f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Vocabulary" sheetId="2" r:id="R4f20a8483e5f45ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Conferences" sheetId="1" r:id="Rcbb51779e80c448f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Vocabulary" sheetId="2" r:id="Rdcc88c89b9d04464"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -91,7 +91,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CoreConferencesTable" displayName="CoreConferencesTable" ref="A1:F34" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CoreConferencesTable" displayName="CoreConferencesTable" ref="A1:F59" headerRowCount="1" totalsRowCount="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Conference"/>
     <x:tableColumn id="2" name="TAGS"/>
@@ -308,7 +308,7 @@
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="F2" s="14" t="str">
-        <x:v>https://neurips.cc/</x:v>
+        <x:v>https://neurips.cc/Conferences/2026</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -328,7 +328,7 @@
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="F3" s="14" t="str">
-        <x:v>https://icml.cc/</x:v>
+        <x:v>https://icml.cc/Conferences/2026</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -348,7 +348,7 @@
         <x:v>Paper-based / OpenReview</x:v>
       </x:c>
       <x:c r="F4" s="14" t="str">
-        <x:v>https://iclr.cc/</x:v>
+        <x:v>https://iclr.cc/Conferences/2027</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -408,7 +408,7 @@
         <x:v>Paper-based / theory-focused</x:v>
       </x:c>
       <x:c r="F7" s="14" t="str">
-        <x:v>https://learningtheory.org/colt2026/</x:v>
+        <x:v>https://learningtheory.org/colt2027/</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -428,7 +428,7 @@
         <x:v>Paper-based / mixed tracks</x:v>
       </x:c>
       <x:c r="F8" s="14" t="str">
-        <x:v>https://ecmlpkdd.org/</x:v>
+        <x:v>https://ecmlpkdd.org/2026/</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -448,7 +448,7 @@
         <x:v>Paper-based / mixed tracks</x:v>
       </x:c>
       <x:c r="F9" s="14" t="str">
-        <x:v>https://www.kdd.org/conferences</x:v>
+        <x:v>https://kdd2026.kdd.org/</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -508,7 +508,7 @@
         <x:v>Paper-based / applied tracks</x:v>
       </x:c>
       <x:c r="F12" s="14" t="str">
-        <x:v>https://dsaa.co/</x:v>
+        <x:v>https://dsaa-2026.vercel.app/</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -579,7 +579,7 @@
         <x:v>Time Series &amp; Sequential Data; Healthcare &amp; Clinical AI; Signal Processing; Explainability &amp; Interpretability</x:v>
       </x:c>
       <x:c r="C16" s="14" t="str">
-        <x:v>S/focused</x:v>
+        <x:v>S</x:v>
       </x:c>
       <x:c r="D16" s="14" t="str">
         <x:v>Moderate-hard</x:v>
@@ -648,7 +648,7 @@
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="F19" s="14" t="str">
-        <x:v>https://biomedicalimaging.org/2026/</x:v>
+        <x:v>https://biomedicalimaging.org/2027/</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -708,7 +708,7 @@
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="F22" s="14" t="str">
-        <x:v>https://ieeeicassp.org/</x:v>
+        <x:v>https://2027.ieeeicassp.org/</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -728,7 +728,7 @@
         <x:v>Paper-based / workshop-style conference</x:v>
       </x:c>
       <x:c r="F23" s="14" t="str">
-        <x:v>https://signalprocessingsociety.org/event-names/mlsp</x:v>
+        <x:v>https://mlsp26.ieeesps.org/</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -748,7 +748,7 @@
         <x:v>Abstract-based / talks highly selective</x:v>
       </x:c>
       <x:c r="F24" s="14" t="str">
-        <x:v>https://www.cosyne.org/</x:v>
+        <x:v>https://www.cosyne.org/cosyne-home</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -808,7 +808,7 @@
         <x:v>Abstract-based</x:v>
       </x:c>
       <x:c r="F27" s="14" t="str">
-        <x:v>https://www.cnsorg.org/</x:v>
+        <x:v>https://www.cnsorg.org/cns-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -828,7 +828,7 @@
         <x:v>Abstract-based / talks selective</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
-        <x:v>https://humanbrainmapping.org/</x:v>
+        <x:v>https://humanbrainmapping.org/ohbm-2027/</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -888,7 +888,7 @@
         <x:v>Abstract-based / specialist venue</x:v>
       </x:c>
       <x:c r="F31" s="14" t="str">
-        <x:v>https://biomag2026.scimeeting.cn/en/web/index/31426</x:v>
+        <x:v>https://mm.scimeeting.cn/en/web/index/31426</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -948,7 +948,7 @@
         <x:v>Paper-based / HCI-focused</x:v>
       </x:c>
       <x:c r="F34" s="14" t="str">
-        <x:v>https://chi2026.acm.org/</x:v>
+        <x:v>https://chi2027.acm.org/</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -971,10 +971,490 @@
         <x:v>https://aaai.org/conference/aaai/aaai-27/</x:v>
       </x:c>
     </x:row>
+    <x:row r="36" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A36" s="12" t="str">
+        <x:v>IJCAI-ECAI</x:v>
+      </x:c>
+      <x:c r="B36" s="12" t="str">
+        <x:v>Machine Learning; Deep Representation Learning; Learning Theory &amp; Statistical Foundations; Fairness &amp; Responsible AI</x:v>
+      </x:c>
+      <x:c r="C36" s="12" t="str">
+        <x:v>XL</x:v>
+      </x:c>
+      <x:c r="D36" s="12" t="str">
+        <x:v>Very hard</x:v>
+      </x:c>
+      <x:c r="E36" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="F36" s="12" t="str">
+        <x:v>https://www.ijcai.org/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A37" s="12" t="str">
+        <x:v>ACML</x:v>
+      </x:c>
+      <x:c r="B37" s="12" t="str">
+        <x:v>Machine Learning; Deep Representation Learning; Learning Theory &amp; Statistical Foundations; Explainability &amp; Interpretability</x:v>
+      </x:c>
+      <x:c r="C37" s="12" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="D37" s="12" t="str">
+        <x:v>Hard</x:v>
+      </x:c>
+      <x:c r="E37" s="12" t="str">
+        <x:v>Paper-based / OpenReview</x:v>
+      </x:c>
+      <x:c r="F37" s="12" t="str">
+        <x:v>https://www.acml-conf.org/2026/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A38" s="12" t="str">
+        <x:v>PAKDD</x:v>
+      </x:c>
+      <x:c r="B38" s="12" t="str">
+        <x:v>Data Mining &amp; Data Science; Machine Learning; Time Series &amp; Sequential Data; Learning Theory &amp; Statistical Foundations</x:v>
+      </x:c>
+      <x:c r="C38" s="12" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="D38" s="12" t="str">
+        <x:v>Hard</x:v>
+      </x:c>
+      <x:c r="E38" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="F38" s="12" t="str">
+        <x:v>https://pakdd.org/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A39" s="12" t="str">
+        <x:v>CIKM</x:v>
+      </x:c>
+      <x:c r="B39" s="12" t="str">
+        <x:v>Data Mining &amp; Data Science; Machine Learning; Time Series &amp; Sequential Data; Human-AI Interaction &amp; Deployment</x:v>
+      </x:c>
+      <x:c r="C39" s="12" t="str">
+        <x:v>XL</x:v>
+      </x:c>
+      <x:c r="D39" s="12" t="str">
+        <x:v>Very hard</x:v>
+      </x:c>
+      <x:c r="E39" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="F39" s="12" t="str">
+        <x:v>https://www.cikmconference.org/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A40" s="12" t="str">
+        <x:v>WSDM</x:v>
+      </x:c>
+      <x:c r="B40" s="12" t="str">
+        <x:v>Data Mining &amp; Data Science; Machine Learning; Fairness &amp; Responsible AI; Human-AI Interaction &amp; Deployment</x:v>
+      </x:c>
+      <x:c r="C40" s="12" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="D40" s="12" t="str">
+        <x:v>Very hard</x:v>
+      </x:c>
+      <x:c r="E40" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="F40" s="12" t="str">
+        <x:v>https://www.wsdm-conference.org/2027/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A41" s="12" t="str">
+        <x:v>IEEE BigData</x:v>
+      </x:c>
+      <x:c r="B41" s="12" t="str">
+        <x:v>Data Mining &amp; Data Science; Machine Learning; Time Series &amp; Sequential Data; Healthcare &amp; Clinical AI</x:v>
+      </x:c>
+      <x:c r="C41" s="12" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="D41" s="12" t="str">
+        <x:v>Moderate-hard</x:v>
+      </x:c>
+      <x:c r="E41" s="12" t="str">
+        <x:v>Paper-based / mixed tracks</x:v>
+      </x:c>
+      <x:c r="F41" s="12" t="str">
+        <x:v>https://bigdataieee.org/BigData2026/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A42" s="12" t="str">
+        <x:v>Discovery Science</x:v>
+      </x:c>
+      <x:c r="B42" s="12" t="str">
+        <x:v>Data Mining &amp; Data Science; Machine Learning; Learning Theory &amp; Statistical Foundations; Time Series &amp; Sequential Data</x:v>
+      </x:c>
+      <x:c r="C42" s="12" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D42" s="12" t="str">
+        <x:v>Hard</x:v>
+      </x:c>
+      <x:c r="E42" s="12" t="str">
+        <x:v>Paper-based / research forum</x:v>
+      </x:c>
+      <x:c r="F42" s="12" t="str">
+        <x:v>https://discovery-science.org/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A43" s="12" t="str">
+        <x:v>IDA</x:v>
+      </x:c>
+      <x:c r="B43" s="12" t="str">
+        <x:v>Data Mining &amp; Data Science; Machine Learning; Probabilistic, Causal &amp; Uncertainty ML; Time Series &amp; Sequential Data</x:v>
+      </x:c>
+      <x:c r="C43" s="12" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D43" s="12" t="str">
+        <x:v>Moderate-hard</x:v>
+      </x:c>
+      <x:c r="E43" s="12" t="str">
+        <x:v>Paper-based / interdisciplinary</x:v>
+      </x:c>
+      <x:c r="F43" s="12" t="str">
+        <x:v>https://www.ida-society.org/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A44" s="12" t="str">
+        <x:v>ADMA</x:v>
+      </x:c>
+      <x:c r="B44" s="12" t="str">
+        <x:v>Data Mining &amp; Data Science; Machine Learning; Time Series &amp; Sequential Data; Explainability &amp; Interpretability</x:v>
+      </x:c>
+      <x:c r="C44" s="12" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D44" s="12" t="str">
+        <x:v>Moderate-hard</x:v>
+      </x:c>
+      <x:c r="E44" s="12" t="str">
+        <x:v>Paper-based / special sessions</x:v>
+      </x:c>
+      <x:c r="F44" s="12" t="str">
+        <x:v>https://adma2026.github.io/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A45" s="12" t="str">
+        <x:v>IJCNN</x:v>
+      </x:c>
+      <x:c r="B45" s="12" t="str">
+        <x:v>Machine Learning; Deep Representation Learning; Learning Theory &amp; Statistical Foundations; Signal Processing</x:v>
+      </x:c>
+      <x:c r="C45" s="12" t="str">
+        <x:v>XL</x:v>
+      </x:c>
+      <x:c r="D45" s="12" t="str">
+        <x:v>Moderate-hard</x:v>
+      </x:c>
+      <x:c r="E45" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="F45" s="12" t="str">
+        <x:v>https://ijcnn.org/2027</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A46" s="12" t="str">
+        <x:v>ICANN</x:v>
+      </x:c>
+      <x:c r="B46" s="12" t="str">
+        <x:v>Machine Learning; Deep Representation Learning; Computational Neuroscience; Signal Processing</x:v>
+      </x:c>
+      <x:c r="C46" s="12" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="D46" s="12" t="str">
+        <x:v>Moderate-hard</x:v>
+      </x:c>
+      <x:c r="E46" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="F46" s="12" t="str">
+        <x:v>https://e-nns.org/icann2026/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A47" s="12" t="str">
+        <x:v>ESANN</x:v>
+      </x:c>
+      <x:c r="B47" s="12" t="str">
+        <x:v>Machine Learning; Deep Representation Learning; Learning Theory &amp; Statistical Foundations; Signal Processing</x:v>
+      </x:c>
+      <x:c r="C47" s="12" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D47" s="12" t="str">
+        <x:v>Hard</x:v>
+      </x:c>
+      <x:c r="E47" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="F47" s="12" t="str">
+        <x:v>https://www.esann.org/node/160</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A48" s="12" t="str">
+        <x:v>ICONIP</x:v>
+      </x:c>
+      <x:c r="B48" s="12" t="str">
+        <x:v>Machine Learning; Deep Representation Learning; Computational Neuroscience; Signal Processing</x:v>
+      </x:c>
+      <x:c r="C48" s="12" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="D48" s="12" t="str">
+        <x:v>Moderate-hard</x:v>
+      </x:c>
+      <x:c r="E48" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="F48" s="12" t="str">
+        <x:v>https://www.iconip2026.org/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A49" s="12" t="str">
+        <x:v>ICPR</x:v>
+      </x:c>
+      <x:c r="B49" s="12" t="str">
+        <x:v>Machine Learning; Deep Representation Learning; Signal Processing; Biomedical Imaging</x:v>
+      </x:c>
+      <x:c r="C49" s="12" t="str">
+        <x:v>XL</x:v>
+      </x:c>
+      <x:c r="D49" s="12" t="str">
+        <x:v>Hard</x:v>
+      </x:c>
+      <x:c r="E49" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="F49" s="12" t="str">
+        <x:v>https://iapr.org/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A50" s="12" t="str">
+        <x:v>ACPR</x:v>
+      </x:c>
+      <x:c r="B50" s="12" t="str">
+        <x:v>Machine Learning; Deep Representation Learning; Signal Processing; Biomedical Imaging</x:v>
+      </x:c>
+      <x:c r="C50" s="12" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D50" s="12" t="str">
+        <x:v>Hard</x:v>
+      </x:c>
+      <x:c r="E50" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="F50" s="12" t="str">
+        <x:v>https://iapr.org/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A51" s="12" t="str">
+        <x:v>S+SSPR</x:v>
+      </x:c>
+      <x:c r="B51" s="12" t="str">
+        <x:v>Machine Learning; Deep Representation Learning; Data Mining &amp; Data Science; Signal Processing</x:v>
+      </x:c>
+      <x:c r="C51" s="12" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D51" s="12" t="str">
+        <x:v>Moderate-hard</x:v>
+      </x:c>
+      <x:c r="E51" s="12" t="str">
+        <x:v>Paper-based / workshop-style conference</x:v>
+      </x:c>
+      <x:c r="F51" s="12" t="str">
+        <x:v>https://ssspr2026.inf.unibe.ch/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A52" s="12" t="str">
+        <x:v>IEEE ICMLA</x:v>
+      </x:c>
+      <x:c r="B52" s="12" t="str">
+        <x:v>Machine Learning; Deep Representation Learning; Data Mining &amp; Data Science; Time Series &amp; Sequential Data</x:v>
+      </x:c>
+      <x:c r="C52" s="12" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D52" s="12" t="str">
+        <x:v>Moderate-hard</x:v>
+      </x:c>
+      <x:c r="E52" s="12" t="str">
+        <x:v>Paper-based / special sessions</x:v>
+      </x:c>
+      <x:c r="F52" s="12" t="str">
+        <x:v>https://www.icmla-conference.org/icmla26/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A53" s="12" t="str">
+        <x:v>IEEE SSCI</x:v>
+      </x:c>
+      <x:c r="B53" s="12" t="str">
+        <x:v>Machine Learning; Deep Representation Learning; Learning Theory &amp; Statistical Foundations; Fairness &amp; Responsible AI</x:v>
+      </x:c>
+      <x:c r="C53" s="12" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="D53" s="12" t="str">
+        <x:v>Moderate-hard</x:v>
+      </x:c>
+      <x:c r="E53" s="12" t="str">
+        <x:v>Paper-based / symposium series</x:v>
+      </x:c>
+      <x:c r="F53" s="12" t="str">
+        <x:v>https://ssci2027generalchairs.github.io/ssci-2027/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A54" s="12" t="str">
+        <x:v>IDEAL</x:v>
+      </x:c>
+      <x:c r="B54" s="12" t="str">
+        <x:v>Machine Learning; Data Mining &amp; Data Science; Deep Representation Learning; Learning Theory &amp; Statistical Foundations</x:v>
+      </x:c>
+      <x:c r="C54" s="12" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D54" s="12" t="str">
+        <x:v>Moderate-hard</x:v>
+      </x:c>
+      <x:c r="E54" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="F54" s="12" t="str">
+        <x:v>https://www.ideal2026.org/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A55" s="12" t="str">
+        <x:v>LOD</x:v>
+      </x:c>
+      <x:c r="B55" s="12" t="str">
+        <x:v>Machine Learning; Data Mining &amp; Data Science; Learning Theory &amp; Statistical Foundations; Time Series &amp; Sequential Data</x:v>
+      </x:c>
+      <x:c r="C55" s="12" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D55" s="12" t="str">
+        <x:v>Moderate-hard</x:v>
+      </x:c>
+      <x:c r="E55" s="12" t="str">
+        <x:v>Paper-based / Springer proceedings</x:v>
+      </x:c>
+      <x:c r="F55" s="12" t="str">
+        <x:v>https://lodconference.org/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A56" s="12" t="str">
+        <x:v>EUSIPCO</x:v>
+      </x:c>
+      <x:c r="B56" s="12" t="str">
+        <x:v>Signal Processing; Machine Learning; Time Series &amp; Sequential Data; EEG/MEG &amp; Neural Signals</x:v>
+      </x:c>
+      <x:c r="C56" s="12" t="str">
+        <x:v>XL</x:v>
+      </x:c>
+      <x:c r="D56" s="12" t="str">
+        <x:v>Hard</x:v>
+      </x:c>
+      <x:c r="E56" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="F56" s="12" t="str">
+        <x:v>https://eusipco2026.org/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A57" s="12" t="str">
+        <x:v>IEEE SSP</x:v>
+      </x:c>
+      <x:c r="B57" s="12" t="str">
+        <x:v>Signal Processing; Machine Learning; Time Series &amp; Sequential Data; Probabilistic, Causal &amp; Uncertainty ML</x:v>
+      </x:c>
+      <x:c r="C57" s="12" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D57" s="12" t="str">
+        <x:v>Hard</x:v>
+      </x:c>
+      <x:c r="E57" s="12" t="str">
+        <x:v>Paper-based / specialist workshop</x:v>
+      </x:c>
+      <x:c r="F57" s="12" t="str">
+        <x:v>https://signalprocessingsociety.org/events/call-proposals-statistical-signal-processing-ssp-2027</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A58" s="12" t="str">
+        <x:v>AALTD</x:v>
+      </x:c>
+      <x:c r="B58" s="12" t="str">
+        <x:v>Time Series &amp; Sequential Data; Data Mining &amp; Data Science; Machine Learning; Explainability &amp; Interpretability</x:v>
+      </x:c>
+      <x:c r="C58" s="12" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="D58" s="12" t="str">
+        <x:v>Moderate-hard</x:v>
+      </x:c>
+      <x:c r="E58" s="12" t="str">
+        <x:v>Workshop / paper-based</x:v>
+      </x:c>
+      <x:c r="F58" s="12" t="str">
+        <x:v>https://ecml-aaltd.github.io/aaltd2026/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A59" s="12" t="str">
+        <x:v>ITISE</x:v>
+      </x:c>
+      <x:c r="B59" s="12" t="str">
+        <x:v>Time Series &amp; Sequential Data; Machine Learning; Data Mining &amp; Data Science; Learning Theory &amp; Statistical Foundations</x:v>
+      </x:c>
+      <x:c r="C59" s="12" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D59" s="12" t="str">
+        <x:v>Moderate-hard</x:v>
+      </x:c>
+      <x:c r="E59" s="12" t="str">
+        <x:v>Paper-based / forecasting-focused</x:v>
+      </x:c>
+      <x:c r="F59" s="12" t="str">
+        <x:v>https://itise.ugr.es/</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c242cb4471d40d3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69680b8eb2934ed0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1126,7 +1606,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5322ae3c56cb4fec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4279c7a2acdd48e7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add EACL and refresh upcoming editions
</commit_message>
<xml_diff>
--- a/data/core_conferences_normalized_tags.xlsx
+++ b/data/core_conferences_normalized_tags.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Conferences" sheetId="1" r:id="Rcbb51779e80c448f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Vocabulary" sheetId="2" r:id="Rdcc88c89b9d04464"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Conferences" sheetId="1" r:id="Rc0f9ba7615944165"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Vocabulary" sheetId="2" r:id="R7ef1cbbf56ba431e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -768,7 +768,7 @@
         <x:v>Mixed: proceedings + extended abstracts</x:v>
       </x:c>
       <x:c r="F25" s="14" t="str">
-        <x:v>https://ccneuro.org/</x:v>
+        <x:v>https://2026.ccneuro.org/</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -988,7 +988,7 @@
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="F36" s="12" t="str">
-        <x:v>https://www.ijcai.org/</x:v>
+        <x:v>https://2026.ijcai.org/</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1048,7 +1048,7 @@
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="F39" s="12" t="str">
-        <x:v>https://www.cikmconference.org/</x:v>
+        <x:v>https://cikm2026.diag.uniroma1.it/</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1208,7 +1208,7 @@
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="F47" s="12" t="str">
-        <x:v>https://www.esann.org/node/160</x:v>
+        <x:v>https://www.esann.org/</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1248,7 +1248,7 @@
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="F49" s="12" t="str">
-        <x:v>https://iapr.org/</x:v>
+        <x:v>https://icpr2026.org/</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1408,7 +1408,7 @@
         <x:v>Paper-based / specialist workshop</x:v>
       </x:c>
       <x:c r="F57" s="12" t="str">
-        <x:v>https://signalprocessingsociety.org/events/call-proposals-statistical-signal-processing-ssp-2027</x:v>
+        <x:v>https://ssp27.ieeesps.org/</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1451,10 +1451,30 @@
         <x:v>https://itise.ugr.es/</x:v>
       </x:c>
     </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="12" t="str">
+        <x:v>EACL</x:v>
+      </x:c>
+      <x:c r="B60" s="12" t="str">
+        <x:v>Natural Language Processing &amp; LLMs; Machine Learning; Deep Representation Learning; Fairness &amp; Responsible AI; Human-AI Interaction &amp; Deployment</x:v>
+      </x:c>
+      <x:c r="C60" s="12" t="str">
+        <x:v>L/XL</x:v>
+      </x:c>
+      <x:c r="D60" s="12" t="str">
+        <x:v>Hard</x:v>
+      </x:c>
+      <x:c r="E60" s="12" t="str">
+        <x:v>Paper-based / ACL Rolling Review</x:v>
+      </x:c>
+      <x:c r="F60" s="12" t="str">
+        <x:v>https://2027.eacl.org/</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69680b8eb2934ed0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re63f4eebc7814514"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1603,10 +1623,18 @@
         <x:v>Human-centered AI, usability, clinical deployment, interfaces, translational use.</x:v>
       </x:c>
     </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="12" t="str">
+        <x:v>Natural Language Processing &amp; LLMs</x:v>
+      </x:c>
+      <x:c r="B18" s="12" t="str">
+        <x:v>Natural language processing, language models, computational linguistics, and LLM systems.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4279c7a2acdd48e7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0de8d75de934d19"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Refresh conference calendar with IDA, AIME, and FMTS
</commit_message>
<xml_diff>
--- a/data/core_conferences_normalized_tags.xlsx
+++ b/data/core_conferences_normalized_tags.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Conferences" sheetId="1" r:id="Rc0f9ba7615944165"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Vocabulary" sheetId="2" r:id="R7ef1cbbf56ba431e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Conferences" sheetId="1" r:id="R2e2cb43f26bc44ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Vocabulary" sheetId="2" r:id="Re2ec369f25de4f62"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -91,7 +91,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CoreConferencesTable" displayName="CoreConferencesTable" ref="A1:F59" headerRowCount="1" totalsRowCount="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CoreConferencesTable" displayName="CoreConferencesTable" ref="A1:F62" headerRowCount="1" totalsRowCount="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Conference"/>
     <x:tableColumn id="2" name="TAGS"/>
@@ -1028,7 +1028,7 @@
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="F38" s="12" t="str">
-        <x:v>https://pakdd.org/</x:v>
+        <x:v>https://pakdd2027.org/</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1448,7 +1448,7 @@
         <x:v>Paper-based / forecasting-focused</x:v>
       </x:c>
       <x:c r="F59" s="12" t="str">
-        <x:v>https://itise.ugr.es/</x:v>
+        <x:v>https://itise.ugr.es/index.html</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
@@ -1471,10 +1471,50 @@
         <x:v>https://2027.eacl.org/</x:v>
       </x:c>
     </x:row>
+    <x:row r="61" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A61" s="12" t="str">
+        <x:v>AIME</x:v>
+      </x:c>
+      <x:c r="B61" s="12" t="str">
+        <x:v>Healthcare &amp; Clinical AI; Machine Learning; Biomedical Imaging; Probabilistic, Causal &amp; Uncertainty ML</x:v>
+      </x:c>
+      <x:c r="C61" s="12" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D61" s="12" t="str">
+        <x:v>Moderate-hard</x:v>
+      </x:c>
+      <x:c r="E61" s="12" t="str">
+        <x:v>Paper-based / clinical AI</x:v>
+      </x:c>
+      <x:c r="F61" s="12" t="str">
+        <x:v>https://aime27.aimedicine.info/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A62" s="12" t="str">
+        <x:v>FMTS @ NeurIPS</x:v>
+      </x:c>
+      <x:c r="B62" s="12" t="str">
+        <x:v>Time Series &amp; Sequential Data; Machine Learning; Deep Representation Learning; Probabilistic, Causal &amp; Uncertainty ML</x:v>
+      </x:c>
+      <x:c r="C62" s="12" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="D62" s="12" t="str">
+        <x:v>Moderate-hard</x:v>
+      </x:c>
+      <x:c r="E62" s="12" t="str">
+        <x:v>Workshop / non-archival short paper</x:v>
+      </x:c>
+      <x:c r="F62" s="12" t="str">
+        <x:v>https://fmts-workshop.github.io/</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re63f4eebc7814514"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ccb6426c8204c07"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1634,7 +1674,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0de8d75de934d19"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89e455f8e2774f49"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add ICORE 2026 rankings to both calendar tabs
</commit_message>
<xml_diff>
--- a/data/core_conferences_normalized_tags.xlsx
+++ b/data/core_conferences_normalized_tags.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Conferences" sheetId="1" r:id="R2e2cb43f26bc44ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Vocabulary" sheetId="2" r:id="Re2ec369f25de4f62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Conferences" sheetId="1" r:id="R5236e086dbf7434b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Vocabulary" sheetId="2" r:id="R63ccbec7b29c4760"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -91,16 +91,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CoreConferencesTable" displayName="CoreConferencesTable" ref="A1:F62" headerRowCount="1" totalsRowCount="0">
-  <x:tableColumns count="6">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="CoreConferencesTable" displayName="CoreConferencesTable" ref="A1:H62" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="8">
     <x:tableColumn id="1" name="Conference"/>
     <x:tableColumn id="2" name="TAGS"/>
     <x:tableColumn id="3" name="SIZE"/>
     <x:tableColumn id="4" name="Acceptance difficulty"/>
-    <x:tableColumn id="5" name="Submission type"/>
-    <x:tableColumn id="6" name="Source"/>
+    <x:tableColumn id="5" name="ICORE 2026"/>
+    <x:tableColumn id="6" name="Submission type"/>
+    <x:tableColumn id="7" name="Source"/>
+    <x:tableColumn id="8" name="ICORE source"/>
   </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
@@ -267,8 +269,10 @@
     <x:col min="2" max="2" width="56" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="10" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="30" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="58" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="31" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="52" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="52" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -285,10 +289,16 @@
         <x:v>Acceptance difficulty</x:v>
       </x:c>
       <x:c r="E1" s="6" t="str">
+        <x:v>ICORE 2026</x:v>
+      </x:c>
+      <x:c r="F1" s="6" t="str">
         <x:v>Submission type</x:v>
       </x:c>
-      <x:c r="F1" s="6" t="str">
+      <x:c r="G1" t="str">
         <x:v>Source</x:v>
+      </x:c>
+      <x:c r="H1" t="str">
+        <x:v>ICORE source</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -305,10 +315,16 @@
         <x:v>Very hard</x:v>
       </x:c>
       <x:c r="E2" s="14" t="str">
-        <x:v>Paper-based</x:v>
+        <x:v>A*</x:v>
       </x:c>
       <x:c r="F2" s="14" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G2" t="str">
         <x:v>https://neurips.cc/Conferences/2026</x:v>
+      </x:c>
+      <x:c r="H2" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/98/</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -325,10 +341,16 @@
         <x:v>Very hard</x:v>
       </x:c>
       <x:c r="E3" s="14" t="str">
-        <x:v>Paper-based</x:v>
+        <x:v>A*</x:v>
       </x:c>
       <x:c r="F3" s="14" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G3" t="str">
         <x:v>https://icml.cc/Conferences/2026</x:v>
+      </x:c>
+      <x:c r="H3" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/1121/</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -345,10 +367,16 @@
         <x:v>Hard</x:v>
       </x:c>
       <x:c r="E4" s="14" t="str">
+        <x:v>A*</x:v>
+      </x:c>
+      <x:c r="F4" s="14" t="str">
         <x:v>Paper-based / OpenReview</x:v>
       </x:c>
-      <x:c r="F4" s="14" t="str">
+      <x:c r="G4" t="str">
         <x:v>https://iclr.cc/Conferences/2027</x:v>
+      </x:c>
+      <x:c r="H4" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/2273/</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -365,10 +393,16 @@
         <x:v>Hard</x:v>
       </x:c>
       <x:c r="E5" s="14" t="str">
-        <x:v>Paper-based</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="F5" s="14" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G5" t="str">
         <x:v>https://aistats.org/</x:v>
+      </x:c>
+      <x:c r="H5" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/913/</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -385,10 +419,16 @@
         <x:v>Hard</x:v>
       </x:c>
       <x:c r="E6" s="14" t="str">
-        <x:v>Paper-based</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="F6" s="14" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G6" t="str">
         <x:v>https://www.auai.org/uai2026/</x:v>
+      </x:c>
+      <x:c r="H6" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/346/</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -405,10 +445,16 @@
         <x:v>Very hard</x:v>
       </x:c>
       <x:c r="E7" s="14" t="str">
+        <x:v>A*</x:v>
+      </x:c>
+      <x:c r="F7" s="14" t="str">
         <x:v>Paper-based / theory-focused</x:v>
       </x:c>
-      <x:c r="F7" s="14" t="str">
+      <x:c r="G7" t="str">
         <x:v>https://learningtheory.org/colt2027/</x:v>
+      </x:c>
+      <x:c r="H7" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/124/</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -425,10 +471,16 @@
         <x:v>Hard</x:v>
       </x:c>
       <x:c r="E8" s="14" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="F8" s="14" t="str">
         <x:v>Paper-based / mixed tracks</x:v>
       </x:c>
-      <x:c r="F8" s="14" t="str">
+      <x:c r="G8" t="str">
         <x:v>https://ecmlpkdd.org/2026/</x:v>
+      </x:c>
+      <x:c r="H8" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/491/</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -445,10 +497,16 @@
         <x:v>Very hard</x:v>
       </x:c>
       <x:c r="E9" s="14" t="str">
+        <x:v>A*</x:v>
+      </x:c>
+      <x:c r="F9" s="14" t="str">
         <x:v>Paper-based / mixed tracks</x:v>
       </x:c>
-      <x:c r="F9" s="14" t="str">
+      <x:c r="G9" t="str">
         <x:v>https://kdd2026.kdd.org/</x:v>
+      </x:c>
+      <x:c r="H9" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/26/</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -465,10 +523,16 @@
         <x:v>Hard</x:v>
       </x:c>
       <x:c r="E10" s="14" t="str">
-        <x:v>Paper-based</x:v>
+        <x:v>A*</x:v>
       </x:c>
       <x:c r="F10" s="14" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G10" t="str">
         <x:v>https://icdm2026.neu.edu.cn/</x:v>
+      </x:c>
+      <x:c r="H10" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/642/</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -485,10 +549,16 @@
         <x:v>Hard</x:v>
       </x:c>
       <x:c r="E11" s="14" t="str">
-        <x:v>Paper-based</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="F11" s="14" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G11" t="str">
         <x:v>https://www.siam.org/conferences-events/siam-conferences/sdm26/</x:v>
+      </x:c>
+      <x:c r="H11" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/1727/</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -505,10 +575,16 @@
         <x:v>Moderate-hard</x:v>
       </x:c>
       <x:c r="E12" s="14" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="F12" s="14" t="str">
         <x:v>Paper-based / applied tracks</x:v>
       </x:c>
-      <x:c r="F12" s="14" t="str">
+      <x:c r="G12" t="str">
         <x:v>https://dsaa-2026.vercel.app/</x:v>
+      </x:c>
+      <x:c r="H12" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/2237/</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -524,12 +600,14 @@
       <x:c r="D13" s="14" t="str">
         <x:v>Hard</x:v>
       </x:c>
-      <x:c r="E13" s="14" t="str">
-        <x:v>Paper-based</x:v>
-      </x:c>
+      <x:c r="E13" s="14" t="str"/>
       <x:c r="F13" s="14" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G13" t="str">
         <x:v>https://mlhc.org/</x:v>
       </x:c>
+      <x:c r="H13" t="str"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="14" t="str">
@@ -544,12 +622,14 @@
       <x:c r="D14" s="14" t="str">
         <x:v>Hard</x:v>
       </x:c>
-      <x:c r="E14" s="14" t="str">
-        <x:v>Paper-based</x:v>
-      </x:c>
+      <x:c r="E14" s="14" t="str"/>
       <x:c r="F14" s="14" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G14" t="str">
         <x:v>https://chil.ahli.cc/</x:v>
       </x:c>
+      <x:c r="H14" t="str"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="14" t="str">
@@ -564,12 +644,14 @@
       <x:c r="D15" s="14" t="str">
         <x:v>Moderate-hard</x:v>
       </x:c>
-      <x:c r="E15" s="14" t="str">
+      <x:c r="E15" s="14" t="str"/>
+      <x:c r="F15" s="14" t="str">
         <x:v>Proceedings + findings tracks</x:v>
       </x:c>
-      <x:c r="F15" s="14" t="str">
+      <x:c r="G15" t="str">
         <x:v>https://ml4h.ahli.cc/</x:v>
       </x:c>
+      <x:c r="H15" t="str"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="14" t="str">
@@ -584,12 +666,14 @@
       <x:c r="D16" s="14" t="str">
         <x:v>Moderate-hard</x:v>
       </x:c>
-      <x:c r="E16" s="14" t="str">
+      <x:c r="E16" s="14" t="str"/>
+      <x:c r="F16" s="14" t="str">
         <x:v>Workshop / paper-based</x:v>
       </x:c>
-      <x:c r="F16" s="14" t="str">
+      <x:c r="G16" t="str">
         <x:v>https://timeseries4health.github.io/</x:v>
       </x:c>
+      <x:c r="H16" t="str"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="14" t="str">
@@ -605,10 +689,16 @@
         <x:v>Hard</x:v>
       </x:c>
       <x:c r="E17" s="14" t="str">
-        <x:v>Paper-based</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="F17" s="14" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G17" t="str">
         <x:v>https://conferences.miccai.org/2026/en/default.asp</x:v>
+      </x:c>
+      <x:c r="H17" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/1607/</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -624,12 +714,14 @@
       <x:c r="D18" s="14" t="str">
         <x:v>Moderate-hard</x:v>
       </x:c>
-      <x:c r="E18" s="14" t="str">
-        <x:v>Paper-based</x:v>
-      </x:c>
+      <x:c r="E18" s="14" t="str"/>
       <x:c r="F18" s="14" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G18" t="str">
         <x:v>https://2026.midl.io/</x:v>
       </x:c>
+      <x:c r="H18" t="str"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="14" t="str">
@@ -644,12 +736,14 @@
       <x:c r="D19" s="14" t="str">
         <x:v>Moderate-hard</x:v>
       </x:c>
-      <x:c r="E19" s="14" t="str">
-        <x:v>Paper-based</x:v>
-      </x:c>
+      <x:c r="E19" s="14" t="str"/>
       <x:c r="F19" s="14" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G19" t="str">
         <x:v>https://biomedicalimaging.org/2027/</x:v>
       </x:c>
+      <x:c r="H19" t="str"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="14" t="str">
@@ -664,12 +758,14 @@
       <x:c r="D20" s="14" t="str">
         <x:v>Moderate-hard</x:v>
       </x:c>
-      <x:c r="E20" s="14" t="str">
-        <x:v>Paper-based</x:v>
-      </x:c>
+      <x:c r="E20" s="14" t="str"/>
       <x:c r="F20" s="14" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G20" t="str">
         <x:v>https://bhi.embs.org/2026/</x:v>
       </x:c>
+      <x:c r="H20" t="str"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="14" t="str">
@@ -684,12 +780,14 @@
       <x:c r="D21" s="14" t="str">
         <x:v>Moderate</x:v>
       </x:c>
-      <x:c r="E21" s="14" t="str">
+      <x:c r="E21" s="14" t="str"/>
+      <x:c r="F21" s="14" t="str">
         <x:v>Paper-based / broad applied venue</x:v>
       </x:c>
-      <x:c r="F21" s="14" t="str">
+      <x:c r="G21" t="str">
         <x:v>https://embc.embs.org/2026/</x:v>
       </x:c>
+      <x:c r="H21" t="str"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="14" t="str">
@@ -704,12 +802,14 @@
       <x:c r="D22" s="14" t="str">
         <x:v>Moderate-hard</x:v>
       </x:c>
-      <x:c r="E22" s="14" t="str">
-        <x:v>Paper-based</x:v>
-      </x:c>
+      <x:c r="E22" s="14" t="str"/>
       <x:c r="F22" s="14" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G22" t="str">
         <x:v>https://2027.ieeeicassp.org/</x:v>
       </x:c>
+      <x:c r="H22" t="str"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="14" t="str">
@@ -724,12 +824,14 @@
       <x:c r="D23" s="14" t="str">
         <x:v>Moderate-hard</x:v>
       </x:c>
-      <x:c r="E23" s="14" t="str">
+      <x:c r="E23" s="14" t="str"/>
+      <x:c r="F23" s="14" t="str">
         <x:v>Paper-based / workshop-style conference</x:v>
       </x:c>
-      <x:c r="F23" s="14" t="str">
+      <x:c r="G23" t="str">
         <x:v>https://mlsp26.ieeesps.org/</x:v>
       </x:c>
+      <x:c r="H23" t="str"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="14" t="str">
@@ -744,12 +846,14 @@
       <x:c r="D24" s="14" t="str">
         <x:v>Hard</x:v>
       </x:c>
-      <x:c r="E24" s="14" t="str">
+      <x:c r="E24" s="14" t="str"/>
+      <x:c r="F24" s="14" t="str">
         <x:v>Abstract-based / talks highly selective</x:v>
       </x:c>
-      <x:c r="F24" s="14" t="str">
+      <x:c r="G24" t="str">
         <x:v>https://www.cosyne.org/cosyne-home</x:v>
       </x:c>
+      <x:c r="H24" t="str"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="14" t="str">
@@ -764,12 +868,14 @@
       <x:c r="D25" s="14" t="str">
         <x:v>Moderate-hard</x:v>
       </x:c>
-      <x:c r="E25" s="14" t="str">
+      <x:c r="E25" s="14" t="str"/>
+      <x:c r="F25" s="14" t="str">
         <x:v>Mixed: proceedings + extended abstracts</x:v>
       </x:c>
-      <x:c r="F25" s="14" t="str">
+      <x:c r="G25" t="str">
         <x:v>https://2026.ccneuro.org/</x:v>
       </x:c>
+      <x:c r="H25" t="str"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="14" t="str">
@@ -784,12 +890,14 @@
       <x:c r="D26" s="14" t="str">
         <x:v>Moderate</x:v>
       </x:c>
-      <x:c r="E26" s="14" t="str">
+      <x:c r="E26" s="14" t="str"/>
+      <x:c r="F26" s="14" t="str">
         <x:v>Abstract-based / talks selective</x:v>
       </x:c>
-      <x:c r="F26" s="14" t="str">
+      <x:c r="G26" t="str">
         <x:v>https://bernstein-network.de/en/bernstein-conference/</x:v>
       </x:c>
+      <x:c r="H26" t="str"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="14" t="str">
@@ -804,12 +912,14 @@
       <x:c r="D27" s="14" t="str">
         <x:v>Moderate</x:v>
       </x:c>
-      <x:c r="E27" s="14" t="str">
+      <x:c r="E27" s="14" t="str"/>
+      <x:c r="F27" s="14" t="str">
         <x:v>Abstract-based</x:v>
       </x:c>
-      <x:c r="F27" s="14" t="str">
+      <x:c r="G27" t="str">
         <x:v>https://www.cnsorg.org/cns-2026</x:v>
       </x:c>
+      <x:c r="H27" t="str"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="14" t="str">
@@ -824,12 +934,14 @@
       <x:c r="D28" s="14" t="str">
         <x:v>Moderate</x:v>
       </x:c>
-      <x:c r="E28" s="14" t="str">
+      <x:c r="E28" s="14" t="str"/>
+      <x:c r="F28" s="14" t="str">
         <x:v>Abstract-based / talks selective</x:v>
       </x:c>
-      <x:c r="F28" s="14" t="str">
+      <x:c r="G28" t="str">
         <x:v>https://humanbrainmapping.org/ohbm-2027/</x:v>
       </x:c>
+      <x:c r="H28" t="str"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="14" t="str">
@@ -844,12 +956,14 @@
       <x:c r="D29" s="14" t="str">
         <x:v>Moderate-hard</x:v>
       </x:c>
-      <x:c r="E29" s="14" t="str">
+      <x:c r="E29" s="14" t="str"/>
+      <x:c r="F29" s="14" t="str">
         <x:v>Paper-based / engineering-focused</x:v>
       </x:c>
-      <x:c r="F29" s="14" t="str">
+      <x:c r="G29" t="str">
         <x:v>https://ieee-ner.org/</x:v>
       </x:c>
+      <x:c r="H29" t="str"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="14" t="str">
@@ -864,12 +978,14 @@
       <x:c r="D30" s="14" t="str">
         <x:v>Moderate</x:v>
       </x:c>
-      <x:c r="E30" s="14" t="str">
+      <x:c r="E30" s="14" t="str"/>
+      <x:c r="F30" s="14" t="str">
         <x:v>Abstract/community-based</x:v>
       </x:c>
-      <x:c r="F30" s="14" t="str">
+      <x:c r="G30" t="str">
         <x:v>https://bcisociety.org/bci-meeting/</x:v>
       </x:c>
+      <x:c r="H30" t="str"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="14" t="str">
@@ -884,12 +1000,14 @@
       <x:c r="D31" s="14" t="str">
         <x:v>Moderate</x:v>
       </x:c>
-      <x:c r="E31" s="14" t="str">
+      <x:c r="E31" s="14" t="str"/>
+      <x:c r="F31" s="14" t="str">
         <x:v>Abstract-based / specialist venue</x:v>
       </x:c>
-      <x:c r="F31" s="14" t="str">
+      <x:c r="G31" t="str">
         <x:v>https://mm.scimeeting.cn/en/web/index/31426</x:v>
       </x:c>
+      <x:c r="H31" t="str"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="14" t="str">
@@ -904,12 +1022,14 @@
       <x:c r="D32" s="14" t="str">
         <x:v>Hard</x:v>
       </x:c>
-      <x:c r="E32" s="14" t="str">
+      <x:c r="E32" s="14" t="str"/>
+      <x:c r="F32" s="14" t="str">
         <x:v>Paper-based / interdisciplinary</x:v>
       </x:c>
-      <x:c r="F32" s="14" t="str">
+      <x:c r="G32" t="str">
         <x:v>https://facctconference.org/</x:v>
       </x:c>
+      <x:c r="H32" t="str"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="14" t="str">
@@ -925,10 +1045,16 @@
         <x:v>Moderate-hard</x:v>
       </x:c>
       <x:c r="E33" s="14" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="F33" s="14" t="str">
         <x:v>Paper-based / interdisciplinary</x:v>
       </x:c>
-      <x:c r="F33" s="14" t="str">
+      <x:c r="G33" t="str">
         <x:v>https://www.aies-conference.com/2026/</x:v>
+      </x:c>
+      <x:c r="H33" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/2354/</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -945,10 +1071,16 @@
         <x:v>Hard</x:v>
       </x:c>
       <x:c r="E34" s="14" t="str">
+        <x:v>A*</x:v>
+      </x:c>
+      <x:c r="F34" s="14" t="str">
         <x:v>Paper-based / HCI-focused</x:v>
       </x:c>
-      <x:c r="F34" s="14" t="str">
+      <x:c r="G34" t="str">
         <x:v>https://chi2027.acm.org/</x:v>
+      </x:c>
+      <x:c r="H34" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/1053/</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -965,10 +1097,16 @@
         <x:v>Very hard</x:v>
       </x:c>
       <x:c r="E35" t="str">
+        <x:v>A*</x:v>
+      </x:c>
+      <x:c r="F35" t="str">
         <x:v>Paper-based / OpenReview</x:v>
       </x:c>
-      <x:c r="F35" t="str">
+      <x:c r="G35" t="str">
         <x:v>https://aaai.org/conference/aaai/aaai-27/</x:v>
+      </x:c>
+      <x:c r="H35" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/1629/</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -984,12 +1122,14 @@
       <x:c r="D36" s="12" t="str">
         <x:v>Very hard</x:v>
       </x:c>
-      <x:c r="E36" s="12" t="str">
-        <x:v>Paper-based</x:v>
-      </x:c>
+      <x:c r="E36" s="12" t="str"/>
       <x:c r="F36" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G36" t="str">
         <x:v>https://2026.ijcai.org/</x:v>
       </x:c>
+      <x:c r="H36" t="str"/>
     </x:row>
     <x:row r="37" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A37" s="12" t="str">
@@ -1005,10 +1145,16 @@
         <x:v>Hard</x:v>
       </x:c>
       <x:c r="E37" s="12" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="F37" s="12" t="str">
         <x:v>Paper-based / OpenReview</x:v>
       </x:c>
-      <x:c r="F37" s="12" t="str">
+      <x:c r="G37" t="str">
         <x:v>https://www.acml-conf.org/2026/</x:v>
+      </x:c>
+      <x:c r="H37" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/2174/</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1025,10 +1171,16 @@
         <x:v>Hard</x:v>
       </x:c>
       <x:c r="E38" s="12" t="str">
-        <x:v>Paper-based</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="F38" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G38" t="str">
         <x:v>https://pakdd2027.org/</x:v>
+      </x:c>
+      <x:c r="H38" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/1667/</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1045,10 +1197,16 @@
         <x:v>Very hard</x:v>
       </x:c>
       <x:c r="E39" s="12" t="str">
-        <x:v>Paper-based</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="F39" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G39" t="str">
         <x:v>https://cikm2026.diag.uniroma1.it/</x:v>
+      </x:c>
+      <x:c r="H39" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/25/</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1065,10 +1223,16 @@
         <x:v>Very hard</x:v>
       </x:c>
       <x:c r="E40" s="12" t="str">
-        <x:v>Paper-based</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="F40" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G40" t="str">
         <x:v>https://www.wsdm-conference.org/2027/</x:v>
+      </x:c>
+      <x:c r="H40" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/31/</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1085,10 +1249,16 @@
         <x:v>Moderate-hard</x:v>
       </x:c>
       <x:c r="E41" s="12" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="F41" s="12" t="str">
         <x:v>Paper-based / mixed tracks</x:v>
       </x:c>
-      <x:c r="F41" s="12" t="str">
+      <x:c r="G41" t="str">
         <x:v>https://bigdataieee.org/BigData2026/</x:v>
+      </x:c>
+      <x:c r="H41" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/2274/</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1105,10 +1275,16 @@
         <x:v>Hard</x:v>
       </x:c>
       <x:c r="E42" s="12" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="F42" s="12" t="str">
         <x:v>Paper-based / research forum</x:v>
       </x:c>
-      <x:c r="F42" s="12" t="str">
+      <x:c r="G42" t="str">
         <x:v>https://discovery-science.org/</x:v>
+      </x:c>
+      <x:c r="H42" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/2191/</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1125,10 +1301,16 @@
         <x:v>Moderate-hard</x:v>
       </x:c>
       <x:c r="E43" s="12" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="F43" s="12" t="str">
         <x:v>Paper-based / interdisciplinary</x:v>
       </x:c>
-      <x:c r="F43" s="12" t="str">
+      <x:c r="G43" t="str">
         <x:v>https://www.ida-society.org/</x:v>
+      </x:c>
+      <x:c r="H43" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/845/</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1145,10 +1327,16 @@
         <x:v>Moderate-hard</x:v>
       </x:c>
       <x:c r="E44" s="12" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="F44" s="12" t="str">
         <x:v>Paper-based / special sessions</x:v>
       </x:c>
-      <x:c r="F44" s="12" t="str">
+      <x:c r="G44" t="str">
         <x:v>https://adma2026.github.io/</x:v>
+      </x:c>
+      <x:c r="H44" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/888/</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1165,10 +1353,16 @@
         <x:v>Moderate-hard</x:v>
       </x:c>
       <x:c r="E45" s="12" t="str">
-        <x:v>Paper-based</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="F45" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G45" t="str">
         <x:v>https://ijcnn.org/2027</x:v>
+      </x:c>
+      <x:c r="H45" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/685/</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1185,10 +1379,16 @@
         <x:v>Moderate-hard</x:v>
       </x:c>
       <x:c r="E46" s="12" t="str">
-        <x:v>Paper-based</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="F46" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G46" t="str">
         <x:v>https://e-nns.org/icann2026/</x:v>
+      </x:c>
+      <x:c r="H46" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/915/</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1205,10 +1405,16 @@
         <x:v>Hard</x:v>
       </x:c>
       <x:c r="E47" s="12" t="str">
-        <x:v>Paper-based</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="F47" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G47" t="str">
         <x:v>https://www.esann.org/</x:v>
+      </x:c>
+      <x:c r="H47" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/512/</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1225,10 +1431,16 @@
         <x:v>Moderate-hard</x:v>
       </x:c>
       <x:c r="E48" s="12" t="str">
-        <x:v>Paper-based</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="F48" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G48" t="str">
         <x:v>https://www.iconip2026.org/</x:v>
+      </x:c>
+      <x:c r="H48" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/1152/</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1245,10 +1457,16 @@
         <x:v>Hard</x:v>
       </x:c>
       <x:c r="E49" s="12" t="str">
-        <x:v>Paper-based</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="F49" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G49" t="str">
         <x:v>https://icpr2026.org/</x:v>
+      </x:c>
+      <x:c r="H49" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/1169/</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1264,12 +1482,14 @@
       <x:c r="D50" s="12" t="str">
         <x:v>Hard</x:v>
       </x:c>
-      <x:c r="E50" s="12" t="str">
-        <x:v>Paper-based</x:v>
-      </x:c>
+      <x:c r="E50" s="12" t="str"/>
       <x:c r="F50" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G50" t="str">
         <x:v>https://iapr.org/</x:v>
       </x:c>
+      <x:c r="H50" t="str"/>
     </x:row>
     <x:row r="51" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A51" s="12" t="str">
@@ -1284,12 +1504,14 @@
       <x:c r="D51" s="12" t="str">
         <x:v>Moderate-hard</x:v>
       </x:c>
-      <x:c r="E51" s="12" t="str">
+      <x:c r="E51" s="12" t="str"/>
+      <x:c r="F51" s="12" t="str">
         <x:v>Paper-based / workshop-style conference</x:v>
       </x:c>
-      <x:c r="F51" s="12" t="str">
+      <x:c r="G51" t="str">
         <x:v>https://ssspr2026.inf.unibe.ch/</x:v>
       </x:c>
+      <x:c r="H51" t="str"/>
     </x:row>
     <x:row r="52" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A52" s="12" t="str">
@@ -1305,10 +1527,16 @@
         <x:v>Moderate-hard</x:v>
       </x:c>
       <x:c r="E52" s="12" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="F52" s="12" t="str">
         <x:v>Paper-based / special sessions</x:v>
       </x:c>
-      <x:c r="F52" s="12" t="str">
+      <x:c r="G52" t="str">
         <x:v>https://www.icmla-conference.org/icmla26/</x:v>
+      </x:c>
+      <x:c r="H52" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/1122/</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1324,12 +1552,14 @@
       <x:c r="D53" s="12" t="str">
         <x:v>Moderate-hard</x:v>
       </x:c>
-      <x:c r="E53" s="12" t="str">
+      <x:c r="E53" s="12" t="str"/>
+      <x:c r="F53" s="12" t="str">
         <x:v>Paper-based / symposium series</x:v>
       </x:c>
-      <x:c r="F53" s="12" t="str">
+      <x:c r="G53" t="str">
         <x:v>https://ssci2027generalchairs.github.io/ssci-2027/</x:v>
       </x:c>
+      <x:c r="H53" t="str"/>
     </x:row>
     <x:row r="54" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A54" s="12" t="str">
@@ -1345,10 +1575,16 @@
         <x:v>Moderate-hard</x:v>
       </x:c>
       <x:c r="E54" s="12" t="str">
-        <x:v>Paper-based</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="F54" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G54" t="str">
         <x:v>https://www.ideal2026.org/</x:v>
+      </x:c>
+      <x:c r="H54" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/1093/</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1364,12 +1600,14 @@
       <x:c r="D55" s="12" t="str">
         <x:v>Moderate-hard</x:v>
       </x:c>
-      <x:c r="E55" s="12" t="str">
+      <x:c r="E55" s="12" t="str"/>
+      <x:c r="F55" s="12" t="str">
         <x:v>Paper-based / Springer proceedings</x:v>
       </x:c>
-      <x:c r="F55" s="12" t="str">
+      <x:c r="G55" t="str">
         <x:v>https://lodconference.org/</x:v>
       </x:c>
+      <x:c r="H55" t="str"/>
     </x:row>
     <x:row r="56" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A56" s="12" t="str">
@@ -1384,12 +1622,14 @@
       <x:c r="D56" s="12" t="str">
         <x:v>Hard</x:v>
       </x:c>
-      <x:c r="E56" s="12" t="str">
-        <x:v>Paper-based</x:v>
-      </x:c>
+      <x:c r="E56" s="12" t="str"/>
       <x:c r="F56" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G56" t="str">
         <x:v>https://eusipco2026.org/</x:v>
       </x:c>
+      <x:c r="H56" t="str"/>
     </x:row>
     <x:row r="57" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A57" s="12" t="str">
@@ -1404,12 +1644,14 @@
       <x:c r="D57" s="12" t="str">
         <x:v>Hard</x:v>
       </x:c>
-      <x:c r="E57" s="12" t="str">
+      <x:c r="E57" s="12" t="str"/>
+      <x:c r="F57" s="12" t="str">
         <x:v>Paper-based / specialist workshop</x:v>
       </x:c>
-      <x:c r="F57" s="12" t="str">
+      <x:c r="G57" t="str">
         <x:v>https://ssp27.ieeesps.org/</x:v>
       </x:c>
+      <x:c r="H57" t="str"/>
     </x:row>
     <x:row r="58" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A58" s="12" t="str">
@@ -1424,12 +1666,14 @@
       <x:c r="D58" s="12" t="str">
         <x:v>Moderate-hard</x:v>
       </x:c>
-      <x:c r="E58" s="12" t="str">
+      <x:c r="E58" s="12" t="str"/>
+      <x:c r="F58" s="12" t="str">
         <x:v>Workshop / paper-based</x:v>
       </x:c>
-      <x:c r="F58" s="12" t="str">
+      <x:c r="G58" t="str">
         <x:v>https://ecml-aaltd.github.io/aaltd2026/</x:v>
       </x:c>
+      <x:c r="H58" t="str"/>
     </x:row>
     <x:row r="59" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A59" s="12" t="str">
@@ -1444,12 +1688,14 @@
       <x:c r="D59" s="12" t="str">
         <x:v>Moderate-hard</x:v>
       </x:c>
-      <x:c r="E59" s="12" t="str">
+      <x:c r="E59" s="12" t="str"/>
+      <x:c r="F59" s="12" t="str">
         <x:v>Paper-based / forecasting-focused</x:v>
       </x:c>
-      <x:c r="F59" s="12" t="str">
+      <x:c r="G59" t="str">
         <x:v>https://itise.ugr.es/index.html</x:v>
       </x:c>
+      <x:c r="H59" t="str"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="12" t="str">
@@ -1465,10 +1711,16 @@
         <x:v>Hard</x:v>
       </x:c>
       <x:c r="E60" s="12" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="F60" s="12" t="str">
         <x:v>Paper-based / ACL Rolling Review</x:v>
       </x:c>
-      <x:c r="F60" s="12" t="str">
+      <x:c r="G60" t="str">
         <x:v>https://2027.eacl.org/</x:v>
+      </x:c>
+      <x:c r="H60" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/468/</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1485,10 +1737,16 @@
         <x:v>Moderate-hard</x:v>
       </x:c>
       <x:c r="E61" s="12" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="F61" s="12" t="str">
         <x:v>Paper-based / clinical AI</x:v>
       </x:c>
-      <x:c r="F61" s="12" t="str">
+      <x:c r="G61" t="str">
         <x:v>https://aime27.aimedicine.info/</x:v>
+      </x:c>
+      <x:c r="H61" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/151/</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1504,17 +1762,19 @@
       <x:c r="D62" s="12" t="str">
         <x:v>Moderate-hard</x:v>
       </x:c>
-      <x:c r="E62" s="12" t="str">
+      <x:c r="E62" s="12" t="str"/>
+      <x:c r="F62" s="12" t="str">
         <x:v>Workshop / non-archival short paper</x:v>
       </x:c>
-      <x:c r="F62" s="12" t="str">
+      <x:c r="G62" t="str">
         <x:v>https://fmts-workshop.github.io/</x:v>
       </x:c>
+      <x:c r="H62" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ccb6426c8204c07"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9988e0f28f1b4db7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1674,7 +1934,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89e455f8e2774f49"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd506e8cf24e14abc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Show actionable submission status and sourced selectivity evidence
</commit_message>
<xml_diff>
--- a/data/core_conferences_normalized_tags.xlsx
+++ b/data/core_conferences_normalized_tags.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Conferences" sheetId="1" r:id="R5236e086dbf7434b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Vocabulary" sheetId="2" r:id="R63ccbec7b29c4760"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Conferences" sheetId="1" r:id="Rab47c390448d4560"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Vocabulary" sheetId="2" r:id="Rd5189bbfb6f64c39"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,6 +14,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="0.0%"/>
+  </x:numFmts>
   <x:fonts count="2">
     <x:font>
       <x:sz val="11"/>
@@ -46,7 +49,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="16">
+  <x:cellXfs count="17">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -83,6 +86,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -91,16 +95,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="CoreConferencesTable" displayName="CoreConferencesTable" ref="A1:H62" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="8">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="CoreConferencesTable" displayName="CoreConferencesTable" ref="A1:N62" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="14">
     <x:tableColumn id="1" name="Conference"/>
     <x:tableColumn id="2" name="TAGS"/>
     <x:tableColumn id="3" name="SIZE"/>
-    <x:tableColumn id="4" name="Acceptance difficulty"/>
+    <x:tableColumn id="4" name="Acceptance band"/>
     <x:tableColumn id="5" name="ICORE 2026"/>
     <x:tableColumn id="6" name="Submission type"/>
     <x:tableColumn id="7" name="Source"/>
     <x:tableColumn id="8" name="ICORE source"/>
+    <x:tableColumn id="9" name="CCF 2026"/>
+    <x:tableColumn id="10" name="CCF source"/>
+    <x:tableColumn id="11" name="Historical acceptance"/>
+    <x:tableColumn id="12" name="Edition"/>
+    <x:tableColumn id="13" name="Track"/>
+    <x:tableColumn id="14" name="Acceptance source"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -268,11 +278,17 @@
     <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="56" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="10" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="19" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="31" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="52" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="52" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="15" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="52" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="23" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="13" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="26" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="52" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -286,7 +302,7 @@
         <x:v>SIZE</x:v>
       </x:c>
       <x:c r="D1" s="6" t="str">
-        <x:v>Acceptance difficulty</x:v>
+        <x:v>Acceptance band</x:v>
       </x:c>
       <x:c r="E1" s="6" t="str">
         <x:v>ICORE 2026</x:v>
@@ -299,6 +315,24 @@
       </x:c>
       <x:c r="H1" t="str">
         <x:v>ICORE source</x:v>
+      </x:c>
+      <x:c r="I1" t="str">
+        <x:v>CCF 2026</x:v>
+      </x:c>
+      <x:c r="J1" t="str">
+        <x:v>CCF source</x:v>
+      </x:c>
+      <x:c r="K1" t="str">
+        <x:v>Historical acceptance</x:v>
+      </x:c>
+      <x:c r="L1" t="str">
+        <x:v>Edition</x:v>
+      </x:c>
+      <x:c r="M1" t="str">
+        <x:v>Track</x:v>
+      </x:c>
+      <x:c r="N1" t="str">
+        <x:v>Acceptance source</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -312,7 +346,7 @@
         <x:v>XXL</x:v>
       </x:c>
       <x:c r="D2" s="14" t="str">
-        <x:v>Very hard</x:v>
+        <x:v>Low</x:v>
       </x:c>
       <x:c r="E2" s="14" t="str">
         <x:v>A*</x:v>
@@ -325,6 +359,24 @@
       </x:c>
       <x:c r="H2" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/98/</x:v>
+      </x:c>
+      <x:c r="I2" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="J2" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=57</x:v>
+      </x:c>
+      <x:c r="K2" s="16" t="n">
+        <x:v>0.2452</x:v>
+      </x:c>
+      <x:c r="L2" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="M2" t="str">
+        <x:v>Main track</x:v>
+      </x:c>
+      <x:c r="N2" t="str">
+        <x:v>https://blog.neurips.cc/2025/09/30/</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -338,7 +390,7 @@
         <x:v>XXL</x:v>
       </x:c>
       <x:c r="D3" s="14" t="str">
-        <x:v>Very hard</x:v>
+        <x:v>Low</x:v>
       </x:c>
       <x:c r="E3" s="14" t="str">
         <x:v>A*</x:v>
@@ -351,6 +403,24 @@
       </x:c>
       <x:c r="H3" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/1121/</x:v>
+      </x:c>
+      <x:c r="I3" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="J3" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=57</x:v>
+      </x:c>
+      <x:c r="K3" s="16" t="n">
+        <x:v>0.27</x:v>
+      </x:c>
+      <x:c r="L3" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="M3" t="str">
+        <x:v>Main track</x:v>
+      </x:c>
+      <x:c r="N3" t="str">
+        <x:v>https://media.icml.cc/Conferences/ICML2025/ICML2025_Fact_Sheet.pdf</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -364,7 +434,7 @@
         <x:v>XXL</x:v>
       </x:c>
       <x:c r="D4" s="14" t="str">
-        <x:v>Hard</x:v>
+        <x:v>Low</x:v>
       </x:c>
       <x:c r="E4" s="14" t="str">
         <x:v>A*</x:v>
@@ -377,6 +447,24 @@
       </x:c>
       <x:c r="H4" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/2273/</x:v>
+      </x:c>
+      <x:c r="I4" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="J4" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=57</x:v>
+      </x:c>
+      <x:c r="K4" s="16" t="n">
+        <x:v>0.27399999999999997</x:v>
+      </x:c>
+      <x:c r="L4" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="M4" t="str">
+        <x:v>Main conference; accepted / valid submissions</x:v>
+      </x:c>
+      <x:c r="N4" t="str">
+        <x:v>https://blog.iclr.cc/2026/</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -390,7 +478,7 @@
         <x:v>L</x:v>
       </x:c>
       <x:c r="D5" s="14" t="str">
-        <x:v>Hard</x:v>
+        <x:v>Low</x:v>
       </x:c>
       <x:c r="E5" s="14" t="str">
         <x:v>A</x:v>
@@ -403,6 +491,24 @@
       </x:c>
       <x:c r="H5" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/913/</x:v>
+      </x:c>
+      <x:c r="I5" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="J5" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=59</x:v>
+      </x:c>
+      <x:c r="K5" s="16" t="n">
+        <x:v>0.281</x:v>
+      </x:c>
+      <x:c r="L5" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="M5" t="str">
+        <x:v>Main conference (590 accepted of 2,102 submitted)</x:v>
+      </x:c>
+      <x:c r="N5" t="str">
+        <x:v>https://www.linkedin.com/posts/asolin_aistats2026-tangier-morocco-activity-7424831733768044544-DjfS</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -416,7 +522,7 @@
         <x:v>M/L</x:v>
       </x:c>
       <x:c r="D6" s="14" t="str">
-        <x:v>Hard</x:v>
+        <x:v>Unknown</x:v>
       </x:c>
       <x:c r="E6" s="14" t="str">
         <x:v>A</x:v>
@@ -430,6 +536,16 @@
       <x:c r="H6" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/346/</x:v>
       </x:c>
+      <x:c r="I6" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J6" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=58</x:v>
+      </x:c>
+      <x:c r="K6" s="16" t="str"/>
+      <x:c r="L6" t="str"/>
+      <x:c r="M6" t="str"/>
+      <x:c r="N6" t="str"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="14" t="str">
@@ -442,7 +558,7 @@
         <x:v>M</x:v>
       </x:c>
       <x:c r="D7" s="14" t="str">
-        <x:v>Very hard</x:v>
+        <x:v>Unknown</x:v>
       </x:c>
       <x:c r="E7" s="14" t="str">
         <x:v>A*</x:v>
@@ -456,6 +572,16 @@
       <x:c r="H7" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/124/</x:v>
       </x:c>
+      <x:c r="I7" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J7" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=58</x:v>
+      </x:c>
+      <x:c r="K7" s="16" t="str"/>
+      <x:c r="L7" t="str"/>
+      <x:c r="M7" t="str"/>
+      <x:c r="N7" t="str"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="14" t="str">
@@ -468,7 +594,7 @@
         <x:v>L</x:v>
       </x:c>
       <x:c r="D8" s="14" t="str">
-        <x:v>Hard</x:v>
+        <x:v>Unknown</x:v>
       </x:c>
       <x:c r="E8" s="14" t="str">
         <x:v>A</x:v>
@@ -482,6 +608,16 @@
       <x:c r="H8" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/491/</x:v>
       </x:c>
+      <x:c r="I8" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J8" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=36</x:v>
+      </x:c>
+      <x:c r="K8" s="16" t="str"/>
+      <x:c r="L8" t="str"/>
+      <x:c r="M8" t="str"/>
+      <x:c r="N8" t="str"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="14" t="str">
@@ -494,7 +630,7 @@
         <x:v>XL</x:v>
       </x:c>
       <x:c r="D9" s="14" t="str">
-        <x:v>Very hard</x:v>
+        <x:v>Very low</x:v>
       </x:c>
       <x:c r="E9" s="14" t="str">
         <x:v>A*</x:v>
@@ -507,6 +643,24 @@
       </x:c>
       <x:c r="H9" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/26/</x:v>
+      </x:c>
+      <x:c r="I9" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="J9" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=35</x:v>
+      </x:c>
+      <x:c r="K9" s="16" t="n">
+        <x:v>0.19</x:v>
+      </x:c>
+      <x:c r="L9" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="M9" t="str">
+        <x:v>Research track, August cycle</x:v>
+      </x:c>
+      <x:c r="N9" t="str">
+        <x:v>https://kdd.org/kdd2025/frequently-asked-questions/</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -520,7 +674,7 @@
         <x:v>M/L</x:v>
       </x:c>
       <x:c r="D10" s="14" t="str">
-        <x:v>Hard</x:v>
+        <x:v>Unknown</x:v>
       </x:c>
       <x:c r="E10" s="14" t="str">
         <x:v>A*</x:v>
@@ -534,6 +688,16 @@
       <x:c r="H10" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/642/</x:v>
       </x:c>
+      <x:c r="I10" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J10" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=36</x:v>
+      </x:c>
+      <x:c r="K10" s="16" t="str"/>
+      <x:c r="L10" t="str"/>
+      <x:c r="M10" t="str"/>
+      <x:c r="N10" t="str"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="14" t="str">
@@ -546,7 +710,7 @@
         <x:v>M</x:v>
       </x:c>
       <x:c r="D11" s="14" t="str">
-        <x:v>Hard</x:v>
+        <x:v>Unknown</x:v>
       </x:c>
       <x:c r="E11" s="14" t="str">
         <x:v>A</x:v>
@@ -560,6 +724,16 @@
       <x:c r="H11" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/1727/</x:v>
       </x:c>
+      <x:c r="I11" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J11" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=36</x:v>
+      </x:c>
+      <x:c r="K11" s="16" t="str"/>
+      <x:c r="L11" t="str"/>
+      <x:c r="M11" t="str"/>
+      <x:c r="N11" t="str"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="14" t="str">
@@ -572,7 +746,7 @@
         <x:v>M</x:v>
       </x:c>
       <x:c r="D12" s="14" t="str">
-        <x:v>Moderate-hard</x:v>
+        <x:v>Unknown</x:v>
       </x:c>
       <x:c r="E12" s="14" t="str">
         <x:v>B</x:v>
@@ -586,6 +760,16 @@
       <x:c r="H12" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/2237/</x:v>
       </x:c>
+      <x:c r="I12" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="J12" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=43</x:v>
+      </x:c>
+      <x:c r="K12" s="16" t="str"/>
+      <x:c r="L12" t="str"/>
+      <x:c r="M12" t="str"/>
+      <x:c r="N12" t="str"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="14" t="str">
@@ -598,16 +782,22 @@
         <x:v>M</x:v>
       </x:c>
       <x:c r="D13" s="14" t="str">
-        <x:v>Hard</x:v>
-      </x:c>
-      <x:c r="E13" s="14" t="str"/>
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E13" s="14"/>
       <x:c r="F13" s="14" t="str">
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G13" t="str">
         <x:v>https://mlhc.org/</x:v>
       </x:c>
-      <x:c r="H13" t="str"/>
+      <x:c r="H13"/>
+      <x:c r="I13" t="str"/>
+      <x:c r="J13" t="str"/>
+      <x:c r="K13" s="16" t="str"/>
+      <x:c r="L13" t="str"/>
+      <x:c r="M13" t="str"/>
+      <x:c r="N13" t="str"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="14" t="str">
@@ -620,16 +810,22 @@
         <x:v>M</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
-        <x:v>Hard</x:v>
-      </x:c>
-      <x:c r="E14" s="14" t="str"/>
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E14" s="14"/>
       <x:c r="F14" s="14" t="str">
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G14" t="str">
         <x:v>https://chil.ahli.cc/</x:v>
       </x:c>
-      <x:c r="H14" t="str"/>
+      <x:c r="H14"/>
+      <x:c r="I14" t="str"/>
+      <x:c r="J14" t="str"/>
+      <x:c r="K14" s="16" t="str"/>
+      <x:c r="L14" t="str"/>
+      <x:c r="M14" t="str"/>
+      <x:c r="N14" t="str"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="14" t="str">
@@ -642,16 +838,22 @@
         <x:v>M</x:v>
       </x:c>
       <x:c r="D15" s="14" t="str">
-        <x:v>Moderate-hard</x:v>
-      </x:c>
-      <x:c r="E15" s="14" t="str"/>
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E15" s="14"/>
       <x:c r="F15" s="14" t="str">
         <x:v>Proceedings + findings tracks</x:v>
       </x:c>
       <x:c r="G15" t="str">
         <x:v>https://ml4h.ahli.cc/</x:v>
       </x:c>
-      <x:c r="H15" t="str"/>
+      <x:c r="H15"/>
+      <x:c r="I15" t="str"/>
+      <x:c r="J15" t="str"/>
+      <x:c r="K15" s="16" t="str"/>
+      <x:c r="L15" t="str"/>
+      <x:c r="M15" t="str"/>
+      <x:c r="N15" t="str"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="14" t="str">
@@ -664,16 +866,22 @@
         <x:v>S</x:v>
       </x:c>
       <x:c r="D16" s="14" t="str">
-        <x:v>Moderate-hard</x:v>
-      </x:c>
-      <x:c r="E16" s="14" t="str"/>
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E16" s="14"/>
       <x:c r="F16" s="14" t="str">
         <x:v>Workshop / paper-based</x:v>
       </x:c>
       <x:c r="G16" t="str">
         <x:v>https://timeseries4health.github.io/</x:v>
       </x:c>
-      <x:c r="H16" t="str"/>
+      <x:c r="H16"/>
+      <x:c r="I16" t="str"/>
+      <x:c r="J16" t="str"/>
+      <x:c r="K16" s="16" t="str"/>
+      <x:c r="L16" t="str"/>
+      <x:c r="M16" t="str"/>
+      <x:c r="N16" t="str"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="14" t="str">
@@ -686,7 +894,7 @@
         <x:v>XL</x:v>
       </x:c>
       <x:c r="D17" s="14" t="str">
-        <x:v>Hard</x:v>
+        <x:v>Low</x:v>
       </x:c>
       <x:c r="E17" s="14" t="str">
         <x:v>A</x:v>
@@ -699,6 +907,24 @@
       </x:c>
       <x:c r="H17" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/1607/</x:v>
+      </x:c>
+      <x:c r="I17" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J17" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=71</x:v>
+      </x:c>
+      <x:c r="K17" s="16" t="n">
+        <x:v>0.29</x:v>
+      </x:c>
+      <x:c r="L17" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="M17" t="str">
+        <x:v>Main conference papers</x:v>
+      </x:c>
+      <x:c r="N17" t="str">
+        <x:v>https://miccai.org/2025/06/20/miccai-quarterly-summer-june-2025/</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -712,16 +938,22 @@
         <x:v>M</x:v>
       </x:c>
       <x:c r="D18" s="14" t="str">
-        <x:v>Moderate-hard</x:v>
-      </x:c>
-      <x:c r="E18" s="14" t="str"/>
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E18" s="14"/>
       <x:c r="F18" s="14" t="str">
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G18" t="str">
         <x:v>https://2026.midl.io/</x:v>
       </x:c>
-      <x:c r="H18" t="str"/>
+      <x:c r="H18"/>
+      <x:c r="I18" t="str"/>
+      <x:c r="J18" t="str"/>
+      <x:c r="K18" s="16" t="str"/>
+      <x:c r="L18" t="str"/>
+      <x:c r="M18" t="str"/>
+      <x:c r="N18" t="str"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="14" t="str">
@@ -734,16 +966,22 @@
         <x:v>L</x:v>
       </x:c>
       <x:c r="D19" s="14" t="str">
-        <x:v>Moderate-hard</x:v>
-      </x:c>
-      <x:c r="E19" s="14" t="str"/>
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E19" s="14"/>
       <x:c r="F19" s="14" t="str">
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G19" t="str">
         <x:v>https://biomedicalimaging.org/2027/</x:v>
       </x:c>
-      <x:c r="H19" t="str"/>
+      <x:c r="H19"/>
+      <x:c r="I19" t="str"/>
+      <x:c r="J19" t="str"/>
+      <x:c r="K19" s="16" t="str"/>
+      <x:c r="L19" t="str"/>
+      <x:c r="M19" t="str"/>
+      <x:c r="N19" t="str"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="14" t="str">
@@ -756,16 +994,22 @@
         <x:v>M</x:v>
       </x:c>
       <x:c r="D20" s="14" t="str">
-        <x:v>Moderate-hard</x:v>
-      </x:c>
-      <x:c r="E20" s="14" t="str"/>
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E20" s="14"/>
       <x:c r="F20" s="14" t="str">
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G20" t="str">
         <x:v>https://bhi.embs.org/2026/</x:v>
       </x:c>
-      <x:c r="H20" t="str"/>
+      <x:c r="H20"/>
+      <x:c r="I20" t="str"/>
+      <x:c r="J20" t="str"/>
+      <x:c r="K20" s="16" t="str"/>
+      <x:c r="L20" t="str"/>
+      <x:c r="M20" t="str"/>
+      <x:c r="N20" t="str"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="14" t="str">
@@ -778,16 +1022,22 @@
         <x:v>XL</x:v>
       </x:c>
       <x:c r="D21" s="14" t="str">
-        <x:v>Moderate</x:v>
-      </x:c>
-      <x:c r="E21" s="14" t="str"/>
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E21" s="14"/>
       <x:c r="F21" s="14" t="str">
         <x:v>Paper-based / broad applied venue</x:v>
       </x:c>
       <x:c r="G21" t="str">
         <x:v>https://embc.embs.org/2026/</x:v>
       </x:c>
-      <x:c r="H21" t="str"/>
+      <x:c r="H21"/>
+      <x:c r="I21" t="str"/>
+      <x:c r="J21" t="str"/>
+      <x:c r="K21" s="16" t="str"/>
+      <x:c r="L21" t="str"/>
+      <x:c r="M21" t="str"/>
+      <x:c r="N21" t="str"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="14" t="str">
@@ -800,16 +1050,34 @@
         <x:v>XL</x:v>
       </x:c>
       <x:c r="D22" s="14" t="str">
-        <x:v>Moderate-hard</x:v>
-      </x:c>
-      <x:c r="E22" s="14" t="str"/>
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E22" s="14"/>
       <x:c r="F22" s="14" t="str">
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G22" t="str">
         <x:v>https://2027.ieeeicassp.org/</x:v>
       </x:c>
-      <x:c r="H22" t="str"/>
+      <x:c r="H22"/>
+      <x:c r="I22" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J22" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=48</x:v>
+      </x:c>
+      <x:c r="K22" s="16" t="n">
+        <x:v>0.429</x:v>
+      </x:c>
+      <x:c r="L22" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="M22" t="str">
+        <x:v>Regular papers overall (nearly 11,200 submitted; close to 4,800 accepted)</x:v>
+      </x:c>
+      <x:c r="N22" t="str">
+        <x:v>https://signalprocessingsociety.org/index.php/newsletter/2026/06/meet-icassp-2026-organizers-ana-isabel-perez-neira-and-xavier-mestre</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="14" t="str">
@@ -822,16 +1090,22 @@
         <x:v>S/M</x:v>
       </x:c>
       <x:c r="D23" s="14" t="str">
-        <x:v>Moderate-hard</x:v>
-      </x:c>
-      <x:c r="E23" s="14" t="str"/>
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E23" s="14"/>
       <x:c r="F23" s="14" t="str">
         <x:v>Paper-based / workshop-style conference</x:v>
       </x:c>
       <x:c r="G23" t="str">
         <x:v>https://mlsp26.ieeesps.org/</x:v>
       </x:c>
-      <x:c r="H23" t="str"/>
+      <x:c r="H23"/>
+      <x:c r="I23" t="str"/>
+      <x:c r="J23" t="str"/>
+      <x:c r="K23" s="16" t="str"/>
+      <x:c r="L23" t="str"/>
+      <x:c r="M23" t="str"/>
+      <x:c r="N23" t="str"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="14" t="str">
@@ -844,16 +1118,22 @@
         <x:v>L</x:v>
       </x:c>
       <x:c r="D24" s="14" t="str">
-        <x:v>Hard</x:v>
-      </x:c>
-      <x:c r="E24" s="14" t="str"/>
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E24" s="14"/>
       <x:c r="F24" s="14" t="str">
         <x:v>Abstract-based / talks highly selective</x:v>
       </x:c>
       <x:c r="G24" t="str">
         <x:v>https://www.cosyne.org/cosyne-home</x:v>
       </x:c>
-      <x:c r="H24" t="str"/>
+      <x:c r="H24"/>
+      <x:c r="I24" t="str"/>
+      <x:c r="J24" t="str"/>
+      <x:c r="K24" s="16" t="str"/>
+      <x:c r="L24" t="str"/>
+      <x:c r="M24" t="str"/>
+      <x:c r="N24" t="str"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="14" t="str">
@@ -866,16 +1146,22 @@
         <x:v>M</x:v>
       </x:c>
       <x:c r="D25" s="14" t="str">
-        <x:v>Moderate-hard</x:v>
-      </x:c>
-      <x:c r="E25" s="14" t="str"/>
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E25" s="14"/>
       <x:c r="F25" s="14" t="str">
         <x:v>Mixed: proceedings + extended abstracts</x:v>
       </x:c>
       <x:c r="G25" t="str">
         <x:v>https://2026.ccneuro.org/</x:v>
       </x:c>
-      <x:c r="H25" t="str"/>
+      <x:c r="H25"/>
+      <x:c r="I25" t="str"/>
+      <x:c r="J25" t="str"/>
+      <x:c r="K25" s="16" t="str"/>
+      <x:c r="L25" t="str"/>
+      <x:c r="M25" t="str"/>
+      <x:c r="N25" t="str"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="14" t="str">
@@ -888,16 +1174,22 @@
         <x:v>M</x:v>
       </x:c>
       <x:c r="D26" s="14" t="str">
-        <x:v>Moderate</x:v>
-      </x:c>
-      <x:c r="E26" s="14" t="str"/>
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E26" s="14"/>
       <x:c r="F26" s="14" t="str">
         <x:v>Abstract-based / talks selective</x:v>
       </x:c>
       <x:c r="G26" t="str">
         <x:v>https://bernstein-network.de/en/bernstein-conference/</x:v>
       </x:c>
-      <x:c r="H26" t="str"/>
+      <x:c r="H26"/>
+      <x:c r="I26" t="str"/>
+      <x:c r="J26" t="str"/>
+      <x:c r="K26" s="16" t="str"/>
+      <x:c r="L26" t="str"/>
+      <x:c r="M26" t="str"/>
+      <x:c r="N26" t="str"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="14" t="str">
@@ -910,16 +1202,22 @@
         <x:v>M</x:v>
       </x:c>
       <x:c r="D27" s="14" t="str">
-        <x:v>Moderate</x:v>
-      </x:c>
-      <x:c r="E27" s="14" t="str"/>
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E27" s="14"/>
       <x:c r="F27" s="14" t="str">
         <x:v>Abstract-based</x:v>
       </x:c>
       <x:c r="G27" t="str">
         <x:v>https://www.cnsorg.org/cns-2026</x:v>
       </x:c>
-      <x:c r="H27" t="str"/>
+      <x:c r="H27"/>
+      <x:c r="I27" t="str"/>
+      <x:c r="J27" t="str"/>
+      <x:c r="K27" s="16" t="str"/>
+      <x:c r="L27" t="str"/>
+      <x:c r="M27" t="str"/>
+      <x:c r="N27" t="str"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="14" t="str">
@@ -932,16 +1230,22 @@
         <x:v>L/XL</x:v>
       </x:c>
       <x:c r="D28" s="14" t="str">
-        <x:v>Moderate</x:v>
-      </x:c>
-      <x:c r="E28" s="14" t="str"/>
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E28" s="14"/>
       <x:c r="F28" s="14" t="str">
         <x:v>Abstract-based / talks selective</x:v>
       </x:c>
       <x:c r="G28" t="str">
         <x:v>https://humanbrainmapping.org/ohbm-2027/</x:v>
       </x:c>
-      <x:c r="H28" t="str"/>
+      <x:c r="H28"/>
+      <x:c r="I28" t="str"/>
+      <x:c r="J28" t="str"/>
+      <x:c r="K28" s="16" t="str"/>
+      <x:c r="L28" t="str"/>
+      <x:c r="M28" t="str"/>
+      <x:c r="N28" t="str"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="14" t="str">
@@ -954,16 +1258,22 @@
         <x:v>M</x:v>
       </x:c>
       <x:c r="D29" s="14" t="str">
-        <x:v>Moderate-hard</x:v>
-      </x:c>
-      <x:c r="E29" s="14" t="str"/>
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E29" s="14"/>
       <x:c r="F29" s="14" t="str">
         <x:v>Paper-based / engineering-focused</x:v>
       </x:c>
       <x:c r="G29" t="str">
         <x:v>https://ieee-ner.org/</x:v>
       </x:c>
-      <x:c r="H29" t="str"/>
+      <x:c r="H29"/>
+      <x:c r="I29" t="str"/>
+      <x:c r="J29" t="str"/>
+      <x:c r="K29" s="16" t="str"/>
+      <x:c r="L29" t="str"/>
+      <x:c r="M29" t="str"/>
+      <x:c r="N29" t="str"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="14" t="str">
@@ -976,16 +1286,22 @@
         <x:v>S/M</x:v>
       </x:c>
       <x:c r="D30" s="14" t="str">
-        <x:v>Moderate</x:v>
-      </x:c>
-      <x:c r="E30" s="14" t="str"/>
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E30" s="14"/>
       <x:c r="F30" s="14" t="str">
         <x:v>Abstract/community-based</x:v>
       </x:c>
       <x:c r="G30" t="str">
         <x:v>https://bcisociety.org/bci-meeting/</x:v>
       </x:c>
-      <x:c r="H30" t="str"/>
+      <x:c r="H30"/>
+      <x:c r="I30" t="str"/>
+      <x:c r="J30" t="str"/>
+      <x:c r="K30" s="16" t="str"/>
+      <x:c r="L30" t="str"/>
+      <x:c r="M30" t="str"/>
+      <x:c r="N30" t="str"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="14" t="str">
@@ -998,16 +1314,22 @@
         <x:v>M</x:v>
       </x:c>
       <x:c r="D31" s="14" t="str">
-        <x:v>Moderate</x:v>
-      </x:c>
-      <x:c r="E31" s="14" t="str"/>
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E31" s="14"/>
       <x:c r="F31" s="14" t="str">
         <x:v>Abstract-based / specialist venue</x:v>
       </x:c>
       <x:c r="G31" t="str">
         <x:v>https://mm.scimeeting.cn/en/web/index/31426</x:v>
       </x:c>
-      <x:c r="H31" t="str"/>
+      <x:c r="H31"/>
+      <x:c r="I31" t="str"/>
+      <x:c r="J31" t="str"/>
+      <x:c r="K31" s="16" t="str"/>
+      <x:c r="L31" t="str"/>
+      <x:c r="M31" t="str"/>
+      <x:c r="N31" t="str"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="14" t="str">
@@ -1020,16 +1342,22 @@
         <x:v>M</x:v>
       </x:c>
       <x:c r="D32" s="14" t="str">
-        <x:v>Hard</x:v>
-      </x:c>
-      <x:c r="E32" s="14" t="str"/>
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E32" s="14"/>
       <x:c r="F32" s="14" t="str">
         <x:v>Paper-based / interdisciplinary</x:v>
       </x:c>
       <x:c r="G32" t="str">
         <x:v>https://facctconference.org/</x:v>
       </x:c>
-      <x:c r="H32" t="str"/>
+      <x:c r="H32"/>
+      <x:c r="I32" t="str"/>
+      <x:c r="J32" t="str"/>
+      <x:c r="K32" s="16" t="str"/>
+      <x:c r="L32" t="str"/>
+      <x:c r="M32" t="str"/>
+      <x:c r="N32" t="str"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="14" t="str">
@@ -1042,7 +1370,7 @@
         <x:v>S/M</x:v>
       </x:c>
       <x:c r="D33" s="14" t="str">
-        <x:v>Moderate-hard</x:v>
+        <x:v>Moderate</x:v>
       </x:c>
       <x:c r="E33" s="14" t="str">
         <x:v>C</x:v>
@@ -1055,6 +1383,20 @@
       </x:c>
       <x:c r="H33" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/2354/</x:v>
+      </x:c>
+      <x:c r="I33" t="str"/>
+      <x:c r="J33" t="str"/>
+      <x:c r="K33" s="16" t="n">
+        <x:v>0.318</x:v>
+      </x:c>
+      <x:c r="L33" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="M33" t="str">
+        <x:v>Main papers (238 accepted of 748 reviewed)</x:v>
+      </x:c>
+      <x:c r="N33" t="str">
+        <x:v>https://aaai.org/wp-content/uploads/2025/10/AIES-2025-Program-10.14.pdf</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -1068,7 +1410,7 @@
         <x:v>XL</x:v>
       </x:c>
       <x:c r="D34" s="14" t="str">
-        <x:v>Hard</x:v>
+        <x:v>Low</x:v>
       </x:c>
       <x:c r="E34" s="14" t="str">
         <x:v>A*</x:v>
@@ -1081,6 +1423,24 @@
       </x:c>
       <x:c r="H34" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/1053/</x:v>
+      </x:c>
+      <x:c r="I34" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="J34" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=64</x:v>
+      </x:c>
+      <x:c r="K34" s="16" t="n">
+        <x:v>0.249</x:v>
+      </x:c>
+      <x:c r="L34" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="M34" t="str">
+        <x:v>Papers track</x:v>
+      </x:c>
+      <x:c r="N34" t="str">
+        <x:v>https://chi2025.acm.org/chi-2025-papers-track-post-pc-outcomes-report/</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -1094,7 +1454,7 @@
         <x:v>XXL</x:v>
       </x:c>
       <x:c r="D35" t="str">
-        <x:v>Very hard</x:v>
+        <x:v>Very low</x:v>
       </x:c>
       <x:c r="E35" t="str">
         <x:v>A*</x:v>
@@ -1107,6 +1467,24 @@
       </x:c>
       <x:c r="H35" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/1629/</x:v>
+      </x:c>
+      <x:c r="I35" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="J35" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=57</x:v>
+      </x:c>
+      <x:c r="K35" s="16" t="n">
+        <x:v>0.175</x:v>
+      </x:c>
+      <x:c r="L35" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="M35" t="str">
+        <x:v>Main technical track</x:v>
+      </x:c>
+      <x:c r="N35" t="str">
+        <x:v>https://aaai.org/wp-content/uploads/2026/01/AAAI-26-Opening-Ceremony.pdf</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1120,16 +1498,22 @@
         <x:v>XL</x:v>
       </x:c>
       <x:c r="D36" s="12" t="str">
-        <x:v>Very hard</x:v>
-      </x:c>
-      <x:c r="E36" s="12" t="str"/>
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E36" s="12"/>
       <x:c r="F36" s="12" t="str">
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G36" t="str">
         <x:v>https://2026.ijcai.org/</x:v>
       </x:c>
-      <x:c r="H36" t="str"/>
+      <x:c r="H36"/>
+      <x:c r="I36" t="str"/>
+      <x:c r="J36" t="str"/>
+      <x:c r="K36" s="16" t="str"/>
+      <x:c r="L36" t="str"/>
+      <x:c r="M36" t="str"/>
+      <x:c r="N36" t="str"/>
     </x:row>
     <x:row r="37" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A37" s="12" t="str">
@@ -1142,7 +1526,7 @@
         <x:v>L</x:v>
       </x:c>
       <x:c r="D37" s="12" t="str">
-        <x:v>Hard</x:v>
+        <x:v>Unknown</x:v>
       </x:c>
       <x:c r="E37" s="12" t="str">
         <x:v>C</x:v>
@@ -1156,6 +1540,16 @@
       <x:c r="H37" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/2174/</x:v>
       </x:c>
+      <x:c r="I37" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="J37" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=59</x:v>
+      </x:c>
+      <x:c r="K37" s="16" t="str"/>
+      <x:c r="L37" t="str"/>
+      <x:c r="M37" t="str"/>
+      <x:c r="N37" t="str"/>
     </x:row>
     <x:row r="38" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A38" s="12" t="str">
@@ -1168,7 +1562,7 @@
         <x:v>L</x:v>
       </x:c>
       <x:c r="D38" s="12" t="str">
-        <x:v>Hard</x:v>
+        <x:v>Unknown</x:v>
       </x:c>
       <x:c r="E38" s="12" t="str">
         <x:v>B</x:v>
@@ -1182,6 +1576,16 @@
       <x:c r="H38" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/1667/</x:v>
       </x:c>
+      <x:c r="I38" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="J38" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=37</x:v>
+      </x:c>
+      <x:c r="K38" s="16" t="str"/>
+      <x:c r="L38" t="str"/>
+      <x:c r="M38" t="str"/>
+      <x:c r="N38" t="str"/>
     </x:row>
     <x:row r="39" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A39" s="12" t="str">
@@ -1194,7 +1598,7 @@
         <x:v>XL</x:v>
       </x:c>
       <x:c r="D39" s="12" t="str">
-        <x:v>Very hard</x:v>
+        <x:v>Unknown</x:v>
       </x:c>
       <x:c r="E39" s="12" t="str">
         <x:v>A</x:v>
@@ -1208,6 +1612,16 @@
       <x:c r="H39" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/25/</x:v>
       </x:c>
+      <x:c r="I39" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J39" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=36</x:v>
+      </x:c>
+      <x:c r="K39" s="16" t="str"/>
+      <x:c r="L39" t="str"/>
+      <x:c r="M39" t="str"/>
+      <x:c r="N39" t="str"/>
     </x:row>
     <x:row r="40" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A40" s="12" t="str">
@@ -1220,7 +1634,7 @@
         <x:v>L</x:v>
       </x:c>
       <x:c r="D40" s="12" t="str">
-        <x:v>Very hard</x:v>
+        <x:v>Unknown</x:v>
       </x:c>
       <x:c r="E40" s="12" t="str">
         <x:v>A</x:v>
@@ -1234,6 +1648,16 @@
       <x:c r="H40" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/31/</x:v>
       </x:c>
+      <x:c r="I40" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J40" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=36</x:v>
+      </x:c>
+      <x:c r="K40" s="16" t="str"/>
+      <x:c r="L40" t="str"/>
+      <x:c r="M40" t="str"/>
+      <x:c r="N40" t="str"/>
     </x:row>
     <x:row r="41" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A41" s="12" t="str">
@@ -1246,7 +1670,7 @@
         <x:v>L</x:v>
       </x:c>
       <x:c r="D41" s="12" t="str">
-        <x:v>Moderate-hard</x:v>
+        <x:v>Unknown</x:v>
       </x:c>
       <x:c r="E41" s="12" t="str">
         <x:v>B</x:v>
@@ -1260,6 +1684,12 @@
       <x:c r="H41" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/2274/</x:v>
       </x:c>
+      <x:c r="I41" t="str"/>
+      <x:c r="J41" t="str"/>
+      <x:c r="K41" s="16" t="str"/>
+      <x:c r="L41" t="str"/>
+      <x:c r="M41" t="str"/>
+      <x:c r="N41" t="str"/>
     </x:row>
     <x:row r="42" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A42" s="12" t="str">
@@ -1272,7 +1702,7 @@
         <x:v>M</x:v>
       </x:c>
       <x:c r="D42" s="12" t="str">
-        <x:v>Hard</x:v>
+        <x:v>Unknown</x:v>
       </x:c>
       <x:c r="E42" s="12" t="str">
         <x:v>B</x:v>
@@ -1286,6 +1716,12 @@
       <x:c r="H42" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/2191/</x:v>
       </x:c>
+      <x:c r="I42" t="str"/>
+      <x:c r="J42" t="str"/>
+      <x:c r="K42" s="16" t="str"/>
+      <x:c r="L42" t="str"/>
+      <x:c r="M42" t="str"/>
+      <x:c r="N42" t="str"/>
     </x:row>
     <x:row r="43" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A43" s="12" t="str">
@@ -1298,7 +1734,7 @@
         <x:v>M</x:v>
       </x:c>
       <x:c r="D43" s="12" t="str">
-        <x:v>Moderate-hard</x:v>
+        <x:v>Unknown</x:v>
       </x:c>
       <x:c r="E43" s="12" t="str">
         <x:v>B</x:v>
@@ -1312,6 +1748,16 @@
       <x:c r="H43" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/845/</x:v>
       </x:c>
+      <x:c r="I43" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="J43" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=55</x:v>
+      </x:c>
+      <x:c r="K43" s="16" t="str"/>
+      <x:c r="L43" t="str"/>
+      <x:c r="M43" t="str"/>
+      <x:c r="N43" t="str"/>
     </x:row>
     <x:row r="44" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A44" s="12" t="str">
@@ -1324,7 +1770,7 @@
         <x:v>M</x:v>
       </x:c>
       <x:c r="D44" s="12" t="str">
-        <x:v>Moderate-hard</x:v>
+        <x:v>Unknown</x:v>
       </x:c>
       <x:c r="E44" s="12" t="str">
         <x:v>C</x:v>
@@ -1338,6 +1784,16 @@
       <x:c r="H44" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/888/</x:v>
       </x:c>
+      <x:c r="I44" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="J44" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=37</x:v>
+      </x:c>
+      <x:c r="K44" s="16" t="str"/>
+      <x:c r="L44" t="str"/>
+      <x:c r="M44" t="str"/>
+      <x:c r="N44" t="str"/>
     </x:row>
     <x:row r="45" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A45" s="12" t="str">
@@ -1350,7 +1806,7 @@
         <x:v>XL</x:v>
       </x:c>
       <x:c r="D45" s="12" t="str">
-        <x:v>Moderate-hard</x:v>
+        <x:v>Unknown</x:v>
       </x:c>
       <x:c r="E45" s="12" t="str">
         <x:v>B</x:v>
@@ -1364,6 +1820,16 @@
       <x:c r="H45" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/685/</x:v>
       </x:c>
+      <x:c r="I45" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="J45" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=60</x:v>
+      </x:c>
+      <x:c r="K45" s="16" t="str"/>
+      <x:c r="L45" t="str"/>
+      <x:c r="M45" t="str"/>
+      <x:c r="N45" t="str"/>
     </x:row>
     <x:row r="46" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A46" s="12" t="str">
@@ -1376,7 +1842,7 @@
         <x:v>L</x:v>
       </x:c>
       <x:c r="D46" s="12" t="str">
-        <x:v>Moderate-hard</x:v>
+        <x:v>Unknown</x:v>
       </x:c>
       <x:c r="E46" s="12" t="str">
         <x:v>C</x:v>
@@ -1390,6 +1856,16 @@
       <x:c r="H46" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/915/</x:v>
       </x:c>
+      <x:c r="I46" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="J46" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=59</x:v>
+      </x:c>
+      <x:c r="K46" s="16" t="str"/>
+      <x:c r="L46" t="str"/>
+      <x:c r="M46" t="str"/>
+      <x:c r="N46" t="str"/>
     </x:row>
     <x:row r="47" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A47" s="12" t="str">
@@ -1402,7 +1878,7 @@
         <x:v>M</x:v>
       </x:c>
       <x:c r="D47" s="12" t="str">
-        <x:v>Hard</x:v>
+        <x:v>Unknown</x:v>
       </x:c>
       <x:c r="E47" s="12" t="str">
         <x:v>B</x:v>
@@ -1416,6 +1892,12 @@
       <x:c r="H47" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/512/</x:v>
       </x:c>
+      <x:c r="I47" t="str"/>
+      <x:c r="J47" t="str"/>
+      <x:c r="K47" s="16" t="str"/>
+      <x:c r="L47" t="str"/>
+      <x:c r="M47" t="str"/>
+      <x:c r="N47" t="str"/>
     </x:row>
     <x:row r="48" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A48" s="12" t="str">
@@ -1428,7 +1910,7 @@
         <x:v>L</x:v>
       </x:c>
       <x:c r="D48" s="12" t="str">
-        <x:v>Moderate-hard</x:v>
+        <x:v>Unknown</x:v>
       </x:c>
       <x:c r="E48" s="12" t="str">
         <x:v>B</x:v>
@@ -1442,6 +1924,16 @@
       <x:c r="H48" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/1152/</x:v>
       </x:c>
+      <x:c r="I48" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="J48" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=60</x:v>
+      </x:c>
+      <x:c r="K48" s="16" t="str"/>
+      <x:c r="L48" t="str"/>
+      <x:c r="M48" t="str"/>
+      <x:c r="N48" t="str"/>
     </x:row>
     <x:row r="49" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A49" s="12" t="str">
@@ -1454,7 +1946,7 @@
         <x:v>XL</x:v>
       </x:c>
       <x:c r="D49" s="12" t="str">
-        <x:v>Hard</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="E49" s="12" t="str">
         <x:v>B</x:v>
@@ -1467,6 +1959,24 @@
       </x:c>
       <x:c r="H49" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/1169/</x:v>
+      </x:c>
+      <x:c r="I49" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="J49" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=60</x:v>
+      </x:c>
+      <x:c r="K49" s="16" t="n">
+        <x:v>0.4426</x:v>
+      </x:c>
+      <x:c r="L49" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="M49" t="str">
+        <x:v>Main conference papers</x:v>
+      </x:c>
+      <x:c r="N49" t="str">
+        <x:v>https://icpr2024.org/book/978-3-031-78347-0_Book_OnlinePDF.pdf</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1480,16 +1990,22 @@
         <x:v>M</x:v>
       </x:c>
       <x:c r="D50" s="12" t="str">
-        <x:v>Hard</x:v>
-      </x:c>
-      <x:c r="E50" s="12" t="str"/>
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E50" s="12"/>
       <x:c r="F50" s="12" t="str">
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G50" t="str">
         <x:v>https://iapr.org/</x:v>
       </x:c>
-      <x:c r="H50" t="str"/>
+      <x:c r="H50"/>
+      <x:c r="I50" t="str"/>
+      <x:c r="J50" t="str"/>
+      <x:c r="K50" s="16" t="str"/>
+      <x:c r="L50" t="str"/>
+      <x:c r="M50" t="str"/>
+      <x:c r="N50" t="str"/>
     </x:row>
     <x:row r="51" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A51" s="12" t="str">
@@ -1502,16 +2018,22 @@
         <x:v>M</x:v>
       </x:c>
       <x:c r="D51" s="12" t="str">
-        <x:v>Moderate-hard</x:v>
-      </x:c>
-      <x:c r="E51" s="12" t="str"/>
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E51" s="12"/>
       <x:c r="F51" s="12" t="str">
         <x:v>Paper-based / workshop-style conference</x:v>
       </x:c>
       <x:c r="G51" t="str">
         <x:v>https://ssspr2026.inf.unibe.ch/</x:v>
       </x:c>
-      <x:c r="H51" t="str"/>
+      <x:c r="H51"/>
+      <x:c r="I51" t="str"/>
+      <x:c r="J51" t="str"/>
+      <x:c r="K51" s="16" t="str"/>
+      <x:c r="L51" t="str"/>
+      <x:c r="M51" t="str"/>
+      <x:c r="N51" t="str"/>
     </x:row>
     <x:row r="52" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A52" s="12" t="str">
@@ -1524,7 +2046,7 @@
         <x:v>M</x:v>
       </x:c>
       <x:c r="D52" s="12" t="str">
-        <x:v>Moderate-hard</x:v>
+        <x:v>Unknown</x:v>
       </x:c>
       <x:c r="E52" s="12" t="str">
         <x:v>C</x:v>
@@ -1538,6 +2060,12 @@
       <x:c r="H52" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/1122/</x:v>
       </x:c>
+      <x:c r="I52" t="str"/>
+      <x:c r="J52" t="str"/>
+      <x:c r="K52" s="16" t="str"/>
+      <x:c r="L52" t="str"/>
+      <x:c r="M52" t="str"/>
+      <x:c r="N52" t="str"/>
     </x:row>
     <x:row r="53" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A53" s="12" t="str">
@@ -1550,16 +2078,22 @@
         <x:v>L</x:v>
       </x:c>
       <x:c r="D53" s="12" t="str">
-        <x:v>Moderate-hard</x:v>
-      </x:c>
-      <x:c r="E53" s="12" t="str"/>
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E53" s="12"/>
       <x:c r="F53" s="12" t="str">
         <x:v>Paper-based / symposium series</x:v>
       </x:c>
       <x:c r="G53" t="str">
         <x:v>https://ssci2027generalchairs.github.io/ssci-2027/</x:v>
       </x:c>
-      <x:c r="H53" t="str"/>
+      <x:c r="H53"/>
+      <x:c r="I53" t="str"/>
+      <x:c r="J53" t="str"/>
+      <x:c r="K53" s="16" t="str"/>
+      <x:c r="L53" t="str"/>
+      <x:c r="M53" t="str"/>
+      <x:c r="N53" t="str"/>
     </x:row>
     <x:row r="54" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A54" s="12" t="str">
@@ -1572,7 +2106,7 @@
         <x:v>M</x:v>
       </x:c>
       <x:c r="D54" s="12" t="str">
-        <x:v>Moderate-hard</x:v>
+        <x:v>Unknown</x:v>
       </x:c>
       <x:c r="E54" s="12" t="str">
         <x:v>C</x:v>
@@ -1586,6 +2120,12 @@
       <x:c r="H54" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/1093/</x:v>
       </x:c>
+      <x:c r="I54" t="str"/>
+      <x:c r="J54" t="str"/>
+      <x:c r="K54" s="16" t="str"/>
+      <x:c r="L54" t="str"/>
+      <x:c r="M54" t="str"/>
+      <x:c r="N54" t="str"/>
     </x:row>
     <x:row r="55" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A55" s="12" t="str">
@@ -1598,16 +2138,22 @@
         <x:v>M</x:v>
       </x:c>
       <x:c r="D55" s="12" t="str">
-        <x:v>Moderate-hard</x:v>
-      </x:c>
-      <x:c r="E55" s="12" t="str"/>
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E55" s="12"/>
       <x:c r="F55" s="12" t="str">
         <x:v>Paper-based / Springer proceedings</x:v>
       </x:c>
       <x:c r="G55" t="str">
         <x:v>https://lodconference.org/</x:v>
       </x:c>
-      <x:c r="H55" t="str"/>
+      <x:c r="H55"/>
+      <x:c r="I55" t="str"/>
+      <x:c r="J55" t="str"/>
+      <x:c r="K55" s="16" t="str"/>
+      <x:c r="L55" t="str"/>
+      <x:c r="M55" t="str"/>
+      <x:c r="N55" t="str"/>
     </x:row>
     <x:row r="56" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A56" s="12" t="str">
@@ -1620,16 +2166,30 @@
         <x:v>XL</x:v>
       </x:c>
       <x:c r="D56" s="12" t="str">
-        <x:v>Hard</x:v>
-      </x:c>
-      <x:c r="E56" s="12" t="str"/>
+        <x:v>Very high</x:v>
+      </x:c>
+      <x:c r="E56" s="12"/>
       <x:c r="F56" s="12" t="str">
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G56" t="str">
         <x:v>https://eusipco2026.org/</x:v>
       </x:c>
-      <x:c r="H56" t="str"/>
+      <x:c r="H56"/>
+      <x:c r="I56" t="str"/>
+      <x:c r="J56" t="str"/>
+      <x:c r="K56" s="16" t="n">
+        <x:v>0.664</x:v>
+      </x:c>
+      <x:c r="L56" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="M56" t="str">
+        <x:v>Conference papers (about 550 of 828)</x:v>
+      </x:c>
+      <x:c r="N56" t="str">
+        <x:v>https://eurasip.org/newsletter/newsletter_2024-09.html</x:v>
+      </x:c>
     </x:row>
     <x:row r="57" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A57" s="12" t="str">
@@ -1642,16 +2202,22 @@
         <x:v>M</x:v>
       </x:c>
       <x:c r="D57" s="12" t="str">
-        <x:v>Hard</x:v>
-      </x:c>
-      <x:c r="E57" s="12" t="str"/>
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E57" s="12"/>
       <x:c r="F57" s="12" t="str">
         <x:v>Paper-based / specialist workshop</x:v>
       </x:c>
       <x:c r="G57" t="str">
         <x:v>https://ssp27.ieeesps.org/</x:v>
       </x:c>
-      <x:c r="H57" t="str"/>
+      <x:c r="H57"/>
+      <x:c r="I57" t="str"/>
+      <x:c r="J57" t="str"/>
+      <x:c r="K57" s="16" t="str"/>
+      <x:c r="L57" t="str"/>
+      <x:c r="M57" t="str"/>
+      <x:c r="N57" t="str"/>
     </x:row>
     <x:row r="58" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A58" s="12" t="str">
@@ -1664,16 +2230,22 @@
         <x:v>S</x:v>
       </x:c>
       <x:c r="D58" s="12" t="str">
-        <x:v>Moderate-hard</x:v>
-      </x:c>
-      <x:c r="E58" s="12" t="str"/>
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E58" s="12"/>
       <x:c r="F58" s="12" t="str">
         <x:v>Workshop / paper-based</x:v>
       </x:c>
       <x:c r="G58" t="str">
         <x:v>https://ecml-aaltd.github.io/aaltd2026/</x:v>
       </x:c>
-      <x:c r="H58" t="str"/>
+      <x:c r="H58"/>
+      <x:c r="I58" t="str"/>
+      <x:c r="J58" t="str"/>
+      <x:c r="K58" s="16" t="str"/>
+      <x:c r="L58" t="str"/>
+      <x:c r="M58" t="str"/>
+      <x:c r="N58" t="str"/>
     </x:row>
     <x:row r="59" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A59" s="12" t="str">
@@ -1686,16 +2258,22 @@
         <x:v>M</x:v>
       </x:c>
       <x:c r="D59" s="12" t="str">
-        <x:v>Moderate-hard</x:v>
-      </x:c>
-      <x:c r="E59" s="12" t="str"/>
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E59" s="12"/>
       <x:c r="F59" s="12" t="str">
         <x:v>Paper-based / forecasting-focused</x:v>
       </x:c>
       <x:c r="G59" t="str">
         <x:v>https://itise.ugr.es/index.html</x:v>
       </x:c>
-      <x:c r="H59" t="str"/>
+      <x:c r="H59"/>
+      <x:c r="I59" t="str"/>
+      <x:c r="J59" t="str"/>
+      <x:c r="K59" s="16" t="str"/>
+      <x:c r="L59" t="str"/>
+      <x:c r="M59" t="str"/>
+      <x:c r="N59" t="str"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="12" t="str">
@@ -1708,7 +2286,7 @@
         <x:v>L/XL</x:v>
       </x:c>
       <x:c r="D60" s="12" t="str">
-        <x:v>Hard</x:v>
+        <x:v>Low</x:v>
       </x:c>
       <x:c r="E60" s="12" t="str">
         <x:v>A</x:v>
@@ -1721,6 +2299,20 @@
       </x:c>
       <x:c r="H60" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/468/</x:v>
+      </x:c>
+      <x:c r="I60" t="str"/>
+      <x:c r="J60" t="str"/>
+      <x:c r="K60" s="16" t="n">
+        <x:v>0.203</x:v>
+      </x:c>
+      <x:c r="L60" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="M60" t="str">
+        <x:v>Main conference (226 accepted of 1,114 candidate papers; Findings excluded)</x:v>
+      </x:c>
+      <x:c r="N60" t="str">
+        <x:v>https://2024.eacl.org/downloads/handbook.pdf</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1734,7 +2326,7 @@
         <x:v>M</x:v>
       </x:c>
       <x:c r="D61" s="12" t="str">
-        <x:v>Moderate-hard</x:v>
+        <x:v>Unknown</x:v>
       </x:c>
       <x:c r="E61" s="12" t="str">
         <x:v>B</x:v>
@@ -1748,6 +2340,12 @@
       <x:c r="H61" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/151/</x:v>
       </x:c>
+      <x:c r="I61" t="str"/>
+      <x:c r="J61" t="str"/>
+      <x:c r="K61" s="16" t="str"/>
+      <x:c r="L61" t="str"/>
+      <x:c r="M61" t="str"/>
+      <x:c r="N61" t="str"/>
     </x:row>
     <x:row r="62" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A62" s="12" t="str">
@@ -1760,21 +2358,27 @@
         <x:v>S</x:v>
       </x:c>
       <x:c r="D62" s="12" t="str">
-        <x:v>Moderate-hard</x:v>
-      </x:c>
-      <x:c r="E62" s="12" t="str"/>
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E62" s="12"/>
       <x:c r="F62" s="12" t="str">
         <x:v>Workshop / non-archival short paper</x:v>
       </x:c>
       <x:c r="G62" t="str">
         <x:v>https://fmts-workshop.github.io/</x:v>
       </x:c>
-      <x:c r="H62" t="str"/>
+      <x:c r="H62"/>
+      <x:c r="I62" t="str"/>
+      <x:c r="J62" t="str"/>
+      <x:c r="K62" s="16" t="str"/>
+      <x:c r="L62" t="str"/>
+      <x:c r="M62" t="str"/>
+      <x:c r="N62" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9988e0f28f1b4db7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba0b69dc0aef4283"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1934,7 +2538,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd506e8cf24e14abc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a97d3f07e974545"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Refresh conference opportunities and recurring editions
</commit_message>
<xml_diff>
--- a/data/core_conferences_normalized_tags.xlsx
+++ b/data/core_conferences_normalized_tags.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Conferences" sheetId="1" r:id="Rab47c390448d4560"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Vocabulary" sheetId="2" r:id="Rd5189bbfb6f64c39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Conferences" sheetId="1" r:id="R2cbae0c569d74e82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Vocabulary" sheetId="2" r:id="R72650b53d031434b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -95,7 +95,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="CoreConferencesTable" displayName="CoreConferencesTable" ref="A1:N62" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="CoreConferencesTable" displayName="CoreConferencesTable" ref="A1:N64" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Conference"/>
     <x:tableColumn id="2" name="TAGS"/>
@@ -522,7 +522,7 @@
         <x:v>M/L</x:v>
       </x:c>
       <x:c r="D6" s="14" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Low (estimated)</x:v>
       </x:c>
       <x:c r="E6" s="14" t="str">
         <x:v>A</x:v>
@@ -543,9 +543,15 @@
         <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=58</x:v>
       </x:c>
       <x:c r="K6" s="16" t="str"/>
-      <x:c r="L6" t="str"/>
-      <x:c r="M6" t="str"/>
-      <x:c r="N6" t="str"/>
+      <x:c r="L6" t="n">
+        <x:v>2021</x:v>
+      </x:c>
+      <x:c r="M6" t="str">
+        <x:v>Main conference papers</x:v>
+      </x:c>
+      <x:c r="N6" t="str">
+        <x:v>https://proceedings.mlr.press/v161/campos21a/campos21a.pdf</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="14" t="str">
@@ -594,7 +600,7 @@
         <x:v>L</x:v>
       </x:c>
       <x:c r="D8" s="14" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Low</x:v>
       </x:c>
       <x:c r="E8" s="14" t="str">
         <x:v>A</x:v>
@@ -614,10 +620,18 @@
       <x:c r="J8" t="str">
         <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=36</x:v>
       </x:c>
-      <x:c r="K8" s="16" t="str"/>
-      <x:c r="L8" t="str"/>
-      <x:c r="M8" t="str"/>
-      <x:c r="N8" t="str"/>
+      <x:c r="K8" s="16" t="n">
+        <x:v>0.239</x:v>
+      </x:c>
+      <x:c r="L8" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="M8" t="str">
+        <x:v>Research and applied data science tracks combined (300 of 1,253)</x:v>
+      </x:c>
+      <x:c r="N8" t="str">
+        <x:v>https://link.springer.com/book/10.1007/978-3-662-72243-5</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="14" t="str">
@@ -710,7 +724,7 @@
         <x:v>M</x:v>
       </x:c>
       <x:c r="D11" s="14" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Low</x:v>
       </x:c>
       <x:c r="E11" s="14" t="str">
         <x:v>A</x:v>
@@ -730,10 +744,18 @@
       <x:c r="J11" t="str">
         <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=36</x:v>
       </x:c>
-      <x:c r="K11" s="16" t="str"/>
-      <x:c r="L11" t="str"/>
-      <x:c r="M11" t="str"/>
-      <x:c r="N11" t="str"/>
+      <x:c r="K11" s="16" t="n">
+        <x:v>0.2955</x:v>
+      </x:c>
+      <x:c r="L11" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="M11" t="str">
+        <x:v>Research papers; program chairs' reported rate</x:v>
+      </x:c>
+      <x:c r="N11" t="str">
+        <x:v>https://epubs.siam.org/doi/pdf/10.1137/1.9781611978032.fm</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="14" t="str">
@@ -784,14 +806,14 @@
       <x:c r="D13" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E13" s="14"/>
+      <x:c r="E13" s="14" t="str"/>
       <x:c r="F13" s="14" t="str">
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G13" t="str">
         <x:v>https://mlhc.org/</x:v>
       </x:c>
-      <x:c r="H13"/>
+      <x:c r="H13" t="str"/>
       <x:c r="I13" t="str"/>
       <x:c r="J13" t="str"/>
       <x:c r="K13" s="16" t="str"/>
@@ -812,14 +834,14 @@
       <x:c r="D14" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E14" s="14"/>
+      <x:c r="E14" s="14" t="str"/>
       <x:c r="F14" s="14" t="str">
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G14" t="str">
         <x:v>https://chil.ahli.cc/</x:v>
       </x:c>
-      <x:c r="H14"/>
+      <x:c r="H14" t="str"/>
       <x:c r="I14" t="str"/>
       <x:c r="J14" t="str"/>
       <x:c r="K14" s="16" t="str"/>
@@ -840,14 +862,14 @@
       <x:c r="D15" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E15" s="14"/>
+      <x:c r="E15" s="14" t="str"/>
       <x:c r="F15" s="14" t="str">
         <x:v>Proceedings + findings tracks</x:v>
       </x:c>
       <x:c r="G15" t="str">
         <x:v>https://ml4h.ahli.cc/</x:v>
       </x:c>
-      <x:c r="H15"/>
+      <x:c r="H15" t="str"/>
       <x:c r="I15" t="str"/>
       <x:c r="J15" t="str"/>
       <x:c r="K15" s="16" t="str"/>
@@ -868,14 +890,14 @@
       <x:c r="D16" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E16" s="14"/>
+      <x:c r="E16" s="14" t="str"/>
       <x:c r="F16" s="14" t="str">
         <x:v>Workshop / paper-based</x:v>
       </x:c>
       <x:c r="G16" t="str">
         <x:v>https://timeseries4health.github.io/</x:v>
       </x:c>
-      <x:c r="H16"/>
+      <x:c r="H16" t="str"/>
       <x:c r="I16" t="str"/>
       <x:c r="J16" t="str"/>
       <x:c r="K16" s="16" t="str"/>
@@ -940,14 +962,14 @@
       <x:c r="D18" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E18" s="14"/>
+      <x:c r="E18" s="14" t="str"/>
       <x:c r="F18" s="14" t="str">
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G18" t="str">
         <x:v>https://2026.midl.io/</x:v>
       </x:c>
-      <x:c r="H18"/>
+      <x:c r="H18" t="str"/>
       <x:c r="I18" t="str"/>
       <x:c r="J18" t="str"/>
       <x:c r="K18" s="16" t="str"/>
@@ -968,14 +990,14 @@
       <x:c r="D19" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E19" s="14"/>
+      <x:c r="E19" s="14" t="str"/>
       <x:c r="F19" s="14" t="str">
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G19" t="str">
         <x:v>https://biomedicalimaging.org/2027/</x:v>
       </x:c>
-      <x:c r="H19"/>
+      <x:c r="H19" t="str"/>
       <x:c r="I19" t="str"/>
       <x:c r="J19" t="str"/>
       <x:c r="K19" s="16" t="str"/>
@@ -996,14 +1018,14 @@
       <x:c r="D20" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E20" s="14"/>
+      <x:c r="E20" s="14" t="str"/>
       <x:c r="F20" s="14" t="str">
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G20" t="str">
         <x:v>https://bhi.embs.org/2026/</x:v>
       </x:c>
-      <x:c r="H20"/>
+      <x:c r="H20" t="str"/>
       <x:c r="I20" t="str"/>
       <x:c r="J20" t="str"/>
       <x:c r="K20" s="16" t="str"/>
@@ -1024,14 +1046,14 @@
       <x:c r="D21" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E21" s="14"/>
+      <x:c r="E21" s="14" t="str"/>
       <x:c r="F21" s="14" t="str">
         <x:v>Paper-based / broad applied venue</x:v>
       </x:c>
       <x:c r="G21" t="str">
         <x:v>https://embc.embs.org/2026/</x:v>
       </x:c>
-      <x:c r="H21"/>
+      <x:c r="H21" t="str"/>
       <x:c r="I21" t="str"/>
       <x:c r="J21" t="str"/>
       <x:c r="K21" s="16" t="str"/>
@@ -1052,14 +1074,14 @@
       <x:c r="D22" s="14" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="E22" s="14"/>
+      <x:c r="E22" s="14" t="str"/>
       <x:c r="F22" s="14" t="str">
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G22" t="str">
         <x:v>https://2027.ieeeicassp.org/</x:v>
       </x:c>
-      <x:c r="H22"/>
+      <x:c r="H22" t="str"/>
       <x:c r="I22" t="str">
         <x:v>B</x:v>
       </x:c>
@@ -1092,14 +1114,14 @@
       <x:c r="D23" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E23" s="14"/>
+      <x:c r="E23" s="14" t="str"/>
       <x:c r="F23" s="14" t="str">
         <x:v>Paper-based / workshop-style conference</x:v>
       </x:c>
       <x:c r="G23" t="str">
         <x:v>https://mlsp26.ieeesps.org/</x:v>
       </x:c>
-      <x:c r="H23"/>
+      <x:c r="H23" t="str"/>
       <x:c r="I23" t="str"/>
       <x:c r="J23" t="str"/>
       <x:c r="K23" s="16" t="str"/>
@@ -1120,14 +1142,14 @@
       <x:c r="D24" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E24" s="14"/>
+      <x:c r="E24" s="14" t="str"/>
       <x:c r="F24" s="14" t="str">
         <x:v>Abstract-based / talks highly selective</x:v>
       </x:c>
       <x:c r="G24" t="str">
         <x:v>https://www.cosyne.org/cosyne-home</x:v>
       </x:c>
-      <x:c r="H24"/>
+      <x:c r="H24" t="str"/>
       <x:c r="I24" t="str"/>
       <x:c r="J24" t="str"/>
       <x:c r="K24" s="16" t="str"/>
@@ -1148,14 +1170,14 @@
       <x:c r="D25" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E25" s="14"/>
+      <x:c r="E25" s="14" t="str"/>
       <x:c r="F25" s="14" t="str">
         <x:v>Mixed: proceedings + extended abstracts</x:v>
       </x:c>
       <x:c r="G25" t="str">
         <x:v>https://2026.ccneuro.org/</x:v>
       </x:c>
-      <x:c r="H25"/>
+      <x:c r="H25" t="str"/>
       <x:c r="I25" t="str"/>
       <x:c r="J25" t="str"/>
       <x:c r="K25" s="16" t="str"/>
@@ -1176,14 +1198,14 @@
       <x:c r="D26" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E26" s="14"/>
+      <x:c r="E26" s="14" t="str"/>
       <x:c r="F26" s="14" t="str">
         <x:v>Abstract-based / talks selective</x:v>
       </x:c>
       <x:c r="G26" t="str">
         <x:v>https://bernstein-network.de/en/bernstein-conference/</x:v>
       </x:c>
-      <x:c r="H26"/>
+      <x:c r="H26" t="str"/>
       <x:c r="I26" t="str"/>
       <x:c r="J26" t="str"/>
       <x:c r="K26" s="16" t="str"/>
@@ -1204,14 +1226,14 @@
       <x:c r="D27" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E27" s="14"/>
+      <x:c r="E27" s="14" t="str"/>
       <x:c r="F27" s="14" t="str">
         <x:v>Abstract-based</x:v>
       </x:c>
       <x:c r="G27" t="str">
         <x:v>https://www.cnsorg.org/cns-2026</x:v>
       </x:c>
-      <x:c r="H27"/>
+      <x:c r="H27" t="str"/>
       <x:c r="I27" t="str"/>
       <x:c r="J27" t="str"/>
       <x:c r="K27" s="16" t="str"/>
@@ -1232,14 +1254,14 @@
       <x:c r="D28" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E28" s="14"/>
+      <x:c r="E28" s="14" t="str"/>
       <x:c r="F28" s="14" t="str">
         <x:v>Abstract-based / talks selective</x:v>
       </x:c>
       <x:c r="G28" t="str">
         <x:v>https://humanbrainmapping.org/ohbm-2027/</x:v>
       </x:c>
-      <x:c r="H28"/>
+      <x:c r="H28" t="str"/>
       <x:c r="I28" t="str"/>
       <x:c r="J28" t="str"/>
       <x:c r="K28" s="16" t="str"/>
@@ -1260,14 +1282,14 @@
       <x:c r="D29" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E29" s="14"/>
+      <x:c r="E29" s="14" t="str"/>
       <x:c r="F29" s="14" t="str">
         <x:v>Paper-based / engineering-focused</x:v>
       </x:c>
       <x:c r="G29" t="str">
         <x:v>https://ieee-ner.org/</x:v>
       </x:c>
-      <x:c r="H29"/>
+      <x:c r="H29" t="str"/>
       <x:c r="I29" t="str"/>
       <x:c r="J29" t="str"/>
       <x:c r="K29" s="16" t="str"/>
@@ -1288,14 +1310,14 @@
       <x:c r="D30" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E30" s="14"/>
+      <x:c r="E30" s="14" t="str"/>
       <x:c r="F30" s="14" t="str">
         <x:v>Abstract/community-based</x:v>
       </x:c>
       <x:c r="G30" t="str">
         <x:v>https://bcisociety.org/bci-meeting/</x:v>
       </x:c>
-      <x:c r="H30"/>
+      <x:c r="H30" t="str"/>
       <x:c r="I30" t="str"/>
       <x:c r="J30" t="str"/>
       <x:c r="K30" s="16" t="str"/>
@@ -1316,14 +1338,14 @@
       <x:c r="D31" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E31" s="14"/>
+      <x:c r="E31" s="14" t="str"/>
       <x:c r="F31" s="14" t="str">
         <x:v>Abstract-based / specialist venue</x:v>
       </x:c>
       <x:c r="G31" t="str">
         <x:v>https://mm.scimeeting.cn/en/web/index/31426</x:v>
       </x:c>
-      <x:c r="H31"/>
+      <x:c r="H31" t="str"/>
       <x:c r="I31" t="str"/>
       <x:c r="J31" t="str"/>
       <x:c r="K31" s="16" t="str"/>
@@ -1344,14 +1366,14 @@
       <x:c r="D32" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E32" s="14"/>
+      <x:c r="E32" s="14" t="str"/>
       <x:c r="F32" s="14" t="str">
         <x:v>Paper-based / interdisciplinary</x:v>
       </x:c>
       <x:c r="G32" t="str">
         <x:v>https://facctconference.org/</x:v>
       </x:c>
-      <x:c r="H32"/>
+      <x:c r="H32" t="str"/>
       <x:c r="I32" t="str"/>
       <x:c r="J32" t="str"/>
       <x:c r="K32" s="16" t="str"/>
@@ -1500,14 +1522,14 @@
       <x:c r="D36" s="12" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E36" s="12"/>
+      <x:c r="E36" s="12" t="str"/>
       <x:c r="F36" s="12" t="str">
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G36" t="str">
         <x:v>https://2026.ijcai.org/</x:v>
       </x:c>
-      <x:c r="H36"/>
+      <x:c r="H36" t="str"/>
       <x:c r="I36" t="str"/>
       <x:c r="J36" t="str"/>
       <x:c r="K36" s="16" t="str"/>
@@ -1517,70 +1539,78 @@
     </x:row>
     <x:row r="37" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A37" s="12" t="str">
-        <x:v>ACML</x:v>
+        <x:v>IJCAI</x:v>
       </x:c>
       <x:c r="B37" s="12" t="str">
-        <x:v>Machine Learning; Deep Representation Learning; Learning Theory &amp; Statistical Foundations; Explainability &amp; Interpretability</x:v>
+        <x:v>Machine Learning; Deep Representation Learning; Learning Theory &amp; Statistical Foundations; Fairness &amp; Responsible AI</x:v>
       </x:c>
       <x:c r="C37" s="12" t="str">
-        <x:v>L</x:v>
+        <x:v>XL</x:v>
       </x:c>
       <x:c r="D37" s="12" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Very low</x:v>
       </x:c>
       <x:c r="E37" s="12" t="str">
-        <x:v>C</x:v>
+        <x:v>A*</x:v>
       </x:c>
       <x:c r="F37" s="12" t="str">
-        <x:v>Paper-based / OpenReview</x:v>
+        <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G37" t="str">
-        <x:v>https://www.acml-conf.org/2026/</x:v>
+        <x:v>https://2027.ijcai.org/</x:v>
       </x:c>
       <x:c r="H37" t="str">
-        <x:v>https://portal.core.edu.au/conf-ranks/2174/</x:v>
+        <x:v>https://portal.core.edu.au/conf-ranks/1313/</x:v>
       </x:c>
       <x:c r="I37" t="str">
-        <x:v>C</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J37" t="str">
-        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=59</x:v>
-      </x:c>
-      <x:c r="K37" s="16" t="str"/>
-      <x:c r="L37" t="str"/>
-      <x:c r="M37" t="str"/>
-      <x:c r="N37" t="str"/>
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=58</x:v>
+      </x:c>
+      <x:c r="K37" s="16" t="n">
+        <x:v>0.14</x:v>
+      </x:c>
+      <x:c r="L37" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="M37" t="str">
+        <x:v>Main conference papers (791 accepted of 5,650 reviewed)</x:v>
+      </x:c>
+      <x:c r="N37" t="str">
+        <x:v>https://2025.ijcai.org/wp-content/uploads/2024/12/IJCAI25-Sponsorship-Infographics.pdf</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A38" s="12" t="str">
-        <x:v>PAKDD</x:v>
+        <x:v>ECAI</x:v>
       </x:c>
       <x:c r="B38" s="12" t="str">
-        <x:v>Data Mining &amp; Data Science; Machine Learning; Time Series &amp; Sequential Data; Learning Theory &amp; Statistical Foundations</x:v>
+        <x:v>Machine Learning; Deep Representation Learning; Learning Theory &amp; Statistical Foundations; Fairness &amp; Responsible AI</x:v>
       </x:c>
       <x:c r="C38" s="12" t="str">
-        <x:v>L</x:v>
+        <x:v>XL</x:v>
       </x:c>
       <x:c r="D38" s="12" t="str">
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="E38" s="12" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="F38" s="12" t="str">
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G38" t="str">
-        <x:v>https://pakdd2027.org/</x:v>
+        <x:v>https://ecai2027.org/</x:v>
       </x:c>
       <x:c r="H38" t="str">
-        <x:v>https://portal.core.edu.au/conf-ranks/1667/</x:v>
+        <x:v>https://portal.core.edu.au/conf-ranks/473/</x:v>
       </x:c>
       <x:c r="I38" t="str">
-        <x:v>C</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J38" t="str">
-        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=37</x:v>
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=58</x:v>
       </x:c>
       <x:c r="K38" s="16" t="str"/>
       <x:c r="L38" t="str"/>
@@ -1589,46 +1619,54 @@
     </x:row>
     <x:row r="39" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A39" s="12" t="str">
-        <x:v>CIKM</x:v>
+        <x:v>ACML</x:v>
       </x:c>
       <x:c r="B39" s="12" t="str">
-        <x:v>Data Mining &amp; Data Science; Machine Learning; Time Series &amp; Sequential Data; Human-AI Interaction &amp; Deployment</x:v>
+        <x:v>Machine Learning; Deep Representation Learning; Learning Theory &amp; Statistical Foundations; Explainability &amp; Interpretability</x:v>
       </x:c>
       <x:c r="C39" s="12" t="str">
-        <x:v>XL</x:v>
+        <x:v>L</x:v>
       </x:c>
       <x:c r="D39" s="12" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Low</x:v>
       </x:c>
       <x:c r="E39" s="12" t="str">
-        <x:v>A</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="F39" s="12" t="str">
-        <x:v>Paper-based</x:v>
+        <x:v>Paper-based / OpenReview</x:v>
       </x:c>
       <x:c r="G39" t="str">
-        <x:v>https://cikm2026.diag.uniroma1.it/</x:v>
+        <x:v>https://www.acml-conf.org/2026/</x:v>
       </x:c>
       <x:c r="H39" t="str">
-        <x:v>https://portal.core.edu.au/conf-ranks/25/</x:v>
+        <x:v>https://portal.core.edu.au/conf-ranks/2174/</x:v>
       </x:c>
       <x:c r="I39" t="str">
-        <x:v>B</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="J39" t="str">
-        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=36</x:v>
-      </x:c>
-      <x:c r="K39" s="16" t="str"/>
-      <x:c r="L39" t="str"/>
-      <x:c r="M39" t="str"/>
-      <x:c r="N39" t="str"/>
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=59</x:v>
+      </x:c>
+      <x:c r="K39" s="16" t="n">
+        <x:v>0.29</x:v>
+      </x:c>
+      <x:c r="L39" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="M39" t="str">
+        <x:v>Conference track (79 accepted of 272 submitted)</x:v>
+      </x:c>
+      <x:c r="N39" t="str">
+        <x:v>https://www.acml-conf.org/</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A40" s="12" t="str">
-        <x:v>WSDM</x:v>
+        <x:v>PAKDD</x:v>
       </x:c>
       <x:c r="B40" s="12" t="str">
-        <x:v>Data Mining &amp; Data Science; Machine Learning; Fairness &amp; Responsible AI; Human-AI Interaction &amp; Deployment</x:v>
+        <x:v>Data Mining &amp; Data Science; Machine Learning; Time Series &amp; Sequential Data; Learning Theory &amp; Statistical Foundations</x:v>
       </x:c>
       <x:c r="C40" s="12" t="str">
         <x:v>L</x:v>
@@ -1637,22 +1675,22 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="E40" s="12" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="F40" s="12" t="str">
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G40" t="str">
-        <x:v>https://www.wsdm-conference.org/2027/</x:v>
+        <x:v>https://pakdd2027.org/</x:v>
       </x:c>
       <x:c r="H40" t="str">
-        <x:v>https://portal.core.edu.au/conf-ranks/31/</x:v>
+        <x:v>https://portal.core.edu.au/conf-ranks/1667/</x:v>
       </x:c>
       <x:c r="I40" t="str">
-        <x:v>B</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="J40" t="str">
-        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=36</x:v>
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=37</x:v>
       </x:c>
       <x:c r="K40" s="16" t="str"/>
       <x:c r="L40" t="str"/>
@@ -1661,77 +1699,99 @@
     </x:row>
     <x:row r="41" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A41" s="12" t="str">
-        <x:v>IEEE BigData</x:v>
+        <x:v>CIKM</x:v>
       </x:c>
       <x:c r="B41" s="12" t="str">
-        <x:v>Data Mining &amp; Data Science; Machine Learning; Time Series &amp; Sequential Data; Healthcare &amp; Clinical AI</x:v>
+        <x:v>Data Mining &amp; Data Science; Machine Learning; Time Series &amp; Sequential Data; Human-AI Interaction &amp; Deployment</x:v>
       </x:c>
       <x:c r="C41" s="12" t="str">
-        <x:v>L</x:v>
+        <x:v>XL</x:v>
       </x:c>
       <x:c r="D41" s="12" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Low</x:v>
       </x:c>
       <x:c r="E41" s="12" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="F41" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G41" t="str">
+        <x:v>https://cikm2026.diag.uniroma1.it/</x:v>
+      </x:c>
+      <x:c r="H41" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/25/</x:v>
+      </x:c>
+      <x:c r="I41" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="F41" s="12" t="str">
-        <x:v>Paper-based / mixed tracks</x:v>
-      </x:c>
-      <x:c r="G41" t="str">
-        <x:v>https://bigdataieee.org/BigData2026/</x:v>
-      </x:c>
-      <x:c r="H41" t="str">
-        <x:v>https://portal.core.edu.au/conf-ranks/2274/</x:v>
-      </x:c>
-      <x:c r="I41" t="str"/>
-      <x:c r="J41" t="str"/>
-      <x:c r="K41" s="16" t="str"/>
-      <x:c r="L41" t="str"/>
-      <x:c r="M41" t="str"/>
-      <x:c r="N41" t="str"/>
+      <x:c r="J41" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=36</x:v>
+      </x:c>
+      <x:c r="K41" s="16" t="n">
+        <x:v>0.27</x:v>
+      </x:c>
+      <x:c r="L41" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="M41" t="str">
+        <x:v>Full research papers (443 accepted of 1,627 submitted)</x:v>
+      </x:c>
+      <x:c r="N41" t="str">
+        <x:v>https://www.sigir.org/wp-content/uploads/2026/02/p18.pdf</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A42" s="12" t="str">
-        <x:v>Discovery Science</x:v>
+        <x:v>WSDM</x:v>
       </x:c>
       <x:c r="B42" s="12" t="str">
-        <x:v>Data Mining &amp; Data Science; Machine Learning; Learning Theory &amp; Statistical Foundations; Time Series &amp; Sequential Data</x:v>
+        <x:v>Data Mining &amp; Data Science; Machine Learning; Fairness &amp; Responsible AI; Human-AI Interaction &amp; Deployment</x:v>
       </x:c>
       <x:c r="C42" s="12" t="str">
-        <x:v>M</x:v>
+        <x:v>L</x:v>
       </x:c>
       <x:c r="D42" s="12" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Very low (estimated)</x:v>
       </x:c>
       <x:c r="E42" s="12" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="F42" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G42" t="str">
+        <x:v>https://www.wsdm-conference.org/2027/</x:v>
+      </x:c>
+      <x:c r="H42" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/31/</x:v>
+      </x:c>
+      <x:c r="I42" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="F42" s="12" t="str">
-        <x:v>Paper-based / research forum</x:v>
-      </x:c>
-      <x:c r="G42" t="str">
-        <x:v>https://discovery-science.org/</x:v>
-      </x:c>
-      <x:c r="H42" t="str">
-        <x:v>https://portal.core.edu.au/conf-ranks/2191/</x:v>
-      </x:c>
-      <x:c r="I42" t="str"/>
-      <x:c r="J42" t="str"/>
+      <x:c r="J42" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=36</x:v>
+      </x:c>
       <x:c r="K42" s="16" t="str"/>
-      <x:c r="L42" t="str"/>
-      <x:c r="M42" t="str"/>
-      <x:c r="N42" t="str"/>
+      <x:c r="L42" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="M42" t="str">
+        <x:v>Research papers</x:v>
+      </x:c>
+      <x:c r="N42" t="str">
+        <x:v>https://www.sigir.org/wp-content/uploads/2023/07/p08.pdf</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A43" s="12" t="str">
-        <x:v>IDA</x:v>
+        <x:v>IEEE BigData</x:v>
       </x:c>
       <x:c r="B43" s="12" t="str">
-        <x:v>Data Mining &amp; Data Science; Machine Learning; Probabilistic, Causal &amp; Uncertainty ML; Time Series &amp; Sequential Data</x:v>
+        <x:v>Data Mining &amp; Data Science; Machine Learning; Time Series &amp; Sequential Data; Healthcare &amp; Clinical AI</x:v>
       </x:c>
       <x:c r="C43" s="12" t="str">
-        <x:v>M</x:v>
+        <x:v>L</x:v>
       </x:c>
       <x:c r="D43" s="12" t="str">
         <x:v>Unknown</x:v>
@@ -1740,20 +1800,16 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="F43" s="12" t="str">
-        <x:v>Paper-based / interdisciplinary</x:v>
+        <x:v>Paper-based / mixed tracks</x:v>
       </x:c>
       <x:c r="G43" t="str">
-        <x:v>https://www.ida-society.org/</x:v>
+        <x:v>https://bigdataieee.org/BigData2026/</x:v>
       </x:c>
       <x:c r="H43" t="str">
-        <x:v>https://portal.core.edu.au/conf-ranks/845/</x:v>
-      </x:c>
-      <x:c r="I43" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="J43" t="str">
-        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=55</x:v>
-      </x:c>
+        <x:v>https://portal.core.edu.au/conf-ranks/2274/</x:v>
+      </x:c>
+      <x:c r="I43" t="str"/>
+      <x:c r="J43" t="str"/>
       <x:c r="K43" s="16" t="str"/>
       <x:c r="L43" t="str"/>
       <x:c r="M43" t="str"/>
@@ -1761,10 +1817,10 @@
     </x:row>
     <x:row r="44" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A44" s="12" t="str">
-        <x:v>ADMA</x:v>
+        <x:v>Discovery Science</x:v>
       </x:c>
       <x:c r="B44" s="12" t="str">
-        <x:v>Data Mining &amp; Data Science; Machine Learning; Time Series &amp; Sequential Data; Explainability &amp; Interpretability</x:v>
+        <x:v>Data Mining &amp; Data Science; Machine Learning; Learning Theory &amp; Statistical Foundations; Time Series &amp; Sequential Data</x:v>
       </x:c>
       <x:c r="C44" s="12" t="str">
         <x:v>M</x:v>
@@ -1773,23 +1829,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="E44" s="12" t="str">
-        <x:v>C</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="F44" s="12" t="str">
-        <x:v>Paper-based / special sessions</x:v>
+        <x:v>Paper-based / research forum</x:v>
       </x:c>
       <x:c r="G44" t="str">
-        <x:v>https://adma2026.github.io/</x:v>
+        <x:v>https://discovery-science.org/</x:v>
       </x:c>
       <x:c r="H44" t="str">
-        <x:v>https://portal.core.edu.au/conf-ranks/888/</x:v>
-      </x:c>
-      <x:c r="I44" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="J44" t="str">
-        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=37</x:v>
-      </x:c>
+        <x:v>https://portal.core.edu.au/conf-ranks/2191/</x:v>
+      </x:c>
+      <x:c r="I44" t="str"/>
+      <x:c r="J44" t="str"/>
       <x:c r="K44" s="16" t="str"/>
       <x:c r="L44" t="str"/>
       <x:c r="M44" t="str"/>
@@ -1797,49 +1849,57 @@
     </x:row>
     <x:row r="45" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A45" s="12" t="str">
-        <x:v>IJCNN</x:v>
+        <x:v>IDA</x:v>
       </x:c>
       <x:c r="B45" s="12" t="str">
-        <x:v>Machine Learning; Deep Representation Learning; Learning Theory &amp; Statistical Foundations; Signal Processing</x:v>
+        <x:v>Data Mining &amp; Data Science; Machine Learning; Probabilistic, Causal &amp; Uncertainty ML; Time Series &amp; Sequential Data</x:v>
       </x:c>
       <x:c r="C45" s="12" t="str">
-        <x:v>XL</x:v>
+        <x:v>M</x:v>
       </x:c>
       <x:c r="D45" s="12" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Moderate</x:v>
       </x:c>
       <x:c r="E45" s="12" t="str">
         <x:v>B</x:v>
       </x:c>
       <x:c r="F45" s="12" t="str">
-        <x:v>Paper-based</x:v>
+        <x:v>Paper-based / interdisciplinary</x:v>
       </x:c>
       <x:c r="G45" t="str">
-        <x:v>https://ijcnn.org/2027</x:v>
+        <x:v>https://www.ida-society.org/</x:v>
       </x:c>
       <x:c r="H45" t="str">
-        <x:v>https://portal.core.edu.au/conf-ranks/685/</x:v>
+        <x:v>https://portal.core.edu.au/conf-ranks/845/</x:v>
       </x:c>
       <x:c r="I45" t="str">
         <x:v>C</x:v>
       </x:c>
       <x:c r="J45" t="str">
-        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=60</x:v>
-      </x:c>
-      <x:c r="K45" s="16" t="str"/>
-      <x:c r="L45" t="str"/>
-      <x:c r="M45" t="str"/>
-      <x:c r="N45" t="str"/>
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=55</x:v>
+      </x:c>
+      <x:c r="K45" s="16" t="n">
+        <x:v>0.3846</x:v>
+      </x:c>
+      <x:c r="L45" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="M45" t="str">
+        <x:v>Full papers (35 accepted of 91 submitted)</x:v>
+      </x:c>
+      <x:c r="N45" t="str">
+        <x:v>https://link.springer.com/book/10.1007/978-3-031-91398-3</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A46" s="12" t="str">
-        <x:v>ICANN</x:v>
+        <x:v>ADMA</x:v>
       </x:c>
       <x:c r="B46" s="12" t="str">
-        <x:v>Machine Learning; Deep Representation Learning; Computational Neuroscience; Signal Processing</x:v>
+        <x:v>Data Mining &amp; Data Science; Machine Learning; Time Series &amp; Sequential Data; Explainability &amp; Interpretability</x:v>
       </x:c>
       <x:c r="C46" s="12" t="str">
-        <x:v>L</x:v>
+        <x:v>M</x:v>
       </x:c>
       <x:c r="D46" s="12" t="str">
         <x:v>Unknown</x:v>
@@ -1848,19 +1908,19 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="F46" s="12" t="str">
-        <x:v>Paper-based</x:v>
+        <x:v>Paper-based / special sessions</x:v>
       </x:c>
       <x:c r="G46" t="str">
-        <x:v>https://e-nns.org/icann2026/</x:v>
+        <x:v>https://adma2026.github.io/</x:v>
       </x:c>
       <x:c r="H46" t="str">
-        <x:v>https://portal.core.edu.au/conf-ranks/915/</x:v>
+        <x:v>https://portal.core.edu.au/conf-ranks/888/</x:v>
       </x:c>
       <x:c r="I46" t="str">
         <x:v>C</x:v>
       </x:c>
       <x:c r="J46" t="str">
-        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=59</x:v>
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=37</x:v>
       </x:c>
       <x:c r="K46" s="16" t="str"/>
       <x:c r="L46" t="str"/>
@@ -1869,13 +1929,13 @@
     </x:row>
     <x:row r="47" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A47" s="12" t="str">
-        <x:v>ESANN</x:v>
+        <x:v>IJCNN</x:v>
       </x:c>
       <x:c r="B47" s="12" t="str">
         <x:v>Machine Learning; Deep Representation Learning; Learning Theory &amp; Statistical Foundations; Signal Processing</x:v>
       </x:c>
       <x:c r="C47" s="12" t="str">
-        <x:v>M</x:v>
+        <x:v>XL</x:v>
       </x:c>
       <x:c r="D47" s="12" t="str">
         <x:v>Unknown</x:v>
@@ -1887,13 +1947,17 @@
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G47" t="str">
-        <x:v>https://www.esann.org/</x:v>
+        <x:v>https://ijcnn.org/2027</x:v>
       </x:c>
       <x:c r="H47" t="str">
-        <x:v>https://portal.core.edu.au/conf-ranks/512/</x:v>
-      </x:c>
-      <x:c r="I47" t="str"/>
-      <x:c r="J47" t="str"/>
+        <x:v>https://portal.core.edu.au/conf-ranks/685/</x:v>
+      </x:c>
+      <x:c r="I47" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="J47" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=60</x:v>
+      </x:c>
       <x:c r="K47" s="16" t="str"/>
       <x:c r="L47" t="str"/>
       <x:c r="M47" t="str"/>
@@ -1901,7 +1965,7 @@
     </x:row>
     <x:row r="48" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A48" s="12" t="str">
-        <x:v>ICONIP</x:v>
+        <x:v>ICANN</x:v>
       </x:c>
       <x:c r="B48" s="12" t="str">
         <x:v>Machine Learning; Deep Representation Learning; Computational Neuroscience; Signal Processing</x:v>
@@ -1913,22 +1977,22 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="E48" s="12" t="str">
-        <x:v>B</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="F48" s="12" t="str">
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G48" t="str">
-        <x:v>https://www.iconip2026.org/</x:v>
+        <x:v>https://e-nns.org/icann2026/</x:v>
       </x:c>
       <x:c r="H48" t="str">
-        <x:v>https://portal.core.edu.au/conf-ranks/1152/</x:v>
+        <x:v>https://portal.core.edu.au/conf-ranks/915/</x:v>
       </x:c>
       <x:c r="I48" t="str">
         <x:v>C</x:v>
       </x:c>
       <x:c r="J48" t="str">
-        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=60</x:v>
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=59</x:v>
       </x:c>
       <x:c r="K48" s="16" t="str"/>
       <x:c r="L48" t="str"/>
@@ -1937,16 +2001,16 @@
     </x:row>
     <x:row r="49" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A49" s="12" t="str">
-        <x:v>ICPR</x:v>
+        <x:v>ESANN</x:v>
       </x:c>
       <x:c r="B49" s="12" t="str">
-        <x:v>Machine Learning; Deep Representation Learning; Signal Processing; Biomedical Imaging</x:v>
+        <x:v>Machine Learning; Deep Representation Learning; Learning Theory &amp; Statistical Foundations; Signal Processing</x:v>
       </x:c>
       <x:c r="C49" s="12" t="str">
-        <x:v>XL</x:v>
+        <x:v>M</x:v>
       </x:c>
       <x:c r="D49" s="12" t="str">
-        <x:v>High</x:v>
+        <x:v>Unknown</x:v>
       </x:c>
       <x:c r="E49" s="12" t="str">
         <x:v>B</x:v>
@@ -1955,53 +2019,49 @@
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G49" t="str">
-        <x:v>https://icpr2026.org/</x:v>
+        <x:v>https://www.esann.org/</x:v>
       </x:c>
       <x:c r="H49" t="str">
-        <x:v>https://portal.core.edu.au/conf-ranks/1169/</x:v>
-      </x:c>
-      <x:c r="I49" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="J49" t="str">
-        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=60</x:v>
-      </x:c>
-      <x:c r="K49" s="16" t="n">
-        <x:v>0.4426</x:v>
-      </x:c>
-      <x:c r="L49" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="M49" t="str">
-        <x:v>Main conference papers</x:v>
-      </x:c>
-      <x:c r="N49" t="str">
-        <x:v>https://icpr2024.org/book/978-3-031-78347-0_Book_OnlinePDF.pdf</x:v>
-      </x:c>
+        <x:v>https://portal.core.edu.au/conf-ranks/512/</x:v>
+      </x:c>
+      <x:c r="I49" t="str"/>
+      <x:c r="J49" t="str"/>
+      <x:c r="K49" s="16" t="str"/>
+      <x:c r="L49" t="str"/>
+      <x:c r="M49" t="str"/>
+      <x:c r="N49" t="str"/>
     </x:row>
     <x:row r="50" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A50" s="12" t="str">
-        <x:v>ACPR</x:v>
+        <x:v>ICONIP</x:v>
       </x:c>
       <x:c r="B50" s="12" t="str">
-        <x:v>Machine Learning; Deep Representation Learning; Signal Processing; Biomedical Imaging</x:v>
+        <x:v>Machine Learning; Deep Representation Learning; Computational Neuroscience; Signal Processing</x:v>
       </x:c>
       <x:c r="C50" s="12" t="str">
-        <x:v>M</x:v>
+        <x:v>L</x:v>
       </x:c>
       <x:c r="D50" s="12" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E50" s="12"/>
+      <x:c r="E50" s="12" t="str">
+        <x:v>B</x:v>
+      </x:c>
       <x:c r="F50" s="12" t="str">
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G50" t="str">
-        <x:v>https://iapr.org/</x:v>
-      </x:c>
-      <x:c r="H50"/>
-      <x:c r="I50" t="str"/>
-      <x:c r="J50" t="str"/>
+        <x:v>https://www.iconip2026.org/</x:v>
+      </x:c>
+      <x:c r="H50" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/1152/</x:v>
+      </x:c>
+      <x:c r="I50" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="J50" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=60</x:v>
+      </x:c>
       <x:c r="K50" s="16" t="str"/>
       <x:c r="L50" t="str"/>
       <x:c r="M50" t="str"/>
@@ -2009,85 +2069,105 @@
     </x:row>
     <x:row r="51" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A51" s="12" t="str">
-        <x:v>S+SSPR</x:v>
+        <x:v>ICPR</x:v>
       </x:c>
       <x:c r="B51" s="12" t="str">
-        <x:v>Machine Learning; Deep Representation Learning; Data Mining &amp; Data Science; Signal Processing</x:v>
+        <x:v>Machine Learning; Deep Representation Learning; Signal Processing; Biomedical Imaging</x:v>
       </x:c>
       <x:c r="C51" s="12" t="str">
-        <x:v>M</x:v>
+        <x:v>XL</x:v>
       </x:c>
       <x:c r="D51" s="12" t="str">
-        <x:v>Unknown</x:v>
-      </x:c>
-      <x:c r="E51" s="12"/>
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E51" s="12" t="str">
+        <x:v>B</x:v>
+      </x:c>
       <x:c r="F51" s="12" t="str">
-        <x:v>Paper-based / workshop-style conference</x:v>
+        <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G51" t="str">
-        <x:v>https://ssspr2026.inf.unibe.ch/</x:v>
-      </x:c>
-      <x:c r="H51"/>
-      <x:c r="I51" t="str"/>
-      <x:c r="J51" t="str"/>
-      <x:c r="K51" s="16" t="str"/>
-      <x:c r="L51" t="str"/>
-      <x:c r="M51" t="str"/>
-      <x:c r="N51" t="str"/>
+        <x:v>https://icpr2026.org/</x:v>
+      </x:c>
+      <x:c r="H51" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/1169/</x:v>
+      </x:c>
+      <x:c r="I51" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="J51" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=60</x:v>
+      </x:c>
+      <x:c r="K51" s="16" t="n">
+        <x:v>0.4426</x:v>
+      </x:c>
+      <x:c r="L51" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="M51" t="str">
+        <x:v>Main conference papers</x:v>
+      </x:c>
+      <x:c r="N51" t="str">
+        <x:v>https://icpr2024.org/book/978-3-031-78347-0_Book_OnlinePDF.pdf</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A52" s="12" t="str">
-        <x:v>IEEE ICMLA</x:v>
+        <x:v>ACPR</x:v>
       </x:c>
       <x:c r="B52" s="12" t="str">
-        <x:v>Machine Learning; Deep Representation Learning; Data Mining &amp; Data Science; Time Series &amp; Sequential Data</x:v>
+        <x:v>Machine Learning; Deep Representation Learning; Signal Processing; Biomedical Imaging</x:v>
       </x:c>
       <x:c r="C52" s="12" t="str">
         <x:v>M</x:v>
       </x:c>
       <x:c r="D52" s="12" t="str">
-        <x:v>Unknown</x:v>
-      </x:c>
-      <x:c r="E52" s="12" t="str">
-        <x:v>C</x:v>
-      </x:c>
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E52" s="12" t="str"/>
       <x:c r="F52" s="12" t="str">
-        <x:v>Paper-based / special sessions</x:v>
+        <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G52" t="str">
-        <x:v>https://www.icmla-conference.org/icmla26/</x:v>
-      </x:c>
-      <x:c r="H52" t="str">
-        <x:v>https://portal.core.edu.au/conf-ranks/1122/</x:v>
-      </x:c>
+        <x:v>https://iapr.org/</x:v>
+      </x:c>
+      <x:c r="H52" t="str"/>
       <x:c r="I52" t="str"/>
       <x:c r="J52" t="str"/>
-      <x:c r="K52" s="16" t="str"/>
-      <x:c r="L52" t="str"/>
-      <x:c r="M52" t="str"/>
-      <x:c r="N52" t="str"/>
+      <x:c r="K52" s="16" t="n">
+        <x:v>0.5085000000000001</x:v>
+      </x:c>
+      <x:c r="L52" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="M52" t="str">
+        <x:v>Full papers (60 accepted of 118 submitted)</x:v>
+      </x:c>
+      <x:c r="N52" t="str">
+        <x:v>https://link.springer.com/book/10.1007/978-981-95-4398-4</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A53" s="12" t="str">
-        <x:v>IEEE SSCI</x:v>
+        <x:v>S+SSPR</x:v>
       </x:c>
       <x:c r="B53" s="12" t="str">
-        <x:v>Machine Learning; Deep Representation Learning; Learning Theory &amp; Statistical Foundations; Fairness &amp; Responsible AI</x:v>
+        <x:v>Machine Learning; Deep Representation Learning; Data Mining &amp; Data Science; Signal Processing</x:v>
       </x:c>
       <x:c r="C53" s="12" t="str">
-        <x:v>L</x:v>
+        <x:v>M</x:v>
       </x:c>
       <x:c r="D53" s="12" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E53" s="12"/>
+      <x:c r="E53" s="12" t="str"/>
       <x:c r="F53" s="12" t="str">
-        <x:v>Paper-based / symposium series</x:v>
+        <x:v>Paper-based / workshop-style conference</x:v>
       </x:c>
       <x:c r="G53" t="str">
-        <x:v>https://ssci2027generalchairs.github.io/ssci-2027/</x:v>
-      </x:c>
-      <x:c r="H53"/>
+        <x:v>https://ssspr2026.inf.unibe.ch/</x:v>
+      </x:c>
+      <x:c r="H53" t="str"/>
       <x:c r="I53" t="str"/>
       <x:c r="J53" t="str"/>
       <x:c r="K53" s="16" t="str"/>
@@ -2097,10 +2177,10 @@
     </x:row>
     <x:row r="54" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A54" s="12" t="str">
-        <x:v>IDEAL</x:v>
+        <x:v>IEEE ICMLA</x:v>
       </x:c>
       <x:c r="B54" s="12" t="str">
-        <x:v>Machine Learning; Data Mining &amp; Data Science; Deep Representation Learning; Learning Theory &amp; Statistical Foundations</x:v>
+        <x:v>Machine Learning; Deep Representation Learning; Data Mining &amp; Data Science; Time Series &amp; Sequential Data</x:v>
       </x:c>
       <x:c r="C54" s="12" t="str">
         <x:v>M</x:v>
@@ -2112,13 +2192,13 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="F54" s="12" t="str">
-        <x:v>Paper-based</x:v>
+        <x:v>Paper-based / special sessions</x:v>
       </x:c>
       <x:c r="G54" t="str">
-        <x:v>https://www.ideal2026.org/</x:v>
+        <x:v>https://www.icmla-conference.org/icmla26/</x:v>
       </x:c>
       <x:c r="H54" t="str">
-        <x:v>https://portal.core.edu.au/conf-ranks/1093/</x:v>
+        <x:v>https://portal.core.edu.au/conf-ranks/1122/</x:v>
       </x:c>
       <x:c r="I54" t="str"/>
       <x:c r="J54" t="str"/>
@@ -2129,25 +2209,25 @@
     </x:row>
     <x:row r="55" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A55" s="12" t="str">
-        <x:v>LOD</x:v>
+        <x:v>IEEE SSCI</x:v>
       </x:c>
       <x:c r="B55" s="12" t="str">
-        <x:v>Machine Learning; Data Mining &amp; Data Science; Learning Theory &amp; Statistical Foundations; Time Series &amp; Sequential Data</x:v>
+        <x:v>Machine Learning; Deep Representation Learning; Learning Theory &amp; Statistical Foundations; Fairness &amp; Responsible AI</x:v>
       </x:c>
       <x:c r="C55" s="12" t="str">
-        <x:v>M</x:v>
+        <x:v>L</x:v>
       </x:c>
       <x:c r="D55" s="12" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E55" s="12"/>
+      <x:c r="E55" s="12" t="str"/>
       <x:c r="F55" s="12" t="str">
-        <x:v>Paper-based / Springer proceedings</x:v>
+        <x:v>Paper-based / symposium series</x:v>
       </x:c>
       <x:c r="G55" t="str">
-        <x:v>https://lodconference.org/</x:v>
-      </x:c>
-      <x:c r="H55"/>
+        <x:v>https://ssci2027generalchairs.github.io/ssci-2027/</x:v>
+      </x:c>
+      <x:c r="H55" t="str"/>
       <x:c r="I55" t="str"/>
       <x:c r="J55" t="str"/>
       <x:c r="K55" s="16" t="str"/>
@@ -2157,46 +2237,42 @@
     </x:row>
     <x:row r="56" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A56" s="12" t="str">
-        <x:v>EUSIPCO</x:v>
+        <x:v>IDEAL</x:v>
       </x:c>
       <x:c r="B56" s="12" t="str">
-        <x:v>Signal Processing; Machine Learning; Time Series &amp; Sequential Data; EEG/MEG &amp; Neural Signals</x:v>
+        <x:v>Machine Learning; Data Mining &amp; Data Science; Deep Representation Learning; Learning Theory &amp; Statistical Foundations</x:v>
       </x:c>
       <x:c r="C56" s="12" t="str">
-        <x:v>XL</x:v>
+        <x:v>M</x:v>
       </x:c>
       <x:c r="D56" s="12" t="str">
-        <x:v>Very high</x:v>
-      </x:c>
-      <x:c r="E56" s="12"/>
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E56" s="12" t="str">
+        <x:v>C</x:v>
+      </x:c>
       <x:c r="F56" s="12" t="str">
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G56" t="str">
-        <x:v>https://eusipco2026.org/</x:v>
-      </x:c>
-      <x:c r="H56"/>
+        <x:v>https://www.ideal2026.org/</x:v>
+      </x:c>
+      <x:c r="H56" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/1093/</x:v>
+      </x:c>
       <x:c r="I56" t="str"/>
       <x:c r="J56" t="str"/>
-      <x:c r="K56" s="16" t="n">
-        <x:v>0.664</x:v>
-      </x:c>
-      <x:c r="L56" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="M56" t="str">
-        <x:v>Conference papers (about 550 of 828)</x:v>
-      </x:c>
-      <x:c r="N56" t="str">
-        <x:v>https://eurasip.org/newsletter/newsletter_2024-09.html</x:v>
-      </x:c>
+      <x:c r="K56" s="16" t="str"/>
+      <x:c r="L56" t="str"/>
+      <x:c r="M56" t="str"/>
+      <x:c r="N56" t="str"/>
     </x:row>
     <x:row r="57" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A57" s="12" t="str">
-        <x:v>IEEE SSP</x:v>
+        <x:v>LOD</x:v>
       </x:c>
       <x:c r="B57" s="12" t="str">
-        <x:v>Signal Processing; Machine Learning; Time Series &amp; Sequential Data; Probabilistic, Causal &amp; Uncertainty ML</x:v>
+        <x:v>Machine Learning; Data Mining &amp; Data Science; Learning Theory &amp; Statistical Foundations; Time Series &amp; Sequential Data</x:v>
       </x:c>
       <x:c r="C57" s="12" t="str">
         <x:v>M</x:v>
@@ -2204,14 +2280,14 @@
       <x:c r="D57" s="12" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E57" s="12"/>
+      <x:c r="E57" s="12" t="str"/>
       <x:c r="F57" s="12" t="str">
-        <x:v>Paper-based / specialist workshop</x:v>
+        <x:v>Paper-based / Springer proceedings</x:v>
       </x:c>
       <x:c r="G57" t="str">
-        <x:v>https://ssp27.ieeesps.org/</x:v>
-      </x:c>
-      <x:c r="H57"/>
+        <x:v>https://ais2026.icas.events/</x:v>
+      </x:c>
+      <x:c r="H57" t="str"/>
       <x:c r="I57" t="str"/>
       <x:c r="J57" t="str"/>
       <x:c r="K57" s="16" t="str"/>
@@ -2221,38 +2297,46 @@
     </x:row>
     <x:row r="58" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A58" s="12" t="str">
-        <x:v>AALTD</x:v>
+        <x:v>EUSIPCO</x:v>
       </x:c>
       <x:c r="B58" s="12" t="str">
-        <x:v>Time Series &amp; Sequential Data; Data Mining &amp; Data Science; Machine Learning; Explainability &amp; Interpretability</x:v>
+        <x:v>Signal Processing; Machine Learning; Time Series &amp; Sequential Data; EEG/MEG &amp; Neural Signals</x:v>
       </x:c>
       <x:c r="C58" s="12" t="str">
-        <x:v>S</x:v>
+        <x:v>XL</x:v>
       </x:c>
       <x:c r="D58" s="12" t="str">
-        <x:v>Unknown</x:v>
-      </x:c>
-      <x:c r="E58" s="12"/>
+        <x:v>Very high</x:v>
+      </x:c>
+      <x:c r="E58" s="12" t="str"/>
       <x:c r="F58" s="12" t="str">
-        <x:v>Workshop / paper-based</x:v>
+        <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G58" t="str">
-        <x:v>https://ecml-aaltd.github.io/aaltd2026/</x:v>
-      </x:c>
-      <x:c r="H58"/>
+        <x:v>https://eusipco2026.org/</x:v>
+      </x:c>
+      <x:c r="H58" t="str"/>
       <x:c r="I58" t="str"/>
       <x:c r="J58" t="str"/>
-      <x:c r="K58" s="16" t="str"/>
-      <x:c r="L58" t="str"/>
-      <x:c r="M58" t="str"/>
-      <x:c r="N58" t="str"/>
+      <x:c r="K58" s="16" t="n">
+        <x:v>0.664</x:v>
+      </x:c>
+      <x:c r="L58" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="M58" t="str">
+        <x:v>Conference papers (about 550 of 828)</x:v>
+      </x:c>
+      <x:c r="N58" t="str">
+        <x:v>https://eurasip.org/newsletter/newsletter_2024-09.html</x:v>
+      </x:c>
     </x:row>
     <x:row r="59" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A59" s="12" t="str">
-        <x:v>ITISE</x:v>
+        <x:v>IEEE SSP</x:v>
       </x:c>
       <x:c r="B59" s="12" t="str">
-        <x:v>Time Series &amp; Sequential Data; Machine Learning; Data Mining &amp; Data Science; Learning Theory &amp; Statistical Foundations</x:v>
+        <x:v>Signal Processing; Machine Learning; Time Series &amp; Sequential Data; Probabilistic, Causal &amp; Uncertainty ML</x:v>
       </x:c>
       <x:c r="C59" s="12" t="str">
         <x:v>M</x:v>
@@ -2260,14 +2344,14 @@
       <x:c r="D59" s="12" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E59" s="12"/>
+      <x:c r="E59" s="12" t="str"/>
       <x:c r="F59" s="12" t="str">
-        <x:v>Paper-based / forecasting-focused</x:v>
+        <x:v>Paper-based / specialist workshop</x:v>
       </x:c>
       <x:c r="G59" t="str">
-        <x:v>https://itise.ugr.es/index.html</x:v>
-      </x:c>
-      <x:c r="H59"/>
+        <x:v>https://ssp27.ieeesps.org/</x:v>
+      </x:c>
+      <x:c r="H59" t="str"/>
       <x:c r="I59" t="str"/>
       <x:c r="J59" t="str"/>
       <x:c r="K59" s="16" t="str"/>
@@ -2277,50 +2361,38 @@
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="12" t="str">
-        <x:v>EACL</x:v>
+        <x:v>AALTD</x:v>
       </x:c>
       <x:c r="B60" s="12" t="str">
-        <x:v>Natural Language Processing &amp; LLMs; Machine Learning; Deep Representation Learning; Fairness &amp; Responsible AI; Human-AI Interaction &amp; Deployment</x:v>
+        <x:v>Time Series &amp; Sequential Data; Data Mining &amp; Data Science; Machine Learning; Explainability &amp; Interpretability</x:v>
       </x:c>
       <x:c r="C60" s="12" t="str">
-        <x:v>L/XL</x:v>
+        <x:v>S</x:v>
       </x:c>
       <x:c r="D60" s="12" t="str">
-        <x:v>Low</x:v>
-      </x:c>
-      <x:c r="E60" s="12" t="str">
-        <x:v>A</x:v>
-      </x:c>
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E60" s="12" t="str"/>
       <x:c r="F60" s="12" t="str">
-        <x:v>Paper-based / ACL Rolling Review</x:v>
+        <x:v>Workshop / paper-based</x:v>
       </x:c>
       <x:c r="G60" t="str">
-        <x:v>https://2027.eacl.org/</x:v>
-      </x:c>
-      <x:c r="H60" t="str">
-        <x:v>https://portal.core.edu.au/conf-ranks/468/</x:v>
-      </x:c>
+        <x:v>https://ecml-aaltd.github.io/aaltd2026/</x:v>
+      </x:c>
+      <x:c r="H60" t="str"/>
       <x:c r="I60" t="str"/>
       <x:c r="J60" t="str"/>
-      <x:c r="K60" s="16" t="n">
-        <x:v>0.203</x:v>
-      </x:c>
-      <x:c r="L60" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="M60" t="str">
-        <x:v>Main conference (226 accepted of 1,114 candidate papers; Findings excluded)</x:v>
-      </x:c>
-      <x:c r="N60" t="str">
-        <x:v>https://2024.eacl.org/downloads/handbook.pdf</x:v>
-      </x:c>
+      <x:c r="K60" s="16" t="str"/>
+      <x:c r="L60" t="str"/>
+      <x:c r="M60" t="str"/>
+      <x:c r="N60" t="str"/>
     </x:row>
     <x:row r="61" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A61" s="12" t="str">
-        <x:v>AIME</x:v>
+        <x:v>ITISE</x:v>
       </x:c>
       <x:c r="B61" s="12" t="str">
-        <x:v>Healthcare &amp; Clinical AI; Machine Learning; Biomedical Imaging; Probabilistic, Causal &amp; Uncertainty ML</x:v>
+        <x:v>Time Series &amp; Sequential Data; Machine Learning; Data Mining &amp; Data Science; Learning Theory &amp; Statistical Foundations</x:v>
       </x:c>
       <x:c r="C61" s="12" t="str">
         <x:v>M</x:v>
@@ -2328,18 +2400,14 @@
       <x:c r="D61" s="12" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E61" s="12" t="str">
-        <x:v>B</x:v>
-      </x:c>
+      <x:c r="E61" s="12" t="str"/>
       <x:c r="F61" s="12" t="str">
-        <x:v>Paper-based / clinical AI</x:v>
+        <x:v>Paper-based / forecasting-focused</x:v>
       </x:c>
       <x:c r="G61" t="str">
-        <x:v>https://aime27.aimedicine.info/</x:v>
-      </x:c>
-      <x:c r="H61" t="str">
-        <x:v>https://portal.core.edu.au/conf-ranks/151/</x:v>
-      </x:c>
+        <x:v>https://itise.ugr.es/index.html</x:v>
+      </x:c>
+      <x:c r="H61" t="str"/>
       <x:c r="I61" t="str"/>
       <x:c r="J61" t="str"/>
       <x:c r="K61" s="16" t="str"/>
@@ -2349,36 +2417,108 @@
     </x:row>
     <x:row r="62" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A62" s="12" t="str">
-        <x:v>FMTS @ NeurIPS</x:v>
+        <x:v>EACL</x:v>
       </x:c>
       <x:c r="B62" s="12" t="str">
-        <x:v>Time Series &amp; Sequential Data; Machine Learning; Deep Representation Learning; Probabilistic, Causal &amp; Uncertainty ML</x:v>
+        <x:v>Natural Language Processing &amp; LLMs; Machine Learning; Deep Representation Learning; Fairness &amp; Responsible AI; Human-AI Interaction &amp; Deployment</x:v>
       </x:c>
       <x:c r="C62" s="12" t="str">
-        <x:v>S</x:v>
+        <x:v>L/XL</x:v>
       </x:c>
       <x:c r="D62" s="12" t="str">
-        <x:v>Unknown</x:v>
-      </x:c>
-      <x:c r="E62" s="12"/>
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="E62" s="12" t="str">
+        <x:v>A</x:v>
+      </x:c>
       <x:c r="F62" s="12" t="str">
-        <x:v>Workshop / non-archival short paper</x:v>
+        <x:v>Paper-based / ACL Rolling Review</x:v>
       </x:c>
       <x:c r="G62" t="str">
-        <x:v>https://fmts-workshop.github.io/</x:v>
-      </x:c>
-      <x:c r="H62"/>
+        <x:v>https://2027.eacl.org/</x:v>
+      </x:c>
+      <x:c r="H62" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/468/</x:v>
+      </x:c>
       <x:c r="I62" t="str"/>
       <x:c r="J62" t="str"/>
-      <x:c r="K62" s="16" t="str"/>
-      <x:c r="L62" t="str"/>
-      <x:c r="M62" t="str"/>
-      <x:c r="N62" t="str"/>
+      <x:c r="K62" s="16" t="n">
+        <x:v>0.203</x:v>
+      </x:c>
+      <x:c r="L62" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="M62" t="str">
+        <x:v>Main conference (226 accepted of 1,114 candidate papers; Findings excluded)</x:v>
+      </x:c>
+      <x:c r="N62" t="str">
+        <x:v>https://2024.eacl.org/downloads/handbook.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" t="str">
+        <x:v>AIME</x:v>
+      </x:c>
+      <x:c r="B63" t="str">
+        <x:v>Healthcare &amp; Clinical AI; Machine Learning; Biomedical Imaging; Probabilistic, Causal &amp; Uncertainty ML</x:v>
+      </x:c>
+      <x:c r="C63" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D63" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E63" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="F63" t="str">
+        <x:v>Paper-based / clinical AI</x:v>
+      </x:c>
+      <x:c r="G63" t="str">
+        <x:v>https://aime27.aimedicine.info/</x:v>
+      </x:c>
+      <x:c r="H63" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/151/</x:v>
+      </x:c>
+      <x:c r="I63" t="str"/>
+      <x:c r="J63" t="str"/>
+      <x:c r="K63" s="16" t="str"/>
+      <x:c r="L63" t="str"/>
+      <x:c r="M63" t="str"/>
+      <x:c r="N63" t="str"/>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" t="str">
+        <x:v>FMTS @ NeurIPS</x:v>
+      </x:c>
+      <x:c r="B64" t="str">
+        <x:v>Time Series &amp; Sequential Data; Machine Learning; Deep Representation Learning; Probabilistic, Causal &amp; Uncertainty ML</x:v>
+      </x:c>
+      <x:c r="C64" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="D64" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E64" t="str"/>
+      <x:c r="F64" t="str">
+        <x:v>Workshop / non-archival short paper</x:v>
+      </x:c>
+      <x:c r="G64" t="str">
+        <x:v>https://fmts-workshop.github.io/</x:v>
+      </x:c>
+      <x:c r="H64" t="str"/>
+      <x:c r="I64" t="str"/>
+      <x:c r="J64" t="str"/>
+      <x:c r="K64" s="16" t="str"/>
+      <x:c r="L64" t="str"/>
+      <x:c r="M64" t="str"/>
+      <x:c r="N64" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba0b69dc0aef4283"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f5d1e1c04f441c0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2538,7 +2678,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a97d3f07e974545"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f15308995474ada"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Launch Venue Radar with hierarchical topics and conference map
</commit_message>
<xml_diff>
--- a/data/core_conferences_normalized_tags.xlsx
+++ b/data/core_conferences_normalized_tags.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Conferences" sheetId="1" r:id="R2cbae0c569d74e82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Vocabulary" sheetId="2" r:id="R72650b53d031434b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Conferences" sheetId="1" r:id="R3c059a25c4fe434e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Vocabulary" sheetId="2" r:id="R0d878d9057754bb5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,8 +14,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="200" formatCode="0.0%"/>
+    <x:numFmt numFmtId="201" formatCode="0"/>
   </x:numFmts>
   <x:fonts count="2">
     <x:font>
@@ -49,7 +50,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="17">
+  <x:cellXfs count="18">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -87,6 +88,7 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -95,7 +97,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="CoreConferencesTable" displayName="CoreConferencesTable" ref="A1:N64" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="CoreConferencesTable" displayName="CoreConferencesTable" ref="A1:N72" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Conference"/>
     <x:tableColumn id="2" name="TAGS"/>
@@ -117,7 +119,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TagVocabularyTable" displayName="TagVocabularyTable" ref="A1:B17" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TagVocabularyTable" displayName="TagVocabularyTable" ref="A1:B27" headerRowCount="1" totalsRowCount="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Standard tag"/>
     <x:tableColumn id="2" name="Definition"/>
@@ -335,7 +337,7 @@
         <x:v>Acceptance source</x:v>
       </x:c>
     </x:row>
-    <x:row r="2">
+    <x:row r="2" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A2" s="14" t="str">
         <x:v>NeurIPS</x:v>
       </x:c>
@@ -369,7 +371,7 @@
       <x:c r="K2" s="16" t="n">
         <x:v>0.2452</x:v>
       </x:c>
-      <x:c r="L2" t="n">
+      <x:c r="L2" s="17" t="n">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="M2" t="str">
@@ -379,7 +381,7 @@
         <x:v>https://blog.neurips.cc/2025/09/30/</x:v>
       </x:c>
     </x:row>
-    <x:row r="3">
+    <x:row r="3" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A3" s="14" t="str">
         <x:v>ICML</x:v>
       </x:c>
@@ -399,7 +401,7 @@
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G3" t="str">
-        <x:v>https://icml.cc/Conferences/2026</x:v>
+        <x:v>https://icml.cc/Conferences/FutureMeetings</x:v>
       </x:c>
       <x:c r="H3" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/1121/</x:v>
@@ -413,7 +415,7 @@
       <x:c r="K3" s="16" t="n">
         <x:v>0.27</x:v>
       </x:c>
-      <x:c r="L3" t="n">
+      <x:c r="L3" s="17" t="n">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="M3" t="str">
@@ -423,12 +425,12 @@
         <x:v>https://media.icml.cc/Conferences/ICML2025/ICML2025_Fact_Sheet.pdf</x:v>
       </x:c>
     </x:row>
-    <x:row r="4">
+    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A4" s="14" t="str">
         <x:v>ICLR</x:v>
       </x:c>
       <x:c r="B4" s="14" t="str">
-        <x:v>Deep Representation Learning; Machine Learning; Explainability &amp; Interpretability; EEG/MEG &amp; Neural Signals</x:v>
+        <x:v>Deep Representation Learning; Machine Learning; Explainability &amp; Interpretability; Robustness &amp; Safety</x:v>
       </x:c>
       <x:c r="C4" s="14" t="str">
         <x:v>XXL</x:v>
@@ -457,7 +459,7 @@
       <x:c r="K4" s="16" t="n">
         <x:v>0.27399999999999997</x:v>
       </x:c>
-      <x:c r="L4" t="n">
+      <x:c r="L4" s="17" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="M4" t="str">
@@ -467,7 +469,7 @@
         <x:v>https://blog.iclr.cc/2026/</x:v>
       </x:c>
     </x:row>
-    <x:row r="5">
+    <x:row r="5" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A5" s="14" t="str">
         <x:v>AISTATS</x:v>
       </x:c>
@@ -487,7 +489,7 @@
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G5" t="str">
-        <x:v>https://aistats.org/</x:v>
+        <x:v>https://aistats.org/aistats2027/index.html</x:v>
       </x:c>
       <x:c r="H5" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/913/</x:v>
@@ -501,7 +503,7 @@
       <x:c r="K5" s="16" t="n">
         <x:v>0.281</x:v>
       </x:c>
-      <x:c r="L5" t="n">
+      <x:c r="L5" s="17" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="M5" t="str">
@@ -511,15 +513,15 @@
         <x:v>https://www.linkedin.com/posts/asolin_aistats2026-tangier-morocco-activity-7424831733768044544-DjfS</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
+    <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A6" s="14" t="str">
         <x:v>UAI</x:v>
       </x:c>
       <x:c r="B6" s="14" t="str">
-        <x:v>Probabilistic, Causal &amp; Uncertainty ML; Machine Learning; Healthcare &amp; Clinical AI; Fairness &amp; Responsible AI</x:v>
+        <x:v>Probabilistic, Causal &amp; Uncertainty ML; Machine Learning; Learning Theory &amp; Statistical Foundations</x:v>
       </x:c>
       <x:c r="C6" s="14" t="str">
-        <x:v>M/L</x:v>
+        <x:v>L</x:v>
       </x:c>
       <x:c r="D6" s="14" t="str">
         <x:v>Low (estimated)</x:v>
@@ -542,8 +544,8 @@
       <x:c r="J6" t="str">
         <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=58</x:v>
       </x:c>
-      <x:c r="K6" s="16" t="str"/>
-      <x:c r="L6" t="n">
+      <x:c r="K6" s="16"/>
+      <x:c r="L6" s="17" t="n">
         <x:v>2021</x:v>
       </x:c>
       <x:c r="M6" t="str">
@@ -553,7 +555,7 @@
         <x:v>https://proceedings.mlr.press/v161/campos21a/campos21a.pdf</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="14" t="str">
         <x:v>COLT</x:v>
       </x:c>
@@ -584,17 +586,17 @@
       <x:c r="J7" t="str">
         <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=58</x:v>
       </x:c>
-      <x:c r="K7" s="16" t="str"/>
-      <x:c r="L7" t="str"/>
-      <x:c r="M7" t="str"/>
-      <x:c r="N7" t="str"/>
-    </x:row>
-    <x:row r="8">
+      <x:c r="K7" s="16"/>
+      <x:c r="L7" s="17"/>
+      <x:c r="M7"/>
+      <x:c r="N7"/>
+    </x:row>
+    <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A8" s="14" t="str">
         <x:v>ECML PKDD</x:v>
       </x:c>
       <x:c r="B8" s="14" t="str">
-        <x:v>Machine Learning; Data Mining &amp; Data Science; Time Series &amp; Sequential Data; Healthcare &amp; Clinical AI</x:v>
+        <x:v>Machine Learning; Data Mining &amp; Data Science; Time Series &amp; Sequential Data; Explainability &amp; Interpretability</x:v>
       </x:c>
       <x:c r="C8" s="14" t="str">
         <x:v>L</x:v>
@@ -609,7 +611,7 @@
         <x:v>Paper-based / mixed tracks</x:v>
       </x:c>
       <x:c r="G8" t="str">
-        <x:v>https://ecmlpkdd.org/2026/</x:v>
+        <x:v>https://ecmlpkdd.org/2027/</x:v>
       </x:c>
       <x:c r="H8" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/491/</x:v>
@@ -623,7 +625,7 @@
       <x:c r="K8" s="16" t="n">
         <x:v>0.239</x:v>
       </x:c>
-      <x:c r="L8" t="n">
+      <x:c r="L8" s="17" t="n">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="M8" t="str">
@@ -633,12 +635,12 @@
         <x:v>https://link.springer.com/book/10.1007/978-3-662-72243-5</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
+    <x:row r="9" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A9" s="14" t="str">
         <x:v>KDD</x:v>
       </x:c>
       <x:c r="B9" s="14" t="str">
-        <x:v>Data Mining &amp; Data Science; Machine Learning; Time Series &amp; Sequential Data; Fairness &amp; Responsible AI</x:v>
+        <x:v>Data Mining &amp; Data Science; Machine Learning; Time Series &amp; Sequential Data; Federated &amp; Distributed Learning</x:v>
       </x:c>
       <x:c r="C9" s="14" t="str">
         <x:v>XL</x:v>
@@ -653,7 +655,7 @@
         <x:v>Paper-based / mixed tracks</x:v>
       </x:c>
       <x:c r="G9" t="str">
-        <x:v>https://kdd2026.kdd.org/</x:v>
+        <x:v>https://kdd2027.kdd.org/</x:v>
       </x:c>
       <x:c r="H9" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/26/</x:v>
@@ -667,7 +669,7 @@
       <x:c r="K9" s="16" t="n">
         <x:v>0.19</x:v>
       </x:c>
-      <x:c r="L9" t="n">
+      <x:c r="L9" s="17" t="n">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="M9" t="str">
@@ -677,15 +679,15 @@
         <x:v>https://kdd.org/kdd2025/frequently-asked-questions/</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
+    <x:row r="10" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A10" s="14" t="str">
         <x:v>ICDM</x:v>
       </x:c>
       <x:c r="B10" s="14" t="str">
-        <x:v>Data Mining &amp; Data Science; Time Series &amp; Sequential Data; Machine Learning; Healthcare &amp; Clinical AI</x:v>
+        <x:v>Data Mining &amp; Data Science; Time Series &amp; Sequential Data; Machine Learning</x:v>
       </x:c>
       <x:c r="C10" s="14" t="str">
-        <x:v>M/L</x:v>
+        <x:v>L</x:v>
       </x:c>
       <x:c r="D10" s="14" t="str">
         <x:v>Unknown</x:v>
@@ -708,12 +710,12 @@
       <x:c r="J10" t="str">
         <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=36</x:v>
       </x:c>
-      <x:c r="K10" s="16" t="str"/>
-      <x:c r="L10" t="str"/>
-      <x:c r="M10" t="str"/>
-      <x:c r="N10" t="str"/>
-    </x:row>
-    <x:row r="11">
+      <x:c r="K10" s="16"/>
+      <x:c r="L10" s="17"/>
+      <x:c r="M10"/>
+      <x:c r="N10"/>
+    </x:row>
+    <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A11" s="14" t="str">
         <x:v>SDM</x:v>
       </x:c>
@@ -747,7 +749,7 @@
       <x:c r="K11" s="16" t="n">
         <x:v>0.2955</x:v>
       </x:c>
-      <x:c r="L11" t="n">
+      <x:c r="L11" s="17" t="n">
         <x:v>2024</x:v>
       </x:c>
       <x:c r="M11" t="str">
@@ -757,12 +759,12 @@
         <x:v>https://epubs.siam.org/doi/pdf/10.1137/1.9781611978032.fm</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
+    <x:row r="12" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A12" s="14" t="str">
         <x:v>DSAA</x:v>
       </x:c>
       <x:c r="B12" s="14" t="str">
-        <x:v>Data Mining &amp; Data Science; Machine Learning; Healthcare &amp; Clinical AI; Human-AI Interaction &amp; Deployment</x:v>
+        <x:v>Data Mining &amp; Data Science; Machine Learning; Time Series &amp; Sequential Data; Human-AI Interaction &amp; Deployment</x:v>
       </x:c>
       <x:c r="C12" s="14" t="str">
         <x:v>M</x:v>
@@ -788,12 +790,12 @@
       <x:c r="J12" t="str">
         <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=43</x:v>
       </x:c>
-      <x:c r="K12" s="16" t="str"/>
-      <x:c r="L12" t="str"/>
-      <x:c r="M12" t="str"/>
-      <x:c r="N12" t="str"/>
-    </x:row>
-    <x:row r="13">
+      <x:c r="K12" s="16"/>
+      <x:c r="L12" s="17"/>
+      <x:c r="M12"/>
+      <x:c r="N12"/>
+    </x:row>
+    <x:row r="13" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A13" s="14" t="str">
         <x:v>MLHC</x:v>
       </x:c>
@@ -806,22 +808,22 @@
       <x:c r="D13" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E13" s="14" t="str"/>
+      <x:c r="E13" s="14"/>
       <x:c r="F13" s="14" t="str">
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G13" t="str">
         <x:v>https://mlhc.org/</x:v>
       </x:c>
-      <x:c r="H13" t="str"/>
-      <x:c r="I13" t="str"/>
-      <x:c r="J13" t="str"/>
-      <x:c r="K13" s="16" t="str"/>
-      <x:c r="L13" t="str"/>
-      <x:c r="M13" t="str"/>
-      <x:c r="N13" t="str"/>
-    </x:row>
-    <x:row r="14">
+      <x:c r="H13"/>
+      <x:c r="I13"/>
+      <x:c r="J13"/>
+      <x:c r="K13" s="16"/>
+      <x:c r="L13" s="17"/>
+      <x:c r="M13"/>
+      <x:c r="N13"/>
+    </x:row>
+    <x:row r="14" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A14" s="14" t="str">
         <x:v>CHIL</x:v>
       </x:c>
@@ -834,22 +836,22 @@
       <x:c r="D14" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E14" s="14" t="str"/>
+      <x:c r="E14" s="14"/>
       <x:c r="F14" s="14" t="str">
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G14" t="str">
         <x:v>https://chil.ahli.cc/</x:v>
       </x:c>
-      <x:c r="H14" t="str"/>
-      <x:c r="I14" t="str"/>
-      <x:c r="J14" t="str"/>
-      <x:c r="K14" s="16" t="str"/>
-      <x:c r="L14" t="str"/>
-      <x:c r="M14" t="str"/>
-      <x:c r="N14" t="str"/>
-    </x:row>
-    <x:row r="15">
+      <x:c r="H14"/>
+      <x:c r="I14"/>
+      <x:c r="J14"/>
+      <x:c r="K14" s="16"/>
+      <x:c r="L14" s="17"/>
+      <x:c r="M14"/>
+      <x:c r="N14"/>
+    </x:row>
+    <x:row r="15" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A15" s="14" t="str">
         <x:v>ML4H</x:v>
       </x:c>
@@ -862,22 +864,22 @@
       <x:c r="D15" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E15" s="14" t="str"/>
+      <x:c r="E15" s="14"/>
       <x:c r="F15" s="14" t="str">
         <x:v>Proceedings + findings tracks</x:v>
       </x:c>
       <x:c r="G15" t="str">
         <x:v>https://ml4h.ahli.cc/</x:v>
       </x:c>
-      <x:c r="H15" t="str"/>
-      <x:c r="I15" t="str"/>
-      <x:c r="J15" t="str"/>
-      <x:c r="K15" s="16" t="str"/>
-      <x:c r="L15" t="str"/>
-      <x:c r="M15" t="str"/>
-      <x:c r="N15" t="str"/>
-    </x:row>
-    <x:row r="16">
+      <x:c r="H15"/>
+      <x:c r="I15"/>
+      <x:c r="J15"/>
+      <x:c r="K15" s="16"/>
+      <x:c r="L15" s="17"/>
+      <x:c r="M15"/>
+      <x:c r="N15"/>
+    </x:row>
+    <x:row r="16" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A16" s="14" t="str">
         <x:v>TS4H</x:v>
       </x:c>
@@ -890,22 +892,22 @@
       <x:c r="D16" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E16" s="14" t="str"/>
+      <x:c r="E16" s="14"/>
       <x:c r="F16" s="14" t="str">
         <x:v>Workshop / paper-based</x:v>
       </x:c>
       <x:c r="G16" t="str">
         <x:v>https://timeseries4health.github.io/</x:v>
       </x:c>
-      <x:c r="H16" t="str"/>
-      <x:c r="I16" t="str"/>
-      <x:c r="J16" t="str"/>
-      <x:c r="K16" s="16" t="str"/>
-      <x:c r="L16" t="str"/>
-      <x:c r="M16" t="str"/>
-      <x:c r="N16" t="str"/>
-    </x:row>
-    <x:row r="17">
+      <x:c r="H16"/>
+      <x:c r="I16"/>
+      <x:c r="J16"/>
+      <x:c r="K16" s="16"/>
+      <x:c r="L16" s="17"/>
+      <x:c r="M16"/>
+      <x:c r="N16"/>
+    </x:row>
+    <x:row r="17" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A17" s="14" t="str">
         <x:v>MICCAI</x:v>
       </x:c>
@@ -925,7 +927,7 @@
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G17" t="str">
-        <x:v>https://conferences.miccai.org/2026/en/default.asp</x:v>
+        <x:v>https://miccai.org/upcoming-conferences/</x:v>
       </x:c>
       <x:c r="H17" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/1607/</x:v>
@@ -939,7 +941,7 @@
       <x:c r="K17" s="16" t="n">
         <x:v>0.29</x:v>
       </x:c>
-      <x:c r="L17" t="n">
+      <x:c r="L17" s="17" t="n">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="M17" t="str">
@@ -949,7 +951,7 @@
         <x:v>https://miccai.org/2025/06/20/miccai-quarterly-summer-june-2025/</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="14" t="str">
         <x:v>MIDL</x:v>
       </x:c>
@@ -962,22 +964,22 @@
       <x:c r="D18" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E18" s="14" t="str"/>
+      <x:c r="E18" s="14"/>
       <x:c r="F18" s="14" t="str">
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G18" t="str">
-        <x:v>https://2026.midl.io/</x:v>
-      </x:c>
-      <x:c r="H18" t="str"/>
-      <x:c r="I18" t="str"/>
-      <x:c r="J18" t="str"/>
-      <x:c r="K18" s="16" t="str"/>
-      <x:c r="L18" t="str"/>
-      <x:c r="M18" t="str"/>
-      <x:c r="N18" t="str"/>
-    </x:row>
-    <x:row r="19">
+        <x:v>https://2027.midl.io/</x:v>
+      </x:c>
+      <x:c r="H18"/>
+      <x:c r="I18"/>
+      <x:c r="J18"/>
+      <x:c r="K18" s="16"/>
+      <x:c r="L18" s="17"/>
+      <x:c r="M18"/>
+      <x:c r="N18"/>
+    </x:row>
+    <x:row r="19" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A19" s="14" t="str">
         <x:v>ISBI</x:v>
       </x:c>
@@ -990,22 +992,22 @@
       <x:c r="D19" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E19" s="14" t="str"/>
+      <x:c r="E19" s="14"/>
       <x:c r="F19" s="14" t="str">
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G19" t="str">
         <x:v>https://biomedicalimaging.org/2027/</x:v>
       </x:c>
-      <x:c r="H19" t="str"/>
-      <x:c r="I19" t="str"/>
-      <x:c r="J19" t="str"/>
-      <x:c r="K19" s="16" t="str"/>
-      <x:c r="L19" t="str"/>
-      <x:c r="M19" t="str"/>
-      <x:c r="N19" t="str"/>
-    </x:row>
-    <x:row r="20">
+      <x:c r="H19"/>
+      <x:c r="I19"/>
+      <x:c r="J19"/>
+      <x:c r="K19" s="16"/>
+      <x:c r="L19" s="17"/>
+      <x:c r="M19"/>
+      <x:c r="N19"/>
+    </x:row>
+    <x:row r="20" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A20" s="14" t="str">
         <x:v>IEEE BHI</x:v>
       </x:c>
@@ -1018,22 +1020,22 @@
       <x:c r="D20" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E20" s="14" t="str"/>
+      <x:c r="E20" s="14"/>
       <x:c r="F20" s="14" t="str">
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G20" t="str">
         <x:v>https://bhi.embs.org/2026/</x:v>
       </x:c>
-      <x:c r="H20" t="str"/>
-      <x:c r="I20" t="str"/>
-      <x:c r="J20" t="str"/>
-      <x:c r="K20" s="16" t="str"/>
-      <x:c r="L20" t="str"/>
-      <x:c r="M20" t="str"/>
-      <x:c r="N20" t="str"/>
-    </x:row>
-    <x:row r="21">
+      <x:c r="H20"/>
+      <x:c r="I20"/>
+      <x:c r="J20"/>
+      <x:c r="K20" s="16"/>
+      <x:c r="L20" s="17"/>
+      <x:c r="M20"/>
+      <x:c r="N20"/>
+    </x:row>
+    <x:row r="21" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A21" s="14" t="str">
         <x:v>IEEE EMBC</x:v>
       </x:c>
@@ -1046,27 +1048,27 @@
       <x:c r="D21" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E21" s="14" t="str"/>
+      <x:c r="E21" s="14"/>
       <x:c r="F21" s="14" t="str">
         <x:v>Paper-based / broad applied venue</x:v>
       </x:c>
       <x:c r="G21" t="str">
-        <x:v>https://embc.embs.org/2026/</x:v>
-      </x:c>
-      <x:c r="H21" t="str"/>
-      <x:c r="I21" t="str"/>
-      <x:c r="J21" t="str"/>
-      <x:c r="K21" s="16" t="str"/>
-      <x:c r="L21" t="str"/>
-      <x:c r="M21" t="str"/>
-      <x:c r="N21" t="str"/>
-    </x:row>
-    <x:row r="22">
+        <x:v>https://embc.embs.org/2027/</x:v>
+      </x:c>
+      <x:c r="H21"/>
+      <x:c r="I21"/>
+      <x:c r="J21"/>
+      <x:c r="K21" s="16"/>
+      <x:c r="L21" s="17"/>
+      <x:c r="M21"/>
+      <x:c r="N21"/>
+    </x:row>
+    <x:row r="22" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A22" s="14" t="str">
         <x:v>ICASSP</x:v>
       </x:c>
       <x:c r="B22" s="14" t="str">
-        <x:v>Signal Processing; Machine Learning; Time Series &amp; Sequential Data; EEG/MEG &amp; Neural Signals</x:v>
+        <x:v>Signal Processing; Machine Learning; Time Series &amp; Sequential Data; Computer Vision &amp; Pattern Recognition</x:v>
       </x:c>
       <x:c r="C22" s="14" t="str">
         <x:v>XL</x:v>
@@ -1074,14 +1076,14 @@
       <x:c r="D22" s="14" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="E22" s="14" t="str"/>
+      <x:c r="E22" s="14"/>
       <x:c r="F22" s="14" t="str">
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G22" t="str">
         <x:v>https://2027.ieeeicassp.org/</x:v>
       </x:c>
-      <x:c r="H22" t="str"/>
+      <x:c r="H22"/>
       <x:c r="I22" t="str">
         <x:v>B</x:v>
       </x:c>
@@ -1091,7 +1093,7 @@
       <x:c r="K22" s="16" t="n">
         <x:v>0.429</x:v>
       </x:c>
-      <x:c r="L22" t="n">
+      <x:c r="L22" s="17" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="M22" t="str">
@@ -1101,35 +1103,35 @@
         <x:v>https://signalprocessingsociety.org/index.php/newsletter/2026/06/meet-icassp-2026-organizers-ana-isabel-perez-neira-and-xavier-mestre</x:v>
       </x:c>
     </x:row>
-    <x:row r="23">
+    <x:row r="23" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A23" s="14" t="str">
         <x:v>IEEE MLSP</x:v>
       </x:c>
       <x:c r="B23" s="14" t="str">
-        <x:v>Machine Learning; Signal Processing; Time Series &amp; Sequential Data; EEG/MEG &amp; Neural Signals</x:v>
+        <x:v>Machine Learning; Signal Processing; Time Series &amp; Sequential Data</x:v>
       </x:c>
       <x:c r="C23" s="14" t="str">
-        <x:v>S/M</x:v>
+        <x:v>M</x:v>
       </x:c>
       <x:c r="D23" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E23" s="14" t="str"/>
+      <x:c r="E23" s="14"/>
       <x:c r="F23" s="14" t="str">
         <x:v>Paper-based / workshop-style conference</x:v>
       </x:c>
       <x:c r="G23" t="str">
-        <x:v>https://mlsp26.ieeesps.org/</x:v>
-      </x:c>
-      <x:c r="H23" t="str"/>
-      <x:c r="I23" t="str"/>
-      <x:c r="J23" t="str"/>
-      <x:c r="K23" s="16" t="str"/>
-      <x:c r="L23" t="str"/>
-      <x:c r="M23" t="str"/>
-      <x:c r="N23" t="str"/>
-    </x:row>
-    <x:row r="24">
+        <x:v>https://signalprocessingsociety.org/tags/mlsp-2027</x:v>
+      </x:c>
+      <x:c r="H23"/>
+      <x:c r="I23"/>
+      <x:c r="J23"/>
+      <x:c r="K23" s="16"/>
+      <x:c r="L23" s="17"/>
+      <x:c r="M23"/>
+      <x:c r="N23"/>
+    </x:row>
+    <x:row r="24" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A24" s="14" t="str">
         <x:v>COSYNE</x:v>
       </x:c>
@@ -1142,22 +1144,22 @@
       <x:c r="D24" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E24" s="14" t="str"/>
+      <x:c r="E24" s="14"/>
       <x:c r="F24" s="14" t="str">
         <x:v>Abstract-based / talks highly selective</x:v>
       </x:c>
       <x:c r="G24" t="str">
-        <x:v>https://www.cosyne.org/cosyne-home</x:v>
-      </x:c>
-      <x:c r="H24" t="str"/>
-      <x:c r="I24" t="str"/>
-      <x:c r="J24" t="str"/>
-      <x:c r="K24" s="16" t="str"/>
-      <x:c r="L24" t="str"/>
-      <x:c r="M24" t="str"/>
-      <x:c r="N24" t="str"/>
-    </x:row>
-    <x:row r="25">
+        <x:v>https://www.cosyne.org/</x:v>
+      </x:c>
+      <x:c r="H24"/>
+      <x:c r="I24"/>
+      <x:c r="J24"/>
+      <x:c r="K24" s="16"/>
+      <x:c r="L24" s="17"/>
+      <x:c r="M24"/>
+      <x:c r="N24"/>
+    </x:row>
+    <x:row r="25" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A25" s="14" t="str">
         <x:v>CCN</x:v>
       </x:c>
@@ -1170,22 +1172,22 @@
       <x:c r="D25" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E25" s="14" t="str"/>
+      <x:c r="E25" s="14"/>
       <x:c r="F25" s="14" t="str">
         <x:v>Mixed: proceedings + extended abstracts</x:v>
       </x:c>
       <x:c r="G25" t="str">
-        <x:v>https://2026.ccneuro.org/</x:v>
-      </x:c>
-      <x:c r="H25" t="str"/>
-      <x:c r="I25" t="str"/>
-      <x:c r="J25" t="str"/>
-      <x:c r="K25" s="16" t="str"/>
-      <x:c r="L25" t="str"/>
-      <x:c r="M25" t="str"/>
-      <x:c r="N25" t="str"/>
-    </x:row>
-    <x:row r="26">
+        <x:v>https://2027.ccneuro.org/</x:v>
+      </x:c>
+      <x:c r="H25"/>
+      <x:c r="I25"/>
+      <x:c r="J25"/>
+      <x:c r="K25" s="16"/>
+      <x:c r="L25" s="17"/>
+      <x:c r="M25"/>
+      <x:c r="N25"/>
+    </x:row>
+    <x:row r="26" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A26" s="14" t="str">
         <x:v>Bernstein Conference</x:v>
       </x:c>
@@ -1198,22 +1200,22 @@
       <x:c r="D26" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E26" s="14" t="str"/>
+      <x:c r="E26" s="14"/>
       <x:c r="F26" s="14" t="str">
         <x:v>Abstract-based / talks selective</x:v>
       </x:c>
       <x:c r="G26" t="str">
-        <x:v>https://bernstein-network.de/en/bernstein-conference/</x:v>
-      </x:c>
-      <x:c r="H26" t="str"/>
-      <x:c r="I26" t="str"/>
-      <x:c r="J26" t="str"/>
-      <x:c r="K26" s="16" t="str"/>
-      <x:c r="L26" t="str"/>
-      <x:c r="M26" t="str"/>
-      <x:c r="N26" t="str"/>
-    </x:row>
-    <x:row r="27">
+        <x:v>https://bernstein-network.de/bernstein-conference/bernstein-conference-2027/</x:v>
+      </x:c>
+      <x:c r="H26"/>
+      <x:c r="I26"/>
+      <x:c r="J26"/>
+      <x:c r="K26" s="16"/>
+      <x:c r="L26" s="17"/>
+      <x:c r="M26"/>
+      <x:c r="N26"/>
+    </x:row>
+    <x:row r="27" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A27" s="14" t="str">
         <x:v>CNS*</x:v>
       </x:c>
@@ -1226,22 +1228,22 @@
       <x:c r="D27" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E27" s="14" t="str"/>
+      <x:c r="E27" s="14"/>
       <x:c r="F27" s="14" t="str">
         <x:v>Abstract-based</x:v>
       </x:c>
       <x:c r="G27" t="str">
-        <x:v>https://www.cnsorg.org/cns-2026</x:v>
-      </x:c>
-      <x:c r="H27" t="str"/>
-      <x:c r="I27" t="str"/>
-      <x:c r="J27" t="str"/>
-      <x:c r="K27" s="16" t="str"/>
-      <x:c r="L27" t="str"/>
-      <x:c r="M27" t="str"/>
-      <x:c r="N27" t="str"/>
-    </x:row>
-    <x:row r="28">
+        <x:v>https://www.cnsorg.org/</x:v>
+      </x:c>
+      <x:c r="H27"/>
+      <x:c r="I27"/>
+      <x:c r="J27"/>
+      <x:c r="K27" s="16"/>
+      <x:c r="L27" s="17"/>
+      <x:c r="M27"/>
+      <x:c r="N27"/>
+    </x:row>
+    <x:row r="28" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A28" s="14" t="str">
         <x:v>OHBM</x:v>
       </x:c>
@@ -1249,27 +1251,27 @@
         <x:v>Neuroimaging &amp; Brain Mapping; EEG/MEG &amp; Neural Signals; Healthcare &amp; Clinical AI; Computational Neuroscience</x:v>
       </x:c>
       <x:c r="C28" s="14" t="str">
-        <x:v>L/XL</x:v>
+        <x:v>XL</x:v>
       </x:c>
       <x:c r="D28" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E28" s="14" t="str"/>
+      <x:c r="E28" s="14"/>
       <x:c r="F28" s="14" t="str">
         <x:v>Abstract-based / talks selective</x:v>
       </x:c>
       <x:c r="G28" t="str">
         <x:v>https://humanbrainmapping.org/ohbm-2027/</x:v>
       </x:c>
-      <x:c r="H28" t="str"/>
-      <x:c r="I28" t="str"/>
-      <x:c r="J28" t="str"/>
-      <x:c r="K28" s="16" t="str"/>
-      <x:c r="L28" t="str"/>
-      <x:c r="M28" t="str"/>
-      <x:c r="N28" t="str"/>
-    </x:row>
-    <x:row r="29">
+      <x:c r="H28"/>
+      <x:c r="I28"/>
+      <x:c r="J28"/>
+      <x:c r="K28" s="16"/>
+      <x:c r="L28" s="17"/>
+      <x:c r="M28"/>
+      <x:c r="N28"/>
+    </x:row>
+    <x:row r="29" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A29" s="14" t="str">
         <x:v>IEEE NER</x:v>
       </x:c>
@@ -1282,22 +1284,22 @@
       <x:c r="D29" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E29" s="14" t="str"/>
+      <x:c r="E29" s="14"/>
       <x:c r="F29" s="14" t="str">
         <x:v>Paper-based / engineering-focused</x:v>
       </x:c>
       <x:c r="G29" t="str">
         <x:v>https://ieee-ner.org/</x:v>
       </x:c>
-      <x:c r="H29" t="str"/>
-      <x:c r="I29" t="str"/>
-      <x:c r="J29" t="str"/>
-      <x:c r="K29" s="16" t="str"/>
-      <x:c r="L29" t="str"/>
-      <x:c r="M29" t="str"/>
-      <x:c r="N29" t="str"/>
-    </x:row>
-    <x:row r="30">
+      <x:c r="H29"/>
+      <x:c r="I29"/>
+      <x:c r="J29"/>
+      <x:c r="K29" s="16"/>
+      <x:c r="L29" s="17"/>
+      <x:c r="M29"/>
+      <x:c r="N29"/>
+    </x:row>
+    <x:row r="30" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A30" s="14" t="str">
         <x:v>International BCI Meeting</x:v>
       </x:c>
@@ -1305,27 +1307,27 @@
         <x:v>BCI &amp; Neurotechnology; EEG/MEG &amp; Neural Signals; Computational Neuroscience; Human-AI Interaction &amp; Deployment</x:v>
       </x:c>
       <x:c r="C30" s="14" t="str">
-        <x:v>S/M</x:v>
+        <x:v>M</x:v>
       </x:c>
       <x:c r="D30" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E30" s="14" t="str"/>
+      <x:c r="E30" s="14"/>
       <x:c r="F30" s="14" t="str">
         <x:v>Abstract/community-based</x:v>
       </x:c>
       <x:c r="G30" t="str">
         <x:v>https://bcisociety.org/bci-meeting/</x:v>
       </x:c>
-      <x:c r="H30" t="str"/>
-      <x:c r="I30" t="str"/>
-      <x:c r="J30" t="str"/>
-      <x:c r="K30" s="16" t="str"/>
-      <x:c r="L30" t="str"/>
-      <x:c r="M30" t="str"/>
-      <x:c r="N30" t="str"/>
-    </x:row>
-    <x:row r="31">
+      <x:c r="H30"/>
+      <x:c r="I30"/>
+      <x:c r="J30"/>
+      <x:c r="K30" s="16"/>
+      <x:c r="L30" s="17"/>
+      <x:c r="M30"/>
+      <x:c r="N30"/>
+    </x:row>
+    <x:row r="31" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A31" s="14" t="str">
         <x:v>BIOMAG</x:v>
       </x:c>
@@ -1338,27 +1340,27 @@
       <x:c r="D31" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E31" s="14" t="str"/>
+      <x:c r="E31" s="14"/>
       <x:c r="F31" s="14" t="str">
         <x:v>Abstract-based / specialist venue</x:v>
       </x:c>
       <x:c r="G31" t="str">
         <x:v>https://mm.scimeeting.cn/en/web/index/31426</x:v>
       </x:c>
-      <x:c r="H31" t="str"/>
-      <x:c r="I31" t="str"/>
-      <x:c r="J31" t="str"/>
-      <x:c r="K31" s="16" t="str"/>
-      <x:c r="L31" t="str"/>
-      <x:c r="M31" t="str"/>
-      <x:c r="N31" t="str"/>
-    </x:row>
-    <x:row r="32">
+      <x:c r="H31"/>
+      <x:c r="I31"/>
+      <x:c r="J31"/>
+      <x:c r="K31" s="16"/>
+      <x:c r="L31" s="17"/>
+      <x:c r="M31"/>
+      <x:c r="N31"/>
+    </x:row>
+    <x:row r="32" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A32" s="14" t="str">
         <x:v>ACM FAccT</x:v>
       </x:c>
       <x:c r="B32" s="14" t="str">
-        <x:v>Fairness &amp; Responsible AI; Explainability &amp; Interpretability; Healthcare &amp; Clinical AI; Human-AI Interaction &amp; Deployment</x:v>
+        <x:v>Fairness &amp; Responsible AI; Explainability &amp; Interpretability; Ethics &amp; Governance; Privacy-preserving ML</x:v>
       </x:c>
       <x:c r="C32" s="14" t="str">
         <x:v>M</x:v>
@@ -1366,30 +1368,30 @@
       <x:c r="D32" s="14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E32" s="14" t="str"/>
+      <x:c r="E32" s="14"/>
       <x:c r="F32" s="14" t="str">
         <x:v>Paper-based / interdisciplinary</x:v>
       </x:c>
       <x:c r="G32" t="str">
         <x:v>https://facctconference.org/</x:v>
       </x:c>
-      <x:c r="H32" t="str"/>
-      <x:c r="I32" t="str"/>
-      <x:c r="J32" t="str"/>
-      <x:c r="K32" s="16" t="str"/>
-      <x:c r="L32" t="str"/>
-      <x:c r="M32" t="str"/>
-      <x:c r="N32" t="str"/>
-    </x:row>
-    <x:row r="33">
+      <x:c r="H32"/>
+      <x:c r="I32"/>
+      <x:c r="J32"/>
+      <x:c r="K32" s="16"/>
+      <x:c r="L32" s="17"/>
+      <x:c r="M32"/>
+      <x:c r="N32"/>
+    </x:row>
+    <x:row r="33" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A33" s="14" t="str">
         <x:v>AIES</x:v>
       </x:c>
       <x:c r="B33" s="14" t="str">
-        <x:v>Fairness &amp; Responsible AI; Human-AI Interaction &amp; Deployment; Machine Learning; Healthcare &amp; Clinical AI</x:v>
+        <x:v>Ethics &amp; Governance; Fairness &amp; Responsible AI; Explainability &amp; Interpretability; Robustness &amp; Safety</x:v>
       </x:c>
       <x:c r="C33" s="14" t="str">
-        <x:v>S/M</x:v>
+        <x:v>M</x:v>
       </x:c>
       <x:c r="D33" s="14" t="str">
         <x:v>Moderate</x:v>
@@ -1406,12 +1408,12 @@
       <x:c r="H33" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/2354/</x:v>
       </x:c>
-      <x:c r="I33" t="str"/>
-      <x:c r="J33" t="str"/>
+      <x:c r="I33"/>
+      <x:c r="J33"/>
       <x:c r="K33" s="16" t="n">
         <x:v>0.318</x:v>
       </x:c>
-      <x:c r="L33" t="n">
+      <x:c r="L33" s="17" t="n">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="M33" t="str">
@@ -1421,12 +1423,12 @@
         <x:v>https://aaai.org/wp-content/uploads/2025/10/AIES-2025-Program-10.14.pdf</x:v>
       </x:c>
     </x:row>
-    <x:row r="34">
+    <x:row r="34" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A34" s="14" t="str">
         <x:v>CHI</x:v>
       </x:c>
       <x:c r="B34" s="14" t="str">
-        <x:v>Human-AI Interaction &amp; Deployment; Explainability &amp; Interpretability; Fairness &amp; Responsible AI; Healthcare &amp; Clinical AI</x:v>
+        <x:v>Human-AI Interaction &amp; Deployment; Explainability &amp; Interpretability; Fairness &amp; Responsible AI</x:v>
       </x:c>
       <x:c r="C34" s="14" t="str">
         <x:v>XL</x:v>
@@ -1455,7 +1457,7 @@
       <x:c r="K34" s="16" t="n">
         <x:v>0.249</x:v>
       </x:c>
-      <x:c r="L34" t="n">
+      <x:c r="L34" s="17" t="n">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="M34" t="str">
@@ -1465,11 +1467,11 @@
         <x:v>https://chi2025.acm.org/chi-2025-papers-track-post-pc-outcomes-report/</x:v>
       </x:c>
     </x:row>
-    <x:row r="35">
+    <x:row r="35" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A35" t="str">
         <x:v>AAAI</x:v>
       </x:c>
-      <x:c r="B35" t="str">
+      <x:c r="B35" s="12" t="str">
         <x:v>Machine Learning; Deep Representation Learning; Data Mining &amp; Data Science; Fairness &amp; Responsible AI</x:v>
       </x:c>
       <x:c r="C35" t="str">
@@ -1499,7 +1501,7 @@
       <x:c r="K35" s="16" t="n">
         <x:v>0.175</x:v>
       </x:c>
-      <x:c r="L35" t="n">
+      <x:c r="L35" s="17" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="M35" t="str">
@@ -1522,20 +1524,20 @@
       <x:c r="D36" s="12" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E36" s="12" t="str"/>
+      <x:c r="E36" s="12"/>
       <x:c r="F36" s="12" t="str">
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G36" t="str">
         <x:v>https://2026.ijcai.org/</x:v>
       </x:c>
-      <x:c r="H36" t="str"/>
-      <x:c r="I36" t="str"/>
-      <x:c r="J36" t="str"/>
-      <x:c r="K36" s="16" t="str"/>
-      <x:c r="L36" t="str"/>
-      <x:c r="M36" t="str"/>
-      <x:c r="N36" t="str"/>
+      <x:c r="H36"/>
+      <x:c r="I36"/>
+      <x:c r="J36"/>
+      <x:c r="K36" s="16"/>
+      <x:c r="L36" s="17"/>
+      <x:c r="M36"/>
+      <x:c r="N36"/>
     </x:row>
     <x:row r="37" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A37" s="12" t="str">
@@ -1571,7 +1573,7 @@
       <x:c r="K37" s="16" t="n">
         <x:v>0.14</x:v>
       </x:c>
-      <x:c r="L37" t="n">
+      <x:c r="L37" s="17" t="n">
         <x:v>2024</x:v>
       </x:c>
       <x:c r="M37" t="str">
@@ -1612,17 +1614,17 @@
       <x:c r="J38" t="str">
         <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=58</x:v>
       </x:c>
-      <x:c r="K38" s="16" t="str"/>
-      <x:c r="L38" t="str"/>
-      <x:c r="M38" t="str"/>
-      <x:c r="N38" t="str"/>
+      <x:c r="K38" s="16"/>
+      <x:c r="L38" s="17"/>
+      <x:c r="M38"/>
+      <x:c r="N38"/>
     </x:row>
     <x:row r="39" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A39" s="12" t="str">
         <x:v>ACML</x:v>
       </x:c>
       <x:c r="B39" s="12" t="str">
-        <x:v>Machine Learning; Deep Representation Learning; Learning Theory &amp; Statistical Foundations; Explainability &amp; Interpretability</x:v>
+        <x:v>Machine Learning; Learning Theory &amp; Statistical Foundations; Explainability &amp; Interpretability; Robustness &amp; Safety</x:v>
       </x:c>
       <x:c r="C39" s="12" t="str">
         <x:v>L</x:v>
@@ -1651,7 +1653,7 @@
       <x:c r="K39" s="16" t="n">
         <x:v>0.29</x:v>
       </x:c>
-      <x:c r="L39" t="n">
+      <x:c r="L39" s="17" t="n">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="M39" t="str">
@@ -1692,17 +1694,17 @@
       <x:c r="J40" t="str">
         <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=37</x:v>
       </x:c>
-      <x:c r="K40" s="16" t="str"/>
-      <x:c r="L40" t="str"/>
-      <x:c r="M40" t="str"/>
-      <x:c r="N40" t="str"/>
+      <x:c r="K40" s="16"/>
+      <x:c r="L40" s="17"/>
+      <x:c r="M40"/>
+      <x:c r="N40"/>
     </x:row>
     <x:row r="41" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A41" s="12" t="str">
         <x:v>CIKM</x:v>
       </x:c>
       <x:c r="B41" s="12" t="str">
-        <x:v>Data Mining &amp; Data Science; Machine Learning; Time Series &amp; Sequential Data; Human-AI Interaction &amp; Deployment</x:v>
+        <x:v>Data Mining &amp; Data Science; Machine Learning; Natural Language Processing &amp; LLMs; Human-AI Interaction &amp; Deployment</x:v>
       </x:c>
       <x:c r="C41" s="12" t="str">
         <x:v>XL</x:v>
@@ -1731,7 +1733,7 @@
       <x:c r="K41" s="16" t="n">
         <x:v>0.27</x:v>
       </x:c>
-      <x:c r="L41" t="n">
+      <x:c r="L41" s="17" t="n">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="M41" t="str">
@@ -1772,8 +1774,8 @@
       <x:c r="J42" t="str">
         <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=36</x:v>
       </x:c>
-      <x:c r="K42" s="16" t="str"/>
-      <x:c r="L42" t="n">
+      <x:c r="K42" s="16"/>
+      <x:c r="L42" s="17" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="M42" t="str">
@@ -1788,7 +1790,7 @@
         <x:v>IEEE BigData</x:v>
       </x:c>
       <x:c r="B43" s="12" t="str">
-        <x:v>Data Mining &amp; Data Science; Machine Learning; Time Series &amp; Sequential Data; Healthcare &amp; Clinical AI</x:v>
+        <x:v>Data Mining &amp; Data Science; Machine Learning; Time Series &amp; Sequential Data; Federated &amp; Distributed Learning</x:v>
       </x:c>
       <x:c r="C43" s="12" t="str">
         <x:v>L</x:v>
@@ -1808,12 +1810,12 @@
       <x:c r="H43" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/2274/</x:v>
       </x:c>
-      <x:c r="I43" t="str"/>
-      <x:c r="J43" t="str"/>
-      <x:c r="K43" s="16" t="str"/>
-      <x:c r="L43" t="str"/>
-      <x:c r="M43" t="str"/>
-      <x:c r="N43" t="str"/>
+      <x:c r="I43"/>
+      <x:c r="J43"/>
+      <x:c r="K43" s="16"/>
+      <x:c r="L43" s="17"/>
+      <x:c r="M43"/>
+      <x:c r="N43"/>
     </x:row>
     <x:row r="44" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A44" s="12" t="str">
@@ -1840,12 +1842,12 @@
       <x:c r="H44" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/2191/</x:v>
       </x:c>
-      <x:c r="I44" t="str"/>
-      <x:c r="J44" t="str"/>
-      <x:c r="K44" s="16" t="str"/>
-      <x:c r="L44" t="str"/>
-      <x:c r="M44" t="str"/>
-      <x:c r="N44" t="str"/>
+      <x:c r="I44"/>
+      <x:c r="J44"/>
+      <x:c r="K44" s="16"/>
+      <x:c r="L44" s="17"/>
+      <x:c r="M44"/>
+      <x:c r="N44"/>
     </x:row>
     <x:row r="45" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A45" s="12" t="str">
@@ -1881,7 +1883,7 @@
       <x:c r="K45" s="16" t="n">
         <x:v>0.3846</x:v>
       </x:c>
-      <x:c r="L45" t="n">
+      <x:c r="L45" s="17" t="n">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="M45" t="str">
@@ -1922,10 +1924,10 @@
       <x:c r="J46" t="str">
         <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=37</x:v>
       </x:c>
-      <x:c r="K46" s="16" t="str"/>
-      <x:c r="L46" t="str"/>
-      <x:c r="M46" t="str"/>
-      <x:c r="N46" t="str"/>
+      <x:c r="K46" s="16"/>
+      <x:c r="L46" s="17"/>
+      <x:c r="M46"/>
+      <x:c r="N46"/>
     </x:row>
     <x:row r="47" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A47" s="12" t="str">
@@ -1958,10 +1960,10 @@
       <x:c r="J47" t="str">
         <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=60</x:v>
       </x:c>
-      <x:c r="K47" s="16" t="str"/>
-      <x:c r="L47" t="str"/>
-      <x:c r="M47" t="str"/>
-      <x:c r="N47" t="str"/>
+      <x:c r="K47" s="16"/>
+      <x:c r="L47" s="17"/>
+      <x:c r="M47"/>
+      <x:c r="N47"/>
     </x:row>
     <x:row r="48" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A48" s="12" t="str">
@@ -1994,10 +1996,10 @@
       <x:c r="J48" t="str">
         <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=59</x:v>
       </x:c>
-      <x:c r="K48" s="16" t="str"/>
-      <x:c r="L48" t="str"/>
-      <x:c r="M48" t="str"/>
-      <x:c r="N48" t="str"/>
+      <x:c r="K48" s="16"/>
+      <x:c r="L48" s="17"/>
+      <x:c r="M48"/>
+      <x:c r="N48"/>
     </x:row>
     <x:row r="49" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A49" s="12" t="str">
@@ -2024,12 +2026,12 @@
       <x:c r="H49" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/512/</x:v>
       </x:c>
-      <x:c r="I49" t="str"/>
-      <x:c r="J49" t="str"/>
-      <x:c r="K49" s="16" t="str"/>
-      <x:c r="L49" t="str"/>
-      <x:c r="M49" t="str"/>
-      <x:c r="N49" t="str"/>
+      <x:c r="I49"/>
+      <x:c r="J49"/>
+      <x:c r="K49" s="16"/>
+      <x:c r="L49" s="17"/>
+      <x:c r="M49"/>
+      <x:c r="N49"/>
     </x:row>
     <x:row r="50" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A50" s="12" t="str">
@@ -2062,17 +2064,17 @@
       <x:c r="J50" t="str">
         <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=60</x:v>
       </x:c>
-      <x:c r="K50" s="16" t="str"/>
-      <x:c r="L50" t="str"/>
-      <x:c r="M50" t="str"/>
-      <x:c r="N50" t="str"/>
+      <x:c r="K50" s="16"/>
+      <x:c r="L50" s="17"/>
+      <x:c r="M50"/>
+      <x:c r="N50"/>
     </x:row>
     <x:row r="51" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A51" s="12" t="str">
         <x:v>ICPR</x:v>
       </x:c>
       <x:c r="B51" s="12" t="str">
-        <x:v>Machine Learning; Deep Representation Learning; Signal Processing; Biomedical Imaging</x:v>
+        <x:v>Computer Vision &amp; Pattern Recognition; Machine Learning; Deep Representation Learning; Biomedical Imaging</x:v>
       </x:c>
       <x:c r="C51" s="12" t="str">
         <x:v>XL</x:v>
@@ -2101,7 +2103,7 @@
       <x:c r="K51" s="16" t="n">
         <x:v>0.4426</x:v>
       </x:c>
-      <x:c r="L51" t="n">
+      <x:c r="L51" s="17" t="n">
         <x:v>2024</x:v>
       </x:c>
       <x:c r="M51" t="str">
@@ -2116,7 +2118,7 @@
         <x:v>ACPR</x:v>
       </x:c>
       <x:c r="B52" s="12" t="str">
-        <x:v>Machine Learning; Deep Representation Learning; Signal Processing; Biomedical Imaging</x:v>
+        <x:v>Computer Vision &amp; Pattern Recognition; Machine Learning; Deep Representation Learning</x:v>
       </x:c>
       <x:c r="C52" s="12" t="str">
         <x:v>M</x:v>
@@ -2124,20 +2126,20 @@
       <x:c r="D52" s="12" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="E52" s="12" t="str"/>
+      <x:c r="E52" s="12"/>
       <x:c r="F52" s="12" t="str">
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G52" t="str">
         <x:v>https://iapr.org/</x:v>
       </x:c>
-      <x:c r="H52" t="str"/>
-      <x:c r="I52" t="str"/>
-      <x:c r="J52" t="str"/>
+      <x:c r="H52"/>
+      <x:c r="I52"/>
+      <x:c r="J52"/>
       <x:c r="K52" s="16" t="n">
         <x:v>0.5085000000000001</x:v>
       </x:c>
-      <x:c r="L52" t="n">
+      <x:c r="L52" s="17" t="n">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="M52" t="str">
@@ -2152,7 +2154,7 @@
         <x:v>S+SSPR</x:v>
       </x:c>
       <x:c r="B53" s="12" t="str">
-        <x:v>Machine Learning; Deep Representation Learning; Data Mining &amp; Data Science; Signal Processing</x:v>
+        <x:v>Computer Vision &amp; Pattern Recognition; Machine Learning; Learning Theory &amp; Statistical Foundations</x:v>
       </x:c>
       <x:c r="C53" s="12" t="str">
         <x:v>M</x:v>
@@ -2160,20 +2162,20 @@
       <x:c r="D53" s="12" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E53" s="12" t="str"/>
+      <x:c r="E53" s="12"/>
       <x:c r="F53" s="12" t="str">
         <x:v>Paper-based / workshop-style conference</x:v>
       </x:c>
       <x:c r="G53" t="str">
         <x:v>https://ssspr2026.inf.unibe.ch/</x:v>
       </x:c>
-      <x:c r="H53" t="str"/>
-      <x:c r="I53" t="str"/>
-      <x:c r="J53" t="str"/>
-      <x:c r="K53" s="16" t="str"/>
-      <x:c r="L53" t="str"/>
-      <x:c r="M53" t="str"/>
-      <x:c r="N53" t="str"/>
+      <x:c r="H53"/>
+      <x:c r="I53"/>
+      <x:c r="J53"/>
+      <x:c r="K53" s="16"/>
+      <x:c r="L53" s="17"/>
+      <x:c r="M53"/>
+      <x:c r="N53"/>
     </x:row>
     <x:row r="54" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A54" s="12" t="str">
@@ -2200,19 +2202,19 @@
       <x:c r="H54" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/1122/</x:v>
       </x:c>
-      <x:c r="I54" t="str"/>
-      <x:c r="J54" t="str"/>
-      <x:c r="K54" s="16" t="str"/>
-      <x:c r="L54" t="str"/>
-      <x:c r="M54" t="str"/>
-      <x:c r="N54" t="str"/>
+      <x:c r="I54"/>
+      <x:c r="J54"/>
+      <x:c r="K54" s="16"/>
+      <x:c r="L54" s="17"/>
+      <x:c r="M54"/>
+      <x:c r="N54"/>
     </x:row>
     <x:row r="55" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A55" s="12" t="str">
         <x:v>IEEE SSCI</x:v>
       </x:c>
       <x:c r="B55" s="12" t="str">
-        <x:v>Machine Learning; Deep Representation Learning; Learning Theory &amp; Statistical Foundations; Fairness &amp; Responsible AI</x:v>
+        <x:v>Machine Learning; Deep Representation Learning; Reinforcement Learning; Control &amp; Robotics</x:v>
       </x:c>
       <x:c r="C55" s="12" t="str">
         <x:v>L</x:v>
@@ -2220,20 +2222,20 @@
       <x:c r="D55" s="12" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E55" s="12" t="str"/>
+      <x:c r="E55" s="12"/>
       <x:c r="F55" s="12" t="str">
         <x:v>Paper-based / symposium series</x:v>
       </x:c>
       <x:c r="G55" t="str">
         <x:v>https://ssci2027generalchairs.github.io/ssci-2027/</x:v>
       </x:c>
-      <x:c r="H55" t="str"/>
-      <x:c r="I55" t="str"/>
-      <x:c r="J55" t="str"/>
-      <x:c r="K55" s="16" t="str"/>
-      <x:c r="L55" t="str"/>
-      <x:c r="M55" t="str"/>
-      <x:c r="N55" t="str"/>
+      <x:c r="H55"/>
+      <x:c r="I55"/>
+      <x:c r="J55"/>
+      <x:c r="K55" s="16"/>
+      <x:c r="L55" s="17"/>
+      <x:c r="M55"/>
+      <x:c r="N55"/>
     </x:row>
     <x:row r="56" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A56" s="12" t="str">
@@ -2260,12 +2262,12 @@
       <x:c r="H56" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/1093/</x:v>
       </x:c>
-      <x:c r="I56" t="str"/>
-      <x:c r="J56" t="str"/>
-      <x:c r="K56" s="16" t="str"/>
-      <x:c r="L56" t="str"/>
-      <x:c r="M56" t="str"/>
-      <x:c r="N56" t="str"/>
+      <x:c r="I56"/>
+      <x:c r="J56"/>
+      <x:c r="K56" s="16"/>
+      <x:c r="L56" s="17"/>
+      <x:c r="M56"/>
+      <x:c r="N56"/>
     </x:row>
     <x:row r="57" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A57" s="12" t="str">
@@ -2280,27 +2282,27 @@
       <x:c r="D57" s="12" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E57" s="12" t="str"/>
+      <x:c r="E57" s="12"/>
       <x:c r="F57" s="12" t="str">
         <x:v>Paper-based / Springer proceedings</x:v>
       </x:c>
       <x:c r="G57" t="str">
         <x:v>https://ais2026.icas.events/</x:v>
       </x:c>
-      <x:c r="H57" t="str"/>
-      <x:c r="I57" t="str"/>
-      <x:c r="J57" t="str"/>
-      <x:c r="K57" s="16" t="str"/>
-      <x:c r="L57" t="str"/>
-      <x:c r="M57" t="str"/>
-      <x:c r="N57" t="str"/>
+      <x:c r="H57"/>
+      <x:c r="I57"/>
+      <x:c r="J57"/>
+      <x:c r="K57" s="16"/>
+      <x:c r="L57" s="17"/>
+      <x:c r="M57"/>
+      <x:c r="N57"/>
     </x:row>
     <x:row r="58" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A58" s="12" t="str">
         <x:v>EUSIPCO</x:v>
       </x:c>
       <x:c r="B58" s="12" t="str">
-        <x:v>Signal Processing; Machine Learning; Time Series &amp; Sequential Data; EEG/MEG &amp; Neural Signals</x:v>
+        <x:v>Signal Processing; Machine Learning; Time Series &amp; Sequential Data; Computer Vision &amp; Pattern Recognition</x:v>
       </x:c>
       <x:c r="C58" s="12" t="str">
         <x:v>XL</x:v>
@@ -2308,20 +2310,20 @@
       <x:c r="D58" s="12" t="str">
         <x:v>Very high</x:v>
       </x:c>
-      <x:c r="E58" s="12" t="str"/>
+      <x:c r="E58" s="12"/>
       <x:c r="F58" s="12" t="str">
         <x:v>Paper-based</x:v>
       </x:c>
       <x:c r="G58" t="str">
-        <x:v>https://eusipco2026.org/</x:v>
-      </x:c>
-      <x:c r="H58" t="str"/>
-      <x:c r="I58" t="str"/>
-      <x:c r="J58" t="str"/>
+        <x:v>https://eusipco2027.de/</x:v>
+      </x:c>
+      <x:c r="H58"/>
+      <x:c r="I58"/>
+      <x:c r="J58"/>
       <x:c r="K58" s="16" t="n">
         <x:v>0.664</x:v>
       </x:c>
-      <x:c r="L58" t="n">
+      <x:c r="L58" s="17" t="n">
         <x:v>2024</x:v>
       </x:c>
       <x:c r="M58" t="str">
@@ -2344,22 +2346,22 @@
       <x:c r="D59" s="12" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E59" s="12" t="str"/>
+      <x:c r="E59" s="12"/>
       <x:c r="F59" s="12" t="str">
         <x:v>Paper-based / specialist workshop</x:v>
       </x:c>
       <x:c r="G59" t="str">
         <x:v>https://ssp27.ieeesps.org/</x:v>
       </x:c>
-      <x:c r="H59" t="str"/>
-      <x:c r="I59" t="str"/>
-      <x:c r="J59" t="str"/>
-      <x:c r="K59" s="16" t="str"/>
-      <x:c r="L59" t="str"/>
-      <x:c r="M59" t="str"/>
-      <x:c r="N59" t="str"/>
-    </x:row>
-    <x:row r="60">
+      <x:c r="H59"/>
+      <x:c r="I59"/>
+      <x:c r="J59"/>
+      <x:c r="K59" s="16"/>
+      <x:c r="L59" s="17"/>
+      <x:c r="M59"/>
+      <x:c r="N59"/>
+    </x:row>
+    <x:row r="60" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A60" s="12" t="str">
         <x:v>AALTD</x:v>
       </x:c>
@@ -2372,20 +2374,20 @@
       <x:c r="D60" s="12" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E60" s="12" t="str"/>
+      <x:c r="E60" s="12"/>
       <x:c r="F60" s="12" t="str">
         <x:v>Workshop / paper-based</x:v>
       </x:c>
       <x:c r="G60" t="str">
         <x:v>https://ecml-aaltd.github.io/aaltd2026/</x:v>
       </x:c>
-      <x:c r="H60" t="str"/>
-      <x:c r="I60" t="str"/>
-      <x:c r="J60" t="str"/>
-      <x:c r="K60" s="16" t="str"/>
-      <x:c r="L60" t="str"/>
-      <x:c r="M60" t="str"/>
-      <x:c r="N60" t="str"/>
+      <x:c r="H60"/>
+      <x:c r="I60"/>
+      <x:c r="J60"/>
+      <x:c r="K60" s="16"/>
+      <x:c r="L60" s="17"/>
+      <x:c r="M60"/>
+      <x:c r="N60"/>
     </x:row>
     <x:row r="61" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A61" s="12" t="str">
@@ -2400,30 +2402,30 @@
       <x:c r="D61" s="12" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E61" s="12" t="str"/>
+      <x:c r="E61" s="12"/>
       <x:c r="F61" s="12" t="str">
         <x:v>Paper-based / forecasting-focused</x:v>
       </x:c>
       <x:c r="G61" t="str">
         <x:v>https://itise.ugr.es/index.html</x:v>
       </x:c>
-      <x:c r="H61" t="str"/>
-      <x:c r="I61" t="str"/>
-      <x:c r="J61" t="str"/>
-      <x:c r="K61" s="16" t="str"/>
-      <x:c r="L61" t="str"/>
-      <x:c r="M61" t="str"/>
-      <x:c r="N61" t="str"/>
+      <x:c r="H61"/>
+      <x:c r="I61"/>
+      <x:c r="J61"/>
+      <x:c r="K61" s="16"/>
+      <x:c r="L61" s="17"/>
+      <x:c r="M61"/>
+      <x:c r="N61"/>
     </x:row>
     <x:row r="62" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A62" s="12" t="str">
         <x:v>EACL</x:v>
       </x:c>
       <x:c r="B62" s="12" t="str">
-        <x:v>Natural Language Processing &amp; LLMs; Machine Learning; Deep Representation Learning; Fairness &amp; Responsible AI; Human-AI Interaction &amp; Deployment</x:v>
+        <x:v>Natural Language Processing &amp; LLMs; Machine Learning; Deep Representation Learning; Human-AI Interaction &amp; Deployment</x:v>
       </x:c>
       <x:c r="C62" s="12" t="str">
-        <x:v>L/XL</x:v>
+        <x:v>XL</x:v>
       </x:c>
       <x:c r="D62" s="12" t="str">
         <x:v>Low</x:v>
@@ -2440,12 +2442,12 @@
       <x:c r="H62" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/468/</x:v>
       </x:c>
-      <x:c r="I62" t="str"/>
-      <x:c r="J62" t="str"/>
+      <x:c r="I62"/>
+      <x:c r="J62"/>
       <x:c r="K62" s="16" t="n">
         <x:v>0.203</x:v>
       </x:c>
-      <x:c r="L62" t="n">
+      <x:c r="L62" s="17" t="n">
         <x:v>2024</x:v>
       </x:c>
       <x:c r="M62" t="str">
@@ -2455,11 +2457,11 @@
         <x:v>https://2024.eacl.org/downloads/handbook.pdf</x:v>
       </x:c>
     </x:row>
-    <x:row r="63">
+    <x:row r="63" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A63" t="str">
         <x:v>AIME</x:v>
       </x:c>
-      <x:c r="B63" t="str">
+      <x:c r="B63" s="12" t="str">
         <x:v>Healthcare &amp; Clinical AI; Machine Learning; Biomedical Imaging; Probabilistic, Causal &amp; Uncertainty ML</x:v>
       </x:c>
       <x:c r="C63" t="str">
@@ -2480,18 +2482,18 @@
       <x:c r="H63" t="str">
         <x:v>https://portal.core.edu.au/conf-ranks/151/</x:v>
       </x:c>
-      <x:c r="I63" t="str"/>
-      <x:c r="J63" t="str"/>
-      <x:c r="K63" s="16" t="str"/>
-      <x:c r="L63" t="str"/>
-      <x:c r="M63" t="str"/>
-      <x:c r="N63" t="str"/>
-    </x:row>
-    <x:row r="64">
+      <x:c r="I63"/>
+      <x:c r="J63"/>
+      <x:c r="K63" s="16"/>
+      <x:c r="L63" s="17"/>
+      <x:c r="M63"/>
+      <x:c r="N63"/>
+    </x:row>
+    <x:row r="64" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A64" t="str">
         <x:v>FMTS @ NeurIPS</x:v>
       </x:c>
-      <x:c r="B64" t="str">
+      <x:c r="B64" s="12" t="str">
         <x:v>Time Series &amp; Sequential Data; Machine Learning; Deep Representation Learning; Probabilistic, Causal &amp; Uncertainty ML</x:v>
       </x:c>
       <x:c r="C64" t="str">
@@ -2500,25 +2502,249 @@
       <x:c r="D64" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="E64" t="str"/>
+      <x:c r="E64"/>
       <x:c r="F64" t="str">
         <x:v>Workshop / non-archival short paper</x:v>
       </x:c>
       <x:c r="G64" t="str">
         <x:v>https://fmts-workshop.github.io/</x:v>
       </x:c>
-      <x:c r="H64" t="str"/>
-      <x:c r="I64" t="str"/>
-      <x:c r="J64" t="str"/>
-      <x:c r="K64" s="16" t="str"/>
-      <x:c r="L64" t="str"/>
-      <x:c r="M64" t="str"/>
-      <x:c r="N64" t="str"/>
+      <x:c r="H64"/>
+      <x:c r="I64"/>
+      <x:c r="J64"/>
+      <x:c r="K64" s="16"/>
+      <x:c r="L64" s="17"/>
+      <x:c r="M64"/>
+      <x:c r="N64"/>
+    </x:row>
+    <x:row r="65" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A65" t="str">
+        <x:v>L4DC</x:v>
+      </x:c>
+      <x:c r="B65" s="12" t="str">
+        <x:v>Machine Learning; Control &amp; Robotics; System Identification &amp; Data-driven Dynamics; Reinforcement Learning</x:v>
+      </x:c>
+      <x:c r="C65" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D65" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E65"/>
+      <x:c r="F65" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G65" t="str">
+        <x:v>https://l4dc2027.control.ee.ethz.ch/home</x:v>
+      </x:c>
+      <x:c r="H65"/>
+      <x:c r="I65"/>
+      <x:c r="J65"/>
+      <x:c r="K65" s="16"/>
+      <x:c r="L65" s="17"/>
+      <x:c r="M65"/>
+      <x:c r="N65"/>
+    </x:row>
+    <x:row r="66" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A66" t="str">
+        <x:v>IFAC SYSID</x:v>
+      </x:c>
+      <x:c r="B66" s="12" t="str">
+        <x:v>System Identification &amp; Data-driven Dynamics; Control &amp; Robotics; Time Series &amp; Sequential Data; Machine Learning</x:v>
+      </x:c>
+      <x:c r="C66" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D66" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E66"/>
+      <x:c r="F66" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G66" t="str">
+        <x:v>https://conferences.ifac-control.org/sysid2027/</x:v>
+      </x:c>
+      <x:c r="H66"/>
+      <x:c r="I66"/>
+      <x:c r="J66"/>
+      <x:c r="K66" s="16"/>
+      <x:c r="L66" s="17"/>
+      <x:c r="M66"/>
+      <x:c r="N66"/>
+    </x:row>
+    <x:row r="67" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A67" t="str">
+        <x:v>ACC</x:v>
+      </x:c>
+      <x:c r="B67" s="12" t="str">
+        <x:v>Control &amp; Robotics; System Identification &amp; Data-driven Dynamics; Reinforcement Learning</x:v>
+      </x:c>
+      <x:c r="C67" t="str">
+        <x:v>XL</x:v>
+      </x:c>
+      <x:c r="D67" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E67"/>
+      <x:c r="F67" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G67" t="str">
+        <x:v>https://acc2027.a2c2.org/</x:v>
+      </x:c>
+      <x:c r="H67"/>
+      <x:c r="I67"/>
+      <x:c r="J67"/>
+      <x:c r="K67" s="16"/>
+      <x:c r="L67" s="17"/>
+      <x:c r="M67"/>
+      <x:c r="N67"/>
+    </x:row>
+    <x:row r="68" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A68" t="str">
+        <x:v>IEEE CDC</x:v>
+      </x:c>
+      <x:c r="B68" s="12" t="str">
+        <x:v>Control &amp; Robotics; System Identification &amp; Data-driven Dynamics; Nonlinear Dynamics &amp; Chaos; Reinforcement Learning</x:v>
+      </x:c>
+      <x:c r="C68" t="str">
+        <x:v>XL</x:v>
+      </x:c>
+      <x:c r="D68" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E68"/>
+      <x:c r="F68" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G68" t="str">
+        <x:v>https://cdc2027.ieeecss.org/</x:v>
+      </x:c>
+      <x:c r="H68"/>
+      <x:c r="I68"/>
+      <x:c r="J68"/>
+      <x:c r="K68" s="16"/>
+      <x:c r="L68" s="17"/>
+      <x:c r="M68"/>
+      <x:c r="N68"/>
+    </x:row>
+    <x:row r="69" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A69" t="str">
+        <x:v>NOLTA</x:v>
+      </x:c>
+      <x:c r="B69" s="12" t="str">
+        <x:v>Nonlinear Dynamics &amp; Chaos; Complex Systems &amp; Network Science; Deep Representation Learning; Control &amp; Robotics</x:v>
+      </x:c>
+      <x:c r="C69" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D69" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E69"/>
+      <x:c r="F69" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G69" t="str">
+        <x:v>https://nolta2026.org/</x:v>
+      </x:c>
+      <x:c r="H69"/>
+      <x:c r="I69"/>
+      <x:c r="J69"/>
+      <x:c r="K69" s="16"/>
+      <x:c r="L69" s="17"/>
+      <x:c r="M69"/>
+      <x:c r="N69"/>
+    </x:row>
+    <x:row r="70" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A70" t="str">
+        <x:v>SIAM DS</x:v>
+      </x:c>
+      <x:c r="B70" s="12" t="str">
+        <x:v>Nonlinear Dynamics &amp; Chaos; Complex Systems &amp; Network Science; System Identification &amp; Data-driven Dynamics; Machine Learning</x:v>
+      </x:c>
+      <x:c r="C70" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="D70" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E70"/>
+      <x:c r="F70" t="str">
+        <x:v>Abstract-based</x:v>
+      </x:c>
+      <x:c r="G70" t="str">
+        <x:v>https://www.siam.org/conferences-events/siam-conferences/ds27/</x:v>
+      </x:c>
+      <x:c r="H70"/>
+      <x:c r="I70"/>
+      <x:c r="J70"/>
+      <x:c r="K70" s="16"/>
+      <x:c r="L70" s="17"/>
+      <x:c r="M70"/>
+      <x:c r="N70"/>
+    </x:row>
+    <x:row r="71" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A71" t="str">
+        <x:v>CCS</x:v>
+      </x:c>
+      <x:c r="B71" s="12" t="str">
+        <x:v>Complex Systems &amp; Network Science; Nonlinear Dynamics &amp; Chaos; Data Mining &amp; Data Science</x:v>
+      </x:c>
+      <x:c r="C71" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="D71" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E71"/>
+      <x:c r="F71" t="str">
+        <x:v>Abstract-based</x:v>
+      </x:c>
+      <x:c r="G71" t="str">
+        <x:v>https://cssociety.org/ccs/</x:v>
+      </x:c>
+      <x:c r="H71"/>
+      <x:c r="I71"/>
+      <x:c r="J71"/>
+      <x:c r="K71" s="16"/>
+      <x:c r="L71" s="17"/>
+      <x:c r="M71"/>
+      <x:c r="N71"/>
+    </x:row>
+    <x:row r="72" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A72" t="str">
+        <x:v>NetSci</x:v>
+      </x:c>
+      <x:c r="B72" s="12" t="str">
+        <x:v>Complex Systems &amp; Network Science; Data Mining &amp; Data Science; Nonlinear Dynamics &amp; Chaos</x:v>
+      </x:c>
+      <x:c r="C72" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="D72" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E72"/>
+      <x:c r="F72" t="str">
+        <x:v>Abstract-based</x:v>
+      </x:c>
+      <x:c r="G72" t="str">
+        <x:v>https://netsci2027.github.io/</x:v>
+      </x:c>
+      <x:c r="H72"/>
+      <x:c r="I72"/>
+      <x:c r="J72"/>
+      <x:c r="K72" s="16"/>
+      <x:c r="L72" s="17"/>
+      <x:c r="M72"/>
+      <x:c r="N72"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f5d1e1c04f441c0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74f89ce4a2ee4071"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2539,146 +2765,226 @@
         <x:v>Definition</x:v>
       </x:c>
     </x:row>
-    <x:row r="2">
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="14" t="str">
         <x:v>Machine Learning</x:v>
       </x:c>
       <x:c r="B2" s="14" t="str">
-        <x:v>General ML methods, algorithms, model development, and applied AI.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
+        <x:v>General ML methods, algorithms, model development, and applied AI. Family: ML &amp; AI.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="14" t="str">
         <x:v>Deep Representation Learning</x:v>
       </x:c>
       <x:c r="B3" s="14" t="str">
-        <x:v>Deep learning, self-supervised learning, latent representations, neural networks.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
+        <x:v>Deep learning, self-supervised learning, latent representations, neural networks. Family: ML &amp; AI.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="14" t="str">
         <x:v>Data Mining &amp; Data Science</x:v>
       </x:c>
       <x:c r="B4" s="14" t="str">
-        <x:v>Knowledge discovery, analytics, applied data science, large-scale data mining.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
+        <x:v>Knowledge discovery, analytics, applied data science, large-scale data mining. Family: Data &amp; Time Series.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="14" t="str">
         <x:v>Time Series &amp; Sequential Data</x:v>
       </x:c>
       <x:c r="B5" s="14" t="str">
-        <x:v>Temporal/sequential data, event streams, longitudinal data, forecasting/classification.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
+        <x:v>Temporal/sequential data, event streams, longitudinal data, forecasting/classification. Family: Data &amp; Time Series.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="14" t="str">
         <x:v>Healthcare &amp; Clinical AI</x:v>
       </x:c>
       <x:c r="B6" s="14" t="str">
-        <x:v>Clinical ML, health data, biomedical informatics, precision/public health.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
+        <x:v>Clinical ML, health data, biomedical informatics, precision/public health. Family: Healthcare &amp; Biomedical AI.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="14" t="str">
         <x:v>Biomedical Imaging</x:v>
       </x:c>
       <x:c r="B7" s="14" t="str">
-        <x:v>Medical image analysis, segmentation, biomedical imaging, clinical imaging.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
+        <x:v>Medical image analysis, segmentation, biomedical imaging, clinical imaging. Family: Healthcare &amp; Biomedical AI.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="14" t="str">
         <x:v>Signal Processing</x:v>
       </x:c>
       <x:c r="B8" s="14" t="str">
-        <x:v>Signal processing methods and ML for signals, including biomedical signals.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
+        <x:v>Signal processing methods and ML for signals, including biomedical signals. Family: Signals &amp; Vision.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="14" t="str">
         <x:v>EEG/MEG &amp; Neural Signals</x:v>
       </x:c>
       <x:c r="B9" s="14" t="str">
-        <x:v>EEG, MEG, OPM-MEG, neural time series, neural decoding from signals.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
+        <x:v>EEG, MEG, OPM-MEG, neural time series, neural decoding from signals. Family: Neuroscience &amp; Neurotechnology.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="14" t="str">
         <x:v>BCI &amp; Neurotechnology</x:v>
       </x:c>
       <x:c r="B10" s="14" t="str">
-        <x:v>Brain-computer interfaces, neuroengineering, neurotechnology, neural devices.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
+        <x:v>Brain-computer interfaces, neuroengineering, neurotechnology, neural devices. Family: Neuroscience &amp; Neurotechnology.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="14" t="str">
         <x:v>Computational Neuroscience</x:v>
       </x:c>
       <x:c r="B11" s="14" t="str">
-        <x:v>Computational/systems/cognitive neuroscience, neural coding, modeling.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
+        <x:v>Computational/systems/cognitive neuroscience, neural coding, modeling. Family: Neuroscience &amp; Neurotechnology.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="14" t="str">
         <x:v>Neuroimaging &amp; Brain Mapping</x:v>
       </x:c>
       <x:c r="B12" s="14" t="str">
-        <x:v>Human brain mapping, fMRI, MRI, MEG neuroimaging, source reconstruction.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
+        <x:v>Human brain mapping, fMRI, MRI, MEG neuroimaging, source reconstruction. Family: Neuroscience &amp; Neurotechnology.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="14" t="str">
         <x:v>Explainability &amp; Interpretability</x:v>
       </x:c>
       <x:c r="B13" s="14" t="str">
-        <x:v>Explainable/interpretable AI, transparency, model explanations.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
+        <x:v>Explainable/interpretable AI, transparency, model explanations. Family: Responsible &amp; Trustworthy AI.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A14" s="14" t="str">
         <x:v>Fairness &amp; Responsible AI</x:v>
       </x:c>
       <x:c r="B14" s="14" t="str">
-        <x:v>Fairness, accountability, ethics, governance, trustworthy/responsible AI.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
+        <x:v>Fairness, accountability, discrimination, and equitable AI. Stable feed key; displayed as Fairness &amp; accountability. Family: Responsible &amp; Trustworthy AI.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="14" t="str">
         <x:v>Probabilistic, Causal &amp; Uncertainty ML</x:v>
       </x:c>
       <x:c r="B15" s="14" t="str">
-        <x:v>Bayesian/probabilistic ML, uncertainty quantification, causal inference.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
+        <x:v>Bayesian/probabilistic ML, uncertainty quantification, causal inference. Family: ML &amp; AI.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="14" t="str">
         <x:v>Learning Theory &amp; Statistical Foundations</x:v>
       </x:c>
       <x:c r="B16" s="14" t="str">
-        <x:v>Statistical learning, learning theory, generalization, theoretical foundations.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
+        <x:v>Statistical learning, learning theory, generalization, theoretical foundations. Family: ML &amp; AI.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="14" t="str">
         <x:v>Human-AI Interaction &amp; Deployment</x:v>
       </x:c>
       <x:c r="B17" s="14" t="str">
-        <x:v>Human-centered AI, usability, clinical deployment, interfaces, translational use.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
+        <x:v>Human-centered AI, usability, clinical deployment, interfaces, translational use. Family: ML &amp; AI.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="12" t="str">
         <x:v>Natural Language Processing &amp; LLMs</x:v>
       </x:c>
       <x:c r="B18" s="12" t="str">
-        <x:v>Natural language processing, language models, computational linguistics, and LLM systems.</x:v>
+        <x:v>Natural language processing, language models, computational linguistics, and LLM systems. Family: ML &amp; AI.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="A19" t="str">
+        <x:v>Reinforcement Learning</x:v>
+      </x:c>
+      <x:c r="B19" s="12" t="str">
+        <x:v>Learning actions and policies from interaction, reward, and feedback. Family: ML &amp; AI.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A20" t="str">
+        <x:v>Federated &amp; Distributed Learning</x:v>
+      </x:c>
+      <x:c r="B20" s="12" t="str">
+        <x:v>Distributed training, federated learning, and collaborative learning systems. Not automatically an ethics tag. Family: ML &amp; AI.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
+      <x:c r="A21" t="str">
+        <x:v>Computer Vision &amp; Pattern Recognition</x:v>
+      </x:c>
+      <x:c r="B21" s="12" t="str">
+        <x:v>Visual understanding, image analysis, recognition, and structured pattern learning. Family: Signals &amp; Vision.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A22" t="str">
+        <x:v>Nonlinear Dynamics &amp; Chaos</x:v>
+      </x:c>
+      <x:c r="B22" s="12" t="str">
+        <x:v>Dynamical systems, bifurcations, chaos, synchronization, and nonlinear modeling. Family: Dynamics, Complex Systems &amp; Control.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A23" t="str">
+        <x:v>Complex Systems &amp; Network Science</x:v>
+      </x:c>
+      <x:c r="B23" s="12" t="str">
+        <x:v>Complex adaptive systems, emergence, network structure, and dynamics on networks. Family: Dynamics, Complex Systems &amp; Control.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A24" t="str">
+        <x:v>Control &amp; Robotics</x:v>
+      </x:c>
+      <x:c r="B24" s="12" t="str">
+        <x:v>Feedback control, automation, decision making, robotics, and learning-based control. Family: Dynamics, Complex Systems &amp; Control.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A25" t="str">
+        <x:v>System Identification &amp; Data-driven Dynamics</x:v>
+      </x:c>
+      <x:c r="B25" s="12" t="str">
+        <x:v>Identifying dynamical models from data, state estimation, and data-driven dynamics. Family: Dynamics, Complex Systems &amp; Control.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="15" hidden="0" customHeight="1">
+      <x:c r="A26" t="str">
+        <x:v>Ethics &amp; Governance</x:v>
+      </x:c>
+      <x:c r="B26" s="12" t="str">
+        <x:v>AI ethics, social impacts, governance, regulation, and responsible research. Family: Responsible &amp; Trustworthy AI.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A27" t="str">
+        <x:v>Privacy-preserving ML</x:v>
+      </x:c>
+      <x:c r="B27" s="12" t="str">
+        <x:v>Privacy, differential privacy, confidential learning, and privacy-preserving computation. Family: Responsible &amp; Trustworthy AI.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="15" hidden="0" customHeight="1">
+      <x:c r="A28" t="str">
+        <x:v>Robustness &amp; Safety</x:v>
+      </x:c>
+      <x:c r="B28" s="12" t="str">
+        <x:v>Reliable and safe AI, adversarial robustness, distribution shift, and model assurance. Family: Responsible &amp; Trustworthy AI.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f15308995474ada"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fe1bad9f7834775"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add 11 conference series and preserve AI Deadlines candidate backlog
</commit_message>
<xml_diff>
--- a/data/core_conferences_normalized_tags.xlsx
+++ b/data/core_conferences_normalized_tags.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Conferences" sheetId="1" r:id="R3c059a25c4fe434e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Vocabulary" sheetId="2" r:id="R0d878d9057754bb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Conferences" sheetId="1" r:id="Rd722c6c1b09b4347"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Vocabulary" sheetId="2" r:id="R656aa7fb54dc4590"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -97,7 +97,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="CoreConferencesTable" displayName="CoreConferencesTable" ref="A1:N72" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="CoreConferencesTable" displayName="CoreConferencesTable" ref="A1:N83" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Conference"/>
     <x:tableColumn id="2" name="TAGS"/>
@@ -119,7 +119,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TagVocabularyTable" displayName="TagVocabularyTable" ref="A1:B27" headerRowCount="1" totalsRowCount="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TagVocabularyTable" displayName="TagVocabularyTable" ref="A1:B30" headerRowCount="1" totalsRowCount="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Standard tag"/>
     <x:tableColumn id="2" name="Definition"/>
@@ -2741,10 +2741,378 @@
       <x:c r="M72"/>
       <x:c r="N72"/>
     </x:row>
+    <x:row r="73" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A73" t="str">
+        <x:v>AutoML</x:v>
+      </x:c>
+      <x:c r="B73" s="12" t="str">
+        <x:v>Machine Learning; Evolutionary Computation &amp; Optimization; Deep Representation Learning; Learning Theory &amp; Statistical Foundations</x:v>
+      </x:c>
+      <x:c r="C73" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D73" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E73"/>
+      <x:c r="F73" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G73" t="str">
+        <x:v>https://2026.automl.cc/</x:v>
+      </x:c>
+      <x:c r="H73"/>
+      <x:c r="I73"/>
+      <x:c r="J73"/>
+      <x:c r="K73" s="16" t="n">
+        <x:v>0.42</x:v>
+      </x:c>
+      <x:c r="L73" s="17" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="M73" t="str">
+        <x:v>Methods and ABCD main tracks (19 accepted of 45 submitted); organizer-reported rounded rate</x:v>
+      </x:c>
+      <x:c r="N73" t="str">
+        <x:v>https://www.linkedin.com/posts/mlindauer_automl-activity-7191396371353022464-i7wW</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A74" t="str">
+        <x:v>LoG</x:v>
+      </x:c>
+      <x:c r="B74" s="12" t="str">
+        <x:v>Machine Learning; Deep Representation Learning; Complex Systems &amp; Network Science; Learning Theory &amp; Statistical Foundations</x:v>
+      </x:c>
+      <x:c r="C74" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D74" t="str">
+        <x:v>Moderate</x:v>
+      </x:c>
+      <x:c r="E74"/>
+      <x:c r="F74" s="12" t="str">
+        <x:v>Paper-based / non-archival extended abstracts</x:v>
+      </x:c>
+      <x:c r="G74" t="str">
+        <x:v>https://logconference.org/</x:v>
+      </x:c>
+      <x:c r="H74"/>
+      <x:c r="I74"/>
+      <x:c r="J74"/>
+      <x:c r="K74" s="16" t="n">
+        <x:v>0.3114</x:v>
+      </x:c>
+      <x:c r="L74" s="17" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="M74" t="str">
+        <x:v>Proceedings full papers (38 accepted of 122 submitted; non-archival abstracts excluded)</x:v>
+      </x:c>
+      <x:c r="N74" t="str">
+        <x:v>https://proceedings.mlr.press/v231/villar24a/villar24a.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A75" t="str">
+        <x:v>CoRL</x:v>
+      </x:c>
+      <x:c r="B75" s="12" t="str">
+        <x:v>Machine Learning; Control &amp; Robotics; Reinforcement Learning; Deep Representation Learning</x:v>
+      </x:c>
+      <x:c r="C75" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="D75" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E75"/>
+      <x:c r="F75" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G75" t="str">
+        <x:v>https://www.corl.org/</x:v>
+      </x:c>
+      <x:c r="H75"/>
+      <x:c r="I75"/>
+      <x:c r="J75"/>
+      <x:c r="K75" s="16"/>
+      <x:c r="L75" s="17"/>
+      <x:c r="M75"/>
+      <x:c r="N75"/>
+    </x:row>
+    <x:row r="76" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A76" t="str">
+        <x:v>GECCO</x:v>
+      </x:c>
+      <x:c r="B76" s="12" t="str">
+        <x:v>Evolutionary Computation &amp; Optimization; Machine Learning; Complex Systems &amp; Network Science</x:v>
+      </x:c>
+      <x:c r="C76" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="D76" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E76" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="F76" s="12" t="str">
+        <x:v>Paper-based / poster papers</x:v>
+      </x:c>
+      <x:c r="G76" t="str">
+        <x:v>https://gecco-2027.sigevo.org/HomePage</x:v>
+      </x:c>
+      <x:c r="H76" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/556/</x:v>
+      </x:c>
+      <x:c r="I76" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="J76" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=59</x:v>
+      </x:c>
+      <x:c r="K76" s="16"/>
+      <x:c r="L76" s="17"/>
+      <x:c r="M76"/>
+      <x:c r="N76"/>
+    </x:row>
+    <x:row r="77" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A77" t="str">
+        <x:v>SaTML</x:v>
+      </x:c>
+      <x:c r="B77" s="12" t="str">
+        <x:v>Robustness &amp; Safety; Privacy-preserving ML; Fairness &amp; Responsible AI; Explainability &amp; Interpretability</x:v>
+      </x:c>
+      <x:c r="C77" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D77" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E77"/>
+      <x:c r="F77" s="12" t="str">
+        <x:v>Paper-based / systematization of knowledge / position papers</x:v>
+      </x:c>
+      <x:c r="G77" t="str">
+        <x:v>https://satml.org/</x:v>
+      </x:c>
+      <x:c r="H77"/>
+      <x:c r="I77"/>
+      <x:c r="J77"/>
+      <x:c r="K77" s="16"/>
+      <x:c r="L77" s="17"/>
+      <x:c r="M77"/>
+      <x:c r="N77"/>
+    </x:row>
+    <x:row r="78" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A78" t="str">
+        <x:v>ProbML</x:v>
+      </x:c>
+      <x:c r="B78" s="12" t="str">
+        <x:v>Probabilistic, Causal &amp; Uncertainty ML; Learning Theory &amp; Statistical Foundations; Machine Learning; Healthcare &amp; Clinical AI</x:v>
+      </x:c>
+      <x:c r="C78" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="D78" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E78"/>
+      <x:c r="F78" s="12" t="str">
+        <x:v>Paper-based / non-archival extended abstracts</x:v>
+      </x:c>
+      <x:c r="G78" t="str">
+        <x:v>https://probml.cc/</x:v>
+      </x:c>
+      <x:c r="H78"/>
+      <x:c r="I78"/>
+      <x:c r="J78"/>
+      <x:c r="K78" s="16"/>
+      <x:c r="L78" s="17"/>
+      <x:c r="M78"/>
+      <x:c r="N78"/>
+    </x:row>
+    <x:row r="79" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A79" t="str">
+        <x:v>AAMAS</x:v>
+      </x:c>
+      <x:c r="B79" s="12" t="str">
+        <x:v>Machine Learning; Reinforcement Learning; Control &amp; Robotics; Human-AI Interaction &amp; Deployment</x:v>
+      </x:c>
+      <x:c r="C79" t="str">
+        <x:v>XL</x:v>
+      </x:c>
+      <x:c r="D79" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="E79" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="F79" s="12" t="str">
+        <x:v>Paper-based / Blue Sky Ideas short papers</x:v>
+      </x:c>
+      <x:c r="G79" t="str">
+        <x:v>https://warwick.ac.uk/fac/sci/dcs/aamas2027/</x:v>
+      </x:c>
+      <x:c r="H79" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/922/</x:v>
+      </x:c>
+      <x:c r="I79" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J79" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=58</x:v>
+      </x:c>
+      <x:c r="K79" s="16" t="n">
+        <x:v>0.255</x:v>
+      </x:c>
+      <x:c r="L79" s="17" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="M79" t="str">
+        <x:v>Main-track full papers; program chairs' reported rate (extended abstracts excluded; withdrawals affect counts)</x:v>
+      </x:c>
+      <x:c r="N79" t="str">
+        <x:v>https://www.ifaamas.org/Proceedings/aamas2026/pdfs/welcome.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A80" t="str">
+        <x:v>MLSys</x:v>
+      </x:c>
+      <x:c r="B80" s="12" t="str">
+        <x:v>ML Systems &amp; Infrastructure; Machine Learning; Federated &amp; Distributed Learning; Natural Language Processing &amp; LLMs</x:v>
+      </x:c>
+      <x:c r="C80" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="D80" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E80"/>
+      <x:c r="F80" s="12" t="str">
+        <x:v>Paper-based / research and industrial tracks</x:v>
+      </x:c>
+      <x:c r="G80" t="str">
+        <x:v>https://mlsys.org/Conferences/2027</x:v>
+      </x:c>
+      <x:c r="H80"/>
+      <x:c r="I80"/>
+      <x:c r="J80"/>
+      <x:c r="K80" s="16"/>
+      <x:c r="L80" s="17"/>
+      <x:c r="M80"/>
+      <x:c r="N80"/>
+    </x:row>
+    <x:row r="81" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A81" t="str">
+        <x:v>CogSci</x:v>
+      </x:c>
+      <x:c r="B81" s="12" t="str">
+        <x:v>Cognitive Science &amp; Computational Cognition; Computational Neuroscience; Machine Learning; Natural Language Processing &amp; LLMs</x:v>
+      </x:c>
+      <x:c r="C81" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="D81" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E81" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="F81" s="12" t="str">
+        <x:v>Paper-based / abstract presentations</x:v>
+      </x:c>
+      <x:c r="G81" t="str">
+        <x:v>https://cognitivesciencesociety.org/cogsci-2027/</x:v>
+      </x:c>
+      <x:c r="H81" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/120/</x:v>
+      </x:c>
+      <x:c r="I81" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J81" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=71</x:v>
+      </x:c>
+      <x:c r="K81" s="16"/>
+      <x:c r="L81" s="17"/>
+      <x:c r="M81"/>
+      <x:c r="N81"/>
+    </x:row>
+    <x:row r="82" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A82" t="str">
+        <x:v>ICIP</x:v>
+      </x:c>
+      <x:c r="B82" s="12" t="str">
+        <x:v>Signal Processing; Computer Vision &amp; Pattern Recognition; Machine Learning; Deep Representation Learning</x:v>
+      </x:c>
+      <x:c r="C82" t="str">
+        <x:v>XL</x:v>
+      </x:c>
+      <x:c r="D82" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E82" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="F82" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G82" t="str">
+        <x:v>https://2027.ieeeicip.org/</x:v>
+      </x:c>
+      <x:c r="H82" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/654/</x:v>
+      </x:c>
+      <x:c r="I82" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="J82" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=49</x:v>
+      </x:c>
+      <x:c r="K82" s="16"/>
+      <x:c r="L82" s="17"/>
+      <x:c r="M82"/>
+      <x:c r="N82"/>
+    </x:row>
+    <x:row r="83" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A83" t="str">
+        <x:v>Interspeech</x:v>
+      </x:c>
+      <x:c r="B83" s="12" t="str">
+        <x:v>Signal Processing; Machine Learning; Deep Representation Learning; Natural Language Processing &amp; LLMs</x:v>
+      </x:c>
+      <x:c r="C83" t="str">
+        <x:v>XL</x:v>
+      </x:c>
+      <x:c r="D83" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E83" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="F83" s="12" t="str">
+        <x:v>Paper-based / interactive demonstration papers</x:v>
+      </x:c>
+      <x:c r="G83" t="str">
+        <x:v>https://interspeech2027.org/</x:v>
+      </x:c>
+      <x:c r="H83" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/494/</x:v>
+      </x:c>
+      <x:c r="I83"/>
+      <x:c r="J83"/>
+      <x:c r="K83" s="16"/>
+      <x:c r="L83" s="17"/>
+      <x:c r="M83"/>
+      <x:c r="N83"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74f89ce4a2ee4071"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4c092a76a394cc7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2981,10 +3349,34 @@
         <x:v>Reliable and safe AI, adversarial robustness, distribution shift, and model assurance. Family: Responsible &amp; Trustworthy AI.</x:v>
       </x:c>
     </x:row>
+    <x:row r="29" ht="15" hidden="0" customHeight="1">
+      <x:c r="A29" t="str">
+        <x:v>Evolutionary Computation &amp; Optimization</x:v>
+      </x:c>
+      <x:c r="B29" s="12" t="str">
+        <x:v>Evolutionary algorithms, genetic programming, neuroevolution, and population-based optimization. Family: ML &amp; AI.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A30" t="str">
+        <x:v>Cognitive Science &amp; Computational Cognition</x:v>
+      </x:c>
+      <x:c r="B30" s="12" t="str">
+        <x:v>Computational models of cognition, learning, perception, language, and reasoning. Family: Neuroscience &amp; Neurotechnology.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="15" hidden="0" customHeight="1">
+      <x:c r="A31" t="str">
+        <x:v>ML Systems &amp; Infrastructure</x:v>
+      </x:c>
+      <x:c r="B31" s="12" t="str">
+        <x:v>Systems for ML and ML for systems, including training, inference, compilers, hardware, and serving. Family: ML &amp; AI.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fe1bad9f7834775"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R91b9c1247b9c4ef3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add curated conference scope profiles and richer topic discovery
</commit_message>
<xml_diff>
--- a/data/core_conferences_normalized_tags.xlsx
+++ b/data/core_conferences_normalized_tags.xlsx
@@ -2,8 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Conferences" sheetId="1" r:id="Rd722c6c1b09b4347"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Vocabulary" sheetId="2" r:id="R656aa7fb54dc4590"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Conferences" sheetId="1" r:id="Rfbc8fc13ca064400"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Vocabulary" sheetId="2" r:id="R72a1277fb2a8431a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conference Scope" sheetId="3" r:id="Rcebdc42a32d4481d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,11 +15,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
+  <x:numFmts count="3">
     <x:numFmt numFmtId="200" formatCode="0.0%"/>
     <x:numFmt numFmtId="201" formatCode="0"/>
+    <x:numFmt numFmtId="202" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
-  <x:fonts count="2">
+  <x:fonts count="3">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -28,6 +30,10 @@
       <x:sz val="11"/>
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:name val="Arial"/>
     </x:font>
   </x:fonts>
   <x:fills count="3">
@@ -50,7 +56,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="18">
+  <x:cellXfs count="24">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -89,6 +95,22 @@
     </x:xf>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -125,6 +147,20 @@
     <x:tableColumn id="2" name="Definition"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ConferenceScope" displayName="ConferenceScope" ref="A1:F31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="Series"/>
+    <x:tableColumn id="2" name="Additional topics"/>
+    <x:tableColumn id="3" name="Scope summary"/>
+    <x:tableColumn id="4" name="Source edition"/>
+    <x:tableColumn id="5" name="Scope sources"/>
+    <x:tableColumn id="6" name="Scope reviewed"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
@@ -3112,7 +3148,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4c092a76a394cc7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16568e3c52dc4540"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3376,7 +3412,639 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R91b9c1247b9c4ef3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6276ba1efc204ab0"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="15.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="33.33000183105469" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="55.560001373291016" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="11.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="38.88999938964844" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12.220000267028809" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="15" hidden="0" customHeight="1">
+      <x:c r="A1" s="23" t="str">
+        <x:v>Series</x:v>
+      </x:c>
+      <x:c r="B1" s="23" t="str">
+        <x:v>Additional topics</x:v>
+      </x:c>
+      <x:c r="C1" s="23" t="str">
+        <x:v>Scope summary</x:v>
+      </x:c>
+      <x:c r="D1" s="23" t="str">
+        <x:v>Source edition</x:v>
+      </x:c>
+      <x:c r="E1" s="23" t="str">
+        <x:v>Scope sources</x:v>
+      </x:c>
+      <x:c r="F1" s="23" t="str">
+        <x:v>Scope reviewed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="60" hidden="0" customHeight="1">
+      <x:c r="A2" s="20" t="str">
+        <x:v>AALTD</x:v>
+      </x:c>
+      <x:c r="B2" s="20" t="str">
+        <x:v>Deep Representation Learning</x:v>
+      </x:c>
+      <x:c r="C2" s="20" t="str">
+        <x:v>Analytics and learning specifically for temporal data: time-series classification, clustering, forecasting, segmentation, anomaly detection, temporal representations, and metric or kernel learning. Includes temporal foundation models, data streams, and explainable temporal analysis. Climate, health, and energy are examples of applications rather than separate defining topic assignments.</x:v>
+      </x:c>
+      <x:c r="D2" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E2" s="20" t="str">
+        <x:v>https://ecml-aaltd.github.io/aaltd2026/</x:v>
+      </x:c>
+      <x:c r="F2" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="72" hidden="0" customHeight="1">
+      <x:c r="A3" s="20" t="str">
+        <x:v>AAMAS</x:v>
+      </x:c>
+      <x:c r="B3" s="20" t="str">
+        <x:v>Deep Representation Learning; Probabilistic, Causal &amp; Uncertainty ML; Evolutionary Computation &amp; Optimization; Complex Systems &amp; Network Science; Ethics &amp; Governance; Explainability &amp; Interpretability</x:v>
+      </x:c>
+      <x:c r="C3" s="20" t="str">
+        <x:v>Autonomous agents and multi-agent systems: learning and adaptation, coordination, game theory, planning, reasoning, agent engineering, and agent-based simulation. Also covers human-agent interaction, robot teams, norms and governance, and generative agents. The contribution should concern agents or their interaction; generic language-model or learning results are not automatically in scope.</x:v>
+      </x:c>
+      <x:c r="D3" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E3" s="20" t="str">
+        <x:v>https://warwick.ac.uk/fac/sci/dcs/aamas2027/calls/call-for-main-track/</x:v>
+      </x:c>
+      <x:c r="F3" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="72" hidden="0" customHeight="1">
+      <x:c r="A4" s="20" t="str">
+        <x:v>ACM FAccT</x:v>
+      </x:c>
+      <x:c r="B4" s="20" t="str">
+        <x:v>Human-AI Interaction &amp; Deployment; Robustness &amp; Safety</x:v>
+      </x:c>
+      <x:c r="C4" s="20" t="str">
+        <x:v>Fairness, accountability, and transparency in computing, combining algorithmic research with sociotechnical, legal, philosophical, and human-centered approaches. Characteristic contributions include audits and evaluation practices, governance, human experiences of systems, and responsible development and deployment. A fairness or accountability question should be substantive, not a passing motivation for generic ML.</x:v>
+      </x:c>
+      <x:c r="D4" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E4" s="20" t="str">
+        <x:v>https://facctconference.org/2026/cfp.html</x:v>
+      </x:c>
+      <x:c r="F4" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="60" hidden="0" customHeight="1">
+      <x:c r="A5" s="20" t="str">
+        <x:v>ACML</x:v>
+      </x:c>
+      <x:c r="B5" s="20" t="str">
+        <x:v>Deep Representation Learning; Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Natural Language Processing &amp; LLMs; Fairness &amp; Responsible AI; Privacy-preserving ML</x:v>
+      </x:c>
+      <x:c r="C5" s="20" t="str">
+        <x:v>Theory and practice of machine learning, including probabilistic methods, representation learning, transfer and meta-learning, reinforcement learning, and learning theory. Generative models, language models, and trustworthy learning extend this core. The broad applications list is not treated as evidence that every application field defines the conference.</x:v>
+      </x:c>
+      <x:c r="D5" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E5" s="20" t="str">
+        <x:v>https://www.acml-conf.org/2026/calls/papers/</x:v>
+      </x:c>
+      <x:c r="F5" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="60" hidden="0" customHeight="1">
+      <x:c r="A6" s="20" t="str">
+        <x:v>AIES</x:v>
+      </x:c>
+      <x:c r="B6" s="20" t="str">
+        <x:v>Human-AI Interaction &amp; Deployment; Privacy-preserving ML</x:v>
+      </x:c>
+      <x:c r="C6" s="20" t="str">
+        <x:v>Ethics and societal consequences of AI, connecting computer science, law and policy, social science, and philosophy. Defining concerns include governance and power, accountability after deployment, value alignment, fairness, human-AI interaction, and institutional practice. Technical work is relevant through a serious ethical or societal contribution.</x:v>
+      </x:c>
+      <x:c r="D6" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E6" s="20" t="str">
+        <x:v>https://www.aies-conference.com/2026/call-for-papers/</x:v>
+      </x:c>
+      <x:c r="F6" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="48" hidden="0" customHeight="1">
+      <x:c r="A7" s="20" t="str">
+        <x:v>AISTATS</x:v>
+      </x:c>
+      <x:c r="B7" s="20" t="str"/>
+      <x:c r="C7" s="20" t="str">
+        <x:v>Research at the interface of artificial intelligence, machine learning, and statistics. Its defining emphasis is on statistical foundations and methodology for learning and inference, rather than a particular application domain. Research bridges statistical reasoning and learning algorithms, with archival contributions to both communities.</x:v>
+      </x:c>
+      <x:c r="D7" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E7" s="20" t="str">
+        <x:v>https://aistats.org/aistats2027/; https://aistats.org/aistats2027/call-for-papers.html</x:v>
+      </x:c>
+      <x:c r="F7" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="72" hidden="0" customHeight="1">
+      <x:c r="A8" s="20" t="str">
+        <x:v>AutoML</x:v>
+      </x:c>
+      <x:c r="B8" s="20" t="str">
+        <x:v>Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Explainability &amp; Interpretability; Natural Language Processing &amp; LLMs; Robustness &amp; Safety</x:v>
+      </x:c>
+      <x:c r="C8" s="20" t="str">
+        <x:v>Automating the construction and configuration of learning systems: hyperparameter optimization, Bayesian optimization, neural architecture search, model selection, meta-learning, and pipeline automation. Includes evolutionary and reinforcement-learning approaches, AutoML for foundation models, and evaluation through applications, benchmarks, challenges, and datasets. Trustworthiness matters specifically in automated ML workflows.</x:v>
+      </x:c>
+      <x:c r="D8" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E8" s="20" t="str">
+        <x:v>https://2026.automl.cc/call-for-papers/</x:v>
+      </x:c>
+      <x:c r="F8" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="72" hidden="0" customHeight="1">
+      <x:c r="A9" s="20" t="str">
+        <x:v>CCN</x:v>
+      </x:c>
+      <x:c r="B9" s="20" t="str">
+        <x:v>Cognitive Science &amp; Computational Cognition; Explainability &amp; Interpretability</x:v>
+      </x:c>
+      <x:c r="C9" s="20" t="str">
+        <x:v>Cognitive computational neuroscience, connecting experiments and models of brain computation with artificial intelligence. Characteristic work compares biological and artificial representations, models perception, cognition and action, studies neural connectivity and dynamics, and uses mechanistic interpretability to understand neural-network models. The aim is understanding computation and behavior across brains and AI systems.</x:v>
+      </x:c>
+      <x:c r="D9" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E9" s="20" t="str">
+        <x:v>https://2027.ccneuro.org/</x:v>
+      </x:c>
+      <x:c r="F9" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="72" hidden="0" customHeight="1">
+      <x:c r="A10" s="20" t="str">
+        <x:v>CHIL</x:v>
+      </x:c>
+      <x:c r="B10" s="20" t="str">
+        <x:v>Explainability &amp; Interpretability; Human-AI Interaction &amp; Deployment; Robustness &amp; Safety; Time Series &amp; Sequential Data</x:v>
+      </x:c>
+      <x:c r="C10" s="20" t="str">
+        <x:v>Machine learning and inference for clinical, public, and population health. Distinguishing areas include causal inference, survival analysis, multimodal health data, generalization across populations, interpretability, and clinical evaluation and deployment. Research may emphasize methods, practical applications, or societal impact. Health-focused inference and evaluation remain the common thread across these tracks.</x:v>
+      </x:c>
+      <x:c r="D10" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E10" s="20" t="str">
+        <x:v>https://chil.ahli.cc/submit/call-for-papers/</x:v>
+      </x:c>
+      <x:c r="F10" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="60" hidden="0" customHeight="1">
+      <x:c r="A11" s="20" t="str">
+        <x:v>CogSci</x:v>
+      </x:c>
+      <x:c r="B11" s="20" t="str"/>
+      <x:c r="C11" s="20" t="str">
+        <x:v>Interdisciplinary study of cognition and the mind, connecting psychology, linguistics, artificial intelligence, neuroscience, philosophy, anthropology, and education. Computational models and experiments should illuminate cognitive processes and behavior. An AI paper belongs here through its contribution to understanding cognition, not solely through a predictive performance improvement.</x:v>
+      </x:c>
+      <x:c r="D11" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E11" s="20" t="str">
+        <x:v>https://cognitivesciencesociety.org/submissions-faq/; https://cognitivesciencesociety.org/</x:v>
+      </x:c>
+      <x:c r="F11" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="60" hidden="0" customHeight="1">
+      <x:c r="A12" s="20" t="str">
+        <x:v>COLT</x:v>
+      </x:c>
+      <x:c r="B12" s="20" t="str">
+        <x:v>Deep Representation Learning; Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Privacy-preserving ML; Fairness &amp; Responsible AI</x:v>
+      </x:c>
+      <x:c r="C12" s="20" t="str">
+        <x:v>Theoretical foundations of learning at the intersection of computer science, statistics, and applied mathematics. Characteristic work studies learnability, sample and computational complexity, online learning, optimization, bandits, and generalization. Neural-network, causal, reinforcement-learning, privacy, and fairness papers belong here when the theoretical contribution is central.</x:v>
+      </x:c>
+      <x:c r="D12" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E12" s="20" t="str">
+        <x:v>https://learningtheory.org/colt2026/cfp.html</x:v>
+      </x:c>
+      <x:c r="F12" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="72" hidden="0" customHeight="1">
+      <x:c r="A13" s="20" t="str">
+        <x:v>CoRL</x:v>
+      </x:c>
+      <x:c r="B13" s="20" t="str">
+        <x:v>Computer Vision &amp; Pattern Recognition; Probabilistic, Causal &amp; Uncertainty ML; Human-AI Interaction &amp; Deployment; Robustness &amp; Safety; Learning Theory &amp; Statistical Foundations</x:v>
+      </x:c>
+      <x:c r="C13" s="20" t="str">
+        <x:v>Machine learning for physical robots, especially imitation and reinforcement learning, learned perception and control, robot foundation models, and learning-based task and motion planning. Includes uncertainty, generalization, safety, human-robot interaction, and datasets grounded in manipulation, navigation, or locomotion. General ML is relevant when it makes a substantive contribution to robot learning.</x:v>
+      </x:c>
+      <x:c r="D13" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E13" s="20" t="str">
+        <x:v>https://www.corl.org/contributions/call-for-papers</x:v>
+      </x:c>
+      <x:c r="F13" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="72" hidden="0" customHeight="1">
+      <x:c r="A14" s="20" t="str">
+        <x:v>EACL</x:v>
+      </x:c>
+      <x:c r="B14" s="20" t="str">
+        <x:v>Explainability &amp; Interpretability; Fairness &amp; Responsible AI; Cognitive Science &amp; Computational Cognition</x:v>
+      </x:c>
+      <x:c r="C14" s="20" t="str">
+        <x:v>Computational linguistics and natural language processing, including language modeling, multilingual processing, translation, dialogue, information extraction, semantics, and linguistic analysis. Human-centered evaluation, interpretability, and bias are relevant within language research. The reviewed 2027 theme strengthens connections to psycholinguistics and cognitive modeling; peripheral application domains are not extra tags.</x:v>
+      </x:c>
+      <x:c r="D14" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E14" s="20" t="str">
+        <x:v>https://2027.eacl.org/calls/papers/</x:v>
+      </x:c>
+      <x:c r="F14" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="60" hidden="0" customHeight="1">
+      <x:c r="A15" s="20" t="str">
+        <x:v>FMTS @ NeurIPS</x:v>
+      </x:c>
+      <x:c r="B15" s="20" t="str">
+        <x:v>System Identification &amp; Data-driven Dynamics; Robustness &amp; Safety</x:v>
+      </x:c>
+      <x:c r="C15" s="20" t="str">
+        <x:v>Foundation models for temporal systems, centered on long-horizon and probabilistic forecasting, temporal pretraining, generative simulation, irregularly sampled and multimodal sequences, and state-space architectures. Reliability is a defining theme: distribution shift, calibrated uncertainty, leakage-aware benchmarks, and consistency of simulated trajectories.</x:v>
+      </x:c>
+      <x:c r="D15" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E15" s="20" t="str">
+        <x:v>https://fmts-workshop.github.io/cfp.html</x:v>
+      </x:c>
+      <x:c r="F15" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="60" hidden="0" customHeight="1">
+      <x:c r="A16" s="20" t="str">
+        <x:v>GECCO</x:v>
+      </x:c>
+      <x:c r="B16" s="20" t="str">
+        <x:v>Deep Representation Learning; Learning Theory &amp; Statistical Foundations</x:v>
+      </x:c>
+      <x:c r="C16" s="20" t="str">
+        <x:v>Genetic and evolutionary computation, including genetic algorithms, genetic programming, swarm intelligence, evolutionary multiobjective and combinatorial optimization, metaheuristics, and neuroevolution. Machine learning is relevant through evolutionary learning and optimization, not as an unrestricted substitute for the conference's evolutionary-computation focus.</x:v>
+      </x:c>
+      <x:c r="D16" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E16" s="20" t="str">
+        <x:v>https://gecco-2027.sigevo.org/Call+for+Papers</x:v>
+      </x:c>
+      <x:c r="F16" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="72" hidden="0" customHeight="1">
+      <x:c r="A17" s="20" t="str">
+        <x:v>ICIP</x:v>
+      </x:c>
+      <x:c r="B17" s="20" t="str"/>
+      <x:c r="C17" s="20" t="str">
+        <x:v>Image and video processing across theory, algorithms, and imaging systems. Characteristic problems include restoration, enhancement, reconstruction, registration, compression, quality assessment, and visual analysis. Learning methods and generative models are relevant when they advance image or video processing. The long list of imaging application domains is intentionally not converted into extra specialist-conference tags.</x:v>
+      </x:c>
+      <x:c r="D17" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E17" s="20" t="str">
+        <x:v>https://2026.ieeeicip.org/topics/</x:v>
+      </x:c>
+      <x:c r="F17" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="60" hidden="0" customHeight="1">
+      <x:c r="A18" s="20" t="str">
+        <x:v>ICLR</x:v>
+      </x:c>
+      <x:c r="B18" s="20" t="str">
+        <x:v>Learning Theory &amp; Statistical Foundations; Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Natural Language Processing &amp; LLMs; Computer Vision &amp; Pattern Recognition; ML Systems &amp; Infrastructure</x:v>
+      </x:c>
+      <x:c r="C18" s="20" t="str">
+        <x:v>Learning representations and understanding deep learning, with an emphasis on self-supervised learning, generative models, transfer and meta-learning, and the optimization and theory of learned representations. Language, vision, probabilistic modeling, and reinforcement learning are substantial areas, rather than unrelated application-domain tags.</x:v>
+      </x:c>
+      <x:c r="D18" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E18" s="20" t="str">
+        <x:v>https://iclr.cc/Conferences/2027/CallForPapers</x:v>
+      </x:c>
+      <x:c r="F18" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="60" hidden="0" customHeight="1">
+      <x:c r="A19" s="20" t="str">
+        <x:v>ICML</x:v>
+      </x:c>
+      <x:c r="B19" s="20" t="str">
+        <x:v>Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Explainability &amp; Interpretability; Robustness &amp; Safety; ML Systems &amp; Infrastructure; Federated &amp; Distributed Learning</x:v>
+      </x:c>
+      <x:c r="C19" s="20" t="str">
+        <x:v>Methodological and theoretical machine learning, including supervised and unsupervised learning, deep generative models, optimization, statistical learning theory, Bayesian methods, and reinforcement learning. Scalable systems and trustworthy learning are established parts of the scope; application papers should offer contributions of wider interest to ML.</x:v>
+      </x:c>
+      <x:c r="D19" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E19" s="20" t="str">
+        <x:v>https://icml.cc/Conferences/2026/CallForPapers</x:v>
+      </x:c>
+      <x:c r="F19" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="60" hidden="0" customHeight="1">
+      <x:c r="A20" s="20" t="str">
+        <x:v>IFAC SYSID</x:v>
+      </x:c>
+      <x:c r="B20" s="20" t="str">
+        <x:v>Nonlinear Dynamics &amp; Chaos; Complex Systems &amp; Network Science</x:v>
+      </x:c>
+      <x:c r="C20" s="20" t="str">
+        <x:v>System identification and data-driven modeling for dynamical systems and control. Characteristic themes include nonlinear identification, model reduction, identification software and benchmarks, learning across systems, and dynamic networks. Application tracks remain grounded in identifying or learning dynamical models, rather than becoming general-purpose domain conferences.</x:v>
+      </x:c>
+      <x:c r="D20" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E20" s="20" t="str">
+        <x:v>https://conferences.ifac-control.org/sysid2027/participate/</x:v>
+      </x:c>
+      <x:c r="F20" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="60" hidden="0" customHeight="1">
+      <x:c r="A21" s="20" t="str">
+        <x:v>Interspeech</x:v>
+      </x:c>
+      <x:c r="B21" s="20" t="str"/>
+      <x:c r="C21" s="20" t="str">
+        <x:v>Speech science and speech technology, linking spoken-language research with computational methods for speech recognition, speech synthesis, and speech communication. Machine learning and language models are relevant through speech and spoken-language problems. The current 2027 overview emphasizes the relationship between speech research and spoken-language technologies.</x:v>
+      </x:c>
+      <x:c r="D21" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E21" s="20" t="str">
+        <x:v>https://interspeech2027.org/</x:v>
+      </x:c>
+      <x:c r="F21" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="60" hidden="0" customHeight="1">
+      <x:c r="A22" s="20" t="str">
+        <x:v>KDD</x:v>
+      </x:c>
+      <x:c r="B22" s="20" t="str">
+        <x:v>Deep Representation Learning; Natural Language Processing &amp; LLMs; Explainability &amp; Interpretability; Privacy-preserving ML; ML Systems &amp; Infrastructure</x:v>
+      </x:c>
+      <x:c r="C22" s="20" t="str">
+        <x:v>Knowledge discovery and data science, centered on extracting useful structure from large, heterogeneous data. Characteristic areas include clustering, structured and relational learning, graph and text mining, recommender systems, scalable data analysis, and responsible data use. Generative AI is relevant when it advances data science, not simply because a paper uses an LLM.</x:v>
+      </x:c>
+      <x:c r="D22" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E22" s="20" t="str">
+        <x:v>https://kdd2027.kdd.org/research-track-call-for-papers/</x:v>
+      </x:c>
+      <x:c r="F22" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="60" hidden="0" customHeight="1">
+      <x:c r="A23" s="20" t="str">
+        <x:v>L4DC</x:v>
+      </x:c>
+      <x:c r="B23" s="20" t="str">
+        <x:v>Learning Theory &amp; Statistical Foundations</x:v>
+      </x:c>
+      <x:c r="C23" s="20" t="str">
+        <x:v>The interface of learning, dynamics, control, and optimization for physical and dynamical systems. Emphasizes foundations and methods for data-driven control and dynamical modeling, including theoretical, empirical, and applied contributions. Pure pattern recognition without a meaningful connection to dynamics or control is not the defining focus.</x:v>
+      </x:c>
+      <x:c r="D23" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E23" s="20" t="str">
+        <x:v>https://l4dc2027.control.ee.ethz.ch/home</x:v>
+      </x:c>
+      <x:c r="F23" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="72" hidden="0" customHeight="1">
+      <x:c r="A24" s="20" t="str">
+        <x:v>LoG</x:v>
+      </x:c>
+      <x:c r="B24" s="20" t="str">
+        <x:v>Probabilistic, Causal &amp; Uncertainty ML; Signal Processing; Robustness &amp; Safety; ML Systems &amp; Infrastructure</x:v>
+      </x:c>
+      <x:c r="C24" s="20" t="str">
+        <x:v>Learning on graphs and geometry: graph neural networks, equivariant models, graph kernels, geometric and graph generative models, and statistical theory for structured data. Graph signal processing, causal graph models, robustness, and scalable graph-learning infrastructure are meaningful extensions. A graph or geometric contribution should remain central, even in an application such as language or molecular modeling.</x:v>
+      </x:c>
+      <x:c r="D24" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E24" s="20" t="str">
+        <x:v>https://logconference.org/cfp/</x:v>
+      </x:c>
+      <x:c r="F24" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="60" hidden="0" customHeight="1">
+      <x:c r="A25" s="20" t="str">
+        <x:v>MIDL</x:v>
+      </x:c>
+      <x:c r="B25" s="20" t="str">
+        <x:v>Computer Vision &amp; Pattern Recognition; Probabilistic, Causal &amp; Uncertainty ML; Explainability &amp; Interpretability; Robustness &amp; Safety; Federated &amp; Distributed Learning</x:v>
+      </x:c>
+      <x:c r="C25" s="20" t="str">
+        <x:v>Deep learning for biomedical image analysis, especially segmentation, detection, reconstruction, registration, generative imaging, and learning from limited labels. Uncertainty, interpretability, multi-site learning, robustness, and clinical validation extend that imaging core. Multimodal foundation models are relevant when grounded in medical imaging.</x:v>
+      </x:c>
+      <x:c r="D25" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E25" s="20" t="str">
+        <x:v>https://2026.midl.io/call-for-papers</x:v>
+      </x:c>
+      <x:c r="F25" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="60" hidden="0" customHeight="1">
+      <x:c r="A26" s="20" t="str">
+        <x:v>MLSys</x:v>
+      </x:c>
+      <x:c r="B26" s="20" t="str">
+        <x:v>Reinforcement Learning; Privacy-preserving ML</x:v>
+      </x:c>
+      <x:c r="C26" s="20" t="str">
+        <x:v>The intersection of machine learning and computer systems, including efficient training, inference and serving, compilers and runtimes, programming abstractions, specialized hardware, distributed learning, and system monitoring. LLM and agentic workloads are considered from a systems perspective. Both systems for ML and ML methods that improve computing systems are relevant.</x:v>
+      </x:c>
+      <x:c r="D26" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E26" s="20" t="str">
+        <x:v>https://mlsys.org/Conferences/2027/CallForResearchPapers</x:v>
+      </x:c>
+      <x:c r="F26" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="60" hidden="0" customHeight="1">
+      <x:c r="A27" s="20" t="str">
+        <x:v>NeurIPS</x:v>
+      </x:c>
+      <x:c r="B27" s="20" t="str">
+        <x:v>Learning Theory &amp; Statistical Foundations; Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Natural Language Processing &amp; LLMs; Computer Vision &amp; Pattern Recognition; ML Systems &amp; Infrastructure</x:v>
+      </x:c>
+      <x:c r="C27" s="20" t="str">
+        <x:v>Broad research in machine learning, especially deep and generative models, statistical foundations, optimization, probabilistic inference, and learning for decision-making. Language, vision, and scalable ML systems are important research communities. Interdisciplinary applications should contribute insight of wider interest to the machine-learning community.</x:v>
+      </x:c>
+      <x:c r="D27" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E27" s="20" t="str">
+        <x:v>https://neurips.cc/Conferences/2026/CallForPapers</x:v>
+      </x:c>
+      <x:c r="F27" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="60" hidden="0" customHeight="1">
+      <x:c r="A28" s="20" t="str">
+        <x:v>NOLTA</x:v>
+      </x:c>
+      <x:c r="B28" s="20" t="str">
+        <x:v>Signal Processing; Evolutionary Computation &amp; Optimization</x:v>
+      </x:c>
+      <x:c r="C28" s="20" t="str">
+        <x:v>Nonlinear theory and its applications, centered on chaos, bifurcations, oscillations, synchronization, nonlinear circuits, and complex networks. Neural computation, evolutionary algorithms, control, and signal processing connect to this nonlinear-systems focus. Individual application examples are not taken as additional specialist identities.</x:v>
+      </x:c>
+      <x:c r="D28" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E28" s="20" t="str">
+        <x:v>https://nolta2026.org/</x:v>
+      </x:c>
+      <x:c r="F28" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="72" hidden="0" customHeight="1">
+      <x:c r="A29" s="20" t="str">
+        <x:v>ProbML</x:v>
+      </x:c>
+      <x:c r="B29" s="20" t="str">
+        <x:v>Deep Representation Learning; Reinforcement Learning; Time Series &amp; Sequential Data; Robustness &amp; Safety</x:v>
+      </x:c>
+      <x:c r="C29" s="20" t="str">
+        <x:v>Probabilistic and Bayesian machine learning, emphasizing approximate inference, variational and Monte Carlo methods, Gaussian processes, graphical and state-space models, calibration, and decisions under uncertainty. Includes Bayesian optimization and uncertainty-aware deep learning. The reviewed 2026 application focus is healthcare and climate; probabilistic reasoning remains essential to a suitable contribution.</x:v>
+      </x:c>
+      <x:c r="D29" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E29" s="20" t="str">
+        <x:v>https://probml.cc/call/</x:v>
+      </x:c>
+      <x:c r="F29" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="60" hidden="0" customHeight="1">
+      <x:c r="A30" s="20" t="str">
+        <x:v>SaTML</x:v>
+      </x:c>
+      <x:c r="B30" s="20" t="str">
+        <x:v>Machine Learning; ML Systems &amp; Infrastructure</x:v>
+      </x:c>
+      <x:c r="C30" s="20" t="str">
+        <x:v>Security, safety, and trustworthiness of machine learning. Characteristic work studies attacks and defenses, privacy, verification, ML-system security, fairness, interpretability, and trustworthy data curation. Theoretical, empirical, and applied papers must engage substantively with a safety or trustworthiness question; merely using an ML model is insufficient.</x:v>
+      </x:c>
+      <x:c r="D30" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E30" s="20" t="str">
+        <x:v>https://satml.org/call-for-papers/</x:v>
+      </x:c>
+      <x:c r="F30" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="60" hidden="0" customHeight="1">
+      <x:c r="A31" s="20" t="str">
+        <x:v>UAI</x:v>
+      </x:c>
+      <x:c r="B31" s="20" t="str">
+        <x:v>Deep Representation Learning; Reinforcement Learning; Time Series &amp; Sequential Data; Explainability &amp; Interpretability; Robustness &amp; Safety</x:v>
+      </x:c>
+      <x:c r="C31" s="20" t="str">
+        <x:v>Learning and reasoning under uncertainty, centered on probabilistic and Bayesian modeling, graphical models, causal inference, approximate inference, and decision theory. Includes Monte Carlo and variational methods, uncertainty quantification, sequential models, and principled analysis of learning algorithms. Uncertainty is the organizing theme, not just another application of general-purpose AI.</x:v>
+      </x:c>
+      <x:c r="D31" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E31" s="20" t="str">
+        <x:v>https://www.auai.org/uai2026/subject_areas; https://www.auai.org/uai2026/call_for_papers</x:v>
+      </x:c>
+      <x:c r="F31" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62005996abd44f46"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add AI, vision, multimedia and biometrics conferences
</commit_message>
<xml_diff>
--- a/data/core_conferences_normalized_tags.xlsx
+++ b/data/core_conferences_normalized_tags.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Conferences" sheetId="1" r:id="Rfbc8fc13ca064400"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Vocabulary" sheetId="2" r:id="R72a1277fb2a8431a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conference Scope" sheetId="3" r:id="Rcebdc42a32d4481d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Conferences" sheetId="1" r:id="R5109e2a6113b4dc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Vocabulary" sheetId="2" r:id="R60990133882a4fa4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conference Scope" sheetId="3" r:id="Rc6fd55c52f23417d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -119,7 +119,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="CoreConferencesTable" displayName="CoreConferencesTable" ref="A1:N83" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="CoreConferencesTable" displayName="CoreConferencesTable" ref="A1:N98" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Conference"/>
     <x:tableColumn id="2" name="TAGS"/>
@@ -141,7 +141,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TagVocabularyTable" displayName="TagVocabularyTable" ref="A1:B30" headerRowCount="1" totalsRowCount="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TagVocabularyTable" displayName="TagVocabularyTable" ref="A1:B35" headerRowCount="1" totalsRowCount="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Standard tag"/>
     <x:tableColumn id="2" name="Definition"/>
@@ -151,7 +151,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ConferenceScope" displayName="ConferenceScope" ref="A1:F31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ConferenceScope" displayName="ConferenceScope" ref="A1:F46" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Series"/>
     <x:tableColumn id="2" name="Additional topics"/>
@@ -3145,10 +3145,570 @@
       <x:c r="M83"/>
       <x:c r="N83"/>
     </x:row>
+    <x:row r="84" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A84" t="str">
+        <x:v>EuroGP</x:v>
+      </x:c>
+      <x:c r="B84" s="12" t="str">
+        <x:v>Evolutionary Computation &amp; Optimization; Machine Learning; Explainability &amp; Interpretability</x:v>
+      </x:c>
+      <x:c r="C84" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="D84" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E84" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="F84" s="12" t="str">
+        <x:v>Paper-based / Springer LNCS</x:v>
+      </x:c>
+      <x:c r="G84" t="str">
+        <x:v>https://www.evostar.org/2027/eurogp/</x:v>
+      </x:c>
+      <x:c r="H84" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/481/</x:v>
+      </x:c>
+      <x:c r="I84"/>
+      <x:c r="J84"/>
+      <x:c r="K84" s="16"/>
+      <x:c r="L84" s="17"/>
+      <x:c r="M84"/>
+      <x:c r="N84"/>
+    </x:row>
+    <x:row r="85" ht="15" hidden="0" customHeight="1">
+      <x:c r="A85" t="str">
+        <x:v>KR</x:v>
+      </x:c>
+      <x:c r="B85" s="12" t="str">
+        <x:v>Knowledge Representation &amp; Reasoning; Explainability &amp; Interpretability</x:v>
+      </x:c>
+      <x:c r="C85" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D85" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E85" t="str">
+        <x:v>A*</x:v>
+      </x:c>
+      <x:c r="F85" s="12" t="str">
+        <x:v>Paper-based / formal and symbolic AI</x:v>
+      </x:c>
+      <x:c r="G85" t="str">
+        <x:v>https://kr.org/</x:v>
+      </x:c>
+      <x:c r="H85" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/1239/</x:v>
+      </x:c>
+      <x:c r="I85" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J85" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=58</x:v>
+      </x:c>
+      <x:c r="K85" s="16"/>
+      <x:c r="L85" s="17"/>
+      <x:c r="M85"/>
+      <x:c r="N85"/>
+    </x:row>
+    <x:row r="86" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A86" t="str">
+        <x:v>ICAPS</x:v>
+      </x:c>
+      <x:c r="B86" s="12" t="str">
+        <x:v>Planning &amp; Search; Knowledge Representation &amp; Reasoning; Machine Learning; Control &amp; Robotics</x:v>
+      </x:c>
+      <x:c r="C86" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D86" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="E86" t="str">
+        <x:v>A*</x:v>
+      </x:c>
+      <x:c r="F86" s="12" t="str">
+        <x:v>Long and short papers / automated planning</x:v>
+      </x:c>
+      <x:c r="G86" t="str">
+        <x:v>https://icaps27.icaps-conference.org/</x:v>
+      </x:c>
+      <x:c r="H86" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/919/</x:v>
+      </x:c>
+      <x:c r="I86" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J86" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=58</x:v>
+      </x:c>
+      <x:c r="K86" s="16" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="L86" s="17" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="M86" t="str">
+        <x:v>Main papers; council minutes report rounded 25% (82 accepted of 335 submitted)</x:v>
+      </x:c>
+      <x:c r="N86" t="str">
+        <x:v>https://www.icaps-conference.org/wp-content/uploads/2025/12/MinutesICAPS2024CouncilMeeting_v2.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A87" t="str">
+        <x:v>3DV</x:v>
+      </x:c>
+      <x:c r="B87" s="12" t="str">
+        <x:v>Computer Vision &amp; Pattern Recognition; Computer Graphics &amp; Visualization; Signal Processing</x:v>
+      </x:c>
+      <x:c r="C87" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D87" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E87"/>
+      <x:c r="F87" s="12" t="str">
+        <x:v>Paper-based / OpenReview</x:v>
+      </x:c>
+      <x:c r="G87" t="str">
+        <x:v>https://3dvconf.github.io/2027/</x:v>
+      </x:c>
+      <x:c r="H87"/>
+      <x:c r="I87" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="J87" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=49</x:v>
+      </x:c>
+      <x:c r="K87" s="16"/>
+      <x:c r="L87" s="17"/>
+      <x:c r="M87"/>
+      <x:c r="N87"/>
+    </x:row>
+    <x:row r="88" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A88" t="str">
+        <x:v>ACM MM</x:v>
+      </x:c>
+      <x:c r="B88" s="12" t="str">
+        <x:v>Multimedia Learning &amp; Retrieval; Computer Vision &amp; Pattern Recognition; Deep Representation Learning; Signal Processing</x:v>
+      </x:c>
+      <x:c r="C88" t="str">
+        <x:v>XL</x:v>
+      </x:c>
+      <x:c r="D88" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E88" t="str">
+        <x:v>A*</x:v>
+      </x:c>
+      <x:c r="F88" s="12" t="str">
+        <x:v>Paper-based / multimedia research</x:v>
+      </x:c>
+      <x:c r="G88" t="str">
+        <x:v>https://www.acmmm.org/</x:v>
+      </x:c>
+      <x:c r="H88" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/37/</x:v>
+      </x:c>
+      <x:c r="I88" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="J88" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=47</x:v>
+      </x:c>
+      <x:c r="K88" s="16"/>
+      <x:c r="L88" s="17"/>
+      <x:c r="M88"/>
+      <x:c r="N88"/>
+    </x:row>
+    <x:row r="89" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A89" t="str">
+        <x:v>ACM SIGGRAPH</x:v>
+      </x:c>
+      <x:c r="B89" s="12" t="str">
+        <x:v>Computer Graphics &amp; Visualization; Machine Learning; Computer Vision &amp; Pattern Recognition</x:v>
+      </x:c>
+      <x:c r="C89" t="str">
+        <x:v>XXL</x:v>
+      </x:c>
+      <x:c r="D89" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E89" t="str">
+        <x:v>A*</x:v>
+      </x:c>
+      <x:c r="F89" s="12" t="str">
+        <x:v>Technical papers / conference and ACM TOG tracks</x:v>
+      </x:c>
+      <x:c r="G89" t="str">
+        <x:v>https://s2027.siggraph.org/</x:v>
+      </x:c>
+      <x:c r="H89" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/38/</x:v>
+      </x:c>
+      <x:c r="I89" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="J89" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=47</x:v>
+      </x:c>
+      <x:c r="K89" s="16"/>
+      <x:c r="L89" s="17"/>
+      <x:c r="M89"/>
+      <x:c r="N89"/>
+    </x:row>
+    <x:row r="90" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A90" t="str">
+        <x:v>BMVC</x:v>
+      </x:c>
+      <x:c r="B90" s="12" t="str">
+        <x:v>Computer Vision &amp; Pattern Recognition; Machine Learning; Deep Representation Learning</x:v>
+      </x:c>
+      <x:c r="C90" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="D90" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E90" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="F90" s="12" t="str">
+        <x:v>Paper-based / BMVA proceedings</x:v>
+      </x:c>
+      <x:c r="G90" t="str">
+        <x:v>https://bmvc2026.bmva.org/</x:v>
+      </x:c>
+      <x:c r="H90" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/296/</x:v>
+      </x:c>
+      <x:c r="I90" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="J90" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=59</x:v>
+      </x:c>
+      <x:c r="K90" s="16"/>
+      <x:c r="L90" s="17"/>
+      <x:c r="M90"/>
+      <x:c r="N90"/>
+    </x:row>
+    <x:row r="91" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A91" t="str">
+        <x:v>CVPR</x:v>
+      </x:c>
+      <x:c r="B91" s="12" t="str">
+        <x:v>Computer Vision &amp; Pattern Recognition; Deep Representation Learning; Machine Learning</x:v>
+      </x:c>
+      <x:c r="C91" t="str">
+        <x:v>XXL</x:v>
+      </x:c>
+      <x:c r="D91" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="E91" t="str">
+        <x:v>A*</x:v>
+      </x:c>
+      <x:c r="F91" s="12" t="str">
+        <x:v>Paper-based / OpenReview</x:v>
+      </x:c>
+      <x:c r="G91" t="str">
+        <x:v>https://cvpr.thecvf.com/Conferences/2027</x:v>
+      </x:c>
+      <x:c r="H91" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/604/</x:v>
+      </x:c>
+      <x:c r="I91" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="J91" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=57</x:v>
+      </x:c>
+      <x:c r="K91" s="16" t="n">
+        <x:v>0.2541</x:v>
+      </x:c>
+      <x:c r="L91" s="17" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="M91" t="str">
+        <x:v>Main technical program (4,089 presentations of 16,092 submissions in the official program release)</x:v>
+      </x:c>
+      <x:c r="N91" t="str">
+        <x:v>https://cvpr.thecvf.com/Conferences/2026/News/Technical_Program</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A92" t="str">
+        <x:v>ECCV</x:v>
+      </x:c>
+      <x:c r="B92" s="12" t="str">
+        <x:v>Computer Vision &amp; Pattern Recognition; Deep Representation Learning; Machine Learning</x:v>
+      </x:c>
+      <x:c r="C92" t="str">
+        <x:v>XXL</x:v>
+      </x:c>
+      <x:c r="D92" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="E92" t="str">
+        <x:v>A*</x:v>
+      </x:c>
+      <x:c r="F92" s="12" t="str">
+        <x:v>Paper-based / Springer proceedings</x:v>
+      </x:c>
+      <x:c r="G92" t="str">
+        <x:v>https://eccv.ecva.net/</x:v>
+      </x:c>
+      <x:c r="H92" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/479/</x:v>
+      </x:c>
+      <x:c r="I92" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J92" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=58</x:v>
+      </x:c>
+      <x:c r="K92" s="16" t="n">
+        <x:v>0.278</x:v>
+      </x:c>
+      <x:c r="L92" s="17" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="M92" t="str">
+        <x:v>Main papers (2,387 accepted of 8,585 valid submissions); calculated from organizer counts</x:v>
+      </x:c>
+      <x:c r="N92" t="str">
+        <x:v>https://eccv.ecva.net/media/eccv-2024/Slides/2822.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A93" t="str">
+        <x:v>EUVIP</x:v>
+      </x:c>
+      <x:c r="B93" s="12" t="str">
+        <x:v>Signal Processing; Computer Vision &amp; Pattern Recognition; Machine Learning; Deep Representation Learning</x:v>
+      </x:c>
+      <x:c r="C93" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="D93" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E93"/>
+      <x:c r="F93" s="12" t="str">
+        <x:v>Paper-based / visual information processing</x:v>
+      </x:c>
+      <x:c r="G93" t="str">
+        <x:v>https://euvip2026.github.io/</x:v>
+      </x:c>
+      <x:c r="H93"/>
+      <x:c r="I93"/>
+      <x:c r="J93"/>
+      <x:c r="K93" s="16"/>
+      <x:c r="L93" s="17"/>
+      <x:c r="M93"/>
+      <x:c r="N93"/>
+    </x:row>
+    <x:row r="94" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A94" t="str">
+        <x:v>FG</x:v>
+      </x:c>
+      <x:c r="B94" s="12" t="str">
+        <x:v>Biometrics &amp; Human Sensing; Computer Vision &amp; Pattern Recognition; Deep Representation Learning; Machine Learning</x:v>
+      </x:c>
+      <x:c r="C94" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D94" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E94" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="F94" s="12" t="str">
+        <x:v>Long and short papers / face, gesture, and body recognition</x:v>
+      </x:c>
+      <x:c r="G94" t="str">
+        <x:v>https://fg2027.ieee-biometrics.org/</x:v>
+      </x:c>
+      <x:c r="H94" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/629/</x:v>
+      </x:c>
+      <x:c r="I94" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="J94" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=59</x:v>
+      </x:c>
+      <x:c r="K94" s="16"/>
+      <x:c r="L94" s="17"/>
+      <x:c r="M94"/>
+      <x:c r="N94"/>
+    </x:row>
+    <x:row r="95" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A95" t="str">
+        <x:v>ICCV</x:v>
+      </x:c>
+      <x:c r="B95" s="12" t="str">
+        <x:v>Computer Vision &amp; Pattern Recognition; Deep Representation Learning; Machine Learning</x:v>
+      </x:c>
+      <x:c r="C95" t="str">
+        <x:v>XXL</x:v>
+      </x:c>
+      <x:c r="D95" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="E95" t="str">
+        <x:v>A*</x:v>
+      </x:c>
+      <x:c r="F95" s="12" t="str">
+        <x:v>Paper-based / OpenReview</x:v>
+      </x:c>
+      <x:c r="G95" t="str">
+        <x:v>https://iccv.thecvf.com/Conferences/2027</x:v>
+      </x:c>
+      <x:c r="H95" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/638/</x:v>
+      </x:c>
+      <x:c r="I95" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="J95" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=57</x:v>
+      </x:c>
+      <x:c r="K95" s="16" t="n">
+        <x:v>0.24</x:v>
+      </x:c>
+      <x:c r="L95" s="17" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="M95" t="str">
+        <x:v>Main papers; chairs' rounded rate (2,701 accepted of 11,239 valid submissions)</x:v>
+      </x:c>
+      <x:c r="N95" t="str">
+        <x:v>https://media.eventhosts.cc/Conferences/ICCV2025/iccv25_main_program.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A96" t="str">
+        <x:v>ICMR</x:v>
+      </x:c>
+      <x:c r="B96" s="12" t="str">
+        <x:v>Multimedia Learning &amp; Retrieval; Computer Vision &amp; Pattern Recognition; Machine Learning; Deep Representation Learning</x:v>
+      </x:c>
+      <x:c r="C96" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D96" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E96" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="F96" s="12" t="str">
+        <x:v>Full and short papers / multimedia retrieval</x:v>
+      </x:c>
+      <x:c r="G96" t="str">
+        <x:v>https://www.icmr2027.org/</x:v>
+      </x:c>
+      <x:c r="H96" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/44/</x:v>
+      </x:c>
+      <x:c r="I96" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J96" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=48</x:v>
+      </x:c>
+      <x:c r="K96" s="16"/>
+      <x:c r="L96" s="17"/>
+      <x:c r="M96"/>
+      <x:c r="N96"/>
+    </x:row>
+    <x:row r="97" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A97" t="str">
+        <x:v>IJCB</x:v>
+      </x:c>
+      <x:c r="B97" s="12" t="str">
+        <x:v>Biometrics &amp; Human Sensing; Computer Vision &amp; Pattern Recognition; Deep Representation Learning; Privacy-preserving ML</x:v>
+      </x:c>
+      <x:c r="C97" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D97" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E97" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="F97" s="12" t="str">
+        <x:v>Paper-based / biometrics and identity science</x:v>
+      </x:c>
+      <x:c r="G97" t="str">
+        <x:v>https://ijcb2027.ieee-biometrics.org/</x:v>
+      </x:c>
+      <x:c r="H97" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/2305/</x:v>
+      </x:c>
+      <x:c r="I97" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="J97" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=60</x:v>
+      </x:c>
+      <x:c r="K97" s="16"/>
+      <x:c r="L97" s="17"/>
+      <x:c r="M97"/>
+      <x:c r="N97"/>
+    </x:row>
+    <x:row r="98" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A98" t="str">
+        <x:v>WACV</x:v>
+      </x:c>
+      <x:c r="B98" s="12" t="str">
+        <x:v>Computer Vision &amp; Pattern Recognition; Machine Learning; Deep Representation Learning</x:v>
+      </x:c>
+      <x:c r="C98" t="str">
+        <x:v>XL</x:v>
+      </x:c>
+      <x:c r="D98" t="str">
+        <x:v>Moderate</x:v>
+      </x:c>
+      <x:c r="E98" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="F98" s="12" t="str">
+        <x:v>Paper-based / two independent submission rounds</x:v>
+      </x:c>
+      <x:c r="G98" t="str">
+        <x:v>https://wacv.thecvf.com/Conferences/2027</x:v>
+      </x:c>
+      <x:c r="H98" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/763/</x:v>
+      </x:c>
+      <x:c r="I98"/>
+      <x:c r="J98"/>
+      <x:c r="K98" s="16" t="n">
+        <x:v>0.33</x:v>
+      </x:c>
+      <x:c r="L98" s="17" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="M98" t="str">
+        <x:v>Main papers across both rounds; chairs' rounded rate (832 accepted of 2,550 submissions)</x:v>
+      </x:c>
+      <x:c r="N98" t="str">
+        <x:v>https://media.eventhosts.cc/Conferences/WACV2026/wacv_2026_program_v18_Digital.pdf</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16568e3c52dc4540"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5dc5d7f55d874962"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3222,7 +3782,7 @@
         <x:v>Signal Processing</x:v>
       </x:c>
       <x:c r="B8" s="14" t="str">
-        <x:v>Signal processing methods and ML for signals, including biomedical signals. Family: Signals &amp; Vision.</x:v>
+        <x:v>Signal processing methods and ML for signals, including biomedical signals. Family: Signals, Vision &amp; Multimedia.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -3326,7 +3886,7 @@
         <x:v>Computer Vision &amp; Pattern Recognition</x:v>
       </x:c>
       <x:c r="B21" s="12" t="str">
-        <x:v>Visual understanding, image analysis, recognition, and structured pattern learning. Family: Signals &amp; Vision.</x:v>
+        <x:v>Visual understanding, image analysis, recognition, and structured pattern learning. Family: Signals, Vision &amp; Multimedia.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -3409,10 +3969,50 @@
         <x:v>Systems for ML and ML for systems, including training, inference, compilers, hardware, and serving. Family: ML &amp; AI.</x:v>
       </x:c>
     </x:row>
+    <x:row r="32" ht="15" hidden="0" customHeight="1">
+      <x:c r="A32" t="str">
+        <x:v>Knowledge Representation &amp; Reasoning</x:v>
+      </x:c>
+      <x:c r="B32" s="12" t="str">
+        <x:v>Formal and symbolic representations of knowledge, logic, automated inference, and reasoning in AI. Family: ML &amp; AI.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="15" hidden="0" customHeight="1">
+      <x:c r="A33" t="str">
+        <x:v>Planning &amp; Search</x:v>
+      </x:c>
+      <x:c r="B33" s="12" t="str">
+        <x:v>Automated planning, scheduling, heuristic search, constraint solving, and sequential decision-making. Family: ML &amp; AI.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A34" t="str">
+        <x:v>Computer Graphics &amp; Visualization</x:v>
+      </x:c>
+      <x:c r="B34" s="12" t="str">
+        <x:v>Rendering, geometry, animation, visual simulation, and visualization, including learning-based methods. Family: Signals, Vision &amp; Multimedia.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A35" t="str">
+        <x:v>Multimedia Learning &amp; Retrieval</x:v>
+      </x:c>
+      <x:c r="B35" s="12" t="str">
+        <x:v>Learning from multiple media, multimodal fusion, content understanding, indexing, search, and retrieval. Family: Signals, Vision &amp; Multimedia.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A36" t="str">
+        <x:v>Biometrics &amp; Human Sensing</x:v>
+      </x:c>
+      <x:c r="B36" s="12" t="str">
+        <x:v>Biometric identity, face and gesture recognition, body motion, behavioral sensing, and biometric evaluation. Family: Signals, Vision &amp; Multimedia.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6276ba1efc204ab0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cb5f4dc5093453e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3449,41 +4049,39 @@
         <x:v>Scope reviewed</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="60" hidden="0" customHeight="1">
+    <x:row r="2" ht="72" hidden="0" customHeight="1">
       <x:c r="A2" s="20" t="str">
-        <x:v>AALTD</x:v>
-      </x:c>
-      <x:c r="B2" s="20" t="str">
-        <x:v>Deep Representation Learning</x:v>
-      </x:c>
+        <x:v>3DV</x:v>
+      </x:c>
+      <x:c r="B2" s="20" t="str"/>
       <x:c r="C2" s="20" t="str">
-        <x:v>Analytics and learning specifically for temporal data: time-series classification, clustering, forecasting, segmentation, anomaly detection, temporal representations, and metric or kernel learning. Includes temporal foundation models, data streams, and explainable temporal analysis. Climate, health, and energy are examples of applications rather than separate defining topic assignments.</x:v>
+        <x:v>Three-dimensional computer vision and graphics, especially sensing, geometric modeling and representations, reconstruction, analysis, rendering, and visualization. It is a focused venue for recovering and understanding 3D structure rather than all of computer vision. Papers combine geometric, imaging, and computational methods; unrelated applications and every possible ML technique are not added as separate scope tags.</x:v>
       </x:c>
       <x:c r="D2" s="21" t="n">
-        <x:v>2026</x:v>
+        <x:v>2027</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>https://ecml-aaltd.github.io/aaltd2026/</x:v>
+        <x:v>https://3dvconf.github.io/2027/; https://3dvconf.github.io/2027/author-guidelines/</x:v>
       </x:c>
       <x:c r="F2" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="72" hidden="0" customHeight="1">
+    <x:row r="3" ht="60" hidden="0" customHeight="1">
       <x:c r="A3" s="20" t="str">
-        <x:v>AAMAS</x:v>
+        <x:v>AALTD</x:v>
       </x:c>
       <x:c r="B3" s="20" t="str">
-        <x:v>Deep Representation Learning; Probabilistic, Causal &amp; Uncertainty ML; Evolutionary Computation &amp; Optimization; Complex Systems &amp; Network Science; Ethics &amp; Governance; Explainability &amp; Interpretability</x:v>
+        <x:v>Deep Representation Learning</x:v>
       </x:c>
       <x:c r="C3" s="20" t="str">
-        <x:v>Autonomous agents and multi-agent systems: learning and adaptation, coordination, game theory, planning, reasoning, agent engineering, and agent-based simulation. Also covers human-agent interaction, robot teams, norms and governance, and generative agents. The contribution should concern agents or their interaction; generic language-model or learning results are not automatically in scope.</x:v>
+        <x:v>Analytics and learning specifically for temporal data: time-series classification, clustering, forecasting, segmentation, anomaly detection, temporal representations, and metric or kernel learning. Includes temporal foundation models, data streams, and explainable temporal analysis. Climate, health, and energy are examples of applications rather than separate defining topic assignments.</x:v>
       </x:c>
       <x:c r="D3" s="21" t="n">
-        <x:v>2027</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="E3" s="20" t="str">
-        <x:v>https://warwick.ac.uk/fac/sci/dcs/aamas2027/calls/call-for-main-track/</x:v>
+        <x:v>https://ecml-aaltd.github.io/aaltd2026/</x:v>
       </x:c>
       <x:c r="F3" s="22" t="n">
         <x:v>46302</x:v>
@@ -3491,155 +4089,157 @@
     </x:row>
     <x:row r="4" ht="72" hidden="0" customHeight="1">
       <x:c r="A4" s="20" t="str">
-        <x:v>ACM FAccT</x:v>
+        <x:v>AAMAS</x:v>
       </x:c>
       <x:c r="B4" s="20" t="str">
-        <x:v>Human-AI Interaction &amp; Deployment; Robustness &amp; Safety</x:v>
+        <x:v>Deep Representation Learning; Probabilistic, Causal &amp; Uncertainty ML; Evolutionary Computation &amp; Optimization; Complex Systems &amp; Network Science; Ethics &amp; Governance; Explainability &amp; Interpretability</x:v>
       </x:c>
       <x:c r="C4" s="20" t="str">
-        <x:v>Fairness, accountability, and transparency in computing, combining algorithmic research with sociotechnical, legal, philosophical, and human-centered approaches. Characteristic contributions include audits and evaluation practices, governance, human experiences of systems, and responsible development and deployment. A fairness or accountability question should be substantive, not a passing motivation for generic ML.</x:v>
+        <x:v>Autonomous agents and multi-agent systems: learning and adaptation, coordination, game theory, planning, reasoning, agent engineering, and agent-based simulation. Also covers human-agent interaction, robot teams, norms and governance, and generative agents. The contribution should concern agents or their interaction; generic language-model or learning results are not automatically in scope.</x:v>
       </x:c>
       <x:c r="D4" s="21" t="n">
-        <x:v>2026</x:v>
+        <x:v>2027</x:v>
       </x:c>
       <x:c r="E4" s="20" t="str">
-        <x:v>https://facctconference.org/2026/cfp.html</x:v>
+        <x:v>https://warwick.ac.uk/fac/sci/dcs/aamas2027/calls/call-for-main-track/</x:v>
       </x:c>
       <x:c r="F4" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="60" hidden="0" customHeight="1">
+    <x:row r="5" ht="72" hidden="0" customHeight="1">
       <x:c r="A5" s="20" t="str">
-        <x:v>ACML</x:v>
+        <x:v>ACM FAccT</x:v>
       </x:c>
       <x:c r="B5" s="20" t="str">
-        <x:v>Deep Representation Learning; Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Natural Language Processing &amp; LLMs; Fairness &amp; Responsible AI; Privacy-preserving ML</x:v>
+        <x:v>Human-AI Interaction &amp; Deployment; Robustness &amp; Safety</x:v>
       </x:c>
       <x:c r="C5" s="20" t="str">
-        <x:v>Theory and practice of machine learning, including probabilistic methods, representation learning, transfer and meta-learning, reinforcement learning, and learning theory. Generative models, language models, and trustworthy learning extend this core. The broad applications list is not treated as evidence that every application field defines the conference.</x:v>
+        <x:v>Fairness, accountability, and transparency in computing, combining algorithmic research with sociotechnical, legal, philosophical, and human-centered approaches. Characteristic contributions include audits and evaluation practices, governance, human experiences of systems, and responsible development and deployment. A fairness or accountability question should be substantive, not a passing motivation for generic ML.</x:v>
       </x:c>
       <x:c r="D5" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E5" s="20" t="str">
-        <x:v>https://www.acml-conf.org/2026/calls/papers/</x:v>
+        <x:v>https://facctconference.org/2026/cfp.html</x:v>
       </x:c>
       <x:c r="F5" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="60" hidden="0" customHeight="1">
+    <x:row r="6" ht="72" hidden="0" customHeight="1">
       <x:c r="A6" s="20" t="str">
-        <x:v>AIES</x:v>
+        <x:v>ACM MM</x:v>
       </x:c>
       <x:c r="B6" s="20" t="str">
-        <x:v>Human-AI Interaction &amp; Deployment; Privacy-preserving ML</x:v>
+        <x:v>Machine Learning; Natural Language Processing &amp; LLMs; Human-AI Interaction &amp; Deployment; Data Mining &amp; Data Science; Explainability &amp; Interpretability</x:v>
       </x:c>
       <x:c r="C6" s="20" t="str">
-        <x:v>Ethics and societal consequences of AI, connecting computer science, law and policy, social science, and philosophy. Defining concerns include governance and power, accountability after deployment, value alignment, fairness, human-AI interaction, and institutional practice. Technical work is relevant through a serious ethical or societal contribution.</x:v>
+        <x:v>Multimedia understanding, learning, generation, and retrieval across image, video, audio, language, and other modalities. Characteristic work includes multimodal fusion, generative and foundation models, scalable indexing and search, cross-modal alignment, and human-centered multimedia experiences. The 2026 steering-committee scope also emphasizes explainability. Healthcare, education, and entertainment are applications, not blanket topical identities.</x:v>
       </x:c>
       <x:c r="D6" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E6" s="20" t="str">
-        <x:v>https://www.aies-conference.com/2026/call-for-papers/</x:v>
+        <x:v>https://2026.acmmm.org/site/topics.html; https://2026.acmmm.org/</x:v>
       </x:c>
       <x:c r="F6" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="48" hidden="0" customHeight="1">
+    <x:row r="7" ht="72" hidden="0" customHeight="1">
       <x:c r="A7" s="20" t="str">
-        <x:v>AISTATS</x:v>
-      </x:c>
-      <x:c r="B7" s="20" t="str"/>
+        <x:v>ACM SIGGRAPH</x:v>
+      </x:c>
+      <x:c r="B7" s="20" t="str">
+        <x:v>Deep Representation Learning; Human-AI Interaction &amp; Deployment</x:v>
+      </x:c>
       <x:c r="C7" s="20" t="str">
-        <x:v>Research at the interface of artificial intelligence, machine learning, and statistics. Its defining emphasis is on statistical foundations and methodology for learning and inference, rather than a particular application domain. Research bridges statistical reasoning and learning algorithms, with archival contributions to both communities.</x:v>
+        <x:v>Computer graphics and interactive techniques, centered on rendering, geometric modeling, animation, physical simulation, imaging, visualization, and immersive visual experiences. Generative AI and machine learning are relevant when they advance visual computing, such as neural rendering and learned animation. Technical papers use integrated conference and ACM TOG journal tracks; this profile does not describe SIGGRAPH Asia or all of AI.</x:v>
       </x:c>
       <x:c r="D7" s="21" t="n">
-        <x:v>2027</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="E7" s="20" t="str">
-        <x:v>https://aistats.org/aistats2027/; https://aistats.org/aistats2027/call-for-papers.html</x:v>
+        <x:v>https://s2026.siggraph.org/program/technical-papers/</x:v>
       </x:c>
       <x:c r="F7" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="72" hidden="0" customHeight="1">
+    <x:row r="8" ht="60" hidden="0" customHeight="1">
       <x:c r="A8" s="20" t="str">
-        <x:v>AutoML</x:v>
+        <x:v>ACML</x:v>
       </x:c>
       <x:c r="B8" s="20" t="str">
-        <x:v>Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Explainability &amp; Interpretability; Natural Language Processing &amp; LLMs; Robustness &amp; Safety</x:v>
+        <x:v>Deep Representation Learning; Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Natural Language Processing &amp; LLMs; Fairness &amp; Responsible AI; Privacy-preserving ML</x:v>
       </x:c>
       <x:c r="C8" s="20" t="str">
-        <x:v>Automating the construction and configuration of learning systems: hyperparameter optimization, Bayesian optimization, neural architecture search, model selection, meta-learning, and pipeline automation. Includes evolutionary and reinforcement-learning approaches, AutoML for foundation models, and evaluation through applications, benchmarks, challenges, and datasets. Trustworthiness matters specifically in automated ML workflows.</x:v>
+        <x:v>Theory and practice of machine learning, including probabilistic methods, representation learning, transfer and meta-learning, reinforcement learning, and learning theory. Generative models, language models, and trustworthy learning extend this core. The broad applications list is not treated as evidence that every application field defines the conference.</x:v>
       </x:c>
       <x:c r="D8" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E8" s="20" t="str">
-        <x:v>https://2026.automl.cc/call-for-papers/</x:v>
+        <x:v>https://www.acml-conf.org/2026/calls/papers/</x:v>
       </x:c>
       <x:c r="F8" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="72" hidden="0" customHeight="1">
+    <x:row r="9" ht="60" hidden="0" customHeight="1">
       <x:c r="A9" s="20" t="str">
-        <x:v>CCN</x:v>
+        <x:v>AIES</x:v>
       </x:c>
       <x:c r="B9" s="20" t="str">
-        <x:v>Cognitive Science &amp; Computational Cognition; Explainability &amp; Interpretability</x:v>
+        <x:v>Human-AI Interaction &amp; Deployment; Privacy-preserving ML</x:v>
       </x:c>
       <x:c r="C9" s="20" t="str">
-        <x:v>Cognitive computational neuroscience, connecting experiments and models of brain computation with artificial intelligence. Characteristic work compares biological and artificial representations, models perception, cognition and action, studies neural connectivity and dynamics, and uses mechanistic interpretability to understand neural-network models. The aim is understanding computation and behavior across brains and AI systems.</x:v>
+        <x:v>Ethics and societal consequences of AI, connecting computer science, law and policy, social science, and philosophy. Defining concerns include governance and power, accountability after deployment, value alignment, fairness, human-AI interaction, and institutional practice. Technical work is relevant through a serious ethical or societal contribution.</x:v>
       </x:c>
       <x:c r="D9" s="21" t="n">
-        <x:v>2027</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="E9" s="20" t="str">
-        <x:v>https://2027.ccneuro.org/</x:v>
+        <x:v>https://www.aies-conference.com/2026/call-for-papers/</x:v>
       </x:c>
       <x:c r="F9" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="72" hidden="0" customHeight="1">
+    <x:row r="10" ht="48" hidden="0" customHeight="1">
       <x:c r="A10" s="20" t="str">
-        <x:v>CHIL</x:v>
-      </x:c>
-      <x:c r="B10" s="20" t="str">
-        <x:v>Explainability &amp; Interpretability; Human-AI Interaction &amp; Deployment; Robustness &amp; Safety; Time Series &amp; Sequential Data</x:v>
-      </x:c>
+        <x:v>AISTATS</x:v>
+      </x:c>
+      <x:c r="B10" s="20" t="str"/>
       <x:c r="C10" s="20" t="str">
-        <x:v>Machine learning and inference for clinical, public, and population health. Distinguishing areas include causal inference, survival analysis, multimodal health data, generalization across populations, interpretability, and clinical evaluation and deployment. Research may emphasize methods, practical applications, or societal impact. Health-focused inference and evaluation remain the common thread across these tracks.</x:v>
+        <x:v>Research at the interface of artificial intelligence, machine learning, and statistics. Its defining emphasis is on statistical foundations and methodology for learning and inference, rather than a particular application domain. Research bridges statistical reasoning and learning algorithms, with archival contributions to both communities.</x:v>
       </x:c>
       <x:c r="D10" s="21" t="n">
-        <x:v>2026</x:v>
+        <x:v>2027</x:v>
       </x:c>
       <x:c r="E10" s="20" t="str">
-        <x:v>https://chil.ahli.cc/submit/call-for-papers/</x:v>
+        <x:v>https://aistats.org/aistats2027/; https://aistats.org/aistats2027/call-for-papers.html</x:v>
       </x:c>
       <x:c r="F10" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="60" hidden="0" customHeight="1">
+    <x:row r="11" ht="72" hidden="0" customHeight="1">
       <x:c r="A11" s="20" t="str">
-        <x:v>CogSci</x:v>
-      </x:c>
-      <x:c r="B11" s="20" t="str"/>
+        <x:v>AutoML</x:v>
+      </x:c>
+      <x:c r="B11" s="20" t="str">
+        <x:v>Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Explainability &amp; Interpretability; Natural Language Processing &amp; LLMs; Robustness &amp; Safety</x:v>
+      </x:c>
       <x:c r="C11" s="20" t="str">
-        <x:v>Interdisciplinary study of cognition and the mind, connecting psychology, linguistics, artificial intelligence, neuroscience, philosophy, anthropology, and education. Computational models and experiments should illuminate cognitive processes and behavior. An AI paper belongs here through its contribution to understanding cognition, not solely through a predictive performance improvement.</x:v>
+        <x:v>Automating the construction and configuration of learning systems: hyperparameter optimization, Bayesian optimization, neural architecture search, model selection, meta-learning, and pipeline automation. Includes evolutionary and reinforcement-learning approaches, AutoML for foundation models, and evaluation through applications, benchmarks, challenges, and datasets. Trustworthiness matters specifically in automated ML workflows.</x:v>
       </x:c>
       <x:c r="D11" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E11" s="20" t="str">
-        <x:v>https://cognitivesciencesociety.org/submissions-faq/; https://cognitivesciencesociety.org/</x:v>
+        <x:v>https://2026.automl.cc/call-for-papers/</x:v>
       </x:c>
       <x:c r="F11" s="22" t="n">
         <x:v>46302</x:v>
@@ -3647,19 +4247,19 @@
     </x:row>
     <x:row r="12" ht="60" hidden="0" customHeight="1">
       <x:c r="A12" s="20" t="str">
-        <x:v>COLT</x:v>
+        <x:v>BMVC</x:v>
       </x:c>
       <x:c r="B12" s="20" t="str">
-        <x:v>Deep Representation Learning; Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Privacy-preserving ML; Fairness &amp; Responsible AI</x:v>
+        <x:v>Signal Processing</x:v>
       </x:c>
       <x:c r="C12" s="20" t="str">
-        <x:v>Theoretical foundations of learning at the intersection of computer science, statistics, and applied mathematics. Characteristic work studies learnability, sample and computational complexity, online learning, optimization, bandits, and generalization. Neural-network, causal, reinforcement-learning, privacy, and fairness papers belong here when the theoretical contribution is central.</x:v>
+        <x:v>Computer vision, image processing, and visual pattern recognition, including visual learning, recognition and segmentation, reconstruction, motion and video analysis, and evaluation of vision methods. The single-track BMVA conference combines methodological and applied vision research. It is an established broad vision venue, not a specialist biomedical-imaging meeting.</x:v>
       </x:c>
       <x:c r="D12" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E12" s="20" t="str">
-        <x:v>https://learningtheory.org/colt2026/cfp.html</x:v>
+        <x:v>https://bmvc2026.bmva.org/calls/call-for-papers/</x:v>
       </x:c>
       <x:c r="F12" s="22" t="n">
         <x:v>46302</x:v>
@@ -3667,19 +4267,19 @@
     </x:row>
     <x:row r="13" ht="72" hidden="0" customHeight="1">
       <x:c r="A13" s="20" t="str">
-        <x:v>CoRL</x:v>
+        <x:v>CCN</x:v>
       </x:c>
       <x:c r="B13" s="20" t="str">
-        <x:v>Computer Vision &amp; Pattern Recognition; Probabilistic, Causal &amp; Uncertainty ML; Human-AI Interaction &amp; Deployment; Robustness &amp; Safety; Learning Theory &amp; Statistical Foundations</x:v>
+        <x:v>Cognitive Science &amp; Computational Cognition; Explainability &amp; Interpretability</x:v>
       </x:c>
       <x:c r="C13" s="20" t="str">
-        <x:v>Machine learning for physical robots, especially imitation and reinforcement learning, learned perception and control, robot foundation models, and learning-based task and motion planning. Includes uncertainty, generalization, safety, human-robot interaction, and datasets grounded in manipulation, navigation, or locomotion. General ML is relevant when it makes a substantive contribution to robot learning.</x:v>
+        <x:v>Cognitive computational neuroscience, connecting experiments and models of brain computation with artificial intelligence. Characteristic work compares biological and artificial representations, models perception, cognition and action, studies neural connectivity and dynamics, and uses mechanistic interpretability to understand neural-network models. The aim is understanding computation and behavior across brains and AI systems.</x:v>
       </x:c>
       <x:c r="D13" s="21" t="n">
-        <x:v>2026</x:v>
+        <x:v>2027</x:v>
       </x:c>
       <x:c r="E13" s="20" t="str">
-        <x:v>https://www.corl.org/contributions/call-for-papers</x:v>
+        <x:v>https://2027.ccneuro.org/</x:v>
       </x:c>
       <x:c r="F13" s="22" t="n">
         <x:v>46302</x:v>
@@ -3687,19 +4287,19 @@
     </x:row>
     <x:row r="14" ht="72" hidden="0" customHeight="1">
       <x:c r="A14" s="20" t="str">
-        <x:v>EACL</x:v>
+        <x:v>CHIL</x:v>
       </x:c>
       <x:c r="B14" s="20" t="str">
-        <x:v>Explainability &amp; Interpretability; Fairness &amp; Responsible AI; Cognitive Science &amp; Computational Cognition</x:v>
+        <x:v>Explainability &amp; Interpretability; Human-AI Interaction &amp; Deployment; Robustness &amp; Safety; Time Series &amp; Sequential Data</x:v>
       </x:c>
       <x:c r="C14" s="20" t="str">
-        <x:v>Computational linguistics and natural language processing, including language modeling, multilingual processing, translation, dialogue, information extraction, semantics, and linguistic analysis. Human-centered evaluation, interpretability, and bias are relevant within language research. The reviewed 2027 theme strengthens connections to psycholinguistics and cognitive modeling; peripheral application domains are not extra tags.</x:v>
+        <x:v>Machine learning and inference for clinical, public, and population health. Distinguishing areas include causal inference, survival analysis, multimodal health data, generalization across populations, interpretability, and clinical evaluation and deployment. Research may emphasize methods, practical applications, or societal impact. Health-focused inference and evaluation remain the common thread across these tracks.</x:v>
       </x:c>
       <x:c r="D14" s="21" t="n">
-        <x:v>2027</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="E14" s="20" t="str">
-        <x:v>https://2027.eacl.org/calls/papers/</x:v>
+        <x:v>https://chil.ahli.cc/submit/call-for-papers/</x:v>
       </x:c>
       <x:c r="F14" s="22" t="n">
         <x:v>46302</x:v>
@@ -3707,19 +4307,17 @@
     </x:row>
     <x:row r="15" ht="60" hidden="0" customHeight="1">
       <x:c r="A15" s="20" t="str">
-        <x:v>FMTS @ NeurIPS</x:v>
-      </x:c>
-      <x:c r="B15" s="20" t="str">
-        <x:v>System Identification &amp; Data-driven Dynamics; Robustness &amp; Safety</x:v>
-      </x:c>
+        <x:v>CogSci</x:v>
+      </x:c>
+      <x:c r="B15" s="20" t="str"/>
       <x:c r="C15" s="20" t="str">
-        <x:v>Foundation models for temporal systems, centered on long-horizon and probabilistic forecasting, temporal pretraining, generative simulation, irregularly sampled and multimodal sequences, and state-space architectures. Reliability is a defining theme: distribution shift, calibrated uncertainty, leakage-aware benchmarks, and consistency of simulated trajectories.</x:v>
+        <x:v>Interdisciplinary study of cognition and the mind, connecting psychology, linguistics, artificial intelligence, neuroscience, philosophy, anthropology, and education. Computational models and experiments should illuminate cognitive processes and behavior. An AI paper belongs here through its contribution to understanding cognition, not solely through a predictive performance improvement.</x:v>
       </x:c>
       <x:c r="D15" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E15" s="20" t="str">
-        <x:v>https://fmts-workshop.github.io/cfp.html</x:v>
+        <x:v>https://cognitivesciencesociety.org/submissions-faq/; https://cognitivesciencesociety.org/</x:v>
       </x:c>
       <x:c r="F15" s="22" t="n">
         <x:v>46302</x:v>
@@ -3727,19 +4325,19 @@
     </x:row>
     <x:row r="16" ht="60" hidden="0" customHeight="1">
       <x:c r="A16" s="20" t="str">
-        <x:v>GECCO</x:v>
+        <x:v>COLT</x:v>
       </x:c>
       <x:c r="B16" s="20" t="str">
-        <x:v>Deep Representation Learning; Learning Theory &amp; Statistical Foundations</x:v>
+        <x:v>Deep Representation Learning; Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Privacy-preserving ML; Fairness &amp; Responsible AI</x:v>
       </x:c>
       <x:c r="C16" s="20" t="str">
-        <x:v>Genetic and evolutionary computation, including genetic algorithms, genetic programming, swarm intelligence, evolutionary multiobjective and combinatorial optimization, metaheuristics, and neuroevolution. Machine learning is relevant through evolutionary learning and optimization, not as an unrestricted substitute for the conference's evolutionary-computation focus.</x:v>
+        <x:v>Theoretical foundations of learning at the intersection of computer science, statistics, and applied mathematics. Characteristic work studies learnability, sample and computational complexity, online learning, optimization, bandits, and generalization. Neural-network, causal, reinforcement-learning, privacy, and fairness papers belong here when the theoretical contribution is central.</x:v>
       </x:c>
       <x:c r="D16" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E16" s="20" t="str">
-        <x:v>https://gecco-2027.sigevo.org/Call+for+Papers</x:v>
+        <x:v>https://learningtheory.org/colt2026/cfp.html</x:v>
       </x:c>
       <x:c r="F16" s="22" t="n">
         <x:v>46302</x:v>
@@ -3747,77 +4345,79 @@
     </x:row>
     <x:row r="17" ht="72" hidden="0" customHeight="1">
       <x:c r="A17" s="20" t="str">
-        <x:v>ICIP</x:v>
-      </x:c>
-      <x:c r="B17" s="20" t="str"/>
+        <x:v>CoRL</x:v>
+      </x:c>
+      <x:c r="B17" s="20" t="str">
+        <x:v>Computer Vision &amp; Pattern Recognition; Probabilistic, Causal &amp; Uncertainty ML; Human-AI Interaction &amp; Deployment; Robustness &amp; Safety; Learning Theory &amp; Statistical Foundations</x:v>
+      </x:c>
       <x:c r="C17" s="20" t="str">
-        <x:v>Image and video processing across theory, algorithms, and imaging systems. Characteristic problems include restoration, enhancement, reconstruction, registration, compression, quality assessment, and visual analysis. Learning methods and generative models are relevant when they advance image or video processing. The long list of imaging application domains is intentionally not converted into extra specialist-conference tags.</x:v>
+        <x:v>Machine learning for physical robots, especially imitation and reinforcement learning, learned perception and control, robot foundation models, and learning-based task and motion planning. Includes uncertainty, generalization, safety, human-robot interaction, and datasets grounded in manipulation, navigation, or locomotion. General ML is relevant when it makes a substantive contribution to robot learning.</x:v>
       </x:c>
       <x:c r="D17" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E17" s="20" t="str">
-        <x:v>https://2026.ieeeicip.org/topics/</x:v>
+        <x:v>https://www.corl.org/contributions/call-for-papers</x:v>
       </x:c>
       <x:c r="F17" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="60" hidden="0" customHeight="1">
+    <x:row r="18" ht="72" hidden="0" customHeight="1">
       <x:c r="A18" s="20" t="str">
-        <x:v>ICLR</x:v>
+        <x:v>CVPR</x:v>
       </x:c>
       <x:c r="B18" s="20" t="str">
-        <x:v>Learning Theory &amp; Statistical Foundations; Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Natural Language Processing &amp; LLMs; Computer Vision &amp; Pattern Recognition; ML Systems &amp; Infrastructure</x:v>
+        <x:v>Computer Graphics &amp; Visualization; Multimedia Learning &amp; Retrieval; Natural Language Processing &amp; LLMs; Biometrics &amp; Human Sensing; Robustness &amp; Safety</x:v>
       </x:c>
       <x:c r="C18" s="20" t="str">
-        <x:v>Learning representations and understanding deep learning, with an emphasis on self-supervised learning, generative models, transfer and meta-learning, and the optimization and theory of learned representations. Language, vision, probabilistic modeling, and reinforcement learning are substantial areas, rather than unrelated application-domain tags.</x:v>
+        <x:v>Broad computer vision and pattern recognition: visual representations, recognition and segmentation, 3D reconstruction, computational imaging, image and video generation, motion and tracking, and vision-language learning. Graphics, multimodal learning, human face/body understanding, and reliable vision are substantial recurring research areas. Peripheral application fields are not tagged merely because a long CFP mentions them.</x:v>
       </x:c>
       <x:c r="D18" s="21" t="n">
         <x:v>2027</x:v>
       </x:c>
       <x:c r="E18" s="20" t="str">
-        <x:v>https://iclr.cc/Conferences/2027/CallForPapers</x:v>
+        <x:v>https://cvpr.thecvf.com/Conferences/2027/CallForPapers</x:v>
       </x:c>
       <x:c r="F18" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="60" hidden="0" customHeight="1">
+    <x:row r="19" ht="72" hidden="0" customHeight="1">
       <x:c r="A19" s="20" t="str">
-        <x:v>ICML</x:v>
+        <x:v>EACL</x:v>
       </x:c>
       <x:c r="B19" s="20" t="str">
-        <x:v>Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Explainability &amp; Interpretability; Robustness &amp; Safety; ML Systems &amp; Infrastructure; Federated &amp; Distributed Learning</x:v>
+        <x:v>Explainability &amp; Interpretability; Fairness &amp; Responsible AI; Cognitive Science &amp; Computational Cognition</x:v>
       </x:c>
       <x:c r="C19" s="20" t="str">
-        <x:v>Methodological and theoretical machine learning, including supervised and unsupervised learning, deep generative models, optimization, statistical learning theory, Bayesian methods, and reinforcement learning. Scalable systems and trustworthy learning are established parts of the scope; application papers should offer contributions of wider interest to ML.</x:v>
+        <x:v>Computational linguistics and natural language processing, including language modeling, multilingual processing, translation, dialogue, information extraction, semantics, and linguistic analysis. Human-centered evaluation, interpretability, and bias are relevant within language research. The reviewed 2027 theme strengthens connections to psycholinguistics and cognitive modeling; peripheral application domains are not extra tags.</x:v>
       </x:c>
       <x:c r="D19" s="21" t="n">
-        <x:v>2026</x:v>
+        <x:v>2027</x:v>
       </x:c>
       <x:c r="E19" s="20" t="str">
-        <x:v>https://icml.cc/Conferences/2026/CallForPapers</x:v>
+        <x:v>https://2027.eacl.org/calls/papers/</x:v>
       </x:c>
       <x:c r="F19" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="60" hidden="0" customHeight="1">
+    <x:row r="20" ht="72" hidden="0" customHeight="1">
       <x:c r="A20" s="20" t="str">
-        <x:v>IFAC SYSID</x:v>
+        <x:v>ECCV</x:v>
       </x:c>
       <x:c r="B20" s="20" t="str">
-        <x:v>Nonlinear Dynamics &amp; Chaos; Complex Systems &amp; Network Science</x:v>
+        <x:v>Computer Graphics &amp; Visualization; Multimedia Learning &amp; Retrieval; Natural Language Processing &amp; LLMs; Biometrics &amp; Human Sensing; Robustness &amp; Safety</x:v>
       </x:c>
       <x:c r="C20" s="20" t="str">
-        <x:v>System identification and data-driven modeling for dynamical systems and control. Characteristic themes include nonlinear identification, model reduction, identification software and benchmarks, learning across systems, and dynamic networks. Application tracks remain grounded in identifying or learning dynamical models, rather than becoming general-purpose domain conferences.</x:v>
+        <x:v>Broad research in visual perception, representation learning, recognition, segmentation, 3D geometry and reconstruction, computational imaging, and image/video synthesis. Vision-language models, multimodal understanding, human motion and appearance, and robust visual systems extend this core. ECCV is the biennial European flagship for computer vision; the scope uses the actual published 2026 CFP, not an invented 2028 call.</x:v>
       </x:c>
       <x:c r="D20" s="21" t="n">
-        <x:v>2027</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="E20" s="20" t="str">
-        <x:v>https://conferences.ifac-control.org/sysid2027/participate/</x:v>
+        <x:v>https://eccv.ecva.net/Conferences/2026/CallForPapers</x:v>
       </x:c>
       <x:c r="F20" s="22" t="n">
         <x:v>46302</x:v>
@@ -3825,77 +4425,79 @@
     </x:row>
     <x:row r="21" ht="60" hidden="0" customHeight="1">
       <x:c r="A21" s="20" t="str">
-        <x:v>Interspeech</x:v>
-      </x:c>
-      <x:c r="B21" s="20" t="str"/>
+        <x:v>EuroGP</x:v>
+      </x:c>
+      <x:c r="B21" s="20" t="str">
+        <x:v>Learning Theory &amp; Statistical Foundations; Deep Representation Learning</x:v>
+      </x:c>
       <x:c r="C21" s="20" t="str">
-        <x:v>Speech science and speech technology, linking spoken-language research with computational methods for speech recognition, speech synthesis, and speech communication. Machine learning and language models are relevant through speech and spoken-language problems. The current 2027 overview emphasizes the relationship between speech research and spoken-language technologies.</x:v>
+        <x:v>Genetic programming and evolutionary program synthesis, including symbolic regression, program representations and operators, surrogate-assisted search, multi-objective evolution, and interpretable learned programs. Evolutionary machine learning, AutoML pipelines, and neuroevolution connect this focused methodological community to ML. Application domains do not define its tags.</x:v>
       </x:c>
       <x:c r="D21" s="21" t="n">
         <x:v>2027</x:v>
       </x:c>
       <x:c r="E21" s="20" t="str">
-        <x:v>https://interspeech2027.org/</x:v>
+        <x:v>https://www.evostar.org/2027/eurogp/</x:v>
       </x:c>
       <x:c r="F21" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="60" hidden="0" customHeight="1">
+    <x:row r="22" ht="72" hidden="0" customHeight="1">
       <x:c r="A22" s="20" t="str">
-        <x:v>KDD</x:v>
+        <x:v>EUVIP</x:v>
       </x:c>
       <x:c r="B22" s="20" t="str">
-        <x:v>Deep Representation Learning; Natural Language Processing &amp; LLMs; Explainability &amp; Interpretability; Privacy-preserving ML; ML Systems &amp; Infrastructure</x:v>
+        <x:v>Multimedia Learning &amp; Retrieval; Computer Graphics &amp; Visualization; Biometrics &amp; Human Sensing; Robustness &amp; Safety</x:v>
       </x:c>
       <x:c r="C22" s="20" t="str">
-        <x:v>Knowledge discovery and data science, centered on extracting useful structure from large, heterogeneous data. Characteristic areas include clustering, structured and relational learning, graph and text mining, recommender systems, scalable data analysis, and responsible data use. Generative AI is relevant when it advances data science, not simply because a paper uses an LLM.</x:v>
+        <x:v>Visual information processing across image, video, 3D, and unconventional sensing modalities. Its defining areas are computational imaging, restoration and enhancement, coding, recognition, multimodal fusion, and subjective/objective quality assessment. Rendering and visualizing data, human/biometric analysis, and robust evaluation are recurring strands. An extensive applications list is not treated as equal coverage of every application domain or every responsible-AI subtopic.</x:v>
       </x:c>
       <x:c r="D22" s="21" t="n">
-        <x:v>2027</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="E22" s="20" t="str">
-        <x:v>https://kdd2027.kdd.org/research-track-call-for-papers/</x:v>
+        <x:v>https://euvip2026.github.io/C4P.pdf; https://euvip2026.github.io/calls/</x:v>
       </x:c>
       <x:c r="F22" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="60" hidden="0" customHeight="1">
+    <x:row r="23" ht="84" hidden="0" customHeight="1">
       <x:c r="A23" s="20" t="str">
-        <x:v>L4DC</x:v>
+        <x:v>FG</x:v>
       </x:c>
       <x:c r="B23" s="20" t="str">
-        <x:v>Learning Theory &amp; Statistical Foundations</x:v>
+        <x:v>Robustness &amp; Safety; Fairness &amp; Responsible AI; Computer Graphics &amp; Visualization; Explainability &amp; Interpretability</x:v>
       </x:c>
       <x:c r="C23" s="20" t="str">
-        <x:v>The interface of learning, dynamics, control, and optimization for physical and dynamical systems. Emphasizes foundations and methods for data-driven control and dynamical modeling, including theoretical, empirical, and applied contributions. Pure pattern recognition without a meaningful connection to dynamics or control is not the defining focus.</x:v>
+        <x:v>Face, gesture, body movement, and human behavior from images and video, including detection, tracking, recognition, facial expression and affect, pose and action analysis, and soft biometrics. Characteristic methods include advanced visual learning, generative modeling and neural rendering, multimodal fusion, and evaluation across demographic and acquisition conditions. Bias, interpretability, and robust recognition are directly tied to human sensing rather than generic application tags.</x:v>
       </x:c>
       <x:c r="D23" s="21" t="n">
         <x:v>2027</x:v>
       </x:c>
       <x:c r="E23" s="20" t="str">
-        <x:v>https://l4dc2027.control.ee.ethz.ch/home</x:v>
+        <x:v>https://fg2027.ieee-biometrics.org/call-for-papers/</x:v>
       </x:c>
       <x:c r="F23" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="72" hidden="0" customHeight="1">
+    <x:row r="24" ht="60" hidden="0" customHeight="1">
       <x:c r="A24" s="20" t="str">
-        <x:v>LoG</x:v>
+        <x:v>FMTS @ NeurIPS</x:v>
       </x:c>
       <x:c r="B24" s="20" t="str">
-        <x:v>Probabilistic, Causal &amp; Uncertainty ML; Signal Processing; Robustness &amp; Safety; ML Systems &amp; Infrastructure</x:v>
+        <x:v>System Identification &amp; Data-driven Dynamics; Robustness &amp; Safety</x:v>
       </x:c>
       <x:c r="C24" s="20" t="str">
-        <x:v>Learning on graphs and geometry: graph neural networks, equivariant models, graph kernels, geometric and graph generative models, and statistical theory for structured data. Graph signal processing, causal graph models, robustness, and scalable graph-learning infrastructure are meaningful extensions. A graph or geometric contribution should remain central, even in an application such as language or molecular modeling.</x:v>
+        <x:v>Foundation models for temporal systems, centered on long-horizon and probabilistic forecasting, temporal pretraining, generative simulation, irregularly sampled and multimodal sequences, and state-space architectures. Reliability is a defining theme: distribution shift, calibrated uncertainty, leakage-aware benchmarks, and consistency of simulated trajectories.</x:v>
       </x:c>
       <x:c r="D24" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E24" s="20" t="str">
-        <x:v>https://logconference.org/cfp/</x:v>
+        <x:v>https://fmts-workshop.github.io/cfp.html</x:v>
       </x:c>
       <x:c r="F24" s="22" t="n">
         <x:v>46302</x:v>
@@ -3903,99 +4505,97 @@
     </x:row>
     <x:row r="25" ht="60" hidden="0" customHeight="1">
       <x:c r="A25" s="20" t="str">
-        <x:v>MIDL</x:v>
+        <x:v>GECCO</x:v>
       </x:c>
       <x:c r="B25" s="20" t="str">
-        <x:v>Computer Vision &amp; Pattern Recognition; Probabilistic, Causal &amp; Uncertainty ML; Explainability &amp; Interpretability; Robustness &amp; Safety; Federated &amp; Distributed Learning</x:v>
+        <x:v>Deep Representation Learning; Learning Theory &amp; Statistical Foundations</x:v>
       </x:c>
       <x:c r="C25" s="20" t="str">
-        <x:v>Deep learning for biomedical image analysis, especially segmentation, detection, reconstruction, registration, generative imaging, and learning from limited labels. Uncertainty, interpretability, multi-site learning, robustness, and clinical validation extend that imaging core. Multimodal foundation models are relevant when grounded in medical imaging.</x:v>
+        <x:v>Genetic and evolutionary computation, including genetic algorithms, genetic programming, swarm intelligence, evolutionary multiobjective and combinatorial optimization, metaheuristics, and neuroevolution. Machine learning is relevant through evolutionary learning and optimization, not as an unrestricted substitute for the conference's evolutionary-computation focus.</x:v>
       </x:c>
       <x:c r="D25" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E25" s="20" t="str">
-        <x:v>https://2026.midl.io/call-for-papers</x:v>
+        <x:v>https://gecco-2027.sigevo.org/Call+for+Papers</x:v>
       </x:c>
       <x:c r="F25" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="60" hidden="0" customHeight="1">
+    <x:row r="26" ht="72" hidden="0" customHeight="1">
       <x:c r="A26" s="20" t="str">
-        <x:v>MLSys</x:v>
+        <x:v>ICAPS</x:v>
       </x:c>
       <x:c r="B26" s="20" t="str">
-        <x:v>Reinforcement Learning; Privacy-preserving ML</x:v>
+        <x:v>Probabilistic, Causal &amp; Uncertainty ML</x:v>
       </x:c>
       <x:c r="C26" s="20" t="str">
-        <x:v>The intersection of machine learning and computer systems, including efficient training, inference and serving, compilers and runtimes, programming abstractions, specialized hardware, distributed learning, and system monitoring. LLM and agentic workloads are considered from a systems perspective. Both systems for ML and ML methods that improve computing systems are relevant.</x:v>
+        <x:v>Automated planning and scheduling, heuristic search, constraint-based reasoning, temporal and hierarchical planning, and planning under uncertainty. Learning and foundation models fit when they substantially advance planning or scheduling, including model acquisition and search guidance. The main CFP explicitly excludes reinforcement-learning papers without a substantive planning contribution; general reward-based learning is not a blanket tag.</x:v>
       </x:c>
       <x:c r="D26" s="21" t="n">
         <x:v>2027</x:v>
       </x:c>
       <x:c r="E26" s="20" t="str">
-        <x:v>https://mlsys.org/Conferences/2027/CallForResearchPapers</x:v>
+        <x:v>https://icaps27.icaps-conference.org/calls/cfp/</x:v>
       </x:c>
       <x:c r="F26" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="60" hidden="0" customHeight="1">
+    <x:row r="27" ht="72" hidden="0" customHeight="1">
       <x:c r="A27" s="20" t="str">
-        <x:v>NeurIPS</x:v>
+        <x:v>ICCV</x:v>
       </x:c>
       <x:c r="B27" s="20" t="str">
-        <x:v>Learning Theory &amp; Statistical Foundations; Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Natural Language Processing &amp; LLMs; Computer Vision &amp; Pattern Recognition; ML Systems &amp; Infrastructure</x:v>
+        <x:v>Computer Graphics &amp; Visualization; Multimedia Learning &amp; Retrieval; Natural Language Processing &amp; LLMs; Biometrics &amp; Human Sensing; Robustness &amp; Safety</x:v>
       </x:c>
       <x:c r="C27" s="20" t="str">
-        <x:v>Broad research in machine learning, especially deep and generative models, statistical foundations, optimization, probabilistic inference, and learning for decision-making. Language, vision, and scalable ML systems are important research communities. Interdisciplinary applications should contribute insight of wider interest to the machine-learning community.</x:v>
+        <x:v>Broad computer vision, from geometry and computational imaging to visual learning, recognition, segmentation, generation, and video understanding. Vision-language and multimodal methods, visual graphics, face/body/gesture analysis, and reliable perception are substantial strands. It is a biennial flagship, not a general AI applications conference. The current scope is grounded in its 2025 CFP because the 2027 call is not yet published.</x:v>
       </x:c>
       <x:c r="D27" s="21" t="n">
-        <x:v>2026</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="E27" s="20" t="str">
-        <x:v>https://neurips.cc/Conferences/2026/CallForPapers</x:v>
+        <x:v>https://iccv.thecvf.com/Conferences/2025/CallForPapers</x:v>
       </x:c>
       <x:c r="F27" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="60" hidden="0" customHeight="1">
+    <x:row r="28" ht="72" hidden="0" customHeight="1">
       <x:c r="A28" s="20" t="str">
-        <x:v>NOLTA</x:v>
-      </x:c>
-      <x:c r="B28" s="20" t="str">
-        <x:v>Signal Processing; Evolutionary Computation &amp; Optimization</x:v>
-      </x:c>
+        <x:v>ICIP</x:v>
+      </x:c>
+      <x:c r="B28" s="20" t="str"/>
       <x:c r="C28" s="20" t="str">
-        <x:v>Nonlinear theory and its applications, centered on chaos, bifurcations, oscillations, synchronization, nonlinear circuits, and complex networks. Neural computation, evolutionary algorithms, control, and signal processing connect to this nonlinear-systems focus. Individual application examples are not taken as additional specialist identities.</x:v>
+        <x:v>Image and video processing across theory, algorithms, and imaging systems. Characteristic problems include restoration, enhancement, reconstruction, registration, compression, quality assessment, and visual analysis. Learning methods and generative models are relevant when they advance image or video processing. The long list of imaging application domains is intentionally not converted into extra specialist-conference tags.</x:v>
       </x:c>
       <x:c r="D28" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E28" s="20" t="str">
-        <x:v>https://nolta2026.org/</x:v>
+        <x:v>https://2026.ieeeicip.org/topics/</x:v>
       </x:c>
       <x:c r="F28" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="72" hidden="0" customHeight="1">
+    <x:row r="29" ht="60" hidden="0" customHeight="1">
       <x:c r="A29" s="20" t="str">
-        <x:v>ProbML</x:v>
+        <x:v>ICLR</x:v>
       </x:c>
       <x:c r="B29" s="20" t="str">
-        <x:v>Deep Representation Learning; Reinforcement Learning; Time Series &amp; Sequential Data; Robustness &amp; Safety</x:v>
+        <x:v>Learning Theory &amp; Statistical Foundations; Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Natural Language Processing &amp; LLMs; Computer Vision &amp; Pattern Recognition; ML Systems &amp; Infrastructure</x:v>
       </x:c>
       <x:c r="C29" s="20" t="str">
-        <x:v>Probabilistic and Bayesian machine learning, emphasizing approximate inference, variational and Monte Carlo methods, Gaussian processes, graphical and state-space models, calibration, and decisions under uncertainty. Includes Bayesian optimization and uncertainty-aware deep learning. The reviewed 2026 application focus is healthcare and climate; probabilistic reasoning remains essential to a suitable contribution.</x:v>
+        <x:v>Learning representations and understanding deep learning, with an emphasis on self-supervised learning, generative models, transfer and meta-learning, and the optimization and theory of learned representations. Language, vision, probabilistic modeling, and reinforcement learning are substantial areas, rather than unrelated application-domain tags.</x:v>
       </x:c>
       <x:c r="D29" s="21" t="n">
-        <x:v>2026</x:v>
+        <x:v>2027</x:v>
       </x:c>
       <x:c r="E29" s="20" t="str">
-        <x:v>https://probml.cc/call/</x:v>
+        <x:v>https://iclr.cc/Conferences/2027/CallForPapers</x:v>
       </x:c>
       <x:c r="F29" s="22" t="n">
         <x:v>46302</x:v>
@@ -4003,48 +4603,346 @@
     </x:row>
     <x:row r="30" ht="60" hidden="0" customHeight="1">
       <x:c r="A30" s="20" t="str">
-        <x:v>SaTML</x:v>
+        <x:v>ICML</x:v>
       </x:c>
       <x:c r="B30" s="20" t="str">
-        <x:v>Machine Learning; ML Systems &amp; Infrastructure</x:v>
+        <x:v>Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Explainability &amp; Interpretability; Robustness &amp; Safety; ML Systems &amp; Infrastructure; Federated &amp; Distributed Learning</x:v>
       </x:c>
       <x:c r="C30" s="20" t="str">
-        <x:v>Security, safety, and trustworthiness of machine learning. Characteristic work studies attacks and defenses, privacy, verification, ML-system security, fairness, interpretability, and trustworthy data curation. Theoretical, empirical, and applied papers must engage substantively with a safety or trustworthiness question; merely using an ML model is insufficient.</x:v>
+        <x:v>Methodological and theoretical machine learning, including supervised and unsupervised learning, deep generative models, optimization, statistical learning theory, Bayesian methods, and reinforcement learning. Scalable systems and trustworthy learning are established parts of the scope; application papers should offer contributions of wider interest to ML.</x:v>
       </x:c>
       <x:c r="D30" s="21" t="n">
-        <x:v>2027</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="E30" s="20" t="str">
-        <x:v>https://satml.org/call-for-papers/</x:v>
+        <x:v>https://icml.cc/Conferences/2026/CallForPapers</x:v>
       </x:c>
       <x:c r="F30" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="60" hidden="0" customHeight="1">
+    <x:row r="31" ht="72" hidden="0" customHeight="1">
       <x:c r="A31" s="20" t="str">
+        <x:v>ICMR</x:v>
+      </x:c>
+      <x:c r="B31" s="20" t="str">
+        <x:v>Data Mining &amp; Data Science; Natural Language Processing &amp; LLMs; Privacy-preserving ML</x:v>
+      </x:c>
+      <x:c r="C31" s="20" t="str">
+        <x:v>Search and retrieval of multimedia and multimodal content. Characteristic work studies indexing, content understanding, query representations, cross-modal matching, relevance feedback, recommendation, and evaluation, with deep learning and multimodal models as important methods. Privacy-aware retrieval and knowledge discovery extend this core. The long applications list is not used to characterize ICMR as a medicine, finance, or travel venue.</x:v>
+      </x:c>
+      <x:c r="D31" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E31" s="20" t="str">
+        <x:v>https://www.icmr2027.org/cfc</x:v>
+      </x:c>
+      <x:c r="F31" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="60" hidden="0" customHeight="1">
+      <x:c r="A32" s="20" t="str">
+        <x:v>IFAC SYSID</x:v>
+      </x:c>
+      <x:c r="B32" s="20" t="str">
+        <x:v>Nonlinear Dynamics &amp; Chaos; Complex Systems &amp; Network Science</x:v>
+      </x:c>
+      <x:c r="C32" s="20" t="str">
+        <x:v>System identification and data-driven modeling for dynamical systems and control. Characteristic themes include nonlinear identification, model reduction, identification software and benchmarks, learning across systems, and dynamic networks. Application tracks remain grounded in identifying or learning dynamical models, rather than becoming general-purpose domain conferences.</x:v>
+      </x:c>
+      <x:c r="D32" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E32" s="20" t="str">
+        <x:v>https://conferences.ifac-control.org/sysid2027/participate/</x:v>
+      </x:c>
+      <x:c r="F32" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="84" hidden="0" customHeight="1">
+      <x:c r="A33" s="20" t="str">
+        <x:v>IJCB</x:v>
+      </x:c>
+      <x:c r="B33" s="20" t="str">
+        <x:v>Machine Learning; Robustness &amp; Safety; Fairness &amp; Responsible AI; Explainability &amp; Interpretability; Federated &amp; Distributed Learning; Signal Processing</x:v>
+      </x:c>
+      <x:c r="C33" s="20" t="str">
+        <x:v>Biometrics and identity science across face, fingerprint, iris, voice, gait, and behavioral modalities. Defining concerns include recognition and verification, multimodal fusion, presentation-attack and deepfake detection, biometric template security, privacy, demographic fairness, and rigorous benchmarking. Learned representations and foundation models are important methods; federated learning belongs here through secure biometric systems. Healthcare, banking, and robotics are applications, not blanket scope tags.</x:v>
+      </x:c>
+      <x:c r="D33" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E33" s="20" t="str">
+        <x:v>https://ijcb2027.ieee-biometrics.org/call-for-papers/</x:v>
+      </x:c>
+      <x:c r="F33" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="60" hidden="0" customHeight="1">
+      <x:c r="A34" s="20" t="str">
+        <x:v>Interspeech</x:v>
+      </x:c>
+      <x:c r="B34" s="20" t="str"/>
+      <x:c r="C34" s="20" t="str">
+        <x:v>Speech science and speech technology, linking spoken-language research with computational methods for speech recognition, speech synthesis, and speech communication. Machine learning and language models are relevant through speech and spoken-language problems. The current 2027 overview emphasizes the relationship between speech research and spoken-language technologies.</x:v>
+      </x:c>
+      <x:c r="D34" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E34" s="20" t="str">
+        <x:v>https://interspeech2027.org/</x:v>
+      </x:c>
+      <x:c r="F34" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="60" hidden="0" customHeight="1">
+      <x:c r="A35" s="20" t="str">
+        <x:v>KDD</x:v>
+      </x:c>
+      <x:c r="B35" s="20" t="str">
+        <x:v>Deep Representation Learning; Natural Language Processing &amp; LLMs; Explainability &amp; Interpretability; Privacy-preserving ML; ML Systems &amp; Infrastructure</x:v>
+      </x:c>
+      <x:c r="C35" s="20" t="str">
+        <x:v>Knowledge discovery and data science, centered on extracting useful structure from large, heterogeneous data. Characteristic areas include clustering, structured and relational learning, graph and text mining, recommender systems, scalable data analysis, and responsible data use. Generative AI is relevant when it advances data science, not simply because a paper uses an LLM.</x:v>
+      </x:c>
+      <x:c r="D35" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E35" s="20" t="str">
+        <x:v>https://kdd2027.kdd.org/research-track-call-for-papers/</x:v>
+      </x:c>
+      <x:c r="F35" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="84" hidden="0" customHeight="1">
+      <x:c r="A36" s="20" t="str">
+        <x:v>KR</x:v>
+      </x:c>
+      <x:c r="B36" s="20" t="str">
+        <x:v>Machine Learning; Probabilistic, Causal &amp; Uncertainty ML; Planning &amp; Search</x:v>
+      </x:c>
+      <x:c r="C36" s="20" t="str">
+        <x:v>Formal and symbolic AI centered on representing knowledge and drawing justified conclusions: knowledge bases, description and non-classical logics, ontologies, non-monotonic reasoning, argumentation, belief revision, and reasoning about actions. Learning, uncertainty, and explanations matter when grounded in knowledge representation or reasoning. The last published CFP includes a KR Meets Machine Learning and Explanation track; this is not a general-purpose ML conference or a confirmed promise of that 2027 track.</x:v>
+      </x:c>
+      <x:c r="D36" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E36" s="20" t="str">
+        <x:v>https://kr.org/KR2026/call_main_track.html; https://kr.org/KR2026/</x:v>
+      </x:c>
+      <x:c r="F36" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="60" hidden="0" customHeight="1">
+      <x:c r="A37" s="20" t="str">
+        <x:v>L4DC</x:v>
+      </x:c>
+      <x:c r="B37" s="20" t="str">
+        <x:v>Learning Theory &amp; Statistical Foundations</x:v>
+      </x:c>
+      <x:c r="C37" s="20" t="str">
+        <x:v>The interface of learning, dynamics, control, and optimization for physical and dynamical systems. Emphasizes foundations and methods for data-driven control and dynamical modeling, including theoretical, empirical, and applied contributions. Pure pattern recognition without a meaningful connection to dynamics or control is not the defining focus.</x:v>
+      </x:c>
+      <x:c r="D37" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E37" s="20" t="str">
+        <x:v>https://l4dc2027.control.ee.ethz.ch/home</x:v>
+      </x:c>
+      <x:c r="F37" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="72" hidden="0" customHeight="1">
+      <x:c r="A38" s="20" t="str">
+        <x:v>LoG</x:v>
+      </x:c>
+      <x:c r="B38" s="20" t="str">
+        <x:v>Probabilistic, Causal &amp; Uncertainty ML; Signal Processing; Robustness &amp; Safety; ML Systems &amp; Infrastructure</x:v>
+      </x:c>
+      <x:c r="C38" s="20" t="str">
+        <x:v>Learning on graphs and geometry: graph neural networks, equivariant models, graph kernels, geometric and graph generative models, and statistical theory for structured data. Graph signal processing, causal graph models, robustness, and scalable graph-learning infrastructure are meaningful extensions. A graph or geometric contribution should remain central, even in an application such as language or molecular modeling.</x:v>
+      </x:c>
+      <x:c r="D38" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E38" s="20" t="str">
+        <x:v>https://logconference.org/cfp/</x:v>
+      </x:c>
+      <x:c r="F38" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="60" hidden="0" customHeight="1">
+      <x:c r="A39" s="20" t="str">
+        <x:v>MIDL</x:v>
+      </x:c>
+      <x:c r="B39" s="20" t="str">
+        <x:v>Computer Vision &amp; Pattern Recognition; Probabilistic, Causal &amp; Uncertainty ML; Explainability &amp; Interpretability; Robustness &amp; Safety; Federated &amp; Distributed Learning</x:v>
+      </x:c>
+      <x:c r="C39" s="20" t="str">
+        <x:v>Deep learning for biomedical image analysis, especially segmentation, detection, reconstruction, registration, generative imaging, and learning from limited labels. Uncertainty, interpretability, multi-site learning, robustness, and clinical validation extend that imaging core. Multimodal foundation models are relevant when grounded in medical imaging.</x:v>
+      </x:c>
+      <x:c r="D39" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E39" s="20" t="str">
+        <x:v>https://2026.midl.io/call-for-papers</x:v>
+      </x:c>
+      <x:c r="F39" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="60" hidden="0" customHeight="1">
+      <x:c r="A40" s="20" t="str">
+        <x:v>MLSys</x:v>
+      </x:c>
+      <x:c r="B40" s="20" t="str">
+        <x:v>Reinforcement Learning; Privacy-preserving ML</x:v>
+      </x:c>
+      <x:c r="C40" s="20" t="str">
+        <x:v>The intersection of machine learning and computer systems, including efficient training, inference and serving, compilers and runtimes, programming abstractions, specialized hardware, distributed learning, and system monitoring. LLM and agentic workloads are considered from a systems perspective. Both systems for ML and ML methods that improve computing systems are relevant.</x:v>
+      </x:c>
+      <x:c r="D40" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E40" s="20" t="str">
+        <x:v>https://mlsys.org/Conferences/2027/CallForResearchPapers</x:v>
+      </x:c>
+      <x:c r="F40" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="60" hidden="0" customHeight="1">
+      <x:c r="A41" s="20" t="str">
+        <x:v>NeurIPS</x:v>
+      </x:c>
+      <x:c r="B41" s="20" t="str">
+        <x:v>Learning Theory &amp; Statistical Foundations; Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Natural Language Processing &amp; LLMs; Computer Vision &amp; Pattern Recognition; ML Systems &amp; Infrastructure</x:v>
+      </x:c>
+      <x:c r="C41" s="20" t="str">
+        <x:v>Broad research in machine learning, especially deep and generative models, statistical foundations, optimization, probabilistic inference, and learning for decision-making. Language, vision, and scalable ML systems are important research communities. Interdisciplinary applications should contribute insight of wider interest to the machine-learning community.</x:v>
+      </x:c>
+      <x:c r="D41" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E41" s="20" t="str">
+        <x:v>https://neurips.cc/Conferences/2026/CallForPapers</x:v>
+      </x:c>
+      <x:c r="F41" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="60" hidden="0" customHeight="1">
+      <x:c r="A42" s="20" t="str">
+        <x:v>NOLTA</x:v>
+      </x:c>
+      <x:c r="B42" s="20" t="str">
+        <x:v>Signal Processing; Evolutionary Computation &amp; Optimization</x:v>
+      </x:c>
+      <x:c r="C42" s="20" t="str">
+        <x:v>Nonlinear theory and its applications, centered on chaos, bifurcations, oscillations, synchronization, nonlinear circuits, and complex networks. Neural computation, evolutionary algorithms, control, and signal processing connect to this nonlinear-systems focus. Individual application examples are not taken as additional specialist identities.</x:v>
+      </x:c>
+      <x:c r="D42" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E42" s="20" t="str">
+        <x:v>https://nolta2026.org/</x:v>
+      </x:c>
+      <x:c r="F42" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="72" hidden="0" customHeight="1">
+      <x:c r="A43" s="20" t="str">
+        <x:v>ProbML</x:v>
+      </x:c>
+      <x:c r="B43" s="20" t="str">
+        <x:v>Deep Representation Learning; Reinforcement Learning; Time Series &amp; Sequential Data; Robustness &amp; Safety</x:v>
+      </x:c>
+      <x:c r="C43" s="20" t="str">
+        <x:v>Probabilistic and Bayesian machine learning, emphasizing approximate inference, variational and Monte Carlo methods, Gaussian processes, graphical and state-space models, calibration, and decisions under uncertainty. Includes Bayesian optimization and uncertainty-aware deep learning. The reviewed 2026 application focus is healthcare and climate; probabilistic reasoning remains essential to a suitable contribution.</x:v>
+      </x:c>
+      <x:c r="D43" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E43" s="20" t="str">
+        <x:v>https://probml.cc/call/</x:v>
+      </x:c>
+      <x:c r="F43" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="60" hidden="0" customHeight="1">
+      <x:c r="A44" s="20" t="str">
+        <x:v>SaTML</x:v>
+      </x:c>
+      <x:c r="B44" s="20" t="str">
+        <x:v>Machine Learning; ML Systems &amp; Infrastructure</x:v>
+      </x:c>
+      <x:c r="C44" s="20" t="str">
+        <x:v>Security, safety, and trustworthiness of machine learning. Characteristic work studies attacks and defenses, privacy, verification, ML-system security, fairness, interpretability, and trustworthy data curation. Theoretical, empirical, and applied papers must engage substantively with a safety or trustworthiness question; merely using an ML model is insufficient.</x:v>
+      </x:c>
+      <x:c r="D44" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E44" s="20" t="str">
+        <x:v>https://satml.org/call-for-papers/</x:v>
+      </x:c>
+      <x:c r="F44" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="60" hidden="0" customHeight="1">
+      <x:c r="A45" s="20" t="str">
         <x:v>UAI</x:v>
       </x:c>
-      <x:c r="B31" s="20" t="str">
+      <x:c r="B45" s="20" t="str">
         <x:v>Deep Representation Learning; Reinforcement Learning; Time Series &amp; Sequential Data; Explainability &amp; Interpretability; Robustness &amp; Safety</x:v>
       </x:c>
-      <x:c r="C31" s="20" t="str">
+      <x:c r="C45" s="20" t="str">
         <x:v>Learning and reasoning under uncertainty, centered on probabilistic and Bayesian modeling, graphical models, causal inference, approximate inference, and decision theory. Includes Monte Carlo and variational methods, uncertainty quantification, sequential models, and principled analysis of learning algorithms. Uncertainty is the organizing theme, not just another application of general-purpose AI.</x:v>
       </x:c>
-      <x:c r="D31" s="21" t="n">
+      <x:c r="D45" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
-      <x:c r="E31" s="20" t="str">
+      <x:c r="E45" s="20" t="str">
         <x:v>https://www.auai.org/uai2026/subject_areas; https://www.auai.org/uai2026/call_for_papers</x:v>
       </x:c>
-      <x:c r="F31" s="22" t="n">
+      <x:c r="F45" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="72" hidden="0" customHeight="1">
+      <x:c r="A46" s="20" t="str">
+        <x:v>WACV</x:v>
+      </x:c>
+      <x:c r="B46" s="20" t="str">
+        <x:v>Signal Processing; Biometrics &amp; Human Sensing; Multimedia Learning &amp; Retrieval</x:v>
+      </x:c>
+      <x:c r="C46" s="20" t="str">
+        <x:v>Applied computer vision and visual learning, with an emphasis on practical recognition, detection, segmentation, image/video analysis, 3D perception, and deployable visual systems. Human analysis and multimodal visual methods are established areas. Compared with the flagship trio, WACV particularly welcomes meaningful application-driven contributions supported by sound evaluation; its two submission rounds are routes, not different fields.</x:v>
+      </x:c>
+      <x:c r="D46" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E46" s="20" t="str">
+        <x:v>https://wacv.thecvf.com/Conferences/2027/CallForPapers</x:v>
+      </x:c>
+      <x:c r="F46" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62005996abd44f46"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f6d0384e27a482c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add language and robotics venues with eight-topic discovery
</commit_message>
<xml_diff>
--- a/data/core_conferences_normalized_tags.xlsx
+++ b/data/core_conferences_normalized_tags.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Conferences" sheetId="1" r:id="R5109e2a6113b4dc8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Vocabulary" sheetId="2" r:id="R60990133882a4fa4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conference Scope" sheetId="3" r:id="Rc6fd55c52f23417d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Conferences" sheetId="1" r:id="R07338374964b43c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Vocabulary" sheetId="2" r:id="R185e42a7a4404346"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conference Scope" sheetId="3" r:id="R9fe1be8fca8d4635"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -119,7 +119,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="CoreConferencesTable" displayName="CoreConferencesTable" ref="A1:N98" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="CoreConferencesTable" displayName="CoreConferencesTable" ref="A1:N114" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Conference"/>
     <x:tableColumn id="2" name="TAGS"/>
@@ -141,7 +141,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TagVocabularyTable" displayName="TagVocabularyTable" ref="A1:B35" headerRowCount="1" totalsRowCount="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TagVocabularyTable" displayName="TagVocabularyTable" ref="A1:B40" headerRowCount="1" totalsRowCount="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Standard tag"/>
     <x:tableColumn id="2" name="Definition"/>
@@ -151,7 +151,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ConferenceScope" displayName="ConferenceScope" ref="A1:F46" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ConferenceScope" displayName="ConferenceScope" ref="A1:F64" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Series"/>
     <x:tableColumn id="2" name="Additional topics"/>
@@ -2818,7 +2818,7 @@
         <x:v>LoG</x:v>
       </x:c>
       <x:c r="B74" s="12" t="str">
-        <x:v>Machine Learning; Deep Representation Learning; Complex Systems &amp; Network Science; Learning Theory &amp; Statistical Foundations</x:v>
+        <x:v>Machine Learning; Deep Representation Learning; Graphs &amp; Graph Learning; Learning Theory &amp; Statistical Foundations</x:v>
       </x:c>
       <x:c r="C74" t="str">
         <x:v>M</x:v>
@@ -2974,7 +2974,7 @@
         <x:v>AAMAS</x:v>
       </x:c>
       <x:c r="B79" s="12" t="str">
-        <x:v>Machine Learning; Reinforcement Learning; Control &amp; Robotics; Human-AI Interaction &amp; Deployment</x:v>
+        <x:v>Machine Learning; Reinforcement Learning; Autonomous Agents &amp; Multiagent Systems; Human-AI Interaction &amp; Deployment</x:v>
       </x:c>
       <x:c r="C79" t="str">
         <x:v>XL</x:v>
@@ -3705,10 +3705,594 @@
         <x:v>https://media.eventhosts.cc/Conferences/WACV2026/wacv_2026_program_v18_Digital.pdf</x:v>
       </x:c>
     </x:row>
+    <x:row r="99" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A99" t="str">
+        <x:v>ACL</x:v>
+      </x:c>
+      <x:c r="B99" s="12" t="str">
+        <x:v>Natural Language Processing &amp; LLMs; Deep Representation Learning; LLM Agents &amp; Tool Use; Information Retrieval &amp; Search</x:v>
+      </x:c>
+      <x:c r="C99" t="str">
+        <x:v>XXL</x:v>
+      </x:c>
+      <x:c r="D99" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="E99" t="str">
+        <x:v>A*</x:v>
+      </x:c>
+      <x:c r="F99" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G99" t="str">
+        <x:v>https://2027.aclweb.org/</x:v>
+      </x:c>
+      <x:c r="H99" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/196/</x:v>
+      </x:c>
+      <x:c r="I99" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="J99" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=57</x:v>
+      </x:c>
+      <x:c r="K99" s="16" t="n">
+        <x:v>0.203</x:v>
+      </x:c>
+      <x:c r="L99" s="17" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="M99" t="str">
+        <x:v>Main conference; chairs' rate over unique ARR submissions (Findings excluded)</x:v>
+      </x:c>
+      <x:c r="N99" t="str">
+        <x:v>https://aclanthology.org/2025.acl-long.0.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A100" t="str">
+        <x:v>EMNLP</x:v>
+      </x:c>
+      <x:c r="B100" s="12" t="str">
+        <x:v>Natural Language Processing &amp; LLMs; Deep Representation Learning; LLM Agents &amp; Tool Use; Information Retrieval &amp; Search</x:v>
+      </x:c>
+      <x:c r="C100" t="str">
+        <x:v>XXL</x:v>
+      </x:c>
+      <x:c r="D100" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="E100" t="str">
+        <x:v>A*</x:v>
+      </x:c>
+      <x:c r="F100" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G100" t="str">
+        <x:v>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</x:v>
+      </x:c>
+      <x:c r="H100" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/448/</x:v>
+      </x:c>
+      <x:c r="I100" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J100" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=58</x:v>
+      </x:c>
+      <x:c r="K100" s="16" t="n">
+        <x:v>0.2216</x:v>
+      </x:c>
+      <x:c r="L100" s="17" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="M100" t="str">
+        <x:v>Main conference (1,811 of 8,174 ARR submissions; desk rejections and withdrawals included, Findings excluded)</x:v>
+      </x:c>
+      <x:c r="N100" t="str">
+        <x:v>https://aclanthology.org/2025.emnlp-main.0.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A101" t="str">
+        <x:v>NAACL</x:v>
+      </x:c>
+      <x:c r="B101" s="12" t="str">
+        <x:v>Natural Language Processing &amp; LLMs; LLM Agents &amp; Tool Use; Information Retrieval &amp; Search; Deep Representation Learning</x:v>
+      </x:c>
+      <x:c r="C101" t="str">
+        <x:v>XL</x:v>
+      </x:c>
+      <x:c r="D101" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="E101" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="F101" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G101" t="str">
+        <x:v>https://2027.naacl.org/</x:v>
+      </x:c>
+      <x:c r="H101" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/1648/</x:v>
+      </x:c>
+      <x:c r="I101" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J101" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=58</x:v>
+      </x:c>
+      <x:c r="K101" s="16" t="n">
+        <x:v>0.22</x:v>
+      </x:c>
+      <x:c r="L101" s="17" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="M101" t="str">
+        <x:v>Main conference; chairs' estimated rate over October ARR papers intending NAACL (not commitment-only rate; Findings excluded)</x:v>
+      </x:c>
+      <x:c r="N101" t="str">
+        <x:v>https://aclanthology.org/2025.naacl-long.0.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A102" t="str">
+        <x:v>COLING</x:v>
+      </x:c>
+      <x:c r="B102" s="12" t="str">
+        <x:v>Natural Language Processing &amp; LLMs; Deep Representation Learning; Knowledge Representation &amp; Reasoning; LLM Agents &amp; Tool Use</x:v>
+      </x:c>
+      <x:c r="C102" t="str">
+        <x:v>XL</x:v>
+      </x:c>
+      <x:c r="D102" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E102" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="F102" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G102" t="str">
+        <x:v>https://2027.coling-iccl.org/</x:v>
+      </x:c>
+      <x:c r="H102" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/949/</x:v>
+      </x:c>
+      <x:c r="I102" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J102" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=58</x:v>
+      </x:c>
+      <x:c r="K102" s="16"/>
+      <x:c r="L102" s="17"/>
+      <x:c r="M102"/>
+      <x:c r="N102"/>
+    </x:row>
+    <x:row r="103" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A103" t="str">
+        <x:v>CoNLL</x:v>
+      </x:c>
+      <x:c r="B103" s="12" t="str">
+        <x:v>Natural Language Processing &amp; LLMs; Cognitive Science &amp; Computational Cognition; Computational Neuroscience; Explainability &amp; Interpretability</x:v>
+      </x:c>
+      <x:c r="C103" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="D103" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E103" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="F103" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G103" t="str">
+        <x:v>https://www.conll.org/</x:v>
+      </x:c>
+      <x:c r="H103" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/371/</x:v>
+      </x:c>
+      <x:c r="I103" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="J103" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=59</x:v>
+      </x:c>
+      <x:c r="K103" s="16"/>
+      <x:c r="L103" s="17"/>
+      <x:c r="M103"/>
+      <x:c r="N103"/>
+    </x:row>
+    <x:row r="104" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A104" t="str">
+        <x:v>LREC</x:v>
+      </x:c>
+      <x:c r="B104" s="12" t="str">
+        <x:v>Natural Language Processing &amp; LLMs; Data Mining &amp; Data Science; Signal Processing</x:v>
+      </x:c>
+      <x:c r="C104" t="str">
+        <x:v>XL</x:v>
+      </x:c>
+      <x:c r="D104" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E104" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="F104" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G104" t="str">
+        <x:v>https://www.elra.info/elra-events/lrec/</x:v>
+      </x:c>
+      <x:c r="H104" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/2092/</x:v>
+      </x:c>
+      <x:c r="I104"/>
+      <x:c r="J104"/>
+      <x:c r="K104" s="16"/>
+      <x:c r="L104" s="17"/>
+      <x:c r="M104"/>
+      <x:c r="N104"/>
+    </x:row>
+    <x:row r="105" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A105" t="str">
+        <x:v>IJCNLP</x:v>
+      </x:c>
+      <x:c r="B105" s="12" t="str">
+        <x:v>Natural Language Processing &amp; LLMs; Deep Representation Learning; LLM Agents &amp; Tool Use; Information Retrieval &amp; Search</x:v>
+      </x:c>
+      <x:c r="C105" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="D105" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E105" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="F105" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G105" t="str">
+        <x:v>https://2026.aaclnet.org/</x:v>
+      </x:c>
+      <x:c r="H105" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/1317/</x:v>
+      </x:c>
+      <x:c r="I105"/>
+      <x:c r="J105"/>
+      <x:c r="K105" s="16"/>
+      <x:c r="L105" s="17"/>
+      <x:c r="M105"/>
+      <x:c r="N105"/>
+    </x:row>
+    <x:row r="106" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A106" t="str">
+        <x:v>SIGIR</x:v>
+      </x:c>
+      <x:c r="B106" s="12" t="str">
+        <x:v>Information Retrieval &amp; Search; Recommender Systems; Natural Language Processing &amp; LLMs; Machine Learning</x:v>
+      </x:c>
+      <x:c r="C106" t="str">
+        <x:v>XL</x:v>
+      </x:c>
+      <x:c r="D106" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E106" t="str">
+        <x:v>A*</x:v>
+      </x:c>
+      <x:c r="F106" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G106" t="str">
+        <x:v>https://sigir2027.org/</x:v>
+      </x:c>
+      <x:c r="H106" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/29/</x:v>
+      </x:c>
+      <x:c r="I106" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="J106" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=35</x:v>
+      </x:c>
+      <x:c r="K106" s="16"/>
+      <x:c r="L106" s="17"/>
+      <x:c r="M106"/>
+      <x:c r="N106"/>
+    </x:row>
+    <x:row r="107" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A107" t="str">
+        <x:v>ECIR</x:v>
+      </x:c>
+      <x:c r="B107" s="12" t="str">
+        <x:v>Information Retrieval &amp; Search; Recommender Systems; Natural Language Processing &amp; LLMs; LLM Agents &amp; Tool Use</x:v>
+      </x:c>
+      <x:c r="C107" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="D107" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E107" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="F107" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G107" t="str">
+        <x:v>https://www.ecir2027.co.uk/</x:v>
+      </x:c>
+      <x:c r="H107" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/483/</x:v>
+      </x:c>
+      <x:c r="I107" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="J107" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=37</x:v>
+      </x:c>
+      <x:c r="K107" s="16"/>
+      <x:c r="L107" s="17"/>
+      <x:c r="M107"/>
+      <x:c r="N107"/>
+    </x:row>
+    <x:row r="108" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A108" t="str">
+        <x:v>RecSys</x:v>
+      </x:c>
+      <x:c r="B108" s="12" t="str">
+        <x:v>Recommender Systems; Machine Learning; Information Retrieval &amp; Search; Human-AI Interaction &amp; Deployment</x:v>
+      </x:c>
+      <x:c r="C108" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="D108" t="str">
+        <x:v>Very low</x:v>
+      </x:c>
+      <x:c r="E108" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="F108" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G108" t="str">
+        <x:v>https://recsys.acm.org/recsys27/</x:v>
+      </x:c>
+      <x:c r="H108" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/28/</x:v>
+      </x:c>
+      <x:c r="I108" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J108" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=36</x:v>
+      </x:c>
+      <x:c r="K108" s="16" t="n">
+        <x:v>0.19</x:v>
+      </x:c>
+      <x:c r="L108" s="17" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="M108" t="str">
+        <x:v>Long papers (49 accepted of 261 submitted); official rounded rate</x:v>
+      </x:c>
+      <x:c r="N108" t="str">
+        <x:v>https://recsys.acm.org/statistics/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A109" t="str">
+        <x:v>WWW</x:v>
+      </x:c>
+      <x:c r="B109" s="12" t="str">
+        <x:v>Information Retrieval &amp; Search; Recommender Systems; Graphs &amp; Graph Learning; LLM Agents &amp; Tool Use</x:v>
+      </x:c>
+      <x:c r="C109" t="str">
+        <x:v>XL</x:v>
+      </x:c>
+      <x:c r="D109" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E109" t="str">
+        <x:v>A*</x:v>
+      </x:c>
+      <x:c r="F109" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G109" t="str">
+        <x:v>https://www2027.thewebconf.org/</x:v>
+      </x:c>
+      <x:c r="H109" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/1548/</x:v>
+      </x:c>
+      <x:c r="I109" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="J109" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=70</x:v>
+      </x:c>
+      <x:c r="K109" s="16"/>
+      <x:c r="L109" s="17"/>
+      <x:c r="M109"/>
+      <x:c r="N109"/>
+    </x:row>
+    <x:row r="110" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A110" t="str">
+        <x:v>COLM</x:v>
+      </x:c>
+      <x:c r="B110" s="12" t="str">
+        <x:v>Natural Language Processing &amp; LLMs; Deep Representation Learning; LLM Agents &amp; Tool Use; Information Retrieval &amp; Search</x:v>
+      </x:c>
+      <x:c r="C110" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="D110" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E110"/>
+      <x:c r="F110" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G110" t="str">
+        <x:v>https://colm.cc/</x:v>
+      </x:c>
+      <x:c r="H110"/>
+      <x:c r="I110"/>
+      <x:c r="J110"/>
+      <x:c r="K110" s="16"/>
+      <x:c r="L110" s="17"/>
+      <x:c r="M110"/>
+      <x:c r="N110"/>
+    </x:row>
+    <x:row r="111" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A111" t="str">
+        <x:v>ISWC</x:v>
+      </x:c>
+      <x:c r="B111" s="12" t="str">
+        <x:v>Knowledge Representation &amp; Reasoning; Graphs &amp; Graph Learning; Data Mining &amp; Data Science; Information Retrieval &amp; Search</x:v>
+      </x:c>
+      <x:c r="C111" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D111" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E111" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="F111" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G111" t="str">
+        <x:v>https://swsa.semanticweb.org/conferences/</x:v>
+      </x:c>
+      <x:c r="H111" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/1338/</x:v>
+      </x:c>
+      <x:c r="I111" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J111" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=36</x:v>
+      </x:c>
+      <x:c r="K111" s="16"/>
+      <x:c r="L111" s="17"/>
+      <x:c r="M111"/>
+      <x:c r="N111"/>
+    </x:row>
+    <x:row r="112" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A112" t="str">
+        <x:v>ICRA</x:v>
+      </x:c>
+      <x:c r="B112" s="12" t="str">
+        <x:v>Control &amp; Robotics; Reinforcement Learning; Computer Vision &amp; Pattern Recognition; System Identification &amp; Data-driven Dynamics</x:v>
+      </x:c>
+      <x:c r="C112" t="str">
+        <x:v>XXL</x:v>
+      </x:c>
+      <x:c r="D112" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E112" t="str">
+        <x:v>A*</x:v>
+      </x:c>
+      <x:c r="F112" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G112" t="str">
+        <x:v>https://2027.ieee-icra.org/</x:v>
+      </x:c>
+      <x:c r="H112" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/2051/</x:v>
+      </x:c>
+      <x:c r="I112" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J112" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=58</x:v>
+      </x:c>
+      <x:c r="K112" s="16"/>
+      <x:c r="L112" s="17"/>
+      <x:c r="M112"/>
+      <x:c r="N112"/>
+    </x:row>
+    <x:row r="113" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A113" t="str">
+        <x:v>RSS</x:v>
+      </x:c>
+      <x:c r="B113" s="12" t="str">
+        <x:v>Control &amp; Robotics; Reinforcement Learning; System Identification &amp; Data-driven Dynamics; Computer Vision &amp; Pattern Recognition</x:v>
+      </x:c>
+      <x:c r="C113" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D113" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E113"/>
+      <x:c r="F113" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G113" t="str">
+        <x:v>https://roboticsconference.org/</x:v>
+      </x:c>
+      <x:c r="H113"/>
+      <x:c r="I113"/>
+      <x:c r="J113"/>
+      <x:c r="K113" s="16"/>
+      <x:c r="L113" s="17"/>
+      <x:c r="M113"/>
+      <x:c r="N113"/>
+    </x:row>
+    <x:row r="114" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A114" t="str">
+        <x:v>SMC</x:v>
+      </x:c>
+      <x:c r="B114" s="12" t="str">
+        <x:v>Control &amp; Robotics; Complex Systems &amp; Network Science; Machine Learning; Human-AI Interaction &amp; Deployment</x:v>
+      </x:c>
+      <x:c r="C114" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="D114" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E114" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="F114" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G114" t="str">
+        <x:v>https://www.ieeesmc.org/conferences/calendar/</x:v>
+      </x:c>
+      <x:c r="H114" t="str">
+        <x:v>https://portal.core.edu.au/conf-ranks/611/</x:v>
+      </x:c>
+      <x:c r="I114" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="J114" t="str">
+        <x:v>https://www.ccf.org.cn/ccf/contentcore/resource/download?ID=112CF3BF7E1140ACEB271ADAED12A67ADFABB8FF099E40C2759502A85C8A281F#page=72</x:v>
+      </x:c>
+      <x:c r="K114" s="16"/>
+      <x:c r="L114" s="17"/>
+      <x:c r="M114"/>
+      <x:c r="N114"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5dc5d7f55d874962"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc9061b32c68406b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3734,7 +4318,7 @@
         <x:v>Machine Learning</x:v>
       </x:c>
       <x:c r="B2" s="14" t="str">
-        <x:v>General ML methods, algorithms, model development, and applied AI. Family: ML &amp; AI.</x:v>
+        <x:v>General ML methods, algorithms, model development, and applied AI. Family: ML &amp; Data Science.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
@@ -3742,7 +4326,7 @@
         <x:v>Deep Representation Learning</x:v>
       </x:c>
       <x:c r="B3" s="14" t="str">
-        <x:v>Deep learning, self-supervised learning, latent representations, neural networks. Family: ML &amp; AI.</x:v>
+        <x:v>Deep learning, self-supervised learning, latent representations, neural networks. Family: ML &amp; Data Science.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
@@ -3750,15 +4334,15 @@
         <x:v>Data Mining &amp; Data Science</x:v>
       </x:c>
       <x:c r="B4" s="14" t="str">
-        <x:v>Knowledge discovery, analytics, applied data science, large-scale data mining. Family: Data &amp; Time Series.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="15" hidden="0" customHeight="1">
+        <x:v>Knowledge discovery, analytics, applied data science, large-scale data mining. Family: ML &amp; Data Science.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A5" s="14" t="str">
         <x:v>Time Series &amp; Sequential Data</x:v>
       </x:c>
       <x:c r="B5" s="14" t="str">
-        <x:v>Temporal/sequential data, event streams, longitudinal data, forecasting/classification. Family: Data &amp; Time Series.</x:v>
+        <x:v>Temporal/sequential data, event streams, longitudinal data, forecasting/classification. Family: Complex Systems, Time Series &amp; Signals.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -3766,7 +4350,7 @@
         <x:v>Healthcare &amp; Clinical AI</x:v>
       </x:c>
       <x:c r="B6" s="14" t="str">
-        <x:v>Clinical ML, health data, biomedical informatics, precision/public health. Family: Healthcare &amp; Biomedical AI.</x:v>
+        <x:v>Clinical ML, health data, biomedical informatics, precision/public health. Family: Healthcare &amp; Biometrics.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -3774,15 +4358,15 @@
         <x:v>Biomedical Imaging</x:v>
       </x:c>
       <x:c r="B7" s="14" t="str">
-        <x:v>Medical image analysis, segmentation, biomedical imaging, clinical imaging. Family: Healthcare &amp; Biomedical AI.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="15" hidden="0" customHeight="1">
+        <x:v>Medical image analysis, segmentation, biomedical imaging, clinical imaging. Family: Healthcare &amp; Biometrics.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A8" s="14" t="str">
         <x:v>Signal Processing</x:v>
       </x:c>
       <x:c r="B8" s="14" t="str">
-        <x:v>Signal processing methods and ML for signals, including biomedical signals. Family: Signals, Vision &amp; Multimedia.</x:v>
+        <x:v>Signal processing methods and ML for signals, including biomedical signals. Family: Complex Systems, Time Series &amp; Signals.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -3838,7 +4422,7 @@
         <x:v>Probabilistic, Causal &amp; Uncertainty ML</x:v>
       </x:c>
       <x:c r="B15" s="14" t="str">
-        <x:v>Bayesian/probabilistic ML, uncertainty quantification, causal inference. Family: ML &amp; AI.</x:v>
+        <x:v>Bayesian/probabilistic ML, uncertainty quantification, causal inference. Family: ML &amp; Data Science.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
@@ -3846,7 +4430,7 @@
         <x:v>Learning Theory &amp; Statistical Foundations</x:v>
       </x:c>
       <x:c r="B16" s="14" t="str">
-        <x:v>Statistical learning, learning theory, generalization, theoretical foundations. Family: ML &amp; AI.</x:v>
+        <x:v>Statistical learning, learning theory, generalization, theoretical foundations. Family: ML &amp; Data Science.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
@@ -3854,15 +4438,15 @@
         <x:v>Human-AI Interaction &amp; Deployment</x:v>
       </x:c>
       <x:c r="B17" s="14" t="str">
-        <x:v>Human-centered AI, usability, clinical deployment, interfaces, translational use. Family: ML &amp; AI.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="15" hidden="0" customHeight="1">
+        <x:v>Human-centered AI, usability, clinical deployment, interfaces, translational use. Family: Responsible &amp; Trustworthy AI.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A18" s="12" t="str">
         <x:v>Natural Language Processing &amp; LLMs</x:v>
       </x:c>
       <x:c r="B18" s="12" t="str">
-        <x:v>Natural language processing, language models, computational linguistics, and LLM systems. Family: ML &amp; AI.</x:v>
+        <x:v>Natural language processing, language models, computational linguistics, and LLM systems. Family: NLP, Agents &amp; Retrieval.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
@@ -3870,7 +4454,7 @@
         <x:v>Reinforcement Learning</x:v>
       </x:c>
       <x:c r="B19" s="12" t="str">
-        <x:v>Learning actions and policies from interaction, reward, and feedback. Family: ML &amp; AI.</x:v>
+        <x:v>Learning actions and policies from interaction, reward, and feedback. Family: RL, Robotics &amp; Control.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -3878,7 +4462,7 @@
         <x:v>Federated &amp; Distributed Learning</x:v>
       </x:c>
       <x:c r="B20" s="12" t="str">
-        <x:v>Distributed training, federated learning, and collaborative learning systems. Not automatically an ethics tag. Family: ML &amp; AI.</x:v>
+        <x:v>Distributed training, federated learning, and collaborative learning systems. Not automatically an ethics tag. Family: ML &amp; Data Science.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
@@ -3886,7 +4470,7 @@
         <x:v>Computer Vision &amp; Pattern Recognition</x:v>
       </x:c>
       <x:c r="B21" s="12" t="str">
-        <x:v>Visual understanding, image analysis, recognition, and structured pattern learning. Family: Signals, Vision &amp; Multimedia.</x:v>
+        <x:v>Visual understanding, image analysis, recognition, and structured pattern learning. Family: Vision &amp; Multimedia.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -3894,7 +4478,7 @@
         <x:v>Nonlinear Dynamics &amp; Chaos</x:v>
       </x:c>
       <x:c r="B22" s="12" t="str">
-        <x:v>Dynamical systems, bifurcations, chaos, synchronization, and nonlinear modeling. Family: Dynamics, Complex Systems &amp; Control.</x:v>
+        <x:v>Dynamical systems, bifurcations, chaos, synchronization, and nonlinear modeling. Family: Complex Systems, Time Series &amp; Signals.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -3902,15 +4486,15 @@
         <x:v>Complex Systems &amp; Network Science</x:v>
       </x:c>
       <x:c r="B23" s="12" t="str">
-        <x:v>Complex adaptive systems, emergence, network structure, and dynamics on networks. Family: Dynamics, Complex Systems &amp; Control.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Complex adaptive systems, emergence, network structure, and dynamics on networks. Family: Complex Systems, Time Series &amp; Signals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" t="str">
         <x:v>Control &amp; Robotics</x:v>
       </x:c>
       <x:c r="B24" s="12" t="str">
-        <x:v>Feedback control, automation, decision making, robotics, and learning-based control. Family: Dynamics, Complex Systems &amp; Control.</x:v>
+        <x:v>Feedback control, automation, decision making, robotics, and learning-based control. Family: RL, Robotics &amp; Control.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -3918,7 +4502,7 @@
         <x:v>System Identification &amp; Data-driven Dynamics</x:v>
       </x:c>
       <x:c r="B25" s="12" t="str">
-        <x:v>Identifying dynamical models from data, state estimation, and data-driven dynamics. Family: Dynamics, Complex Systems &amp; Control.</x:v>
+        <x:v>Identifying dynamical models from data, state estimation, and data-driven dynamics. Family: Complex Systems, Time Series &amp; Signals.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">
@@ -3945,12 +4529,12 @@
         <x:v>Reliable and safe AI, adversarial robustness, distribution shift, and model assurance. Family: Responsible &amp; Trustworthy AI.</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="15" hidden="0" customHeight="1">
+    <x:row r="29" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A29" t="str">
         <x:v>Evolutionary Computation &amp; Optimization</x:v>
       </x:c>
       <x:c r="B29" s="12" t="str">
-        <x:v>Evolutionary algorithms, genetic programming, neuroevolution, and population-based optimization. Family: ML &amp; AI.</x:v>
+        <x:v>Evolutionary algorithms, genetic programming, neuroevolution, and population-based optimization. Family: ML &amp; Data Science.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -3961,28 +4545,28 @@
         <x:v>Computational models of cognition, learning, perception, language, and reasoning. Family: Neuroscience &amp; Neurotechnology.</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="15" hidden="0" customHeight="1">
+    <x:row r="31" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A31" t="str">
         <x:v>ML Systems &amp; Infrastructure</x:v>
       </x:c>
       <x:c r="B31" s="12" t="str">
-        <x:v>Systems for ML and ML for systems, including training, inference, compilers, hardware, and serving. Family: ML &amp; AI.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="15" hidden="0" customHeight="1">
+        <x:v>Systems for ML and ML for systems, including training, inference, compilers, hardware, and serving. Family: ML &amp; Data Science.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A32" t="str">
         <x:v>Knowledge Representation &amp; Reasoning</x:v>
       </x:c>
       <x:c r="B32" s="12" t="str">
-        <x:v>Formal and symbolic representations of knowledge, logic, automated inference, and reasoning in AI. Family: ML &amp; AI.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="15" hidden="0" customHeight="1">
+        <x:v>Formal and symbolic representations of knowledge, logic, automated inference, and reasoning in AI. Family: ML &amp; Data Science.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A33" t="str">
         <x:v>Planning &amp; Search</x:v>
       </x:c>
       <x:c r="B33" s="12" t="str">
-        <x:v>Automated planning, scheduling, heuristic search, constraint solving, and sequential decision-making. Family: ML &amp; AI.</x:v>
+        <x:v>Automated planning, scheduling, heuristic search, constraint solving, and sequential decision-making. Family: RL, Robotics &amp; Control.</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -3990,7 +4574,7 @@
         <x:v>Computer Graphics &amp; Visualization</x:v>
       </x:c>
       <x:c r="B34" s="12" t="str">
-        <x:v>Rendering, geometry, animation, visual simulation, and visualization, including learning-based methods. Family: Signals, Vision &amp; Multimedia.</x:v>
+        <x:v>Rendering, geometry, animation, visual simulation, and visualization, including learning-based methods. Family: Vision &amp; Multimedia.</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -3998,7 +4582,7 @@
         <x:v>Multimedia Learning &amp; Retrieval</x:v>
       </x:c>
       <x:c r="B35" s="12" t="str">
-        <x:v>Learning from multiple media, multimodal fusion, content understanding, indexing, search, and retrieval. Family: Signals, Vision &amp; Multimedia.</x:v>
+        <x:v>Learning from multiple media, multimodal fusion, content understanding, indexing, search, and retrieval. Family: Vision &amp; Multimedia.</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -4006,13 +4590,53 @@
         <x:v>Biometrics &amp; Human Sensing</x:v>
       </x:c>
       <x:c r="B36" s="12" t="str">
-        <x:v>Biometric identity, face and gesture recognition, body motion, behavioral sensing, and biometric evaluation. Family: Signals, Vision &amp; Multimedia.</x:v>
+        <x:v>Biometric identity, face and gesture recognition, body motion, behavioral sensing, and biometric evaluation. Family: Healthcare &amp; Biometrics.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A37" t="str">
+        <x:v>Autonomous Agents &amp; Multiagent Systems</x:v>
+      </x:c>
+      <x:c r="B37" s="12" t="str">
+        <x:v>Autonomous agents, coordination, negotiation, communication, and multiagent systems. Distinct from LLM tool use. Family: NLP, Agents &amp; Retrieval.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A38" t="str">
+        <x:v>LLM Agents &amp; Tool Use</x:v>
+      </x:c>
+      <x:c r="B38" s="12" t="str">
+        <x:v>Language-model agents, tool use, agentic workflows, and language-mediated agent communication. Family: NLP, Agents &amp; Retrieval.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A39" t="str">
+        <x:v>Information Retrieval &amp; Search</x:v>
+      </x:c>
+      <x:c r="B39" s="12" t="str">
+        <x:v>Search, ranking, information access, conversational retrieval, and retrieval-augmented generation. Family: NLP, Agents &amp; Retrieval.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A40" t="str">
+        <x:v>Recommender Systems</x:v>
+      </x:c>
+      <x:c r="B40" s="12" t="str">
+        <x:v>Personalization, recommendation models, user-item interaction, and recommendation evaluation. Family: NLP, Agents &amp; Retrieval.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A41" t="str">
+        <x:v>Graphs &amp; Graph Learning</x:v>
+      </x:c>
+      <x:c r="B41" s="12" t="str">
+        <x:v>Graph mining, graph representation learning, graph neural networks, and learning on structured networks. Family: Complex Systems, Time Series &amp; Signals.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cb5f4dc5093453e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7261d0a80e942ff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4092,7 +4716,7 @@
         <x:v>AAMAS</x:v>
       </x:c>
       <x:c r="B4" s="20" t="str">
-        <x:v>Deep Representation Learning; Probabilistic, Causal &amp; Uncertainty ML; Evolutionary Computation &amp; Optimization; Complex Systems &amp; Network Science; Ethics &amp; Governance; Explainability &amp; Interpretability</x:v>
+        <x:v>Deep Representation Learning; Probabilistic, Causal &amp; Uncertainty ML; Control &amp; Robotics; Complex Systems &amp; Network Science; Ethics &amp; Governance; Explainability &amp; Interpretability</x:v>
       </x:c>
       <x:c r="C4" s="20" t="str">
         <x:v>Autonomous agents and multi-agent systems: learning and adaptation, coordination, game theory, planning, reasoning, agent engineering, and agent-based simulation. Also covers human-agent interaction, robot teams, norms and governance, and generative agents. The contribution should concern agents or their interaction; generic language-model or learning results are not automatically in scope.</x:v>
@@ -4109,19 +4733,19 @@
     </x:row>
     <x:row r="5" ht="72" hidden="0" customHeight="1">
       <x:c r="A5" s="20" t="str">
-        <x:v>ACM FAccT</x:v>
+        <x:v>ACL</x:v>
       </x:c>
       <x:c r="B5" s="20" t="str">
-        <x:v>Human-AI Interaction &amp; Deployment; Robustness &amp; Safety</x:v>
+        <x:v>Cognitive Science &amp; Computational Cognition; Explainability &amp; Interpretability; Fairness &amp; Responsible AI; Human-AI Interaction &amp; Deployment; Knowledge Representation &amp; Reasoning</x:v>
       </x:c>
       <x:c r="C5" s="20" t="str">
-        <x:v>Fairness, accountability, and transparency in computing, combining algorithmic research with sociotechnical, legal, philosophical, and human-centered approaches. Characteristic contributions include audits and evaluation practices, governance, human experiences of systems, and responsible development and deployment. A fairness or accountability question should be substantive, not a passing motivation for generic ML.</x:v>
+        <x:v>Computational linguistics and language processing: language modeling, linguistic structure, multilinguality and translation, generation, dialogue, resources, and evaluation. Language-grounded agent and retrieval work is relevant. The 2027 theme examines homogenization and knowledge collapse in LLMs. A language contribution remains central; general medical or robotics applications do not make this a specialist venue.</x:v>
       </x:c>
       <x:c r="D5" s="21" t="n">
-        <x:v>2026</x:v>
+        <x:v>2027</x:v>
       </x:c>
       <x:c r="E5" s="20" t="str">
-        <x:v>https://facctconference.org/2026/cfp.html</x:v>
+        <x:v>https://2027.aclweb.org/calls/main/</x:v>
       </x:c>
       <x:c r="F5" s="22" t="n">
         <x:v>46302</x:v>
@@ -4129,19 +4753,19 @@
     </x:row>
     <x:row r="6" ht="72" hidden="0" customHeight="1">
       <x:c r="A6" s="20" t="str">
-        <x:v>ACM MM</x:v>
+        <x:v>ACM FAccT</x:v>
       </x:c>
       <x:c r="B6" s="20" t="str">
-        <x:v>Machine Learning; Natural Language Processing &amp; LLMs; Human-AI Interaction &amp; Deployment; Data Mining &amp; Data Science; Explainability &amp; Interpretability</x:v>
+        <x:v>Human-AI Interaction &amp; Deployment; Robustness &amp; Safety</x:v>
       </x:c>
       <x:c r="C6" s="20" t="str">
-        <x:v>Multimedia understanding, learning, generation, and retrieval across image, video, audio, language, and other modalities. Characteristic work includes multimodal fusion, generative and foundation models, scalable indexing and search, cross-modal alignment, and human-centered multimedia experiences. The 2026 steering-committee scope also emphasizes explainability. Healthcare, education, and entertainment are applications, not blanket topical identities.</x:v>
+        <x:v>Fairness, accountability, and transparency in computing, combining algorithmic research with sociotechnical, legal, philosophical, and human-centered approaches. Characteristic contributions include audits and evaluation practices, governance, human experiences of systems, and responsible development and deployment. A fairness or accountability question should be substantive, not a passing motivation for generic ML.</x:v>
       </x:c>
       <x:c r="D6" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E6" s="20" t="str">
-        <x:v>https://2026.acmmm.org/site/topics.html; https://2026.acmmm.org/</x:v>
+        <x:v>https://facctconference.org/2026/cfp.html</x:v>
       </x:c>
       <x:c r="F6" s="22" t="n">
         <x:v>46302</x:v>
@@ -4149,39 +4773,39 @@
     </x:row>
     <x:row r="7" ht="72" hidden="0" customHeight="1">
       <x:c r="A7" s="20" t="str">
-        <x:v>ACM SIGGRAPH</x:v>
+        <x:v>ACM MM</x:v>
       </x:c>
       <x:c r="B7" s="20" t="str">
-        <x:v>Deep Representation Learning; Human-AI Interaction &amp; Deployment</x:v>
+        <x:v>Machine Learning; Natural Language Processing &amp; LLMs; Human-AI Interaction &amp; Deployment; Data Mining &amp; Data Science; Explainability &amp; Interpretability</x:v>
       </x:c>
       <x:c r="C7" s="20" t="str">
-        <x:v>Computer graphics and interactive techniques, centered on rendering, geometric modeling, animation, physical simulation, imaging, visualization, and immersive visual experiences. Generative AI and machine learning are relevant when they advance visual computing, such as neural rendering and learned animation. Technical papers use integrated conference and ACM TOG journal tracks; this profile does not describe SIGGRAPH Asia or all of AI.</x:v>
+        <x:v>Multimedia understanding, learning, generation, and retrieval across image, video, audio, language, and other modalities. Characteristic work includes multimodal fusion, generative and foundation models, scalable indexing and search, cross-modal alignment, and human-centered multimedia experiences. The 2026 steering-committee scope also emphasizes explainability. Healthcare, education, and entertainment are applications, not blanket topical identities.</x:v>
       </x:c>
       <x:c r="D7" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E7" s="20" t="str">
-        <x:v>https://s2026.siggraph.org/program/technical-papers/</x:v>
+        <x:v>https://2026.acmmm.org/site/topics.html; https://2026.acmmm.org/</x:v>
       </x:c>
       <x:c r="F7" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="60" hidden="0" customHeight="1">
+    <x:row r="8" ht="72" hidden="0" customHeight="1">
       <x:c r="A8" s="20" t="str">
-        <x:v>ACML</x:v>
+        <x:v>ACM SIGGRAPH</x:v>
       </x:c>
       <x:c r="B8" s="20" t="str">
-        <x:v>Deep Representation Learning; Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Natural Language Processing &amp; LLMs; Fairness &amp; Responsible AI; Privacy-preserving ML</x:v>
+        <x:v>Deep Representation Learning; Human-AI Interaction &amp; Deployment</x:v>
       </x:c>
       <x:c r="C8" s="20" t="str">
-        <x:v>Theory and practice of machine learning, including probabilistic methods, representation learning, transfer and meta-learning, reinforcement learning, and learning theory. Generative models, language models, and trustworthy learning extend this core. The broad applications list is not treated as evidence that every application field defines the conference.</x:v>
+        <x:v>Computer graphics and interactive techniques, centered on rendering, geometric modeling, animation, physical simulation, imaging, visualization, and immersive visual experiences. Generative AI and machine learning are relevant when they advance visual computing, such as neural rendering and learned animation. Technical papers use integrated conference and ACM TOG journal tracks; this profile does not describe SIGGRAPH Asia or all of AI.</x:v>
       </x:c>
       <x:c r="D8" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E8" s="20" t="str">
-        <x:v>https://www.acml-conf.org/2026/calls/papers/</x:v>
+        <x:v>https://s2026.siggraph.org/program/technical-papers/</x:v>
       </x:c>
       <x:c r="F8" s="22" t="n">
         <x:v>46302</x:v>
@@ -4189,97 +4813,97 @@
     </x:row>
     <x:row r="9" ht="60" hidden="0" customHeight="1">
       <x:c r="A9" s="20" t="str">
-        <x:v>AIES</x:v>
+        <x:v>ACML</x:v>
       </x:c>
       <x:c r="B9" s="20" t="str">
-        <x:v>Human-AI Interaction &amp; Deployment; Privacy-preserving ML</x:v>
+        <x:v>Deep Representation Learning; Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Natural Language Processing &amp; LLMs; Fairness &amp; Responsible AI; Privacy-preserving ML</x:v>
       </x:c>
       <x:c r="C9" s="20" t="str">
-        <x:v>Ethics and societal consequences of AI, connecting computer science, law and policy, social science, and philosophy. Defining concerns include governance and power, accountability after deployment, value alignment, fairness, human-AI interaction, and institutional practice. Technical work is relevant through a serious ethical or societal contribution.</x:v>
+        <x:v>Theory and practice of machine learning, including probabilistic methods, representation learning, transfer and meta-learning, reinforcement learning, and learning theory. Generative models, language models, and trustworthy learning extend this core. The broad applications list is not treated as evidence that every application field defines the conference.</x:v>
       </x:c>
       <x:c r="D9" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E9" s="20" t="str">
+        <x:v>https://www.acml-conf.org/2026/calls/papers/</x:v>
+      </x:c>
+      <x:c r="F9" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="60" hidden="0" customHeight="1">
+      <x:c r="A10" s="20" t="str">
+        <x:v>AIES</x:v>
+      </x:c>
+      <x:c r="B10" s="20" t="str">
+        <x:v>Human-AI Interaction &amp; Deployment; Privacy-preserving ML</x:v>
+      </x:c>
+      <x:c r="C10" s="20" t="str">
+        <x:v>Ethics and societal consequences of AI, connecting computer science, law and policy, social science, and philosophy. Defining concerns include governance and power, accountability after deployment, value alignment, fairness, human-AI interaction, and institutional practice. Technical work is relevant through a serious ethical or societal contribution.</x:v>
+      </x:c>
+      <x:c r="D10" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E10" s="20" t="str">
         <x:v>https://www.aies-conference.com/2026/call-for-papers/</x:v>
       </x:c>
-      <x:c r="F9" s="22" t="n">
-        <x:v>46302</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="48" hidden="0" customHeight="1">
-      <x:c r="A10" s="20" t="str">
+      <x:c r="F10" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="48" hidden="0" customHeight="1">
+      <x:c r="A11" s="20" t="str">
         <x:v>AISTATS</x:v>
       </x:c>
-      <x:c r="B10" s="20" t="str"/>
-      <x:c r="C10" s="20" t="str">
+      <x:c r="B11" s="20" t="str"/>
+      <x:c r="C11" s="20" t="str">
         <x:v>Research at the interface of artificial intelligence, machine learning, and statistics. Its defining emphasis is on statistical foundations and methodology for learning and inference, rather than a particular application domain. Research bridges statistical reasoning and learning algorithms, with archival contributions to both communities.</x:v>
       </x:c>
-      <x:c r="D10" s="21" t="n">
+      <x:c r="D11" s="21" t="n">
         <x:v>2027</x:v>
       </x:c>
-      <x:c r="E10" s="20" t="str">
+      <x:c r="E11" s="20" t="str">
         <x:v>https://aistats.org/aistats2027/; https://aistats.org/aistats2027/call-for-papers.html</x:v>
       </x:c>
-      <x:c r="F10" s="22" t="n">
-        <x:v>46302</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="72" hidden="0" customHeight="1">
-      <x:c r="A11" s="20" t="str">
+      <x:c r="F11" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="72" hidden="0" customHeight="1">
+      <x:c r="A12" s="20" t="str">
         <x:v>AutoML</x:v>
       </x:c>
-      <x:c r="B11" s="20" t="str">
+      <x:c r="B12" s="20" t="str">
         <x:v>Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Explainability &amp; Interpretability; Natural Language Processing &amp; LLMs; Robustness &amp; Safety</x:v>
       </x:c>
-      <x:c r="C11" s="20" t="str">
+      <x:c r="C12" s="20" t="str">
         <x:v>Automating the construction and configuration of learning systems: hyperparameter optimization, Bayesian optimization, neural architecture search, model selection, meta-learning, and pipeline automation. Includes evolutionary and reinforcement-learning approaches, AutoML for foundation models, and evaluation through applications, benchmarks, challenges, and datasets. Trustworthiness matters specifically in automated ML workflows.</x:v>
-      </x:c>
-      <x:c r="D11" s="21" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="E11" s="20" t="str">
-        <x:v>https://2026.automl.cc/call-for-papers/</x:v>
-      </x:c>
-      <x:c r="F11" s="22" t="n">
-        <x:v>46302</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="60" hidden="0" customHeight="1">
-      <x:c r="A12" s="20" t="str">
-        <x:v>BMVC</x:v>
-      </x:c>
-      <x:c r="B12" s="20" t="str">
-        <x:v>Signal Processing</x:v>
-      </x:c>
-      <x:c r="C12" s="20" t="str">
-        <x:v>Computer vision, image processing, and visual pattern recognition, including visual learning, recognition and segmentation, reconstruction, motion and video analysis, and evaluation of vision methods. The single-track BMVA conference combines methodological and applied vision research. It is an established broad vision venue, not a specialist biomedical-imaging meeting.</x:v>
       </x:c>
       <x:c r="D12" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E12" s="20" t="str">
+        <x:v>https://2026.automl.cc/call-for-papers/</x:v>
+      </x:c>
+      <x:c r="F12" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="60" hidden="0" customHeight="1">
+      <x:c r="A13" s="20" t="str">
+        <x:v>BMVC</x:v>
+      </x:c>
+      <x:c r="B13" s="20" t="str">
+        <x:v>Signal Processing</x:v>
+      </x:c>
+      <x:c r="C13" s="20" t="str">
+        <x:v>Computer vision, image processing, and visual pattern recognition, including visual learning, recognition and segmentation, reconstruction, motion and video analysis, and evaluation of vision methods. The single-track BMVA conference combines methodological and applied vision research. It is an established broad vision venue, not a specialist biomedical-imaging meeting.</x:v>
+      </x:c>
+      <x:c r="D13" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E13" s="20" t="str">
         <x:v>https://bmvc2026.bmva.org/calls/call-for-papers/</x:v>
-      </x:c>
-      <x:c r="F12" s="22" t="n">
-        <x:v>46302</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="72" hidden="0" customHeight="1">
-      <x:c r="A13" s="20" t="str">
-        <x:v>CCN</x:v>
-      </x:c>
-      <x:c r="B13" s="20" t="str">
-        <x:v>Cognitive Science &amp; Computational Cognition; Explainability &amp; Interpretability</x:v>
-      </x:c>
-      <x:c r="C13" s="20" t="str">
-        <x:v>Cognitive computational neuroscience, connecting experiments and models of brain computation with artificial intelligence. Characteristic work compares biological and artificial representations, models perception, cognition and action, studies neural connectivity and dynamics, and uses mechanistic interpretability to understand neural-network models. The aim is understanding computation and behavior across brains and AI systems.</x:v>
-      </x:c>
-      <x:c r="D13" s="21" t="n">
-        <x:v>2027</x:v>
-      </x:c>
-      <x:c r="E13" s="20" t="str">
-        <x:v>https://2027.ccneuro.org/</x:v>
       </x:c>
       <x:c r="F13" s="22" t="n">
         <x:v>46302</x:v>
@@ -4287,37 +4911,39 @@
     </x:row>
     <x:row r="14" ht="72" hidden="0" customHeight="1">
       <x:c r="A14" s="20" t="str">
+        <x:v>CCN</x:v>
+      </x:c>
+      <x:c r="B14" s="20" t="str">
+        <x:v>Cognitive Science &amp; Computational Cognition; Explainability &amp; Interpretability</x:v>
+      </x:c>
+      <x:c r="C14" s="20" t="str">
+        <x:v>Cognitive computational neuroscience, connecting experiments and models of brain computation with artificial intelligence. Characteristic work compares biological and artificial representations, models perception, cognition and action, studies neural connectivity and dynamics, and uses mechanistic interpretability to understand neural-network models. The aim is understanding computation and behavior across brains and AI systems.</x:v>
+      </x:c>
+      <x:c r="D14" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E14" s="20" t="str">
+        <x:v>https://2027.ccneuro.org/</x:v>
+      </x:c>
+      <x:c r="F14" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="72" hidden="0" customHeight="1">
+      <x:c r="A15" s="20" t="str">
         <x:v>CHIL</x:v>
       </x:c>
-      <x:c r="B14" s="20" t="str">
+      <x:c r="B15" s="20" t="str">
         <x:v>Explainability &amp; Interpretability; Human-AI Interaction &amp; Deployment; Robustness &amp; Safety; Time Series &amp; Sequential Data</x:v>
       </x:c>
-      <x:c r="C14" s="20" t="str">
+      <x:c r="C15" s="20" t="str">
         <x:v>Machine learning and inference for clinical, public, and population health. Distinguishing areas include causal inference, survival analysis, multimodal health data, generalization across populations, interpretability, and clinical evaluation and deployment. Research may emphasize methods, practical applications, or societal impact. Health-focused inference and evaluation remain the common thread across these tracks.</x:v>
-      </x:c>
-      <x:c r="D14" s="21" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="E14" s="20" t="str">
-        <x:v>https://chil.ahli.cc/submit/call-for-papers/</x:v>
-      </x:c>
-      <x:c r="F14" s="22" t="n">
-        <x:v>46302</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="60" hidden="0" customHeight="1">
-      <x:c r="A15" s="20" t="str">
-        <x:v>CogSci</x:v>
-      </x:c>
-      <x:c r="B15" s="20" t="str"/>
-      <x:c r="C15" s="20" t="str">
-        <x:v>Interdisciplinary study of cognition and the mind, connecting psychology, linguistics, artificial intelligence, neuroscience, philosophy, anthropology, and education. Computational models and experiments should illuminate cognitive processes and behavior. An AI paper belongs here through its contribution to understanding cognition, not solely through a predictive performance improvement.</x:v>
       </x:c>
       <x:c r="D15" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E15" s="20" t="str">
-        <x:v>https://cognitivesciencesociety.org/submissions-faq/; https://cognitivesciencesociety.org/</x:v>
+        <x:v>https://chil.ahli.cc/submit/call-for-papers/</x:v>
       </x:c>
       <x:c r="F15" s="22" t="n">
         <x:v>46302</x:v>
@@ -4325,99 +4951,97 @@
     </x:row>
     <x:row r="16" ht="60" hidden="0" customHeight="1">
       <x:c r="A16" s="20" t="str">
-        <x:v>COLT</x:v>
+        <x:v>CIKM</x:v>
       </x:c>
       <x:c r="B16" s="20" t="str">
-        <x:v>Deep Representation Learning; Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Privacy-preserving ML; Fairness &amp; Responsible AI</x:v>
+        <x:v>Information Retrieval &amp; Search; Recommender Systems; Knowledge Representation &amp; Reasoning; Graphs &amp; Graph Learning; LLM Agents &amp; Tool Use</x:v>
       </x:c>
       <x:c r="C16" s="20" t="str">
-        <x:v>Theoretical foundations of learning at the intersection of computer science, statistics, and applied mathematics. Characteristic work studies learnability, sample and computational complexity, online learning, optimization, bandits, and generalization. Neural-network, causal, reinforcement-learning, privacy, and fairness papers belong here when the theoretical contribution is central.</x:v>
+        <x:v>Information retrieval, knowledge management, data mining and database systems, with a strong focus on effective information access and knowledge at scale. The 2026 organizer description emphasizes AI for information access, knowledge representation, personalization and evaluation. Agentic and graph methods are relevant through these information and knowledge problems.</x:v>
       </x:c>
       <x:c r="D16" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E16" s="20" t="str">
-        <x:v>https://learningtheory.org/colt2026/cfp.html</x:v>
+        <x:v>https://cikm2026.diag.uniroma1.it/</x:v>
       </x:c>
       <x:c r="F16" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="72" hidden="0" customHeight="1">
+    <x:row r="17" ht="60" hidden="0" customHeight="1">
       <x:c r="A17" s="20" t="str">
-        <x:v>CoRL</x:v>
-      </x:c>
-      <x:c r="B17" s="20" t="str">
-        <x:v>Computer Vision &amp; Pattern Recognition; Probabilistic, Causal &amp; Uncertainty ML; Human-AI Interaction &amp; Deployment; Robustness &amp; Safety; Learning Theory &amp; Statistical Foundations</x:v>
-      </x:c>
+        <x:v>CogSci</x:v>
+      </x:c>
+      <x:c r="B17" s="20" t="str"/>
       <x:c r="C17" s="20" t="str">
-        <x:v>Machine learning for physical robots, especially imitation and reinforcement learning, learned perception and control, robot foundation models, and learning-based task and motion planning. Includes uncertainty, generalization, safety, human-robot interaction, and datasets grounded in manipulation, navigation, or locomotion. General ML is relevant when it makes a substantive contribution to robot learning.</x:v>
+        <x:v>Interdisciplinary study of cognition and the mind, connecting psychology, linguistics, artificial intelligence, neuroscience, philosophy, anthropology, and education. Computational models and experiments should illuminate cognitive processes and behavior. An AI paper belongs here through its contribution to understanding cognition, not solely through a predictive performance improvement.</x:v>
       </x:c>
       <x:c r="D17" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E17" s="20" t="str">
-        <x:v>https://www.corl.org/contributions/call-for-papers</x:v>
+        <x:v>https://cognitivesciencesociety.org/submissions-faq/; https://cognitivesciencesociety.org/</x:v>
       </x:c>
       <x:c r="F17" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="72" hidden="0" customHeight="1">
+    <x:row r="18" ht="60" hidden="0" customHeight="1">
       <x:c r="A18" s="20" t="str">
-        <x:v>CVPR</x:v>
+        <x:v>COLING</x:v>
       </x:c>
       <x:c r="B18" s="20" t="str">
-        <x:v>Computer Graphics &amp; Visualization; Multimedia Learning &amp; Retrieval; Natural Language Processing &amp; LLMs; Biometrics &amp; Human Sensing; Robustness &amp; Safety</x:v>
+        <x:v>Information Retrieval &amp; Search; Cognitive Science &amp; Computational Cognition; Explainability &amp; Interpretability; Fairness &amp; Responsible AI</x:v>
       </x:c>
       <x:c r="C18" s="20" t="str">
-        <x:v>Broad computer vision and pattern recognition: visual representations, recognition and segmentation, 3D reconstruction, computational imaging, image and video generation, motion and tracking, and vision-language learning. Graphics, multimodal learning, human face/body understanding, and reliable vision are substantial recurring research areas. Peripheral application fields are not tagged merely because a long CFP mentions them.</x:v>
+        <x:v>Computational linguistics and language processing spanning linguistic theory, multilinguality, semantics and structured prediction, language models, dialogue, and empirical evaluation. Agentic language systems and knowledge-grounded NLP are relevant; the defining contribution should concern language, not a peripheral application domain.</x:v>
       </x:c>
       <x:c r="D18" s="21" t="n">
         <x:v>2027</x:v>
       </x:c>
       <x:c r="E18" s="20" t="str">
-        <x:v>https://cvpr.thecvf.com/Conferences/2027/CallForPapers</x:v>
+        <x:v>https://2027.coling-iccl.org/calls/main_conference_papers/</x:v>
       </x:c>
       <x:c r="F18" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="72" hidden="0" customHeight="1">
+    <x:row r="19" ht="60" hidden="0" customHeight="1">
       <x:c r="A19" s="20" t="str">
-        <x:v>EACL</x:v>
+        <x:v>COLM</x:v>
       </x:c>
       <x:c r="B19" s="20" t="str">
-        <x:v>Explainability &amp; Interpretability; Fairness &amp; Responsible AI; Cognitive Science &amp; Computational Cognition</x:v>
+        <x:v>Learning Theory &amp; Statistical Foundations; Explainability &amp; Interpretability; Robustness &amp; Safety; Fairness &amp; Responsible AI; Multimedia Learning &amp; Retrieval</x:v>
       </x:c>
       <x:c r="C19" s="20" t="str">
-        <x:v>Computational linguistics and natural language processing, including language modeling, multilingual processing, translation, dialogue, information extraction, semantics, and linguistic analysis. Human-centered evaluation, interpretability, and bias are relevant within language research. The reviewed 2027 theme strengthens connections to psycholinguistics and cognitive modeling; peripheral application domains are not extra tags.</x:v>
+        <x:v>Language-model foundations and methods: training and architecture, data and scaling, inference and generation, evaluation, reasoning, retrieval augmentation, and tool-using language agents. Alignment, interpretability, and multimodal language models are meaningful extensions. A central language-model contribution distinguishes the conference from generic AI applications.</x:v>
       </x:c>
       <x:c r="D19" s="21" t="n">
-        <x:v>2027</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="E19" s="20" t="str">
-        <x:v>https://2027.eacl.org/calls/papers/</x:v>
+        <x:v>https://colm.cc/Conferences/2026/CallForPapers</x:v>
       </x:c>
       <x:c r="F19" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="72" hidden="0" customHeight="1">
+    <x:row r="20" ht="60" hidden="0" customHeight="1">
       <x:c r="A20" s="20" t="str">
-        <x:v>ECCV</x:v>
+        <x:v>COLT</x:v>
       </x:c>
       <x:c r="B20" s="20" t="str">
-        <x:v>Computer Graphics &amp; Visualization; Multimedia Learning &amp; Retrieval; Natural Language Processing &amp; LLMs; Biometrics &amp; Human Sensing; Robustness &amp; Safety</x:v>
+        <x:v>Deep Representation Learning; Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Privacy-preserving ML; Fairness &amp; Responsible AI</x:v>
       </x:c>
       <x:c r="C20" s="20" t="str">
-        <x:v>Broad research in visual perception, representation learning, recognition, segmentation, 3D geometry and reconstruction, computational imaging, and image/video synthesis. Vision-language models, multimodal understanding, human motion and appearance, and robust visual systems extend this core. ECCV is the biennial European flagship for computer vision; the scope uses the actual published 2026 CFP, not an invented 2028 call.</x:v>
+        <x:v>Theoretical foundations of learning at the intersection of computer science, statistics, and applied mathematics. Characteristic work studies learnability, sample and computational complexity, online learning, optimization, bandits, and generalization. Neural-network, causal, reinforcement-learning, privacy, and fairness papers belong here when the theoretical contribution is central.</x:v>
       </x:c>
       <x:c r="D20" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E20" s="20" t="str">
-        <x:v>https://eccv.ecva.net/Conferences/2026/CallForPapers</x:v>
+        <x:v>https://learningtheory.org/colt2026/cfp.html</x:v>
       </x:c>
       <x:c r="F20" s="22" t="n">
         <x:v>46302</x:v>
@@ -4425,19 +5049,19 @@
     </x:row>
     <x:row r="21" ht="60" hidden="0" customHeight="1">
       <x:c r="A21" s="20" t="str">
-        <x:v>EuroGP</x:v>
+        <x:v>CoNLL</x:v>
       </x:c>
       <x:c r="B21" s="20" t="str">
-        <x:v>Learning Theory &amp; Statistical Foundations; Deep Representation Learning</x:v>
+        <x:v>Deep Representation Learning; Multimedia Learning &amp; Retrieval</x:v>
       </x:c>
       <x:c r="C21" s="20" t="str">
-        <x:v>Genetic programming and evolutionary program synthesis, including symbolic regression, program representations and operators, surrogate-assisted search, multi-objective evolution, and interpretable learned programs. Evolutionary machine learning, AutoML pipelines, and neuroevolution connect this focused methodological community to ML. Application domains do not define its tags.</x:v>
+        <x:v>Scientifically, cognitively, and linguistically motivated computational language learning. Characteristic work concerns language acquisition, psycholinguistics, grammars and meaning, multilinguality, language and the brain, and grounded language models. This is a focused scientific NLP venue rather than a generic empirical language-model benchmark conference.</x:v>
       </x:c>
       <x:c r="D21" s="21" t="n">
-        <x:v>2027</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="E21" s="20" t="str">
-        <x:v>https://www.evostar.org/2027/eurogp/</x:v>
+        <x:v>https://www.conll.org/2026</x:v>
       </x:c>
       <x:c r="F21" s="22" t="n">
         <x:v>46302</x:v>
@@ -4445,197 +5069,199 @@
     </x:row>
     <x:row r="22" ht="72" hidden="0" customHeight="1">
       <x:c r="A22" s="20" t="str">
-        <x:v>EUVIP</x:v>
+        <x:v>CoRL</x:v>
       </x:c>
       <x:c r="B22" s="20" t="str">
-        <x:v>Multimedia Learning &amp; Retrieval; Computer Graphics &amp; Visualization; Biometrics &amp; Human Sensing; Robustness &amp; Safety</x:v>
+        <x:v>Computer Vision &amp; Pattern Recognition; Probabilistic, Causal &amp; Uncertainty ML; Human-AI Interaction &amp; Deployment; Robustness &amp; Safety; Learning Theory &amp; Statistical Foundations</x:v>
       </x:c>
       <x:c r="C22" s="20" t="str">
-        <x:v>Visual information processing across image, video, 3D, and unconventional sensing modalities. Its defining areas are computational imaging, restoration and enhancement, coding, recognition, multimodal fusion, and subjective/objective quality assessment. Rendering and visualizing data, human/biometric analysis, and robust evaluation are recurring strands. An extensive applications list is not treated as equal coverage of every application domain or every responsible-AI subtopic.</x:v>
+        <x:v>Machine learning for physical robots, especially imitation and reinforcement learning, learned perception and control, robot foundation models, and learning-based task and motion planning. Includes uncertainty, generalization, safety, human-robot interaction, and datasets grounded in manipulation, navigation, or locomotion. General ML is relevant when it makes a substantive contribution to robot learning.</x:v>
       </x:c>
       <x:c r="D22" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E22" s="20" t="str">
-        <x:v>https://euvip2026.github.io/C4P.pdf; https://euvip2026.github.io/calls/</x:v>
+        <x:v>https://www.corl.org/contributions/call-for-papers</x:v>
       </x:c>
       <x:c r="F22" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="84" hidden="0" customHeight="1">
+    <x:row r="23" ht="72" hidden="0" customHeight="1">
       <x:c r="A23" s="20" t="str">
-        <x:v>FG</x:v>
+        <x:v>CVPR</x:v>
       </x:c>
       <x:c r="B23" s="20" t="str">
-        <x:v>Robustness &amp; Safety; Fairness &amp; Responsible AI; Computer Graphics &amp; Visualization; Explainability &amp; Interpretability</x:v>
+        <x:v>Computer Graphics &amp; Visualization; Multimedia Learning &amp; Retrieval; Natural Language Processing &amp; LLMs; Biometrics &amp; Human Sensing; Robustness &amp; Safety</x:v>
       </x:c>
       <x:c r="C23" s="20" t="str">
-        <x:v>Face, gesture, body movement, and human behavior from images and video, including detection, tracking, recognition, facial expression and affect, pose and action analysis, and soft biometrics. Characteristic methods include advanced visual learning, generative modeling and neural rendering, multimodal fusion, and evaluation across demographic and acquisition conditions. Bias, interpretability, and robust recognition are directly tied to human sensing rather than generic application tags.</x:v>
+        <x:v>Broad computer vision and pattern recognition: visual representations, recognition and segmentation, 3D reconstruction, computational imaging, image and video generation, motion and tracking, and vision-language learning. Graphics, multimodal learning, human face/body understanding, and reliable vision are substantial recurring research areas. Peripheral application fields are not tagged merely because a long CFP mentions them.</x:v>
       </x:c>
       <x:c r="D23" s="21" t="n">
         <x:v>2027</x:v>
       </x:c>
       <x:c r="E23" s="20" t="str">
-        <x:v>https://fg2027.ieee-biometrics.org/call-for-papers/</x:v>
+        <x:v>https://cvpr.thecvf.com/Conferences/2027/CallForPapers</x:v>
       </x:c>
       <x:c r="F23" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="60" hidden="0" customHeight="1">
+    <x:row r="24" ht="72" hidden="0" customHeight="1">
       <x:c r="A24" s="20" t="str">
-        <x:v>FMTS @ NeurIPS</x:v>
+        <x:v>EACL</x:v>
       </x:c>
       <x:c r="B24" s="20" t="str">
-        <x:v>System Identification &amp; Data-driven Dynamics; Robustness &amp; Safety</x:v>
+        <x:v>Explainability &amp; Interpretability; Fairness &amp; Responsible AI; Cognitive Science &amp; Computational Cognition</x:v>
       </x:c>
       <x:c r="C24" s="20" t="str">
-        <x:v>Foundation models for temporal systems, centered on long-horizon and probabilistic forecasting, temporal pretraining, generative simulation, irregularly sampled and multimodal sequences, and state-space architectures. Reliability is a defining theme: distribution shift, calibrated uncertainty, leakage-aware benchmarks, and consistency of simulated trajectories.</x:v>
+        <x:v>Computational linguistics and natural language processing, including language modeling, multilingual processing, translation, dialogue, information extraction, semantics, and linguistic analysis. Human-centered evaluation, interpretability, and bias are relevant within language research. The reviewed 2027 theme strengthens connections to psycholinguistics and cognitive modeling; peripheral application domains are not extra tags.</x:v>
       </x:c>
       <x:c r="D24" s="21" t="n">
-        <x:v>2026</x:v>
+        <x:v>2027</x:v>
       </x:c>
       <x:c r="E24" s="20" t="str">
-        <x:v>https://fmts-workshop.github.io/cfp.html</x:v>
+        <x:v>https://2027.eacl.org/calls/papers/</x:v>
       </x:c>
       <x:c r="F24" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="60" hidden="0" customHeight="1">
+    <x:row r="25" ht="72" hidden="0" customHeight="1">
       <x:c r="A25" s="20" t="str">
-        <x:v>GECCO</x:v>
+        <x:v>ECCV</x:v>
       </x:c>
       <x:c r="B25" s="20" t="str">
-        <x:v>Deep Representation Learning; Learning Theory &amp; Statistical Foundations</x:v>
+        <x:v>Computer Graphics &amp; Visualization; Multimedia Learning &amp; Retrieval; Natural Language Processing &amp; LLMs; Biometrics &amp; Human Sensing; Robustness &amp; Safety</x:v>
       </x:c>
       <x:c r="C25" s="20" t="str">
-        <x:v>Genetic and evolutionary computation, including genetic algorithms, genetic programming, swarm intelligence, evolutionary multiobjective and combinatorial optimization, metaheuristics, and neuroevolution. Machine learning is relevant through evolutionary learning and optimization, not as an unrestricted substitute for the conference's evolutionary-computation focus.</x:v>
+        <x:v>Broad research in visual perception, representation learning, recognition, segmentation, 3D geometry and reconstruction, computational imaging, and image/video synthesis. Vision-language models, multimodal understanding, human motion and appearance, and robust visual systems extend this core. ECCV is the biennial European flagship for computer vision; the scope uses the actual published 2026 CFP, not an invented 2028 call.</x:v>
       </x:c>
       <x:c r="D25" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E25" s="20" t="str">
-        <x:v>https://gecco-2027.sigevo.org/Call+for+Papers</x:v>
+        <x:v>https://eccv.ecva.net/Conferences/2026/CallForPapers</x:v>
       </x:c>
       <x:c r="F25" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="72" hidden="0" customHeight="1">
+    <x:row r="26" ht="60" hidden="0" customHeight="1">
       <x:c r="A26" s="20" t="str">
-        <x:v>ICAPS</x:v>
+        <x:v>ECIR</x:v>
       </x:c>
       <x:c r="B26" s="20" t="str">
-        <x:v>Probabilistic, Causal &amp; Uncertainty ML</x:v>
+        <x:v>Human-AI Interaction &amp; Deployment; Explainability &amp; Interpretability; Fairness &amp; Responsible AI; Multimedia Learning &amp; Retrieval</x:v>
       </x:c>
       <x:c r="C26" s="20" t="str">
-        <x:v>Automated planning and scheduling, heuristic search, constraint-based reasoning, temporal and hierarchical planning, and planning under uncertainty. Learning and foundation models fit when they substantially advance planning or scheduling, including model acquisition and search guidance. The main CFP explicitly excludes reinforcement-learning papers without a substantive planning contribution; general reward-based learning is not a blanket tag.</x:v>
+        <x:v>Information retrieval and ranking, recommendation, conversational search and RAG, user information interaction, system efficiency, and rigorous evaluation. The 2027 call explicitly includes language models and agentic retrieval workflows. Replicability and research-resource papers are distinct routes. Fairness and explainability concern information access rather than generic responsible-AI topics.</x:v>
       </x:c>
       <x:c r="D26" s="21" t="n">
         <x:v>2027</x:v>
       </x:c>
       <x:c r="E26" s="20" t="str">
-        <x:v>https://icaps27.icaps-conference.org/calls/cfp/</x:v>
+        <x:v>https://www.ecir2027.co.uk/call-for-full-papers</x:v>
       </x:c>
       <x:c r="F26" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="72" hidden="0" customHeight="1">
+    <x:row r="27" ht="60" hidden="0" customHeight="1">
       <x:c r="A27" s="20" t="str">
-        <x:v>ICCV</x:v>
+        <x:v>EMNLP</x:v>
       </x:c>
       <x:c r="B27" s="20" t="str">
-        <x:v>Computer Graphics &amp; Visualization; Multimedia Learning &amp; Retrieval; Natural Language Processing &amp; LLMs; Biometrics &amp; Human Sensing; Robustness &amp; Safety</x:v>
+        <x:v>Explainability &amp; Interpretability; Fairness &amp; Responsible AI; Robustness &amp; Safety; Human-AI Interaction &amp; Deployment</x:v>
       </x:c>
       <x:c r="C27" s="20" t="str">
-        <x:v>Broad computer vision, from geometry and computational imaging to visual learning, recognition, segmentation, generation, and video understanding. Vision-language and multimodal methods, visual graphics, face/body/gesture analysis, and reliable perception are substantial strands. It is a biennial flagship, not a general AI applications conference. The current scope is grounded in its 2025 CFP because the 2027 call is not yet published.</x:v>
+        <x:v>Empirical methods for language modeling and NLP, including generation, information extraction, multilinguality, dialogue, retrieval, and model evaluation. Interpretability, bias, and safety matter within language systems. Curated coverage emphasizes language methods and evidence rather than every application listed in the CFP.</x:v>
       </x:c>
       <x:c r="D27" s="21" t="n">
-        <x:v>2025</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="E27" s="20" t="str">
-        <x:v>https://iccv.thecvf.com/Conferences/2025/CallForPapers</x:v>
+        <x:v>https://2026.emnlp.org/calls/main_conference_papers/</x:v>
       </x:c>
       <x:c r="F27" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="72" hidden="0" customHeight="1">
+    <x:row r="28" ht="60" hidden="0" customHeight="1">
       <x:c r="A28" s="20" t="str">
-        <x:v>ICIP</x:v>
-      </x:c>
-      <x:c r="B28" s="20" t="str"/>
+        <x:v>EuroGP</x:v>
+      </x:c>
+      <x:c r="B28" s="20" t="str">
+        <x:v>Learning Theory &amp; Statistical Foundations; Deep Representation Learning</x:v>
+      </x:c>
       <x:c r="C28" s="20" t="str">
-        <x:v>Image and video processing across theory, algorithms, and imaging systems. Characteristic problems include restoration, enhancement, reconstruction, registration, compression, quality assessment, and visual analysis. Learning methods and generative models are relevant when they advance image or video processing. The long list of imaging application domains is intentionally not converted into extra specialist-conference tags.</x:v>
+        <x:v>Genetic programming and evolutionary program synthesis, including symbolic regression, program representations and operators, surrogate-assisted search, multi-objective evolution, and interpretable learned programs. Evolutionary machine learning, AutoML pipelines, and neuroevolution connect this focused methodological community to ML. Application domains do not define its tags.</x:v>
       </x:c>
       <x:c r="D28" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E28" s="20" t="str">
+        <x:v>https://www.evostar.org/2027/eurogp/</x:v>
+      </x:c>
+      <x:c r="F28" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="72" hidden="0" customHeight="1">
+      <x:c r="A29" s="20" t="str">
+        <x:v>EUVIP</x:v>
+      </x:c>
+      <x:c r="B29" s="20" t="str">
+        <x:v>Multimedia Learning &amp; Retrieval; Computer Graphics &amp; Visualization; Biometrics &amp; Human Sensing; Robustness &amp; Safety</x:v>
+      </x:c>
+      <x:c r="C29" s="20" t="str">
+        <x:v>Visual information processing across image, video, 3D, and unconventional sensing modalities. Its defining areas are computational imaging, restoration and enhancement, coding, recognition, multimodal fusion, and subjective/objective quality assessment. Rendering and visualizing data, human/biometric analysis, and robust evaluation are recurring strands. An extensive applications list is not treated as equal coverage of every application domain or every responsible-AI subtopic.</x:v>
+      </x:c>
+      <x:c r="D29" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
-      <x:c r="E28" s="20" t="str">
-        <x:v>https://2026.ieeeicip.org/topics/</x:v>
-      </x:c>
-      <x:c r="F28" s="22" t="n">
-        <x:v>46302</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="60" hidden="0" customHeight="1">
-      <x:c r="A29" s="20" t="str">
-        <x:v>ICLR</x:v>
-      </x:c>
-      <x:c r="B29" s="20" t="str">
-        <x:v>Learning Theory &amp; Statistical Foundations; Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Natural Language Processing &amp; LLMs; Computer Vision &amp; Pattern Recognition; ML Systems &amp; Infrastructure</x:v>
-      </x:c>
-      <x:c r="C29" s="20" t="str">
-        <x:v>Learning representations and understanding deep learning, with an emphasis on self-supervised learning, generative models, transfer and meta-learning, and the optimization and theory of learned representations. Language, vision, probabilistic modeling, and reinforcement learning are substantial areas, rather than unrelated application-domain tags.</x:v>
-      </x:c>
-      <x:c r="D29" s="21" t="n">
+      <x:c r="E29" s="20" t="str">
+        <x:v>https://euvip2026.github.io/C4P.pdf; https://euvip2026.github.io/calls/</x:v>
+      </x:c>
+      <x:c r="F29" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="84" hidden="0" customHeight="1">
+      <x:c r="A30" s="20" t="str">
+        <x:v>FG</x:v>
+      </x:c>
+      <x:c r="B30" s="20" t="str">
+        <x:v>Robustness &amp; Safety; Fairness &amp; Responsible AI; Computer Graphics &amp; Visualization; Explainability &amp; Interpretability</x:v>
+      </x:c>
+      <x:c r="C30" s="20" t="str">
+        <x:v>Face, gesture, body movement, and human behavior from images and video, including detection, tracking, recognition, facial expression and affect, pose and action analysis, and soft biometrics. Characteristic methods include advanced visual learning, generative modeling and neural rendering, multimodal fusion, and evaluation across demographic and acquisition conditions. Bias, interpretability, and robust recognition are directly tied to human sensing rather than generic application tags.</x:v>
+      </x:c>
+      <x:c r="D30" s="21" t="n">
         <x:v>2027</x:v>
       </x:c>
-      <x:c r="E29" s="20" t="str">
-        <x:v>https://iclr.cc/Conferences/2027/CallForPapers</x:v>
-      </x:c>
-      <x:c r="F29" s="22" t="n">
-        <x:v>46302</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" ht="60" hidden="0" customHeight="1">
-      <x:c r="A30" s="20" t="str">
-        <x:v>ICML</x:v>
-      </x:c>
-      <x:c r="B30" s="20" t="str">
-        <x:v>Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Explainability &amp; Interpretability; Robustness &amp; Safety; ML Systems &amp; Infrastructure; Federated &amp; Distributed Learning</x:v>
-      </x:c>
-      <x:c r="C30" s="20" t="str">
-        <x:v>Methodological and theoretical machine learning, including supervised and unsupervised learning, deep generative models, optimization, statistical learning theory, Bayesian methods, and reinforcement learning. Scalable systems and trustworthy learning are established parts of the scope; application papers should offer contributions of wider interest to ML.</x:v>
-      </x:c>
-      <x:c r="D30" s="21" t="n">
+      <x:c r="E30" s="20" t="str">
+        <x:v>https://fg2027.ieee-biometrics.org/call-for-papers/</x:v>
+      </x:c>
+      <x:c r="F30" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="60" hidden="0" customHeight="1">
+      <x:c r="A31" s="20" t="str">
+        <x:v>FMTS @ NeurIPS</x:v>
+      </x:c>
+      <x:c r="B31" s="20" t="str">
+        <x:v>System Identification &amp; Data-driven Dynamics; Robustness &amp; Safety</x:v>
+      </x:c>
+      <x:c r="C31" s="20" t="str">
+        <x:v>Foundation models for temporal systems, centered on long-horizon and probabilistic forecasting, temporal pretraining, generative simulation, irregularly sampled and multimodal sequences, and state-space architectures. Reliability is a defining theme: distribution shift, calibrated uncertainty, leakage-aware benchmarks, and consistency of simulated trajectories.</x:v>
+      </x:c>
+      <x:c r="D31" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
-      <x:c r="E30" s="20" t="str">
-        <x:v>https://icml.cc/Conferences/2026/CallForPapers</x:v>
-      </x:c>
-      <x:c r="F30" s="22" t="n">
-        <x:v>46302</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="72" hidden="0" customHeight="1">
-      <x:c r="A31" s="20" t="str">
-        <x:v>ICMR</x:v>
-      </x:c>
-      <x:c r="B31" s="20" t="str">
-        <x:v>Data Mining &amp; Data Science; Natural Language Processing &amp; LLMs; Privacy-preserving ML</x:v>
-      </x:c>
-      <x:c r="C31" s="20" t="str">
-        <x:v>Search and retrieval of multimedia and multimodal content. Characteristic work studies indexing, content understanding, query representations, cross-modal matching, relevance feedback, recommendation, and evaluation, with deep learning and multimodal models as important methods. Privacy-aware retrieval and knowledge discovery extend this core. The long applications list is not used to characterize ICMR as a medicine, finance, or travel venue.</x:v>
-      </x:c>
-      <x:c r="D31" s="21" t="n">
-        <x:v>2027</x:v>
-      </x:c>
       <x:c r="E31" s="20" t="str">
-        <x:v>https://www.icmr2027.org/cfc</x:v>
+        <x:v>https://fmts-workshop.github.io/cfp.html</x:v>
       </x:c>
       <x:c r="F31" s="22" t="n">
         <x:v>46302</x:v>
@@ -4643,97 +5269,97 @@
     </x:row>
     <x:row r="32" ht="60" hidden="0" customHeight="1">
       <x:c r="A32" s="20" t="str">
-        <x:v>IFAC SYSID</x:v>
+        <x:v>GECCO</x:v>
       </x:c>
       <x:c r="B32" s="20" t="str">
-        <x:v>Nonlinear Dynamics &amp; Chaos; Complex Systems &amp; Network Science</x:v>
+        <x:v>Deep Representation Learning; Learning Theory &amp; Statistical Foundations</x:v>
       </x:c>
       <x:c r="C32" s="20" t="str">
-        <x:v>System identification and data-driven modeling for dynamical systems and control. Characteristic themes include nonlinear identification, model reduction, identification software and benchmarks, learning across systems, and dynamic networks. Application tracks remain grounded in identifying or learning dynamical models, rather than becoming general-purpose domain conferences.</x:v>
+        <x:v>Genetic and evolutionary computation, including genetic algorithms, genetic programming, swarm intelligence, evolutionary multiobjective and combinatorial optimization, metaheuristics, and neuroevolution. Machine learning is relevant through evolutionary learning and optimization, not as an unrestricted substitute for the conference's evolutionary-computation focus.</x:v>
       </x:c>
       <x:c r="D32" s="21" t="n">
-        <x:v>2027</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="E32" s="20" t="str">
-        <x:v>https://conferences.ifac-control.org/sysid2027/participate/</x:v>
+        <x:v>https://gecco-2027.sigevo.org/Call+for+Papers</x:v>
       </x:c>
       <x:c r="F32" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="84" hidden="0" customHeight="1">
+    <x:row r="33" ht="72" hidden="0" customHeight="1">
       <x:c r="A33" s="20" t="str">
-        <x:v>IJCB</x:v>
+        <x:v>ICAPS</x:v>
       </x:c>
       <x:c r="B33" s="20" t="str">
-        <x:v>Machine Learning; Robustness &amp; Safety; Fairness &amp; Responsible AI; Explainability &amp; Interpretability; Federated &amp; Distributed Learning; Signal Processing</x:v>
+        <x:v>Probabilistic, Causal &amp; Uncertainty ML</x:v>
       </x:c>
       <x:c r="C33" s="20" t="str">
-        <x:v>Biometrics and identity science across face, fingerprint, iris, voice, gait, and behavioral modalities. Defining concerns include recognition and verification, multimodal fusion, presentation-attack and deepfake detection, biometric template security, privacy, demographic fairness, and rigorous benchmarking. Learned representations and foundation models are important methods; federated learning belongs here through secure biometric systems. Healthcare, banking, and robotics are applications, not blanket scope tags.</x:v>
+        <x:v>Automated planning and scheduling, heuristic search, constraint-based reasoning, temporal and hierarchical planning, and planning under uncertainty. Learning and foundation models fit when they substantially advance planning or scheduling, including model acquisition and search guidance. The main CFP explicitly excludes reinforcement-learning papers without a substantive planning contribution; general reward-based learning is not a blanket tag.</x:v>
       </x:c>
       <x:c r="D33" s="21" t="n">
         <x:v>2027</x:v>
       </x:c>
       <x:c r="E33" s="20" t="str">
-        <x:v>https://ijcb2027.ieee-biometrics.org/call-for-papers/</x:v>
+        <x:v>https://icaps27.icaps-conference.org/calls/cfp/</x:v>
       </x:c>
       <x:c r="F33" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="34" ht="60" hidden="0" customHeight="1">
+    <x:row r="34" ht="72" hidden="0" customHeight="1">
       <x:c r="A34" s="20" t="str">
-        <x:v>Interspeech</x:v>
-      </x:c>
-      <x:c r="B34" s="20" t="str"/>
+        <x:v>ICCV</x:v>
+      </x:c>
+      <x:c r="B34" s="20" t="str">
+        <x:v>Computer Graphics &amp; Visualization; Multimedia Learning &amp; Retrieval; Natural Language Processing &amp; LLMs; Biometrics &amp; Human Sensing; Robustness &amp; Safety</x:v>
+      </x:c>
       <x:c r="C34" s="20" t="str">
-        <x:v>Speech science and speech technology, linking spoken-language research with computational methods for speech recognition, speech synthesis, and speech communication. Machine learning and language models are relevant through speech and spoken-language problems. The current 2027 overview emphasizes the relationship between speech research and spoken-language technologies.</x:v>
+        <x:v>Broad computer vision, from geometry and computational imaging to visual learning, recognition, segmentation, generation, and video understanding. Vision-language and multimodal methods, visual graphics, face/body/gesture analysis, and reliable perception are substantial strands. It is a biennial flagship, not a general AI applications conference. The current scope is grounded in its 2025 CFP because the 2027 call is not yet published.</x:v>
       </x:c>
       <x:c r="D34" s="21" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="E34" s="20" t="str">
+        <x:v>https://iccv.thecvf.com/Conferences/2025/CallForPapers</x:v>
+      </x:c>
+      <x:c r="F34" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="72" hidden="0" customHeight="1">
+      <x:c r="A35" s="20" t="str">
+        <x:v>ICIP</x:v>
+      </x:c>
+      <x:c r="B35" s="20" t="str"/>
+      <x:c r="C35" s="20" t="str">
+        <x:v>Image and video processing across theory, algorithms, and imaging systems. Characteristic problems include restoration, enhancement, reconstruction, registration, compression, quality assessment, and visual analysis. Learning methods and generative models are relevant when they advance image or video processing. The long list of imaging application domains is intentionally not converted into extra specialist-conference tags.</x:v>
+      </x:c>
+      <x:c r="D35" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E35" s="20" t="str">
+        <x:v>https://2026.ieeeicip.org/topics/</x:v>
+      </x:c>
+      <x:c r="F35" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="60" hidden="0" customHeight="1">
+      <x:c r="A36" s="20" t="str">
+        <x:v>ICLR</x:v>
+      </x:c>
+      <x:c r="B36" s="20" t="str">
+        <x:v>Learning Theory &amp; Statistical Foundations; Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Natural Language Processing &amp; LLMs; Computer Vision &amp; Pattern Recognition; ML Systems &amp; Infrastructure</x:v>
+      </x:c>
+      <x:c r="C36" s="20" t="str">
+        <x:v>Learning representations and understanding deep learning, with an emphasis on self-supervised learning, generative models, transfer and meta-learning, and the optimization and theory of learned representations. Language, vision, probabilistic modeling, and reinforcement learning are substantial areas, rather than unrelated application-domain tags.</x:v>
+      </x:c>
+      <x:c r="D36" s="21" t="n">
         <x:v>2027</x:v>
       </x:c>
-      <x:c r="E34" s="20" t="str">
-        <x:v>https://interspeech2027.org/</x:v>
-      </x:c>
-      <x:c r="F34" s="22" t="n">
-        <x:v>46302</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35" ht="60" hidden="0" customHeight="1">
-      <x:c r="A35" s="20" t="str">
-        <x:v>KDD</x:v>
-      </x:c>
-      <x:c r="B35" s="20" t="str">
-        <x:v>Deep Representation Learning; Natural Language Processing &amp; LLMs; Explainability &amp; Interpretability; Privacy-preserving ML; ML Systems &amp; Infrastructure</x:v>
-      </x:c>
-      <x:c r="C35" s="20" t="str">
-        <x:v>Knowledge discovery and data science, centered on extracting useful structure from large, heterogeneous data. Characteristic areas include clustering, structured and relational learning, graph and text mining, recommender systems, scalable data analysis, and responsible data use. Generative AI is relevant when it advances data science, not simply because a paper uses an LLM.</x:v>
-      </x:c>
-      <x:c r="D35" s="21" t="n">
-        <x:v>2027</x:v>
-      </x:c>
-      <x:c r="E35" s="20" t="str">
-        <x:v>https://kdd2027.kdd.org/research-track-call-for-papers/</x:v>
-      </x:c>
-      <x:c r="F35" s="22" t="n">
-        <x:v>46302</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36" ht="84" hidden="0" customHeight="1">
-      <x:c r="A36" s="20" t="str">
-        <x:v>KR</x:v>
-      </x:c>
-      <x:c r="B36" s="20" t="str">
-        <x:v>Machine Learning; Probabilistic, Causal &amp; Uncertainty ML; Planning &amp; Search</x:v>
-      </x:c>
-      <x:c r="C36" s="20" t="str">
-        <x:v>Formal and symbolic AI centered on representing knowledge and drawing justified conclusions: knowledge bases, description and non-classical logics, ontologies, non-monotonic reasoning, argumentation, belief revision, and reasoning about actions. Learning, uncertainty, and explanations matter when grounded in knowledge representation or reasoning. The last published CFP includes a KR Meets Machine Learning and Explanation track; this is not a general-purpose ML conference or a confirmed promise of that 2027 track.</x:v>
-      </x:c>
-      <x:c r="D36" s="21" t="n">
-        <x:v>2026</x:v>
-      </x:c>
       <x:c r="E36" s="20" t="str">
-        <x:v>https://kr.org/KR2026/call_main_track.html; https://kr.org/KR2026/</x:v>
+        <x:v>https://iclr.cc/Conferences/2027/CallForPapers</x:v>
       </x:c>
       <x:c r="F36" s="22" t="n">
         <x:v>46302</x:v>
@@ -4741,19 +5367,19 @@
     </x:row>
     <x:row r="37" ht="60" hidden="0" customHeight="1">
       <x:c r="A37" s="20" t="str">
-        <x:v>L4DC</x:v>
+        <x:v>ICML</x:v>
       </x:c>
       <x:c r="B37" s="20" t="str">
-        <x:v>Learning Theory &amp; Statistical Foundations</x:v>
+        <x:v>Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Explainability &amp; Interpretability; Robustness &amp; Safety; ML Systems &amp; Infrastructure; Federated &amp; Distributed Learning</x:v>
       </x:c>
       <x:c r="C37" s="20" t="str">
-        <x:v>The interface of learning, dynamics, control, and optimization for physical and dynamical systems. Emphasizes foundations and methods for data-driven control and dynamical modeling, including theoretical, empirical, and applied contributions. Pure pattern recognition without a meaningful connection to dynamics or control is not the defining focus.</x:v>
+        <x:v>Methodological and theoretical machine learning, including supervised and unsupervised learning, deep generative models, optimization, statistical learning theory, Bayesian methods, and reinforcement learning. Scalable systems and trustworthy learning are established parts of the scope; application papers should offer contributions of wider interest to ML.</x:v>
       </x:c>
       <x:c r="D37" s="21" t="n">
-        <x:v>2027</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="E37" s="20" t="str">
-        <x:v>https://l4dc2027.control.ee.ethz.ch/home</x:v>
+        <x:v>https://icml.cc/Conferences/2026/CallForPapers</x:v>
       </x:c>
       <x:c r="F37" s="22" t="n">
         <x:v>46302</x:v>
@@ -4761,19 +5387,19 @@
     </x:row>
     <x:row r="38" ht="72" hidden="0" customHeight="1">
       <x:c r="A38" s="20" t="str">
-        <x:v>LoG</x:v>
+        <x:v>ICMR</x:v>
       </x:c>
       <x:c r="B38" s="20" t="str">
-        <x:v>Probabilistic, Causal &amp; Uncertainty ML; Signal Processing; Robustness &amp; Safety; ML Systems &amp; Infrastructure</x:v>
+        <x:v>Data Mining &amp; Data Science; Natural Language Processing &amp; LLMs; Privacy-preserving ML</x:v>
       </x:c>
       <x:c r="C38" s="20" t="str">
-        <x:v>Learning on graphs and geometry: graph neural networks, equivariant models, graph kernels, geometric and graph generative models, and statistical theory for structured data. Graph signal processing, causal graph models, robustness, and scalable graph-learning infrastructure are meaningful extensions. A graph or geometric contribution should remain central, even in an application such as language or molecular modeling.</x:v>
+        <x:v>Search and retrieval of multimedia and multimodal content. Characteristic work studies indexing, content understanding, query representations, cross-modal matching, relevance feedback, recommendation, and evaluation, with deep learning and multimodal models as important methods. Privacy-aware retrieval and knowledge discovery extend this core. The long applications list is not used to characterize ICMR as a medicine, finance, or travel venue.</x:v>
       </x:c>
       <x:c r="D38" s="21" t="n">
-        <x:v>2026</x:v>
+        <x:v>2027</x:v>
       </x:c>
       <x:c r="E38" s="20" t="str">
-        <x:v>https://logconference.org/cfp/</x:v>
+        <x:v>https://www.icmr2027.org/cfc</x:v>
       </x:c>
       <x:c r="F38" s="22" t="n">
         <x:v>46302</x:v>
@@ -4781,19 +5407,19 @@
     </x:row>
     <x:row r="39" ht="60" hidden="0" customHeight="1">
       <x:c r="A39" s="20" t="str">
-        <x:v>MIDL</x:v>
+        <x:v>ICRA</x:v>
       </x:c>
       <x:c r="B39" s="20" t="str">
-        <x:v>Computer Vision &amp; Pattern Recognition; Probabilistic, Causal &amp; Uncertainty ML; Explainability &amp; Interpretability; Robustness &amp; Safety; Federated &amp; Distributed Learning</x:v>
+        <x:v>Planning &amp; Search; Deep Representation Learning; Human-AI Interaction &amp; Deployment; Robustness &amp; Safety</x:v>
       </x:c>
       <x:c r="C39" s="20" t="str">
-        <x:v>Deep learning for biomedical image analysis, especially segmentation, detection, reconstruction, registration, generative imaging, and learning from limited labels. Uncertainty, interpretability, multi-site learning, robustness, and clinical validation extend that imaging core. Multimodal foundation models are relevant when grounded in medical imaging.</x:v>
+        <x:v>Robotics and automation across perception, motion and manipulation, planning and control, human-robot interaction, and autonomous systems. Learning-based robotics, reinforcement and imitation learning, and data-driven models are relevant when they advance physical robotic capability. Generic ML with no robotics connection is not the core remit.</x:v>
       </x:c>
       <x:c r="D39" s="21" t="n">
-        <x:v>2026</x:v>
+        <x:v>2027</x:v>
       </x:c>
       <x:c r="E39" s="20" t="str">
-        <x:v>https://2026.midl.io/call-for-papers</x:v>
+        <x:v>https://2027.ieee-icra.org/contribute/call-for-icra-2027-papers-now-accepting-submissions/</x:v>
       </x:c>
       <x:c r="F39" s="22" t="n">
         <x:v>46302</x:v>
@@ -4801,39 +5427,39 @@
     </x:row>
     <x:row r="40" ht="60" hidden="0" customHeight="1">
       <x:c r="A40" s="20" t="str">
-        <x:v>MLSys</x:v>
+        <x:v>IFAC SYSID</x:v>
       </x:c>
       <x:c r="B40" s="20" t="str">
-        <x:v>Reinforcement Learning; Privacy-preserving ML</x:v>
+        <x:v>Nonlinear Dynamics &amp; Chaos; Complex Systems &amp; Network Science</x:v>
       </x:c>
       <x:c r="C40" s="20" t="str">
-        <x:v>The intersection of machine learning and computer systems, including efficient training, inference and serving, compilers and runtimes, programming abstractions, specialized hardware, distributed learning, and system monitoring. LLM and agentic workloads are considered from a systems perspective. Both systems for ML and ML methods that improve computing systems are relevant.</x:v>
+        <x:v>System identification and data-driven modeling for dynamical systems and control. Characteristic themes include nonlinear identification, model reduction, identification software and benchmarks, learning across systems, and dynamic networks. Application tracks remain grounded in identifying or learning dynamical models, rather than becoming general-purpose domain conferences.</x:v>
       </x:c>
       <x:c r="D40" s="21" t="n">
         <x:v>2027</x:v>
       </x:c>
       <x:c r="E40" s="20" t="str">
-        <x:v>https://mlsys.org/Conferences/2027/CallForResearchPapers</x:v>
+        <x:v>https://conferences.ifac-control.org/sysid2027/participate/</x:v>
       </x:c>
       <x:c r="F40" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="41" ht="60" hidden="0" customHeight="1">
+    <x:row r="41" ht="84" hidden="0" customHeight="1">
       <x:c r="A41" s="20" t="str">
-        <x:v>NeurIPS</x:v>
+        <x:v>IJCB</x:v>
       </x:c>
       <x:c r="B41" s="20" t="str">
-        <x:v>Learning Theory &amp; Statistical Foundations; Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Natural Language Processing &amp; LLMs; Computer Vision &amp; Pattern Recognition; ML Systems &amp; Infrastructure</x:v>
+        <x:v>Machine Learning; Robustness &amp; Safety; Fairness &amp; Responsible AI; Explainability &amp; Interpretability; Federated &amp; Distributed Learning; Signal Processing</x:v>
       </x:c>
       <x:c r="C41" s="20" t="str">
-        <x:v>Broad research in machine learning, especially deep and generative models, statistical foundations, optimization, probabilistic inference, and learning for decision-making. Language, vision, and scalable ML systems are important research communities. Interdisciplinary applications should contribute insight of wider interest to the machine-learning community.</x:v>
+        <x:v>Biometrics and identity science across face, fingerprint, iris, voice, gait, and behavioral modalities. Defining concerns include recognition and verification, multimodal fusion, presentation-attack and deepfake detection, biometric template security, privacy, demographic fairness, and rigorous benchmarking. Learned representations and foundation models are important methods; federated learning belongs here through secure biometric systems. Healthcare, banking, and robotics are applications, not blanket scope tags.</x:v>
       </x:c>
       <x:c r="D41" s="21" t="n">
-        <x:v>2026</x:v>
+        <x:v>2027</x:v>
       </x:c>
       <x:c r="E41" s="20" t="str">
-        <x:v>https://neurips.cc/Conferences/2026/CallForPapers</x:v>
+        <x:v>https://ijcb2027.ieee-biometrics.org/call-for-papers/</x:v>
       </x:c>
       <x:c r="F41" s="22" t="n">
         <x:v>46302</x:v>
@@ -4841,39 +5467,37 @@
     </x:row>
     <x:row r="42" ht="60" hidden="0" customHeight="1">
       <x:c r="A42" s="20" t="str">
-        <x:v>NOLTA</x:v>
+        <x:v>IJCNLP</x:v>
       </x:c>
       <x:c r="B42" s="20" t="str">
-        <x:v>Signal Processing; Evolutionary Computation &amp; Optimization</x:v>
+        <x:v>Cognitive Science &amp; Computational Cognition; Explainability &amp; Interpretability; Fairness &amp; Responsible AI; Human-AI Interaction &amp; Deployment</x:v>
       </x:c>
       <x:c r="C42" s="20" t="str">
-        <x:v>Nonlinear theory and its applications, centered on chaos, bifurcations, oscillations, synchronization, nonlinear circuits, and complex networks. Neural computation, evolutionary algorithms, control, and signal processing connect to this nonlinear-systems focus. Individual application examples are not taken as additional specialist identities.</x:v>
+        <x:v>Computational linguistics and natural-language technologies in the Asia-Pacific community, including multilingual and low-resource NLP, language modeling, generation, dialogue, structured prediction, and evaluation. The 2026 edition is jointly organized as AACL-IJCNLP. Alias identity is preserved without inheriting the separate ACL conference ranking.</x:v>
       </x:c>
       <x:c r="D42" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E42" s="20" t="str">
-        <x:v>https://nolta2026.org/</x:v>
+        <x:v>https://2026.aaclnet.org/calls/main_conference_papers/</x:v>
       </x:c>
       <x:c r="F42" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="43" ht="72" hidden="0" customHeight="1">
+    <x:row r="43" ht="60" hidden="0" customHeight="1">
       <x:c r="A43" s="20" t="str">
-        <x:v>ProbML</x:v>
-      </x:c>
-      <x:c r="B43" s="20" t="str">
-        <x:v>Deep Representation Learning; Reinforcement Learning; Time Series &amp; Sequential Data; Robustness &amp; Safety</x:v>
-      </x:c>
+        <x:v>Interspeech</x:v>
+      </x:c>
+      <x:c r="B43" s="20" t="str"/>
       <x:c r="C43" s="20" t="str">
-        <x:v>Probabilistic and Bayesian machine learning, emphasizing approximate inference, variational and Monte Carlo methods, Gaussian processes, graphical and state-space models, calibration, and decisions under uncertainty. Includes Bayesian optimization and uncertainty-aware deep learning. The reviewed 2026 application focus is healthcare and climate; probabilistic reasoning remains essential to a suitable contribution.</x:v>
+        <x:v>Speech science and speech technology, linking spoken-language research with computational methods for speech recognition, speech synthesis, and speech communication. Machine learning and language models are relevant through speech and spoken-language problems. The current 2027 overview emphasizes the relationship between speech research and spoken-language technologies.</x:v>
       </x:c>
       <x:c r="D43" s="21" t="n">
-        <x:v>2026</x:v>
+        <x:v>2027</x:v>
       </x:c>
       <x:c r="E43" s="20" t="str">
-        <x:v>https://probml.cc/call/</x:v>
+        <x:v>https://interspeech2027.org/</x:v>
       </x:c>
       <x:c r="F43" s="22" t="n">
         <x:v>46302</x:v>
@@ -4881,19 +5505,19 @@
     </x:row>
     <x:row r="44" ht="60" hidden="0" customHeight="1">
       <x:c r="A44" s="20" t="str">
-        <x:v>SaTML</x:v>
+        <x:v>ISWC</x:v>
       </x:c>
       <x:c r="B44" s="20" t="str">
-        <x:v>Machine Learning; ML Systems &amp; Infrastructure</x:v>
+        <x:v>Machine Learning; Explainability &amp; Interpretability</x:v>
       </x:c>
       <x:c r="C44" s="20" t="str">
-        <x:v>Security, safety, and trustworthiness of machine learning. Characteristic work studies attacks and defenses, privacy, verification, ML-system security, fairness, interpretability, and trustworthy data curation. Theoretical, empirical, and applied papers must engage substantively with a safety or trustworthiness question; merely using an ML model is insufficient.</x:v>
+        <x:v>Semantic Web and linked-data research: ontologies, knowledge graphs, representation and reasoning, semantic integration, querying, and knowledge-supported AI. Graph learning is relevant through semantic data and knowledge structures; this is not the IEEE wearable-computing symposium with the same acronym.</x:v>
       </x:c>
       <x:c r="D44" s="21" t="n">
-        <x:v>2027</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="E44" s="20" t="str">
-        <x:v>https://satml.org/call-for-papers/</x:v>
+        <x:v>https://iswc2026.semanticweb.org/calls/research</x:v>
       </x:c>
       <x:c r="F44" s="22" t="n">
         <x:v>46302</x:v>
@@ -4901,48 +5525,408 @@
     </x:row>
     <x:row r="45" ht="60" hidden="0" customHeight="1">
       <x:c r="A45" s="20" t="str">
+        <x:v>KDD</x:v>
+      </x:c>
+      <x:c r="B45" s="20" t="str">
+        <x:v>Deep Representation Learning; Natural Language Processing &amp; LLMs; Explainability &amp; Interpretability; Privacy-preserving ML; ML Systems &amp; Infrastructure</x:v>
+      </x:c>
+      <x:c r="C45" s="20" t="str">
+        <x:v>Knowledge discovery and data science, centered on extracting useful structure from large, heterogeneous data. Characteristic areas include clustering, structured and relational learning, graph and text mining, recommender systems, scalable data analysis, and responsible data use. Generative AI is relevant when it advances data science, not simply because a paper uses an LLM.</x:v>
+      </x:c>
+      <x:c r="D45" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E45" s="20" t="str">
+        <x:v>https://kdd2027.kdd.org/research-track-call-for-papers/</x:v>
+      </x:c>
+      <x:c r="F45" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="84" hidden="0" customHeight="1">
+      <x:c r="A46" s="20" t="str">
+        <x:v>KR</x:v>
+      </x:c>
+      <x:c r="B46" s="20" t="str">
+        <x:v>Machine Learning; Probabilistic, Causal &amp; Uncertainty ML; Planning &amp; Search</x:v>
+      </x:c>
+      <x:c r="C46" s="20" t="str">
+        <x:v>Formal and symbolic AI centered on representing knowledge and drawing justified conclusions: knowledge bases, description and non-classical logics, ontologies, non-monotonic reasoning, argumentation, belief revision, and reasoning about actions. Learning, uncertainty, and explanations matter when grounded in knowledge representation or reasoning. The last published CFP includes a KR Meets Machine Learning and Explanation track; this is not a general-purpose ML conference or a confirmed promise of that 2027 track.</x:v>
+      </x:c>
+      <x:c r="D46" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E46" s="20" t="str">
+        <x:v>https://kr.org/KR2026/call_main_track.html; https://kr.org/KR2026/</x:v>
+      </x:c>
+      <x:c r="F46" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="60" hidden="0" customHeight="1">
+      <x:c r="A47" s="20" t="str">
+        <x:v>L4DC</x:v>
+      </x:c>
+      <x:c r="B47" s="20" t="str">
+        <x:v>Learning Theory &amp; Statistical Foundations</x:v>
+      </x:c>
+      <x:c r="C47" s="20" t="str">
+        <x:v>The interface of learning, dynamics, control, and optimization for physical and dynamical systems. Emphasizes foundations and methods for data-driven control and dynamical modeling, including theoretical, empirical, and applied contributions. Pure pattern recognition without a meaningful connection to dynamics or control is not the defining focus.</x:v>
+      </x:c>
+      <x:c r="D47" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E47" s="20" t="str">
+        <x:v>https://l4dc2027.control.ee.ethz.ch/home</x:v>
+      </x:c>
+      <x:c r="F47" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="72" hidden="0" customHeight="1">
+      <x:c r="A48" s="20" t="str">
+        <x:v>LoG</x:v>
+      </x:c>
+      <x:c r="B48" s="20" t="str">
+        <x:v>Complex Systems &amp; Network Science; Probabilistic, Causal &amp; Uncertainty ML; Signal Processing; Robustness &amp; Safety; ML Systems &amp; Infrastructure</x:v>
+      </x:c>
+      <x:c r="C48" s="20" t="str">
+        <x:v>Learning on graphs and geometry: graph neural networks, equivariant models, graph kernels, geometric and graph generative models, and statistical theory for structured data. Graph signal processing, causal graph models, robustness, and scalable graph-learning infrastructure are meaningful extensions. A graph or geometric contribution should remain central, even in an application such as language or molecular modeling.</x:v>
+      </x:c>
+      <x:c r="D48" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E48" s="20" t="str">
+        <x:v>https://logconference.org/cfp/</x:v>
+      </x:c>
+      <x:c r="F48" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="60" hidden="0" customHeight="1">
+      <x:c r="A49" s="20" t="str">
+        <x:v>LREC</x:v>
+      </x:c>
+      <x:c r="B49" s="20" t="str">
+        <x:v>Multimedia Learning &amp; Retrieval; Fairness &amp; Responsible AI</x:v>
+      </x:c>
+      <x:c r="C49" s="20" t="str">
+        <x:v>Language resources, annotation, corpora and datasets, speech and multimodal resources, benchmarking, and evaluation for human-language technologies. Contributions often create or analyze reusable resources and methods for linguistic coverage and reliable assessment. The breadth of language applications is summarized without treating every domain as a defining topic.</x:v>
+      </x:c>
+      <x:c r="D49" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E49" s="20" t="str">
+        <x:v>https://lrec2026.info/third-call-for-papers/</x:v>
+      </x:c>
+      <x:c r="F49" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="60" hidden="0" customHeight="1">
+      <x:c r="A50" s="20" t="str">
+        <x:v>MIDL</x:v>
+      </x:c>
+      <x:c r="B50" s="20" t="str">
+        <x:v>Computer Vision &amp; Pattern Recognition; Probabilistic, Causal &amp; Uncertainty ML; Explainability &amp; Interpretability; Robustness &amp; Safety; Federated &amp; Distributed Learning</x:v>
+      </x:c>
+      <x:c r="C50" s="20" t="str">
+        <x:v>Deep learning for biomedical image analysis, especially segmentation, detection, reconstruction, registration, generative imaging, and learning from limited labels. Uncertainty, interpretability, multi-site learning, robustness, and clinical validation extend that imaging core. Multimodal foundation models are relevant when grounded in medical imaging.</x:v>
+      </x:c>
+      <x:c r="D50" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E50" s="20" t="str">
+        <x:v>https://2026.midl.io/call-for-papers</x:v>
+      </x:c>
+      <x:c r="F50" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="60" hidden="0" customHeight="1">
+      <x:c r="A51" s="20" t="str">
+        <x:v>MLSys</x:v>
+      </x:c>
+      <x:c r="B51" s="20" t="str">
+        <x:v>Reinforcement Learning; Privacy-preserving ML</x:v>
+      </x:c>
+      <x:c r="C51" s="20" t="str">
+        <x:v>The intersection of machine learning and computer systems, including efficient training, inference and serving, compilers and runtimes, programming abstractions, specialized hardware, distributed learning, and system monitoring. LLM and agentic workloads are considered from a systems perspective. Both systems for ML and ML methods that improve computing systems are relevant.</x:v>
+      </x:c>
+      <x:c r="D51" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E51" s="20" t="str">
+        <x:v>https://mlsys.org/Conferences/2027/CallForResearchPapers</x:v>
+      </x:c>
+      <x:c r="F51" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="60" hidden="0" customHeight="1">
+      <x:c r="A52" s="20" t="str">
+        <x:v>NAACL</x:v>
+      </x:c>
+      <x:c r="B52" s="20" t="str">
+        <x:v>Autonomous Agents &amp; Multiagent Systems; Cognitive Science &amp; Computational Cognition; Fairness &amp; Responsible AI; Robustness &amp; Safety; Human-AI Interaction &amp; Deployment</x:v>
+      </x:c>
+      <x:c r="C52" s="20" t="str">
+        <x:v>Language technologies and computational linguistics across the Americas community, covering multilingual and low-resource NLP, language models, dialogue, retrieval, evaluation, and linguistic analysis. The 2027 theme concerns language as a medium for agentic communication, not merely running multiple models. General application domains are not standalone specialist tags.</x:v>
+      </x:c>
+      <x:c r="D52" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E52" s="20" t="str">
+        <x:v>https://2027.naacl.org/calls/main_conference_papers/</x:v>
+      </x:c>
+      <x:c r="F52" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="60" hidden="0" customHeight="1">
+      <x:c r="A53" s="20" t="str">
+        <x:v>NeurIPS</x:v>
+      </x:c>
+      <x:c r="B53" s="20" t="str">
+        <x:v>Learning Theory &amp; Statistical Foundations; Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Natural Language Processing &amp; LLMs; Computer Vision &amp; Pattern Recognition; ML Systems &amp; Infrastructure</x:v>
+      </x:c>
+      <x:c r="C53" s="20" t="str">
+        <x:v>Broad research in machine learning, especially deep and generative models, statistical foundations, optimization, probabilistic inference, and learning for decision-making. Language, vision, and scalable ML systems are important research communities. Interdisciplinary applications should contribute insight of wider interest to the machine-learning community.</x:v>
+      </x:c>
+      <x:c r="D53" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E53" s="20" t="str">
+        <x:v>https://neurips.cc/Conferences/2026/CallForPapers</x:v>
+      </x:c>
+      <x:c r="F53" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="60" hidden="0" customHeight="1">
+      <x:c r="A54" s="20" t="str">
+        <x:v>NOLTA</x:v>
+      </x:c>
+      <x:c r="B54" s="20" t="str">
+        <x:v>Signal Processing; Evolutionary Computation &amp; Optimization</x:v>
+      </x:c>
+      <x:c r="C54" s="20" t="str">
+        <x:v>Nonlinear theory and its applications, centered on chaos, bifurcations, oscillations, synchronization, nonlinear circuits, and complex networks. Neural computation, evolutionary algorithms, control, and signal processing connect to this nonlinear-systems focus. Individual application examples are not taken as additional specialist identities.</x:v>
+      </x:c>
+      <x:c r="D54" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E54" s="20" t="str">
+        <x:v>https://nolta2026.org/</x:v>
+      </x:c>
+      <x:c r="F54" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="72" hidden="0" customHeight="1">
+      <x:c r="A55" s="20" t="str">
+        <x:v>ProbML</x:v>
+      </x:c>
+      <x:c r="B55" s="20" t="str">
+        <x:v>Deep Representation Learning; Reinforcement Learning; Time Series &amp; Sequential Data; Robustness &amp; Safety</x:v>
+      </x:c>
+      <x:c r="C55" s="20" t="str">
+        <x:v>Probabilistic and Bayesian machine learning, emphasizing approximate inference, variational and Monte Carlo methods, Gaussian processes, graphical and state-space models, calibration, and decisions under uncertainty. Includes Bayesian optimization and uncertainty-aware deep learning. The reviewed 2026 application focus is healthcare and climate; probabilistic reasoning remains essential to a suitable contribution.</x:v>
+      </x:c>
+      <x:c r="D55" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E55" s="20" t="str">
+        <x:v>https://probml.cc/call/</x:v>
+      </x:c>
+      <x:c r="F55" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="60" hidden="0" customHeight="1">
+      <x:c r="A56" s="20" t="str">
+        <x:v>RecSys</x:v>
+      </x:c>
+      <x:c r="B56" s="20" t="str">
+        <x:v>Time Series &amp; Sequential Data; Natural Language Processing &amp; LLMs; Fairness &amp; Responsible AI; Explainability &amp; Interpretability</x:v>
+      </x:c>
+      <x:c r="C56" s="20" t="str">
+        <x:v>Recommendation and personalization: user-item modeling, collaborative and content-based methods, sequential and conversational recommendation, evaluation, and deployed recommendation systems. Human and economic impacts matter alongside algorithms. Sequential data is relevant specifically through recommendation behavior; this is not a general forecasting conference.</x:v>
+      </x:c>
+      <x:c r="D56" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E56" s="20" t="str">
+        <x:v>https://recsys.acm.org/recsys26/call/</x:v>
+      </x:c>
+      <x:c r="F56" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="60" hidden="0" customHeight="1">
+      <x:c r="A57" s="20" t="str">
+        <x:v>RSS</x:v>
+      </x:c>
+      <x:c r="B57" s="20" t="str">
+        <x:v>Planning &amp; Search; Deep Representation Learning; Probabilistic, Causal &amp; Uncertainty ML; Robustness &amp; Safety</x:v>
+      </x:c>
+      <x:c r="C57" s="20" t="str">
+        <x:v>Focused robotics research linking perception, learning, planning, control, manipulation, and robot-system science. Reinforcement and imitation learning, model-based behavior, and reliable autonomous systems are characteristic intersections. The 2027 review process emphasizes a scientifically developed robotic hypothesis through gated initial and invited final submissions.</x:v>
+      </x:c>
+      <x:c r="D57" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E57" s="20" t="str">
+        <x:v>https://roboticsconference.org/information/cfp/</x:v>
+      </x:c>
+      <x:c r="F57" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="60" hidden="0" customHeight="1">
+      <x:c r="A58" s="20" t="str">
+        <x:v>SaTML</x:v>
+      </x:c>
+      <x:c r="B58" s="20" t="str">
+        <x:v>Machine Learning; ML Systems &amp; Infrastructure</x:v>
+      </x:c>
+      <x:c r="C58" s="20" t="str">
+        <x:v>Security, safety, and trustworthiness of machine learning. Characteristic work studies attacks and defenses, privacy, verification, ML-system security, fairness, interpretability, and trustworthy data curation. Theoretical, empirical, and applied papers must engage substantively with a safety or trustworthiness question; merely using an ML model is insufficient.</x:v>
+      </x:c>
+      <x:c r="D58" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E58" s="20" t="str">
+        <x:v>https://satml.org/call-for-papers/</x:v>
+      </x:c>
+      <x:c r="F58" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="72" hidden="0" customHeight="1">
+      <x:c r="A59" s="20" t="str">
+        <x:v>SIGIR</x:v>
+      </x:c>
+      <x:c r="B59" s="20" t="str">
+        <x:v>Multimedia Learning &amp; Retrieval; Human-AI Interaction &amp; Deployment; Fairness &amp; Responsible AI; ML Systems &amp; Infrastructure</x:v>
+      </x:c>
+      <x:c r="C59" s="20" t="str">
+        <x:v>Information access, search and ranking, query and content understanding, recommendation, conversational and multimodal retrieval, and evaluation of retrieval systems. Learning and language models are relevant through an information-retrieval contribution, including retrieval-augmented generation. The 2027 detailed track pages contain organizer placeholders; scope should be rechecked when finalized.</x:v>
+      </x:c>
+      <x:c r="D59" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E59" s="20" t="str">
+        <x:v>https://sigir2027.org/pages/submit-full.html</x:v>
+      </x:c>
+      <x:c r="F59" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="60" hidden="0" customHeight="1">
+      <x:c r="A60" s="20" t="str">
+        <x:v>SMC</x:v>
+      </x:c>
+      <x:c r="B60" s="20" t="str">
+        <x:v>Reinforcement Learning; System Identification &amp; Data-driven Dynamics; BCI &amp; Neurotechnology; Cognitive Science &amp; Computational Cognition</x:v>
+      </x:c>
+      <x:c r="C60" s="20" t="str">
+        <x:v>Systems science, cybernetics, and human-machine systems. Characteristic ML-facing work includes intelligent and learning-based control, autonomous systems, adaptive decision-making, and human-AI interaction; brain-machine interfaces and cognitive systems are meaningful extensions. Its interdisciplinary remit is curated without tagging every industrial application as a core specialty.</x:v>
+      </x:c>
+      <x:c r="D60" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E60" s="20" t="str">
+        <x:v>https://www.ieeesmc2026.org/call-for-papers</x:v>
+      </x:c>
+      <x:c r="F60" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="60" hidden="0" customHeight="1">
+      <x:c r="A61" s="20" t="str">
         <x:v>UAI</x:v>
       </x:c>
-      <x:c r="B45" s="20" t="str">
+      <x:c r="B61" s="20" t="str">
         <x:v>Deep Representation Learning; Reinforcement Learning; Time Series &amp; Sequential Data; Explainability &amp; Interpretability; Robustness &amp; Safety</x:v>
       </x:c>
-      <x:c r="C45" s="20" t="str">
+      <x:c r="C61" s="20" t="str">
         <x:v>Learning and reasoning under uncertainty, centered on probabilistic and Bayesian modeling, graphical models, causal inference, approximate inference, and decision theory. Includes Monte Carlo and variational methods, uncertainty quantification, sequential models, and principled analysis of learning algorithms. Uncertainty is the organizing theme, not just another application of general-purpose AI.</x:v>
       </x:c>
-      <x:c r="D45" s="21" t="n">
+      <x:c r="D61" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
-      <x:c r="E45" s="20" t="str">
+      <x:c r="E61" s="20" t="str">
         <x:v>https://www.auai.org/uai2026/subject_areas; https://www.auai.org/uai2026/call_for_papers</x:v>
       </x:c>
-      <x:c r="F45" s="22" t="n">
-        <x:v>46302</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="46" ht="72" hidden="0" customHeight="1">
-      <x:c r="A46" s="20" t="str">
+      <x:c r="F61" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="72" hidden="0" customHeight="1">
+      <x:c r="A62" s="20" t="str">
         <x:v>WACV</x:v>
       </x:c>
-      <x:c r="B46" s="20" t="str">
+      <x:c r="B62" s="20" t="str">
         <x:v>Signal Processing; Biometrics &amp; Human Sensing; Multimedia Learning &amp; Retrieval</x:v>
       </x:c>
-      <x:c r="C46" s="20" t="str">
+      <x:c r="C62" s="20" t="str">
         <x:v>Applied computer vision and visual learning, with an emphasis on practical recognition, detection, segmentation, image/video analysis, 3D perception, and deployable visual systems. Human analysis and multimodal visual methods are established areas. Compared with the flagship trio, WACV particularly welcomes meaningful application-driven contributions supported by sound evaluation; its two submission rounds are routes, not different fields.</x:v>
       </x:c>
-      <x:c r="D46" s="21" t="n">
+      <x:c r="D62" s="21" t="n">
         <x:v>2027</x:v>
       </x:c>
-      <x:c r="E46" s="20" t="str">
+      <x:c r="E62" s="20" t="str">
         <x:v>https://wacv.thecvf.com/Conferences/2027/CallForPapers</x:v>
       </x:c>
-      <x:c r="F46" s="22" t="n">
+      <x:c r="F62" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="60" hidden="0" customHeight="1">
+      <x:c r="A63" s="20" t="str">
+        <x:v>WSDM</x:v>
+      </x:c>
+      <x:c r="B63" s="20" t="str">
+        <x:v>Information Retrieval &amp; Search; Recommender Systems; Graphs &amp; Graph Learning; LLM Agents &amp; Tool Use; Natural Language Processing &amp; LLMs</x:v>
+      </x:c>
+      <x:c r="C63" s="20" t="str">
+        <x:v>Web search, ranking, recommendation and mining of web and social data. Characteristic extensions include large-scale graph analysis, conversational retrieval, foundation-model and agentic web systems, and fairness and privacy in information access. The broad emerging-applications inventory is not treated as evidence that WSDM is a specialist healthcare or climate venue.</x:v>
+      </x:c>
+      <x:c r="D63" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E63" s="20" t="str">
+        <x:v>https://www.wsdm-conference.org/2027/cffp.html</x:v>
+      </x:c>
+      <x:c r="F63" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="60" hidden="0" customHeight="1">
+      <x:c r="A64" s="20" t="str">
+        <x:v>WWW</x:v>
+      </x:c>
+      <x:c r="B64" s="20" t="str">
+        <x:v>Knowledge Representation &amp; Reasoning; Data Mining &amp; Data Science; Fairness &amp; Responsible AI; Privacy-preserving ML; Ethics &amp; Governance</x:v>
+      </x:c>
+      <x:c r="C64" s="20" t="str">
+        <x:v>Research on the Web as infrastructure and a socio-technical ecosystem. Characteristic ML-facing tracks include search and recommendation, retrieval-augmented and agentic information access, graph learning, and semantic knowledge. Responsible Web and privacy research are substantive strands. Merely using a web dataset or API is explicitly insufficient topical relevance.</x:v>
+      </x:c>
+      <x:c r="D64" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E64" s="20" t="str">
+        <x:v>https://www2027.thewebconf.org/research-track-papers/</x:v>
+      </x:c>
+      <x:c r="F64" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f6d0384e27a482c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0475ca36bdfd4304"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add complex systems and neuroscience conference series
</commit_message>
<xml_diff>
--- a/data/core_conferences_normalized_tags.xlsx
+++ b/data/core_conferences_normalized_tags.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Conferences" sheetId="1" r:id="R07338374964b43c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Vocabulary" sheetId="2" r:id="R185e42a7a4404346"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conference Scope" sheetId="3" r:id="R9fe1be8fca8d4635"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Conferences" sheetId="1" r:id="Rdaf34c59c6194604"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Vocabulary" sheetId="2" r:id="R89910889990f421e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conference Scope" sheetId="3" r:id="R2dab23f348df4c26"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -119,7 +119,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="CoreConferencesTable" displayName="CoreConferencesTable" ref="A1:N114" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="CoreConferencesTable" displayName="CoreConferencesTable" ref="A1:N130" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Conference"/>
     <x:tableColumn id="2" name="TAGS"/>
@@ -141,7 +141,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TagVocabularyTable" displayName="TagVocabularyTable" ref="A1:B40" headerRowCount="1" totalsRowCount="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TagVocabularyTable" displayName="TagVocabularyTable" ref="A1:B43" headerRowCount="1" totalsRowCount="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Standard tag"/>
     <x:tableColumn id="2" name="Definition"/>
@@ -151,7 +151,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ConferenceScope" displayName="ConferenceScope" ref="A1:F64" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ConferenceScope" displayName="ConferenceScope" ref="A1:F80" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Series"/>
     <x:tableColumn id="2" name="Additional topics"/>
@@ -4289,10 +4289,458 @@
       <x:c r="M114"/>
       <x:c r="N114"/>
     </x:row>
+    <x:row r="115" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A115" t="str">
+        <x:v>COMPLEX NETWORKS</x:v>
+      </x:c>
+      <x:c r="B115" s="12" t="str">
+        <x:v>Complex Systems &amp; Network Science; Graphs &amp; Graph Learning; Nonlinear Dynamics &amp; Chaos; Data Mining &amp; Data Science</x:v>
+      </x:c>
+      <x:c r="C115" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="D115" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E115"/>
+      <x:c r="F115" s="12" t="str">
+        <x:v>Paper-based + extended abstracts</x:v>
+      </x:c>
+      <x:c r="G115" t="str">
+        <x:v>https://complexnetworks.org/</x:v>
+      </x:c>
+      <x:c r="H115"/>
+      <x:c r="I115"/>
+      <x:c r="J115"/>
+      <x:c r="K115" s="16"/>
+      <x:c r="L115" s="17"/>
+      <x:c r="M115"/>
+      <x:c r="N115"/>
+    </x:row>
+    <x:row r="116" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A116" t="str">
+        <x:v>CompleNet</x:v>
+      </x:c>
+      <x:c r="B116" s="12" t="str">
+        <x:v>Complex Systems &amp; Network Science; Graphs &amp; Graph Learning; Nonlinear Dynamics &amp; Chaos; Computational Neuroscience</x:v>
+      </x:c>
+      <x:c r="C116" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D116" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E116"/>
+      <x:c r="F116" s="12" t="str">
+        <x:v>Full/short papers + extended abstracts</x:v>
+      </x:c>
+      <x:c r="G116" t="str">
+        <x:v>https://complenet.github.io/</x:v>
+      </x:c>
+      <x:c r="H116"/>
+      <x:c r="I116"/>
+      <x:c r="J116"/>
+      <x:c r="K116" s="16"/>
+      <x:c r="L116" s="17"/>
+      <x:c r="M116"/>
+      <x:c r="N116"/>
+    </x:row>
+    <x:row r="117" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A117" t="str">
+        <x:v>ALIFE</x:v>
+      </x:c>
+      <x:c r="B117" s="12" t="str">
+        <x:v>Artificial Life &amp; Adaptive Systems; Complex Systems &amp; Network Science; Evolutionary Computation &amp; Optimization; Cognitive Science &amp; Computational Cognition</x:v>
+      </x:c>
+      <x:c r="C117" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="D117" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E117"/>
+      <x:c r="F117" s="12" t="str">
+        <x:v>Full papers + non-archival abstracts</x:v>
+      </x:c>
+      <x:c r="G117" t="str">
+        <x:v>https://alife.vscht.cz/</x:v>
+      </x:c>
+      <x:c r="H117"/>
+      <x:c r="I117"/>
+      <x:c r="J117"/>
+      <x:c r="K117" s="16"/>
+      <x:c r="L117" s="17"/>
+      <x:c r="M117"/>
+      <x:c r="N117"/>
+    </x:row>
+    <x:row r="118" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A118" t="str">
+        <x:v>NODYCON</x:v>
+      </x:c>
+      <x:c r="B118" s="12" t="str">
+        <x:v>Nonlinear Dynamics &amp; Chaos; System Identification &amp; Data-driven Dynamics; Control &amp; Robotics; Complex Systems &amp; Network Science</x:v>
+      </x:c>
+      <x:c r="C118" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="D118" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E118"/>
+      <x:c r="F118" s="12" t="str">
+        <x:v>Abstract-based + selected journal papers</x:v>
+      </x:c>
+      <x:c r="G118" t="str">
+        <x:v>https://nodycon2026.app.earendelplatform.com/</x:v>
+      </x:c>
+      <x:c r="H118"/>
+      <x:c r="I118"/>
+      <x:c r="J118"/>
+      <x:c r="K118" s="16"/>
+      <x:c r="L118" s="17"/>
+      <x:c r="M118"/>
+      <x:c r="N118"/>
+    </x:row>
+    <x:row r="119" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A119" t="str">
+        <x:v>NICE</x:v>
+      </x:c>
+      <x:c r="B119" s="12" t="str">
+        <x:v>Neuromorphic &amp; Brain-inspired Computing; Computational Neuroscience; Machine Learning; BCI &amp; Neurotechnology</x:v>
+      </x:c>
+      <x:c r="C119" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D119" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E119"/>
+      <x:c r="F119" s="12" t="str">
+        <x:v>Research papers + late-breaking abstracts</x:v>
+      </x:c>
+      <x:c r="G119" t="str">
+        <x:v>https://niceworkshop.org/nice-2027/</x:v>
+      </x:c>
+      <x:c r="H119"/>
+      <x:c r="I119"/>
+      <x:c r="J119"/>
+      <x:c r="K119" s="16"/>
+      <x:c r="L119" s="17"/>
+      <x:c r="M119"/>
+      <x:c r="N119"/>
+    </x:row>
+    <x:row r="120" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A120" t="str">
+        <x:v>SAB</x:v>
+      </x:c>
+      <x:c r="B120" s="12" t="str">
+        <x:v>Artificial Life &amp; Adaptive Systems; Computational Neuroscience; Cognitive Science &amp; Computational Cognition; Control &amp; Robotics</x:v>
+      </x:c>
+      <x:c r="C120" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D120" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E120"/>
+      <x:c r="F120" s="12" t="str">
+        <x:v>Reviewed papers + non-archival contributions</x:v>
+      </x:c>
+      <x:c r="G120" t="str">
+        <x:v>https://sab-conference.org/</x:v>
+      </x:c>
+      <x:c r="H120"/>
+      <x:c r="I120"/>
+      <x:c r="J120"/>
+      <x:c r="K120" s="16"/>
+      <x:c r="L120" s="17"/>
+      <x:c r="M120"/>
+      <x:c r="N120"/>
+    </x:row>
+    <x:row r="121" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A121" t="str">
+        <x:v>BCI Winter</x:v>
+      </x:c>
+      <x:c r="B121" s="12" t="str">
+        <x:v>BCI &amp; Neurotechnology; EEG/MEG &amp; Neural Signals; Signal Processing; Machine Learning</x:v>
+      </x:c>
+      <x:c r="C121" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D121" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E121"/>
+      <x:c r="F121" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G121" t="str">
+        <x:v>https://brain.korea.ac.kr/bci2027/</x:v>
+      </x:c>
+      <x:c r="H121"/>
+      <x:c r="I121"/>
+      <x:c r="J121"/>
+      <x:c r="K121" s="16"/>
+      <x:c r="L121" s="17"/>
+      <x:c r="M121"/>
+      <x:c r="N121"/>
+    </x:row>
+    <x:row r="122" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A122" t="str">
+        <x:v>IEEE BioCAS</x:v>
+      </x:c>
+      <x:c r="B122" s="12" t="str">
+        <x:v>Healthcare &amp; Clinical AI; BCI &amp; Neurotechnology; Signal Processing; Neuromorphic &amp; Brain-inspired Computing</x:v>
+      </x:c>
+      <x:c r="C122" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D122" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E122"/>
+      <x:c r="F122" s="12" t="str">
+        <x:v>Paper-based</x:v>
+      </x:c>
+      <x:c r="G122" t="str">
+        <x:v>https://2027.ieee-biocas.org/</x:v>
+      </x:c>
+      <x:c r="H122"/>
+      <x:c r="I122"/>
+      <x:c r="J122"/>
+      <x:c r="K122" s="16"/>
+      <x:c r="L122" s="17"/>
+      <x:c r="M122"/>
+      <x:c r="N122"/>
+    </x:row>
+    <x:row r="123" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A123" t="str">
+        <x:v>ICCN</x:v>
+      </x:c>
+      <x:c r="B123" s="12" t="str">
+        <x:v>Computational Neuroscience; Cognitive Science &amp; Computational Cognition; Nonlinear Dynamics &amp; Chaos; Complex Systems &amp; Network Science</x:v>
+      </x:c>
+      <x:c r="C123" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D123" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E123"/>
+      <x:c r="F123" s="12" t="str">
+        <x:v>Abstract-based; publication unconfirmed</x:v>
+      </x:c>
+      <x:c r="G123" t="str">
+        <x:v>https://iccn2026.jp/</x:v>
+      </x:c>
+      <x:c r="H123"/>
+      <x:c r="I123"/>
+      <x:c r="J123"/>
+      <x:c r="K123" s="16"/>
+      <x:c r="L123" s="17"/>
+      <x:c r="M123"/>
+      <x:c r="N123"/>
+    </x:row>
+    <x:row r="124" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A124" t="str">
+        <x:v>AREADNE</x:v>
+      </x:c>
+      <x:c r="B124" s="12" t="str">
+        <x:v>Systems &amp; Experimental Neuroscience; Computational Neuroscience; BCI &amp; Neurotechnology</x:v>
+      </x:c>
+      <x:c r="C124" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="D124" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E124"/>
+      <x:c r="F124" s="12" t="str">
+        <x:v>Abstract-based</x:v>
+      </x:c>
+      <x:c r="G124" t="str">
+        <x:v>https://areadne.org/</x:v>
+      </x:c>
+      <x:c r="H124"/>
+      <x:c r="I124"/>
+      <x:c r="J124"/>
+      <x:c r="K124" s="16"/>
+      <x:c r="L124" s="17"/>
+      <x:c r="M124"/>
+      <x:c r="N124"/>
+    </x:row>
+    <x:row r="125" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A125" t="str">
+        <x:v>SfN Neuroscience</x:v>
+      </x:c>
+      <x:c r="B125" s="12" t="str">
+        <x:v>Systems &amp; Experimental Neuroscience; Computational Neuroscience; Cognitive Science &amp; Computational Cognition; Neuroimaging &amp; Brain Mapping</x:v>
+      </x:c>
+      <x:c r="C125" t="str">
+        <x:v>XXL</x:v>
+      </x:c>
+      <x:c r="D125" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E125"/>
+      <x:c r="F125" s="12" t="str">
+        <x:v>Abstract-based</x:v>
+      </x:c>
+      <x:c r="G125" t="str">
+        <x:v>https://www.sfn.org/meetings</x:v>
+      </x:c>
+      <x:c r="H125"/>
+      <x:c r="I125"/>
+      <x:c r="J125"/>
+      <x:c r="K125" s="16"/>
+      <x:c r="L125" s="17"/>
+      <x:c r="M125"/>
+      <x:c r="N125"/>
+    </x:row>
+    <x:row r="126" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A126" t="str">
+        <x:v>Dynamics Days Europe</x:v>
+      </x:c>
+      <x:c r="B126" s="12" t="str">
+        <x:v>Nonlinear Dynamics &amp; Chaos; Complex Systems &amp; Network Science; Time Series &amp; Sequential Data; System Identification &amp; Data-driven Dynamics</x:v>
+      </x:c>
+      <x:c r="C126" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="D126" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E126"/>
+      <x:c r="F126" s="12" t="str">
+        <x:v>Abstract-based</x:v>
+      </x:c>
+      <x:c r="G126" t="str">
+        <x:v>https://www.dynamicsdays.org/</x:v>
+      </x:c>
+      <x:c r="H126"/>
+      <x:c r="I126"/>
+      <x:c r="J126"/>
+      <x:c r="K126" s="16"/>
+      <x:c r="L126" s="17"/>
+      <x:c r="M126"/>
+      <x:c r="N126"/>
+    </x:row>
+    <x:row r="127" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A127" t="str">
+        <x:v>Dynamics Days US</x:v>
+      </x:c>
+      <x:c r="B127" s="12" t="str">
+        <x:v>Nonlinear Dynamics &amp; Chaos; Complex Systems &amp; Network Science; System Identification &amp; Data-driven Dynamics</x:v>
+      </x:c>
+      <x:c r="C127" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D127" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E127"/>
+      <x:c r="F127" s="12" t="str">
+        <x:v>Abstract-based</x:v>
+      </x:c>
+      <x:c r="G127" t="str">
+        <x:v>https://www.ddays.org/2027/</x:v>
+      </x:c>
+      <x:c r="H127"/>
+      <x:c r="I127"/>
+      <x:c r="J127"/>
+      <x:c r="K127" s="16"/>
+      <x:c r="L127" s="17"/>
+      <x:c r="M127"/>
+      <x:c r="N127"/>
+    </x:row>
+    <x:row r="128" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A128" t="str">
+        <x:v>Dynamics Days LAC</x:v>
+      </x:c>
+      <x:c r="B128" s="12" t="str">
+        <x:v>Nonlinear Dynamics &amp; Chaos; Complex Systems &amp; Network Science; Time Series &amp; Sequential Data; Computational Neuroscience</x:v>
+      </x:c>
+      <x:c r="C128" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D128" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E128"/>
+      <x:c r="F128" s="12" t="str">
+        <x:v>Abstract-based</x:v>
+      </x:c>
+      <x:c r="G128" t="str">
+        <x:v>https://fisica.ufpr.br/DDaysLAC2026/index.html</x:v>
+      </x:c>
+      <x:c r="H128"/>
+      <x:c r="I128"/>
+      <x:c r="J128"/>
+      <x:c r="K128" s="16"/>
+      <x:c r="L128" s="17"/>
+      <x:c r="M128"/>
+      <x:c r="N128"/>
+    </x:row>
+    <x:row r="129" ht="15" hidden="0" customHeight="1">
+      <x:c r="A129" t="str">
+        <x:v>Dynamics Days Asia-Pacific</x:v>
+      </x:c>
+      <x:c r="B129" s="12" t="str">
+        <x:v>Nonlinear Dynamics &amp; Chaos; Complex Systems &amp; Network Science</x:v>
+      </x:c>
+      <x:c r="C129" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D129" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E129"/>
+      <x:c r="F129" s="12" t="str">
+        <x:v>Talks/abstracts; next call unannounced</x:v>
+      </x:c>
+      <x:c r="G129" t="str">
+        <x:v>https://www2.yukawa.kyoto-u.ac.jp/~frontier24/DDAP13/</x:v>
+      </x:c>
+      <x:c r="H129"/>
+      <x:c r="I129"/>
+      <x:c r="J129"/>
+      <x:c r="K129" s="16"/>
+      <x:c r="L129" s="17"/>
+      <x:c r="M129"/>
+      <x:c r="N129"/>
+    </x:row>
+    <x:row r="130" ht="15" hidden="0" customHeight="1">
+      <x:c r="A130" t="str">
+        <x:v>Dynamics Days CAC</x:v>
+      </x:c>
+      <x:c r="B130" s="12" t="str">
+        <x:v>Nonlinear Dynamics &amp; Chaos; Complex Systems &amp; Network Science</x:v>
+      </x:c>
+      <x:c r="C130" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D130" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E130"/>
+      <x:c r="F130" s="12" t="str">
+        <x:v>Abstract-based</x:v>
+      </x:c>
+      <x:c r="G130" t="str">
+        <x:v>https://physics-congress.kz/dynamics_days</x:v>
+      </x:c>
+      <x:c r="H130"/>
+      <x:c r="I130"/>
+      <x:c r="J130"/>
+      <x:c r="K130" s="16"/>
+      <x:c r="L130" s="17"/>
+      <x:c r="M130"/>
+      <x:c r="N130"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc9061b32c68406b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R751491f2e50e428a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4633,10 +5081,34 @@
         <x:v>Graph mining, graph representation learning, graph neural networks, and learning on structured networks. Family: Complex Systems, Time Series &amp; Signals.</x:v>
       </x:c>
     </x:row>
+    <x:row r="42" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A42" t="str">
+        <x:v>Artificial Life &amp; Adaptive Systems</x:v>
+      </x:c>
+      <x:c r="B42" s="12" t="str">
+        <x:v>Artificial life, emergence, adaptive behavior, embodied intelligence, and living or life-like systems. Family: Complex Systems, Time Series &amp; Signals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A43" t="str">
+        <x:v>Neuromorphic &amp; Brain-inspired Computing</x:v>
+      </x:c>
+      <x:c r="B43" s="12" t="str">
+        <x:v>Brain-inspired computation, spiking neural networks, neuromorphic hardware, and neural computing systems. Family: Neuroscience &amp; Neurotechnology.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A44" t="str">
+        <x:v>Systems &amp; Experimental Neuroscience</x:v>
+      </x:c>
+      <x:c r="B44" s="12" t="str">
+        <x:v>Experimental and systems neuroscience, neural populations, circuits, behavior, and neural coding. Family: Neuroscience &amp; Neurotechnology.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7261d0a80e942ff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18651688988d4b8a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4869,139 +5341,141 @@
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="72" hidden="0" customHeight="1">
+    <x:row r="12" ht="48" hidden="0" customHeight="1">
       <x:c r="A12" s="20" t="str">
-        <x:v>AutoML</x:v>
+        <x:v>ALIFE</x:v>
       </x:c>
       <x:c r="B12" s="20" t="str">
-        <x:v>Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Explainability &amp; Interpretability; Natural Language Processing &amp; LLMs; Robustness &amp; Safety</x:v>
+        <x:v>Autonomous Agents &amp; Multiagent Systems; Control &amp; Robotics; Machine Learning</x:v>
       </x:c>
       <x:c r="C12" s="20" t="str">
-        <x:v>Automating the construction and configuration of learning systems: hyperparameter optimization, Bayesian optimization, neural architecture search, model selection, meta-learning, and pipeline automation. Includes evolutionary and reinforcement-learning approaches, AutoML for foundation models, and evaluation through applications, benchmarks, challenges, and datasets. Trustworthiness matters specifically in automated ML workflows.</x:v>
+        <x:v>Artificial life and life-like processes in computational, robotic and biological systems. Central questions concern emergence, evolution, adaptation, embodied intelligence and cognition. Relevant ML work studies adaptive agents, evolutionary learning and computational models of living systems; it is not a general-purpose AI conference.</x:v>
       </x:c>
       <x:c r="D12" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E12" s="20" t="str">
-        <x:v>https://2026.automl.cc/call-for-papers/</x:v>
+        <x:v>https://2026.alife.org/call-for-papers/; https://alife.org/conference/alife-2027/</x:v>
       </x:c>
       <x:c r="F12" s="22" t="n">
-        <x:v>46302</x:v>
+        <x:v>46303</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="60" hidden="0" customHeight="1">
       <x:c r="A13" s="20" t="str">
-        <x:v>BMVC</x:v>
+        <x:v>AREADNE</x:v>
       </x:c>
       <x:c r="B13" s="20" t="str">
-        <x:v>Signal Processing</x:v>
+        <x:v>Cognitive Science &amp; Computational Cognition</x:v>
       </x:c>
       <x:c r="C13" s="20" t="str">
-        <x:v>Computer vision, image processing, and visual pattern recognition, including visual learning, recognition and segmentation, reconstruction, motion and video analysis, and evaluation of vision methods. The single-track BMVA conference combines methodological and applied vision research. It is an established broad vision venue, not a specialist biomedical-imaging meeting.</x:v>
+        <x:v>Encoding and decoding of neural ensembles, with emphasis on systems neuroscience, neural population recordings, neural representations, computation and links to behavior. It is a focused experimental/computational neuroscience meeting rather than a general neuroscience congress. Contributions are reviewed abstracts for talks and posters; its proceedings book is a collection of abstracts.</x:v>
       </x:c>
       <x:c r="D13" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E13" s="20" t="str">
-        <x:v>https://bmvc2026.bmva.org/calls/call-for-papers/</x:v>
+        <x:v>https://areadne.org/</x:v>
       </x:c>
       <x:c r="F13" s="22" t="n">
-        <x:v>46302</x:v>
+        <x:v>46303</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="72" hidden="0" customHeight="1">
       <x:c r="A14" s="20" t="str">
-        <x:v>CCN</x:v>
+        <x:v>AutoML</x:v>
       </x:c>
       <x:c r="B14" s="20" t="str">
-        <x:v>Cognitive Science &amp; Computational Cognition; Explainability &amp; Interpretability</x:v>
+        <x:v>Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Explainability &amp; Interpretability; Natural Language Processing &amp; LLMs; Robustness &amp; Safety</x:v>
       </x:c>
       <x:c r="C14" s="20" t="str">
-        <x:v>Cognitive computational neuroscience, connecting experiments and models of brain computation with artificial intelligence. Characteristic work compares biological and artificial representations, models perception, cognition and action, studies neural connectivity and dynamics, and uses mechanistic interpretability to understand neural-network models. The aim is understanding computation and behavior across brains and AI systems.</x:v>
+        <x:v>Automating the construction and configuration of learning systems: hyperparameter optimization, Bayesian optimization, neural architecture search, model selection, meta-learning, and pipeline automation. Includes evolutionary and reinforcement-learning approaches, AutoML for foundation models, and evaluation through applications, benchmarks, challenges, and datasets. Trustworthiness matters specifically in automated ML workflows.</x:v>
       </x:c>
       <x:c r="D14" s="21" t="n">
-        <x:v>2027</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="E14" s="20" t="str">
-        <x:v>https://2027.ccneuro.org/</x:v>
+        <x:v>https://2026.automl.cc/call-for-papers/</x:v>
       </x:c>
       <x:c r="F14" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="72" hidden="0" customHeight="1">
+    <x:row r="15" ht="60" hidden="0" customHeight="1">
       <x:c r="A15" s="20" t="str">
-        <x:v>CHIL</x:v>
+        <x:v>BCI Winter</x:v>
       </x:c>
       <x:c r="B15" s="20" t="str">
-        <x:v>Explainability &amp; Interpretability; Human-AI Interaction &amp; Deployment; Robustness &amp; Safety; Time Series &amp; Sequential Data</x:v>
+        <x:v>Healthcare &amp; Clinical AI; Neuroimaging &amp; Brain Mapping</x:v>
       </x:c>
       <x:c r="C15" s="20" t="str">
-        <x:v>Machine learning and inference for clinical, public, and population health. Distinguishing areas include causal inference, survival analysis, multimodal health data, generalization across populations, interpretability, and clinical evaluation and deployment. Research may emphasize methods, practical applications, or societal impact. Health-focused inference and evaluation remain the common thread across these tracks.</x:v>
+        <x:v>Brain-computer interfaces, neural signal decoding, multimodal brain measurements, neurofeedback and adaptive interfaces. Machine learning is central to biosignal classification and decoding; neurorehabilitation and interaction with real or virtual environments are characteristic applications. IEEE-style reviewed research papers are the established publication route.</x:v>
       </x:c>
       <x:c r="D15" s="21" t="n">
-        <x:v>2026</x:v>
+        <x:v>2027</x:v>
       </x:c>
       <x:c r="E15" s="20" t="str">
-        <x:v>https://chil.ahli.cc/submit/call-for-papers/</x:v>
+        <x:v>https://brain.korea.ac.kr/bci2027/callforpaper.php; https://brain.korea.ac.kr/bci2026/assets/CFP_BCI2026.pdf</x:v>
       </x:c>
       <x:c r="F15" s="22" t="n">
-        <x:v>46302</x:v>
+        <x:v>46303</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="60" hidden="0" customHeight="1">
       <x:c r="A16" s="20" t="str">
-        <x:v>CIKM</x:v>
+        <x:v>BMVC</x:v>
       </x:c>
       <x:c r="B16" s="20" t="str">
-        <x:v>Information Retrieval &amp; Search; Recommender Systems; Knowledge Representation &amp; Reasoning; Graphs &amp; Graph Learning; LLM Agents &amp; Tool Use</x:v>
+        <x:v>Signal Processing</x:v>
       </x:c>
       <x:c r="C16" s="20" t="str">
-        <x:v>Information retrieval, knowledge management, data mining and database systems, with a strong focus on effective information access and knowledge at scale. The 2026 organizer description emphasizes AI for information access, knowledge representation, personalization and evaluation. Agentic and graph methods are relevant through these information and knowledge problems.</x:v>
+        <x:v>Computer vision, image processing, and visual pattern recognition, including visual learning, recognition and segmentation, reconstruction, motion and video analysis, and evaluation of vision methods. The single-track BMVA conference combines methodological and applied vision research. It is an established broad vision venue, not a specialist biomedical-imaging meeting.</x:v>
       </x:c>
       <x:c r="D16" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E16" s="20" t="str">
-        <x:v>https://cikm2026.diag.uniroma1.it/</x:v>
+        <x:v>https://bmvc2026.bmva.org/calls/call-for-papers/</x:v>
       </x:c>
       <x:c r="F16" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="60" hidden="0" customHeight="1">
+    <x:row r="17" ht="72" hidden="0" customHeight="1">
       <x:c r="A17" s="20" t="str">
-        <x:v>CogSci</x:v>
-      </x:c>
-      <x:c r="B17" s="20" t="str"/>
+        <x:v>CCN</x:v>
+      </x:c>
+      <x:c r="B17" s="20" t="str">
+        <x:v>Cognitive Science &amp; Computational Cognition; Explainability &amp; Interpretability</x:v>
+      </x:c>
       <x:c r="C17" s="20" t="str">
-        <x:v>Interdisciplinary study of cognition and the mind, connecting psychology, linguistics, artificial intelligence, neuroscience, philosophy, anthropology, and education. Computational models and experiments should illuminate cognitive processes and behavior. An AI paper belongs here through its contribution to understanding cognition, not solely through a predictive performance improvement.</x:v>
+        <x:v>Cognitive computational neuroscience, connecting experiments and models of brain computation with artificial intelligence. Characteristic work compares biological and artificial representations, models perception, cognition and action, studies neural connectivity and dynamics, and uses mechanistic interpretability to understand neural-network models. The aim is understanding computation and behavior across brains and AI systems.</x:v>
       </x:c>
       <x:c r="D17" s="21" t="n">
-        <x:v>2026</x:v>
+        <x:v>2027</x:v>
       </x:c>
       <x:c r="E17" s="20" t="str">
-        <x:v>https://cognitivesciencesociety.org/submissions-faq/; https://cognitivesciencesociety.org/</x:v>
+        <x:v>https://2027.ccneuro.org/</x:v>
       </x:c>
       <x:c r="F17" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="60" hidden="0" customHeight="1">
+    <x:row r="18" ht="72" hidden="0" customHeight="1">
       <x:c r="A18" s="20" t="str">
-        <x:v>COLING</x:v>
+        <x:v>CHIL</x:v>
       </x:c>
       <x:c r="B18" s="20" t="str">
-        <x:v>Information Retrieval &amp; Search; Cognitive Science &amp; Computational Cognition; Explainability &amp; Interpretability; Fairness &amp; Responsible AI</x:v>
+        <x:v>Explainability &amp; Interpretability; Human-AI Interaction &amp; Deployment; Robustness &amp; Safety; Time Series &amp; Sequential Data</x:v>
       </x:c>
       <x:c r="C18" s="20" t="str">
-        <x:v>Computational linguistics and language processing spanning linguistic theory, multilinguality, semantics and structured prediction, language models, dialogue, and empirical evaluation. Agentic language systems and knowledge-grounded NLP are relevant; the defining contribution should concern language, not a peripheral application domain.</x:v>
+        <x:v>Machine learning and inference for clinical, public, and population health. Distinguishing areas include causal inference, survival analysis, multimodal health data, generalization across populations, interpretability, and clinical evaluation and deployment. Research may emphasize methods, practical applications, or societal impact. Health-focused inference and evaluation remain the common thread across these tracks.</x:v>
       </x:c>
       <x:c r="D18" s="21" t="n">
-        <x:v>2027</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="E18" s="20" t="str">
-        <x:v>https://2027.coling-iccl.org/calls/main_conference_papers/</x:v>
+        <x:v>https://chil.ahli.cc/submit/call-for-papers/</x:v>
       </x:c>
       <x:c r="F18" s="22" t="n">
         <x:v>46302</x:v>
@@ -5009,19 +5483,19 @@
     </x:row>
     <x:row r="19" ht="60" hidden="0" customHeight="1">
       <x:c r="A19" s="20" t="str">
-        <x:v>COLM</x:v>
+        <x:v>CIKM</x:v>
       </x:c>
       <x:c r="B19" s="20" t="str">
-        <x:v>Learning Theory &amp; Statistical Foundations; Explainability &amp; Interpretability; Robustness &amp; Safety; Fairness &amp; Responsible AI; Multimedia Learning &amp; Retrieval</x:v>
+        <x:v>Information Retrieval &amp; Search; Recommender Systems; Knowledge Representation &amp; Reasoning; Graphs &amp; Graph Learning; LLM Agents &amp; Tool Use</x:v>
       </x:c>
       <x:c r="C19" s="20" t="str">
-        <x:v>Language-model foundations and methods: training and architecture, data and scaling, inference and generation, evaluation, reasoning, retrieval augmentation, and tool-using language agents. Alignment, interpretability, and multimodal language models are meaningful extensions. A central language-model contribution distinguishes the conference from generic AI applications.</x:v>
+        <x:v>Information retrieval, knowledge management, data mining and database systems, with a strong focus on effective information access and knowledge at scale. The 2026 organizer description emphasizes AI for information access, knowledge representation, personalization and evaluation. Agentic and graph methods are relevant through these information and knowledge problems.</x:v>
       </x:c>
       <x:c r="D19" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E19" s="20" t="str">
-        <x:v>https://colm.cc/Conferences/2026/CallForPapers</x:v>
+        <x:v>https://cikm2026.diag.uniroma1.it/</x:v>
       </x:c>
       <x:c r="F19" s="22" t="n">
         <x:v>46302</x:v>
@@ -5029,19 +5503,17 @@
     </x:row>
     <x:row r="20" ht="60" hidden="0" customHeight="1">
       <x:c r="A20" s="20" t="str">
-        <x:v>COLT</x:v>
-      </x:c>
-      <x:c r="B20" s="20" t="str">
-        <x:v>Deep Representation Learning; Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Privacy-preserving ML; Fairness &amp; Responsible AI</x:v>
-      </x:c>
+        <x:v>CogSci</x:v>
+      </x:c>
+      <x:c r="B20" s="20" t="str"/>
       <x:c r="C20" s="20" t="str">
-        <x:v>Theoretical foundations of learning at the intersection of computer science, statistics, and applied mathematics. Characteristic work studies learnability, sample and computational complexity, online learning, optimization, bandits, and generalization. Neural-network, causal, reinforcement-learning, privacy, and fairness papers belong here when the theoretical contribution is central.</x:v>
+        <x:v>Interdisciplinary study of cognition and the mind, connecting psychology, linguistics, artificial intelligence, neuroscience, philosophy, anthropology, and education. Computational models and experiments should illuminate cognitive processes and behavior. An AI paper belongs here through its contribution to understanding cognition, not solely through a predictive performance improvement.</x:v>
       </x:c>
       <x:c r="D20" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E20" s="20" t="str">
-        <x:v>https://learningtheory.org/colt2026/cfp.html</x:v>
+        <x:v>https://cognitivesciencesociety.org/submissions-faq/; https://cognitivesciencesociety.org/</x:v>
       </x:c>
       <x:c r="F20" s="22" t="n">
         <x:v>46302</x:v>
@@ -5049,279 +5521,277 @@
     </x:row>
     <x:row r="21" ht="60" hidden="0" customHeight="1">
       <x:c r="A21" s="20" t="str">
-        <x:v>CoNLL</x:v>
+        <x:v>COLING</x:v>
       </x:c>
       <x:c r="B21" s="20" t="str">
-        <x:v>Deep Representation Learning; Multimedia Learning &amp; Retrieval</x:v>
+        <x:v>Information Retrieval &amp; Search; Cognitive Science &amp; Computational Cognition; Explainability &amp; Interpretability; Fairness &amp; Responsible AI</x:v>
       </x:c>
       <x:c r="C21" s="20" t="str">
-        <x:v>Scientifically, cognitively, and linguistically motivated computational language learning. Characteristic work concerns language acquisition, psycholinguistics, grammars and meaning, multilinguality, language and the brain, and grounded language models. This is a focused scientific NLP venue rather than a generic empirical language-model benchmark conference.</x:v>
+        <x:v>Computational linguistics and language processing spanning linguistic theory, multilinguality, semantics and structured prediction, language models, dialogue, and empirical evaluation. Agentic language systems and knowledge-grounded NLP are relevant; the defining contribution should concern language, not a peripheral application domain.</x:v>
       </x:c>
       <x:c r="D21" s="21" t="n">
-        <x:v>2026</x:v>
+        <x:v>2027</x:v>
       </x:c>
       <x:c r="E21" s="20" t="str">
-        <x:v>https://www.conll.org/2026</x:v>
+        <x:v>https://2027.coling-iccl.org/calls/main_conference_papers/</x:v>
       </x:c>
       <x:c r="F21" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="72" hidden="0" customHeight="1">
+    <x:row r="22" ht="60" hidden="0" customHeight="1">
       <x:c r="A22" s="20" t="str">
-        <x:v>CoRL</x:v>
+        <x:v>COLM</x:v>
       </x:c>
       <x:c r="B22" s="20" t="str">
-        <x:v>Computer Vision &amp; Pattern Recognition; Probabilistic, Causal &amp; Uncertainty ML; Human-AI Interaction &amp; Deployment; Robustness &amp; Safety; Learning Theory &amp; Statistical Foundations</x:v>
+        <x:v>Learning Theory &amp; Statistical Foundations; Explainability &amp; Interpretability; Robustness &amp; Safety; Fairness &amp; Responsible AI; Multimedia Learning &amp; Retrieval</x:v>
       </x:c>
       <x:c r="C22" s="20" t="str">
-        <x:v>Machine learning for physical robots, especially imitation and reinforcement learning, learned perception and control, robot foundation models, and learning-based task and motion planning. Includes uncertainty, generalization, safety, human-robot interaction, and datasets grounded in manipulation, navigation, or locomotion. General ML is relevant when it makes a substantive contribution to robot learning.</x:v>
+        <x:v>Language-model foundations and methods: training and architecture, data and scaling, inference and generation, evaluation, reasoning, retrieval augmentation, and tool-using language agents. Alignment, interpretability, and multimodal language models are meaningful extensions. A central language-model contribution distinguishes the conference from generic AI applications.</x:v>
       </x:c>
       <x:c r="D22" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E22" s="20" t="str">
-        <x:v>https://www.corl.org/contributions/call-for-papers</x:v>
+        <x:v>https://colm.cc/Conferences/2026/CallForPapers</x:v>
       </x:c>
       <x:c r="F22" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="72" hidden="0" customHeight="1">
+    <x:row r="23" ht="60" hidden="0" customHeight="1">
       <x:c r="A23" s="20" t="str">
-        <x:v>CVPR</x:v>
+        <x:v>COLT</x:v>
       </x:c>
       <x:c r="B23" s="20" t="str">
-        <x:v>Computer Graphics &amp; Visualization; Multimedia Learning &amp; Retrieval; Natural Language Processing &amp; LLMs; Biometrics &amp; Human Sensing; Robustness &amp; Safety</x:v>
+        <x:v>Deep Representation Learning; Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Privacy-preserving ML; Fairness &amp; Responsible AI</x:v>
       </x:c>
       <x:c r="C23" s="20" t="str">
-        <x:v>Broad computer vision and pattern recognition: visual representations, recognition and segmentation, 3D reconstruction, computational imaging, image and video generation, motion and tracking, and vision-language learning. Graphics, multimodal learning, human face/body understanding, and reliable vision are substantial recurring research areas. Peripheral application fields are not tagged merely because a long CFP mentions them.</x:v>
+        <x:v>Theoretical foundations of learning at the intersection of computer science, statistics, and applied mathematics. Characteristic work studies learnability, sample and computational complexity, online learning, optimization, bandits, and generalization. Neural-network, causal, reinforcement-learning, privacy, and fairness papers belong here when the theoretical contribution is central.</x:v>
       </x:c>
       <x:c r="D23" s="21" t="n">
-        <x:v>2027</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="E23" s="20" t="str">
-        <x:v>https://cvpr.thecvf.com/Conferences/2027/CallForPapers</x:v>
+        <x:v>https://learningtheory.org/colt2026/cfp.html</x:v>
       </x:c>
       <x:c r="F23" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="72" hidden="0" customHeight="1">
+    <x:row r="24" ht="48" hidden="0" customHeight="1">
       <x:c r="A24" s="20" t="str">
-        <x:v>EACL</x:v>
+        <x:v>CompleNet</x:v>
       </x:c>
       <x:c r="B24" s="20" t="str">
-        <x:v>Explainability &amp; Interpretability; Fairness &amp; Responsible AI; Cognitive Science &amp; Computational Cognition</x:v>
+        <x:v>Time Series &amp; Sequential Data; Data Mining &amp; Data Science; Machine Learning</x:v>
       </x:c>
       <x:c r="C24" s="20" t="str">
-        <x:v>Computational linguistics and natural language processing, including language modeling, multilingual processing, translation, dialogue, information extraction, semantics, and linguistic analysis. Human-centered evaluation, interpretability, and bias are relevant within language research. The reviewed 2027 theme strengthens connections to psycholinguistics and cognitive modeling; peripheral application domains are not extra tags.</x:v>
+        <x:v>Network science across mathematical, biological, technological and social systems, with characteristic interests in network dynamics, community structure, temporal and multilayer networks, network neuroscience and learning on networks. Long and short reviewed papers are distinct from abstract-only presentations.</x:v>
       </x:c>
       <x:c r="D24" s="21" t="n">
         <x:v>2027</x:v>
       </x:c>
       <x:c r="E24" s="20" t="str">
-        <x:v>https://2027.eacl.org/calls/papers/</x:v>
+        <x:v>https://complenet.github.io/cfp.html</x:v>
       </x:c>
       <x:c r="F24" s="22" t="n">
-        <x:v>46302</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="72" hidden="0" customHeight="1">
+        <x:v>46303</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="60" hidden="0" customHeight="1">
       <x:c r="A25" s="20" t="str">
-        <x:v>ECCV</x:v>
+        <x:v>COMPLEX NETWORKS</x:v>
       </x:c>
       <x:c r="B25" s="20" t="str">
-        <x:v>Computer Graphics &amp; Visualization; Multimedia Learning &amp; Retrieval; Natural Language Processing &amp; LLMs; Biometrics &amp; Human Sensing; Robustness &amp; Safety</x:v>
+        <x:v>Time Series &amp; Sequential Data; Machine Learning; Computational Neuroscience</x:v>
       </x:c>
       <x:c r="C25" s="20" t="str">
-        <x:v>Broad research in visual perception, representation learning, recognition, segmentation, 3D geometry and reconstruction, computational imaging, and image/video synthesis. Vision-language models, multimodal understanding, human motion and appearance, and robust visual systems extend this core. ECCV is the biennial European flagship for computer vision; the scope uses the actual published 2026 CFP, not an invented 2028 call.</x:v>
+        <x:v>Structure, inference and dynamics of complex networks, including community structure, multilayer and temporal networks, spreading processes, graph learning and network neuroscience. Network methods, rather than a broad inventory of every application, characterize the meeting. Full papers and extended abstracts have separate publication outcomes.</x:v>
       </x:c>
       <x:c r="D25" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E25" s="20" t="str">
-        <x:v>https://eccv.ecva.net/Conferences/2026/CallForPapers</x:v>
+        <x:v>https://complexnetworks.org/submission/</x:v>
       </x:c>
       <x:c r="F25" s="22" t="n">
-        <x:v>46302</x:v>
+        <x:v>46303</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="60" hidden="0" customHeight="1">
       <x:c r="A26" s="20" t="str">
-        <x:v>ECIR</x:v>
+        <x:v>CoNLL</x:v>
       </x:c>
       <x:c r="B26" s="20" t="str">
-        <x:v>Human-AI Interaction &amp; Deployment; Explainability &amp; Interpretability; Fairness &amp; Responsible AI; Multimedia Learning &amp; Retrieval</x:v>
+        <x:v>Deep Representation Learning; Multimedia Learning &amp; Retrieval</x:v>
       </x:c>
       <x:c r="C26" s="20" t="str">
-        <x:v>Information retrieval and ranking, recommendation, conversational search and RAG, user information interaction, system efficiency, and rigorous evaluation. The 2027 call explicitly includes language models and agentic retrieval workflows. Replicability and research-resource papers are distinct routes. Fairness and explainability concern information access rather than generic responsible-AI topics.</x:v>
+        <x:v>Scientifically, cognitively, and linguistically motivated computational language learning. Characteristic work concerns language acquisition, psycholinguistics, grammars and meaning, multilinguality, language and the brain, and grounded language models. This is a focused scientific NLP venue rather than a generic empirical language-model benchmark conference.</x:v>
       </x:c>
       <x:c r="D26" s="21" t="n">
-        <x:v>2027</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="E26" s="20" t="str">
-        <x:v>https://www.ecir2027.co.uk/call-for-full-papers</x:v>
+        <x:v>https://www.conll.org/2026</x:v>
       </x:c>
       <x:c r="F26" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="60" hidden="0" customHeight="1">
+    <x:row r="27" ht="72" hidden="0" customHeight="1">
       <x:c r="A27" s="20" t="str">
-        <x:v>EMNLP</x:v>
+        <x:v>CoRL</x:v>
       </x:c>
       <x:c r="B27" s="20" t="str">
-        <x:v>Explainability &amp; Interpretability; Fairness &amp; Responsible AI; Robustness &amp; Safety; Human-AI Interaction &amp; Deployment</x:v>
+        <x:v>Computer Vision &amp; Pattern Recognition; Probabilistic, Causal &amp; Uncertainty ML; Human-AI Interaction &amp; Deployment; Robustness &amp; Safety; Learning Theory &amp; Statistical Foundations</x:v>
       </x:c>
       <x:c r="C27" s="20" t="str">
-        <x:v>Empirical methods for language modeling and NLP, including generation, information extraction, multilinguality, dialogue, retrieval, and model evaluation. Interpretability, bias, and safety matter within language systems. Curated coverage emphasizes language methods and evidence rather than every application listed in the CFP.</x:v>
+        <x:v>Machine learning for physical robots, especially imitation and reinforcement learning, learned perception and control, robot foundation models, and learning-based task and motion planning. Includes uncertainty, generalization, safety, human-robot interaction, and datasets grounded in manipulation, navigation, or locomotion. General ML is relevant when it makes a substantive contribution to robot learning.</x:v>
       </x:c>
       <x:c r="D27" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E27" s="20" t="str">
-        <x:v>https://2026.emnlp.org/calls/main_conference_papers/</x:v>
+        <x:v>https://www.corl.org/contributions/call-for-papers</x:v>
       </x:c>
       <x:c r="F27" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="60" hidden="0" customHeight="1">
+    <x:row r="28" ht="72" hidden="0" customHeight="1">
       <x:c r="A28" s="20" t="str">
-        <x:v>EuroGP</x:v>
+        <x:v>CVPR</x:v>
       </x:c>
       <x:c r="B28" s="20" t="str">
-        <x:v>Learning Theory &amp; Statistical Foundations; Deep Representation Learning</x:v>
+        <x:v>Computer Graphics &amp; Visualization; Multimedia Learning &amp; Retrieval; Natural Language Processing &amp; LLMs; Biometrics &amp; Human Sensing; Robustness &amp; Safety</x:v>
       </x:c>
       <x:c r="C28" s="20" t="str">
-        <x:v>Genetic programming and evolutionary program synthesis, including symbolic regression, program representations and operators, surrogate-assisted search, multi-objective evolution, and interpretable learned programs. Evolutionary machine learning, AutoML pipelines, and neuroevolution connect this focused methodological community to ML. Application domains do not define its tags.</x:v>
+        <x:v>Broad computer vision and pattern recognition: visual representations, recognition and segmentation, 3D reconstruction, computational imaging, image and video generation, motion and tracking, and vision-language learning. Graphics, multimodal learning, human face/body understanding, and reliable vision are substantial recurring research areas. Peripheral application fields are not tagged merely because a long CFP mentions them.</x:v>
       </x:c>
       <x:c r="D28" s="21" t="n">
         <x:v>2027</x:v>
       </x:c>
       <x:c r="E28" s="20" t="str">
-        <x:v>https://www.evostar.org/2027/eurogp/</x:v>
+        <x:v>https://cvpr.thecvf.com/Conferences/2027/CallForPapers</x:v>
       </x:c>
       <x:c r="F28" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="72" hidden="0" customHeight="1">
+    <x:row r="29" ht="48" hidden="0" customHeight="1">
       <x:c r="A29" s="20" t="str">
-        <x:v>EUVIP</x:v>
+        <x:v>Dynamics Days Asia-Pacific</x:v>
       </x:c>
       <x:c r="B29" s="20" t="str">
-        <x:v>Multimedia Learning &amp; Retrieval; Computer Graphics &amp; Visualization; Biometrics &amp; Human Sensing; Robustness &amp; Safety</x:v>
+        <x:v>Machine Learning</x:v>
       </x:c>
       <x:c r="C29" s="20" t="str">
-        <x:v>Visual information processing across image, video, 3D, and unconventional sensing modalities. Its defining areas are computational imaging, restoration and enhancement, coding, recognition, multimodal fusion, and subjective/objective quality assessment. Rendering and visualizing data, human/biometric analysis, and robust evaluation are recurring strands. An extensive applications list is not treated as equal coverage of every application domain or every responsible-AI subtopic.</x:v>
+        <x:v>Nonlinear dynamics and nonequilibrium complex systems, including chaos, collective behavior, statistical physics and dynamics of learning. The latest verified meeting was linked to a broader Yukawa Institute workshop; its invited-talk format should not be mistaken for a verified open full-paper call.</x:v>
       </x:c>
       <x:c r="D29" s="21" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E29" s="20" t="str">
+        <x:v>https://www2.yukawa.kyoto-u.ac.jp/~frontier24/DDAP13/; https://dynamicsdays.info/ap/</x:v>
+      </x:c>
+      <x:c r="F29" s="22" t="n">
+        <x:v>46303</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="60" hidden="0" customHeight="1">
+      <x:c r="A30" s="20" t="str">
+        <x:v>Dynamics Days CAC</x:v>
+      </x:c>
+      <x:c r="B30" s="20" t="str"/>
+      <x:c r="C30" s="20" t="str">
+        <x:v>Fundamental nonlinear science and complex-system physics, including chaos, collective dynamics, statistical physics and biological systems. The Central Asian and Caucasian meeting promotes collaboration across nonlinear science and its physical applications. Its oral/poster submission form uses paper terminology, but the official date table specifies abstract submissions.</x:v>
+      </x:c>
+      <x:c r="D30" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
-      <x:c r="E29" s="20" t="str">
-        <x:v>https://euvip2026.github.io/C4P.pdf; https://euvip2026.github.io/calls/</x:v>
-      </x:c>
-      <x:c r="F29" s="22" t="n">
-        <x:v>46302</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" ht="84" hidden="0" customHeight="1">
-      <x:c r="A30" s="20" t="str">
-        <x:v>FG</x:v>
-      </x:c>
-      <x:c r="B30" s="20" t="str">
-        <x:v>Robustness &amp; Safety; Fairness &amp; Responsible AI; Computer Graphics &amp; Visualization; Explainability &amp; Interpretability</x:v>
-      </x:c>
-      <x:c r="C30" s="20" t="str">
-        <x:v>Face, gesture, body movement, and human behavior from images and video, including detection, tracking, recognition, facial expression and affect, pose and action analysis, and soft biometrics. Characteristic methods include advanced visual learning, generative modeling and neural rendering, multimodal fusion, and evaluation across demographic and acquisition conditions. Bias, interpretability, and robust recognition are directly tied to human sensing rather than generic application tags.</x:v>
-      </x:c>
-      <x:c r="D30" s="21" t="n">
-        <x:v>2027</x:v>
-      </x:c>
       <x:c r="E30" s="20" t="str">
-        <x:v>https://fg2027.ieee-biometrics.org/call-for-papers/</x:v>
+        <x:v>https://physics-congress.kz/dynamics_days</x:v>
       </x:c>
       <x:c r="F30" s="22" t="n">
-        <x:v>46302</x:v>
+        <x:v>46303</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="60" hidden="0" customHeight="1">
       <x:c r="A31" s="20" t="str">
-        <x:v>FMTS @ NeurIPS</x:v>
+        <x:v>Dynamics Days Europe</x:v>
       </x:c>
       <x:c r="B31" s="20" t="str">
-        <x:v>System Identification &amp; Data-driven Dynamics; Robustness &amp; Safety</x:v>
+        <x:v>Machine Learning; Computational Neuroscience; Control &amp; Robotics; Graphs &amp; Graph Learning</x:v>
       </x:c>
       <x:c r="C31" s="20" t="str">
-        <x:v>Foundation models for temporal systems, centered on long-horizon and probabilistic forecasting, temporal pretraining, generative simulation, irregularly sampled and multimodal sequences, and state-space architectures. Reliability is a defining theme: distribution shift, calibrated uncertainty, leakage-aware benchmarks, and consistency of simulated trajectories.</x:v>
+        <x:v>Theory and applications of nonlinear dynamics: chaos, bifurcations, synchronization, pattern formation, complex networks, stochastic dynamics and time-series analysis. ML and neurodynamics are characteristic interdisciplinary extensions. Contributed talks and posters use abstracts, while minisymposium proposals are organizer activity.</x:v>
       </x:c>
       <x:c r="D31" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E31" s="20" t="str">
-        <x:v>https://fmts-workshop.github.io/cfp.html</x:v>
+        <x:v>https://dde-2026.sci-meet.net/abstract-submission-2</x:v>
       </x:c>
       <x:c r="F31" s="22" t="n">
-        <x:v>46302</x:v>
+        <x:v>46303</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="60" hidden="0" customHeight="1">
       <x:c r="A32" s="20" t="str">
-        <x:v>GECCO</x:v>
+        <x:v>Dynamics Days LAC</x:v>
       </x:c>
       <x:c r="B32" s="20" t="str">
-        <x:v>Deep Representation Learning; Learning Theory &amp; Statistical Foundations</x:v>
+        <x:v>Machine Learning; Graphs &amp; Graph Learning; Control &amp; Robotics</x:v>
       </x:c>
       <x:c r="C32" s="20" t="str">
-        <x:v>Genetic and evolutionary computation, including genetic algorithms, genetic programming, swarm intelligence, evolutionary multiobjective and combinatorial optimization, metaheuristics, and neuroevolution. Machine learning is relevant through evolutionary learning and optimization, not as an unrestricted substitute for the conference's evolutionary-computation focus.</x:v>
+        <x:v>Nonlinear and complex systems across disciplines, including chaos, synchronization, networks, time series, neurodynamics and learning-based modeling. The Latin American and Caribbean meeting supports contributed scientific talks and posters through abstracts, with an explicit interest in cross-disciplinary nonlinear science.</x:v>
       </x:c>
       <x:c r="D32" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E32" s="20" t="str">
-        <x:v>https://gecco-2027.sigevo.org/Call+for+Papers</x:v>
+        <x:v>https://fisica.ufpr.br/DDaysLAC2026/page1.html</x:v>
       </x:c>
       <x:c r="F32" s="22" t="n">
-        <x:v>46302</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="72" hidden="0" customHeight="1">
+        <x:v>46303</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="48" hidden="0" customHeight="1">
       <x:c r="A33" s="20" t="str">
-        <x:v>ICAPS</x:v>
+        <x:v>Dynamics Days US</x:v>
       </x:c>
       <x:c r="B33" s="20" t="str">
-        <x:v>Probabilistic, Causal &amp; Uncertainty ML</x:v>
+        <x:v>Computational Neuroscience; Time Series &amp; Sequential Data</x:v>
       </x:c>
       <x:c r="C33" s="20" t="str">
-        <x:v>Automated planning and scheduling, heuristic search, constraint-based reasoning, temporal and hierarchical planning, and planning under uncertainty. Learning and foundation models fit when they substantially advance planning or scheduling, including model acquisition and search guidance. The main CFP explicitly excludes reinforcement-learning papers without a substantive planning contribution; general reward-based learning is not a blanket tag.</x:v>
+        <x:v>Single-track nonlinear science meeting on chaos, dynamical systems and their interdisciplinary applications. Contributed abstract selection and poster discussion connect mathematical methods with physical, biological and neural systems. It is an abstract-based meeting, not a routine archival full-paper proceedings venue.</x:v>
       </x:c>
       <x:c r="D33" s="21" t="n">
         <x:v>2027</x:v>
       </x:c>
       <x:c r="E33" s="20" t="str">
-        <x:v>https://icaps27.icaps-conference.org/calls/cfp/</x:v>
+        <x:v>https://www.ddays.org/2027/; https://www.ddays.org/2027/abstract-submission/</x:v>
       </x:c>
       <x:c r="F33" s="22" t="n">
-        <x:v>46302</x:v>
+        <x:v>46303</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="72" hidden="0" customHeight="1">
       <x:c r="A34" s="20" t="str">
-        <x:v>ICCV</x:v>
+        <x:v>EACL</x:v>
       </x:c>
       <x:c r="B34" s="20" t="str">
-        <x:v>Computer Graphics &amp; Visualization; Multimedia Learning &amp; Retrieval; Natural Language Processing &amp; LLMs; Biometrics &amp; Human Sensing; Robustness &amp; Safety</x:v>
+        <x:v>Explainability &amp; Interpretability; Fairness &amp; Responsible AI; Cognitive Science &amp; Computational Cognition</x:v>
       </x:c>
       <x:c r="C34" s="20" t="str">
-        <x:v>Broad computer vision, from geometry and computational imaging to visual learning, recognition, segmentation, generation, and video understanding. Vision-language and multimodal methods, visual graphics, face/body/gesture analysis, and reliable perception are substantial strands. It is a biennial flagship, not a general AI applications conference. The current scope is grounded in its 2025 CFP because the 2027 call is not yet published.</x:v>
+        <x:v>Computational linguistics and natural language processing, including language modeling, multilingual processing, translation, dialogue, information extraction, semantics, and linguistic analysis. Human-centered evaluation, interpretability, and bias are relevant within language research. The reviewed 2027 theme strengthens connections to psycholinguistics and cognitive modeling; peripheral application domains are not extra tags.</x:v>
       </x:c>
       <x:c r="D34" s="21" t="n">
-        <x:v>2025</x:v>
+        <x:v>2027</x:v>
       </x:c>
       <x:c r="E34" s="20" t="str">
-        <x:v>https://iccv.thecvf.com/Conferences/2025/CallForPapers</x:v>
+        <x:v>https://2027.eacl.org/calls/papers/</x:v>
       </x:c>
       <x:c r="F34" s="22" t="n">
         <x:v>46302</x:v>
@@ -5329,17 +5799,19 @@
     </x:row>
     <x:row r="35" ht="72" hidden="0" customHeight="1">
       <x:c r="A35" s="20" t="str">
-        <x:v>ICIP</x:v>
-      </x:c>
-      <x:c r="B35" s="20" t="str"/>
+        <x:v>ECCV</x:v>
+      </x:c>
+      <x:c r="B35" s="20" t="str">
+        <x:v>Computer Graphics &amp; Visualization; Multimedia Learning &amp; Retrieval; Natural Language Processing &amp; LLMs; Biometrics &amp; Human Sensing; Robustness &amp; Safety</x:v>
+      </x:c>
       <x:c r="C35" s="20" t="str">
-        <x:v>Image and video processing across theory, algorithms, and imaging systems. Characteristic problems include restoration, enhancement, reconstruction, registration, compression, quality assessment, and visual analysis. Learning methods and generative models are relevant when they advance image or video processing. The long list of imaging application domains is intentionally not converted into extra specialist-conference tags.</x:v>
+        <x:v>Broad research in visual perception, representation learning, recognition, segmentation, 3D geometry and reconstruction, computational imaging, and image/video synthesis. Vision-language models, multimodal understanding, human motion and appearance, and robust visual systems extend this core. ECCV is the biennial European flagship for computer vision; the scope uses the actual published 2026 CFP, not an invented 2028 call.</x:v>
       </x:c>
       <x:c r="D35" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E35" s="20" t="str">
-        <x:v>https://2026.ieeeicip.org/topics/</x:v>
+        <x:v>https://eccv.ecva.net/Conferences/2026/CallForPapers</x:v>
       </x:c>
       <x:c r="F35" s="22" t="n">
         <x:v>46302</x:v>
@@ -5347,19 +5819,19 @@
     </x:row>
     <x:row r="36" ht="60" hidden="0" customHeight="1">
       <x:c r="A36" s="20" t="str">
-        <x:v>ICLR</x:v>
+        <x:v>ECIR</x:v>
       </x:c>
       <x:c r="B36" s="20" t="str">
-        <x:v>Learning Theory &amp; Statistical Foundations; Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Natural Language Processing &amp; LLMs; Computer Vision &amp; Pattern Recognition; ML Systems &amp; Infrastructure</x:v>
+        <x:v>Human-AI Interaction &amp; Deployment; Explainability &amp; Interpretability; Fairness &amp; Responsible AI; Multimedia Learning &amp; Retrieval</x:v>
       </x:c>
       <x:c r="C36" s="20" t="str">
-        <x:v>Learning representations and understanding deep learning, with an emphasis on self-supervised learning, generative models, transfer and meta-learning, and the optimization and theory of learned representations. Language, vision, probabilistic modeling, and reinforcement learning are substantial areas, rather than unrelated application-domain tags.</x:v>
+        <x:v>Information retrieval and ranking, recommendation, conversational search and RAG, user information interaction, system efficiency, and rigorous evaluation. The 2027 call explicitly includes language models and agentic retrieval workflows. Replicability and research-resource papers are distinct routes. Fairness and explainability concern information access rather than generic responsible-AI topics.</x:v>
       </x:c>
       <x:c r="D36" s="21" t="n">
         <x:v>2027</x:v>
       </x:c>
       <x:c r="E36" s="20" t="str">
-        <x:v>https://iclr.cc/Conferences/2027/CallForPapers</x:v>
+        <x:v>https://www.ecir2027.co.uk/call-for-full-papers</x:v>
       </x:c>
       <x:c r="F36" s="22" t="n">
         <x:v>46302</x:v>
@@ -5367,99 +5839,99 @@
     </x:row>
     <x:row r="37" ht="60" hidden="0" customHeight="1">
       <x:c r="A37" s="20" t="str">
-        <x:v>ICML</x:v>
+        <x:v>EMNLP</x:v>
       </x:c>
       <x:c r="B37" s="20" t="str">
-        <x:v>Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Explainability &amp; Interpretability; Robustness &amp; Safety; ML Systems &amp; Infrastructure; Federated &amp; Distributed Learning</x:v>
+        <x:v>Explainability &amp; Interpretability; Fairness &amp; Responsible AI; Robustness &amp; Safety; Human-AI Interaction &amp; Deployment</x:v>
       </x:c>
       <x:c r="C37" s="20" t="str">
-        <x:v>Methodological and theoretical machine learning, including supervised and unsupervised learning, deep generative models, optimization, statistical learning theory, Bayesian methods, and reinforcement learning. Scalable systems and trustworthy learning are established parts of the scope; application papers should offer contributions of wider interest to ML.</x:v>
+        <x:v>Empirical methods for language modeling and NLP, including generation, information extraction, multilinguality, dialogue, retrieval, and model evaluation. Interpretability, bias, and safety matter within language systems. Curated coverage emphasizes language methods and evidence rather than every application listed in the CFP.</x:v>
       </x:c>
       <x:c r="D37" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E37" s="20" t="str">
-        <x:v>https://icml.cc/Conferences/2026/CallForPapers</x:v>
+        <x:v>https://2026.emnlp.org/calls/main_conference_papers/</x:v>
       </x:c>
       <x:c r="F37" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="38" ht="72" hidden="0" customHeight="1">
+    <x:row r="38" ht="60" hidden="0" customHeight="1">
       <x:c r="A38" s="20" t="str">
-        <x:v>ICMR</x:v>
+        <x:v>EuroGP</x:v>
       </x:c>
       <x:c r="B38" s="20" t="str">
-        <x:v>Data Mining &amp; Data Science; Natural Language Processing &amp; LLMs; Privacy-preserving ML</x:v>
+        <x:v>Learning Theory &amp; Statistical Foundations; Deep Representation Learning</x:v>
       </x:c>
       <x:c r="C38" s="20" t="str">
-        <x:v>Search and retrieval of multimedia and multimodal content. Characteristic work studies indexing, content understanding, query representations, cross-modal matching, relevance feedback, recommendation, and evaluation, with deep learning and multimodal models as important methods. Privacy-aware retrieval and knowledge discovery extend this core. The long applications list is not used to characterize ICMR as a medicine, finance, or travel venue.</x:v>
+        <x:v>Genetic programming and evolutionary program synthesis, including symbolic regression, program representations and operators, surrogate-assisted search, multi-objective evolution, and interpretable learned programs. Evolutionary machine learning, AutoML pipelines, and neuroevolution connect this focused methodological community to ML. Application domains do not define its tags.</x:v>
       </x:c>
       <x:c r="D38" s="21" t="n">
         <x:v>2027</x:v>
       </x:c>
       <x:c r="E38" s="20" t="str">
-        <x:v>https://www.icmr2027.org/cfc</x:v>
+        <x:v>https://www.evostar.org/2027/eurogp/</x:v>
       </x:c>
       <x:c r="F38" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="39" ht="60" hidden="0" customHeight="1">
+    <x:row r="39" ht="72" hidden="0" customHeight="1">
       <x:c r="A39" s="20" t="str">
-        <x:v>ICRA</x:v>
+        <x:v>EUVIP</x:v>
       </x:c>
       <x:c r="B39" s="20" t="str">
-        <x:v>Planning &amp; Search; Deep Representation Learning; Human-AI Interaction &amp; Deployment; Robustness &amp; Safety</x:v>
+        <x:v>Multimedia Learning &amp; Retrieval; Computer Graphics &amp; Visualization; Biometrics &amp; Human Sensing; Robustness &amp; Safety</x:v>
       </x:c>
       <x:c r="C39" s="20" t="str">
-        <x:v>Robotics and automation across perception, motion and manipulation, planning and control, human-robot interaction, and autonomous systems. Learning-based robotics, reinforcement and imitation learning, and data-driven models are relevant when they advance physical robotic capability. Generic ML with no robotics connection is not the core remit.</x:v>
+        <x:v>Visual information processing across image, video, 3D, and unconventional sensing modalities. Its defining areas are computational imaging, restoration and enhancement, coding, recognition, multimodal fusion, and subjective/objective quality assessment. Rendering and visualizing data, human/biometric analysis, and robust evaluation are recurring strands. An extensive applications list is not treated as equal coverage of every application domain or every responsible-AI subtopic.</x:v>
       </x:c>
       <x:c r="D39" s="21" t="n">
-        <x:v>2027</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="E39" s="20" t="str">
-        <x:v>https://2027.ieee-icra.org/contribute/call-for-icra-2027-papers-now-accepting-submissions/</x:v>
+        <x:v>https://euvip2026.github.io/C4P.pdf; https://euvip2026.github.io/calls/</x:v>
       </x:c>
       <x:c r="F39" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="40" ht="60" hidden="0" customHeight="1">
+    <x:row r="40" ht="84" hidden="0" customHeight="1">
       <x:c r="A40" s="20" t="str">
-        <x:v>IFAC SYSID</x:v>
+        <x:v>FG</x:v>
       </x:c>
       <x:c r="B40" s="20" t="str">
-        <x:v>Nonlinear Dynamics &amp; Chaos; Complex Systems &amp; Network Science</x:v>
+        <x:v>Robustness &amp; Safety; Fairness &amp; Responsible AI; Computer Graphics &amp; Visualization; Explainability &amp; Interpretability</x:v>
       </x:c>
       <x:c r="C40" s="20" t="str">
-        <x:v>System identification and data-driven modeling for dynamical systems and control. Characteristic themes include nonlinear identification, model reduction, identification software and benchmarks, learning across systems, and dynamic networks. Application tracks remain grounded in identifying or learning dynamical models, rather than becoming general-purpose domain conferences.</x:v>
+        <x:v>Face, gesture, body movement, and human behavior from images and video, including detection, tracking, recognition, facial expression and affect, pose and action analysis, and soft biometrics. Characteristic methods include advanced visual learning, generative modeling and neural rendering, multimodal fusion, and evaluation across demographic and acquisition conditions. Bias, interpretability, and robust recognition are directly tied to human sensing rather than generic application tags.</x:v>
       </x:c>
       <x:c r="D40" s="21" t="n">
         <x:v>2027</x:v>
       </x:c>
       <x:c r="E40" s="20" t="str">
-        <x:v>https://conferences.ifac-control.org/sysid2027/participate/</x:v>
+        <x:v>https://fg2027.ieee-biometrics.org/call-for-papers/</x:v>
       </x:c>
       <x:c r="F40" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="41" ht="84" hidden="0" customHeight="1">
+    <x:row r="41" ht="60" hidden="0" customHeight="1">
       <x:c r="A41" s="20" t="str">
-        <x:v>IJCB</x:v>
+        <x:v>FMTS @ NeurIPS</x:v>
       </x:c>
       <x:c r="B41" s="20" t="str">
-        <x:v>Machine Learning; Robustness &amp; Safety; Fairness &amp; Responsible AI; Explainability &amp; Interpretability; Federated &amp; Distributed Learning; Signal Processing</x:v>
+        <x:v>System Identification &amp; Data-driven Dynamics; Robustness &amp; Safety</x:v>
       </x:c>
       <x:c r="C41" s="20" t="str">
-        <x:v>Biometrics and identity science across face, fingerprint, iris, voice, gait, and behavioral modalities. Defining concerns include recognition and verification, multimodal fusion, presentation-attack and deepfake detection, biometric template security, privacy, demographic fairness, and rigorous benchmarking. Learned representations and foundation models are important methods; federated learning belongs here through secure biometric systems. Healthcare, banking, and robotics are applications, not blanket scope tags.</x:v>
+        <x:v>Foundation models for temporal systems, centered on long-horizon and probabilistic forecasting, temporal pretraining, generative simulation, irregularly sampled and multimodal sequences, and state-space architectures. Reliability is a defining theme: distribution shift, calibrated uncertainty, leakage-aware benchmarks, and consistency of simulated trajectories.</x:v>
       </x:c>
       <x:c r="D41" s="21" t="n">
-        <x:v>2027</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="E41" s="20" t="str">
-        <x:v>https://ijcb2027.ieee-biometrics.org/call-for-papers/</x:v>
+        <x:v>https://fmts-workshop.github.io/cfp.html</x:v>
       </x:c>
       <x:c r="F41" s="22" t="n">
         <x:v>46302</x:v>
@@ -5467,37 +5939,39 @@
     </x:row>
     <x:row r="42" ht="60" hidden="0" customHeight="1">
       <x:c r="A42" s="20" t="str">
-        <x:v>IJCNLP</x:v>
+        <x:v>GECCO</x:v>
       </x:c>
       <x:c r="B42" s="20" t="str">
-        <x:v>Cognitive Science &amp; Computational Cognition; Explainability &amp; Interpretability; Fairness &amp; Responsible AI; Human-AI Interaction &amp; Deployment</x:v>
+        <x:v>Deep Representation Learning; Learning Theory &amp; Statistical Foundations</x:v>
       </x:c>
       <x:c r="C42" s="20" t="str">
-        <x:v>Computational linguistics and natural-language technologies in the Asia-Pacific community, including multilingual and low-resource NLP, language modeling, generation, dialogue, structured prediction, and evaluation. The 2026 edition is jointly organized as AACL-IJCNLP. Alias identity is preserved without inheriting the separate ACL conference ranking.</x:v>
+        <x:v>Genetic and evolutionary computation, including genetic algorithms, genetic programming, swarm intelligence, evolutionary multiobjective and combinatorial optimization, metaheuristics, and neuroevolution. Machine learning is relevant through evolutionary learning and optimization, not as an unrestricted substitute for the conference's evolutionary-computation focus.</x:v>
       </x:c>
       <x:c r="D42" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E42" s="20" t="str">
-        <x:v>https://2026.aaclnet.org/calls/main_conference_papers/</x:v>
+        <x:v>https://gecco-2027.sigevo.org/Call+for+Papers</x:v>
       </x:c>
       <x:c r="F42" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="43" ht="60" hidden="0" customHeight="1">
+    <x:row r="43" ht="72" hidden="0" customHeight="1">
       <x:c r="A43" s="20" t="str">
-        <x:v>Interspeech</x:v>
-      </x:c>
-      <x:c r="B43" s="20" t="str"/>
+        <x:v>ICAPS</x:v>
+      </x:c>
+      <x:c r="B43" s="20" t="str">
+        <x:v>Probabilistic, Causal &amp; Uncertainty ML</x:v>
+      </x:c>
       <x:c r="C43" s="20" t="str">
-        <x:v>Speech science and speech technology, linking spoken-language research with computational methods for speech recognition, speech synthesis, and speech communication. Machine learning and language models are relevant through speech and spoken-language problems. The current 2027 overview emphasizes the relationship between speech research and spoken-language technologies.</x:v>
+        <x:v>Automated planning and scheduling, heuristic search, constraint-based reasoning, temporal and hierarchical planning, and planning under uncertainty. Learning and foundation models fit when they substantially advance planning or scheduling, including model acquisition and search guidance. The main CFP explicitly excludes reinforcement-learning papers without a substantive planning contribution; general reward-based learning is not a blanket tag.</x:v>
       </x:c>
       <x:c r="D43" s="21" t="n">
         <x:v>2027</x:v>
       </x:c>
       <x:c r="E43" s="20" t="str">
-        <x:v>https://interspeech2027.org/</x:v>
+        <x:v>https://icaps27.icaps-conference.org/calls/cfp/</x:v>
       </x:c>
       <x:c r="F43" s="22" t="n">
         <x:v>46302</x:v>
@@ -5505,59 +5979,57 @@
     </x:row>
     <x:row r="44" ht="60" hidden="0" customHeight="1">
       <x:c r="A44" s="20" t="str">
-        <x:v>ISWC</x:v>
+        <x:v>ICCN</x:v>
       </x:c>
       <x:c r="B44" s="20" t="str">
-        <x:v>Machine Learning; Explainability &amp; Interpretability</x:v>
+        <x:v>Systems &amp; Experimental Neuroscience</x:v>
       </x:c>
       <x:c r="C44" s="20" t="str">
-        <x:v>Semantic Web and linked-data research: ontologies, knowledge graphs, representation and reasoning, semantic integration, querying, and knowledge-supported AI. Graph learning is relevant through semantic data and knowledge structures; this is not the IEEE wearable-computing symposium with the same acronym.</x:v>
+        <x:v>Cognitive neurodynamics and the relation between neural dynamics, computation, cognition and behavior. The meeting connects theoretical and computational neuroscience with nonlinear dynamics and complex neural systems. Current submission and publication details require organizer confirmation; historical edited proceedings are not a guarantee for 2026.</x:v>
       </x:c>
       <x:c r="D44" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E44" s="20" t="str">
-        <x:v>https://iswc2026.semanticweb.org/calls/research</x:v>
+        <x:v>https://iccn2026.jp/; https://link.springer.com/book/10.1007/978-981-16-0317-4</x:v>
       </x:c>
       <x:c r="F44" s="22" t="n">
-        <x:v>46302</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="45" ht="60" hidden="0" customHeight="1">
+        <x:v>46303</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="72" hidden="0" customHeight="1">
       <x:c r="A45" s="20" t="str">
-        <x:v>KDD</x:v>
+        <x:v>ICCV</x:v>
       </x:c>
       <x:c r="B45" s="20" t="str">
-        <x:v>Deep Representation Learning; Natural Language Processing &amp; LLMs; Explainability &amp; Interpretability; Privacy-preserving ML; ML Systems &amp; Infrastructure</x:v>
+        <x:v>Computer Graphics &amp; Visualization; Multimedia Learning &amp; Retrieval; Natural Language Processing &amp; LLMs; Biometrics &amp; Human Sensing; Robustness &amp; Safety</x:v>
       </x:c>
       <x:c r="C45" s="20" t="str">
-        <x:v>Knowledge discovery and data science, centered on extracting useful structure from large, heterogeneous data. Characteristic areas include clustering, structured and relational learning, graph and text mining, recommender systems, scalable data analysis, and responsible data use. Generative AI is relevant when it advances data science, not simply because a paper uses an LLM.</x:v>
+        <x:v>Broad computer vision, from geometry and computational imaging to visual learning, recognition, segmentation, generation, and video understanding. Vision-language and multimodal methods, visual graphics, face/body/gesture analysis, and reliable perception are substantial strands. It is a biennial flagship, not a general AI applications conference. The current scope is grounded in its 2025 CFP because the 2027 call is not yet published.</x:v>
       </x:c>
       <x:c r="D45" s="21" t="n">
-        <x:v>2027</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="E45" s="20" t="str">
-        <x:v>https://kdd2027.kdd.org/research-track-call-for-papers/</x:v>
+        <x:v>https://iccv.thecvf.com/Conferences/2025/CallForPapers</x:v>
       </x:c>
       <x:c r="F45" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="46" ht="84" hidden="0" customHeight="1">
+    <x:row r="46" ht="72" hidden="0" customHeight="1">
       <x:c r="A46" s="20" t="str">
-        <x:v>KR</x:v>
-      </x:c>
-      <x:c r="B46" s="20" t="str">
-        <x:v>Machine Learning; Probabilistic, Causal &amp; Uncertainty ML; Planning &amp; Search</x:v>
-      </x:c>
+        <x:v>ICIP</x:v>
+      </x:c>
+      <x:c r="B46" s="20" t="str"/>
       <x:c r="C46" s="20" t="str">
-        <x:v>Formal and symbolic AI centered on representing knowledge and drawing justified conclusions: knowledge bases, description and non-classical logics, ontologies, non-monotonic reasoning, argumentation, belief revision, and reasoning about actions. Learning, uncertainty, and explanations matter when grounded in knowledge representation or reasoning. The last published CFP includes a KR Meets Machine Learning and Explanation track; this is not a general-purpose ML conference or a confirmed promise of that 2027 track.</x:v>
+        <x:v>Image and video processing across theory, algorithms, and imaging systems. Characteristic problems include restoration, enhancement, reconstruction, registration, compression, quality assessment, and visual analysis. Learning methods and generative models are relevant when they advance image or video processing. The long list of imaging application domains is intentionally not converted into extra specialist-conference tags.</x:v>
       </x:c>
       <x:c r="D46" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E46" s="20" t="str">
-        <x:v>https://kr.org/KR2026/call_main_track.html; https://kr.org/KR2026/</x:v>
+        <x:v>https://2026.ieeeicip.org/topics/</x:v>
       </x:c>
       <x:c r="F46" s="22" t="n">
         <x:v>46302</x:v>
@@ -5565,59 +6037,59 @@
     </x:row>
     <x:row r="47" ht="60" hidden="0" customHeight="1">
       <x:c r="A47" s="20" t="str">
-        <x:v>L4DC</x:v>
+        <x:v>ICLR</x:v>
       </x:c>
       <x:c r="B47" s="20" t="str">
-        <x:v>Learning Theory &amp; Statistical Foundations</x:v>
+        <x:v>Learning Theory &amp; Statistical Foundations; Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Natural Language Processing &amp; LLMs; Computer Vision &amp; Pattern Recognition; ML Systems &amp; Infrastructure</x:v>
       </x:c>
       <x:c r="C47" s="20" t="str">
-        <x:v>The interface of learning, dynamics, control, and optimization for physical and dynamical systems. Emphasizes foundations and methods for data-driven control and dynamical modeling, including theoretical, empirical, and applied contributions. Pure pattern recognition without a meaningful connection to dynamics or control is not the defining focus.</x:v>
+        <x:v>Learning representations and understanding deep learning, with an emphasis on self-supervised learning, generative models, transfer and meta-learning, and the optimization and theory of learned representations. Language, vision, probabilistic modeling, and reinforcement learning are substantial areas, rather than unrelated application-domain tags.</x:v>
       </x:c>
       <x:c r="D47" s="21" t="n">
         <x:v>2027</x:v>
       </x:c>
       <x:c r="E47" s="20" t="str">
-        <x:v>https://l4dc2027.control.ee.ethz.ch/home</x:v>
+        <x:v>https://iclr.cc/Conferences/2027/CallForPapers</x:v>
       </x:c>
       <x:c r="F47" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="48" ht="72" hidden="0" customHeight="1">
+    <x:row r="48" ht="60" hidden="0" customHeight="1">
       <x:c r="A48" s="20" t="str">
-        <x:v>LoG</x:v>
+        <x:v>ICML</x:v>
       </x:c>
       <x:c r="B48" s="20" t="str">
-        <x:v>Complex Systems &amp; Network Science; Probabilistic, Causal &amp; Uncertainty ML; Signal Processing; Robustness &amp; Safety; ML Systems &amp; Infrastructure</x:v>
+        <x:v>Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Explainability &amp; Interpretability; Robustness &amp; Safety; ML Systems &amp; Infrastructure; Federated &amp; Distributed Learning</x:v>
       </x:c>
       <x:c r="C48" s="20" t="str">
-        <x:v>Learning on graphs and geometry: graph neural networks, equivariant models, graph kernels, geometric and graph generative models, and statistical theory for structured data. Graph signal processing, causal graph models, robustness, and scalable graph-learning infrastructure are meaningful extensions. A graph or geometric contribution should remain central, even in an application such as language or molecular modeling.</x:v>
+        <x:v>Methodological and theoretical machine learning, including supervised and unsupervised learning, deep generative models, optimization, statistical learning theory, Bayesian methods, and reinforcement learning. Scalable systems and trustworthy learning are established parts of the scope; application papers should offer contributions of wider interest to ML.</x:v>
       </x:c>
       <x:c r="D48" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E48" s="20" t="str">
-        <x:v>https://logconference.org/cfp/</x:v>
+        <x:v>https://icml.cc/Conferences/2026/CallForPapers</x:v>
       </x:c>
       <x:c r="F48" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="49" ht="60" hidden="0" customHeight="1">
+    <x:row r="49" ht="72" hidden="0" customHeight="1">
       <x:c r="A49" s="20" t="str">
-        <x:v>LREC</x:v>
+        <x:v>ICMR</x:v>
       </x:c>
       <x:c r="B49" s="20" t="str">
-        <x:v>Multimedia Learning &amp; Retrieval; Fairness &amp; Responsible AI</x:v>
+        <x:v>Data Mining &amp; Data Science; Natural Language Processing &amp; LLMs; Privacy-preserving ML</x:v>
       </x:c>
       <x:c r="C49" s="20" t="str">
-        <x:v>Language resources, annotation, corpora and datasets, speech and multimodal resources, benchmarking, and evaluation for human-language technologies. Contributions often create or analyze reusable resources and methods for linguistic coverage and reliable assessment. The breadth of language applications is summarized without treating every domain as a defining topic.</x:v>
+        <x:v>Search and retrieval of multimedia and multimodal content. Characteristic work studies indexing, content understanding, query representations, cross-modal matching, relevance feedback, recommendation, and evaluation, with deep learning and multimodal models as important methods. Privacy-aware retrieval and knowledge discovery extend this core. The long applications list is not used to characterize ICMR as a medicine, finance, or travel venue.</x:v>
       </x:c>
       <x:c r="D49" s="21" t="n">
-        <x:v>2026</x:v>
+        <x:v>2027</x:v>
       </x:c>
       <x:c r="E49" s="20" t="str">
-        <x:v>https://lrec2026.info/third-call-for-papers/</x:v>
+        <x:v>https://www.icmr2027.org/cfc</x:v>
       </x:c>
       <x:c r="F49" s="22" t="n">
         <x:v>46302</x:v>
@@ -5625,19 +6097,19 @@
     </x:row>
     <x:row r="50" ht="60" hidden="0" customHeight="1">
       <x:c r="A50" s="20" t="str">
-        <x:v>MIDL</x:v>
+        <x:v>ICRA</x:v>
       </x:c>
       <x:c r="B50" s="20" t="str">
-        <x:v>Computer Vision &amp; Pattern Recognition; Probabilistic, Causal &amp; Uncertainty ML; Explainability &amp; Interpretability; Robustness &amp; Safety; Federated &amp; Distributed Learning</x:v>
+        <x:v>Planning &amp; Search; Deep Representation Learning; Human-AI Interaction &amp; Deployment; Robustness &amp; Safety</x:v>
       </x:c>
       <x:c r="C50" s="20" t="str">
-        <x:v>Deep learning for biomedical image analysis, especially segmentation, detection, reconstruction, registration, generative imaging, and learning from limited labels. Uncertainty, interpretability, multi-site learning, robustness, and clinical validation extend that imaging core. Multimodal foundation models are relevant when grounded in medical imaging.</x:v>
+        <x:v>Robotics and automation across perception, motion and manipulation, planning and control, human-robot interaction, and autonomous systems. Learning-based robotics, reinforcement and imitation learning, and data-driven models are relevant when they advance physical robotic capability. Generic ML with no robotics connection is not the core remit.</x:v>
       </x:c>
       <x:c r="D50" s="21" t="n">
-        <x:v>2026</x:v>
+        <x:v>2027</x:v>
       </x:c>
       <x:c r="E50" s="20" t="str">
-        <x:v>https://2026.midl.io/call-for-papers</x:v>
+        <x:v>https://2027.ieee-icra.org/contribute/call-for-icra-2027-papers-now-accepting-submissions/</x:v>
       </x:c>
       <x:c r="F50" s="22" t="n">
         <x:v>46302</x:v>
@@ -5645,59 +6117,59 @@
     </x:row>
     <x:row r="51" ht="60" hidden="0" customHeight="1">
       <x:c r="A51" s="20" t="str">
-        <x:v>MLSys</x:v>
+        <x:v>IEEE BioCAS</x:v>
       </x:c>
       <x:c r="B51" s="20" t="str">
-        <x:v>Reinforcement Learning; Privacy-preserving ML</x:v>
+        <x:v>EEG/MEG &amp; Neural Signals; Machine Learning; ML Systems &amp; Infrastructure</x:v>
       </x:c>
       <x:c r="C51" s="20" t="str">
-        <x:v>The intersection of machine learning and computer systems, including efficient training, inference and serving, compilers and runtimes, programming abstractions, specialized hardware, distributed learning, and system monitoring. LLM and agentic workloads are considered from a systems perspective. Both systems for ML and ML methods that improve computing systems are relevant.</x:v>
+        <x:v>Biomedical circuits, integrated systems and medical devices spanning biosignal acquisition and processing, neural interfaces, implants, bioelectronics and low-power or on-device biomedical computation. Brain-inspired hardware and machine learning are relevant when tied to biomedical engineering, rather than as generic algorithms.</x:v>
       </x:c>
       <x:c r="D51" s="21" t="n">
-        <x:v>2027</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="E51" s="20" t="str">
-        <x:v>https://mlsys.org/Conferences/2027/CallForResearchPapers</x:v>
+        <x:v>https://2026.ieee-biocas.org/2026/pages_submission/call_for_papers.vm; https://2027.ieee-biocas.org/</x:v>
       </x:c>
       <x:c r="F51" s="22" t="n">
-        <x:v>46302</x:v>
+        <x:v>46303</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="60" hidden="0" customHeight="1">
       <x:c r="A52" s="20" t="str">
-        <x:v>NAACL</x:v>
+        <x:v>IFAC SYSID</x:v>
       </x:c>
       <x:c r="B52" s="20" t="str">
-        <x:v>Autonomous Agents &amp; Multiagent Systems; Cognitive Science &amp; Computational Cognition; Fairness &amp; Responsible AI; Robustness &amp; Safety; Human-AI Interaction &amp; Deployment</x:v>
+        <x:v>Nonlinear Dynamics &amp; Chaos; Complex Systems &amp; Network Science</x:v>
       </x:c>
       <x:c r="C52" s="20" t="str">
-        <x:v>Language technologies and computational linguistics across the Americas community, covering multilingual and low-resource NLP, language models, dialogue, retrieval, evaluation, and linguistic analysis. The 2027 theme concerns language as a medium for agentic communication, not merely running multiple models. General application domains are not standalone specialist tags.</x:v>
+        <x:v>System identification and data-driven modeling for dynamical systems and control. Characteristic themes include nonlinear identification, model reduction, identification software and benchmarks, learning across systems, and dynamic networks. Application tracks remain grounded in identifying or learning dynamical models, rather than becoming general-purpose domain conferences.</x:v>
       </x:c>
       <x:c r="D52" s="21" t="n">
         <x:v>2027</x:v>
       </x:c>
       <x:c r="E52" s="20" t="str">
-        <x:v>https://2027.naacl.org/calls/main_conference_papers/</x:v>
+        <x:v>https://conferences.ifac-control.org/sysid2027/participate/</x:v>
       </x:c>
       <x:c r="F52" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="53" ht="60" hidden="0" customHeight="1">
+    <x:row r="53" ht="84" hidden="0" customHeight="1">
       <x:c r="A53" s="20" t="str">
-        <x:v>NeurIPS</x:v>
+        <x:v>IJCB</x:v>
       </x:c>
       <x:c r="B53" s="20" t="str">
-        <x:v>Learning Theory &amp; Statistical Foundations; Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Natural Language Processing &amp; LLMs; Computer Vision &amp; Pattern Recognition; ML Systems &amp; Infrastructure</x:v>
+        <x:v>Machine Learning; Robustness &amp; Safety; Fairness &amp; Responsible AI; Explainability &amp; Interpretability; Federated &amp; Distributed Learning; Signal Processing</x:v>
       </x:c>
       <x:c r="C53" s="20" t="str">
-        <x:v>Broad research in machine learning, especially deep and generative models, statistical foundations, optimization, probabilistic inference, and learning for decision-making. Language, vision, and scalable ML systems are important research communities. Interdisciplinary applications should contribute insight of wider interest to the machine-learning community.</x:v>
+        <x:v>Biometrics and identity science across face, fingerprint, iris, voice, gait, and behavioral modalities. Defining concerns include recognition and verification, multimodal fusion, presentation-attack and deepfake detection, biometric template security, privacy, demographic fairness, and rigorous benchmarking. Learned representations and foundation models are important methods; federated learning belongs here through secure biometric systems. Healthcare, banking, and robotics are applications, not blanket scope tags.</x:v>
       </x:c>
       <x:c r="D53" s="21" t="n">
-        <x:v>2026</x:v>
+        <x:v>2027</x:v>
       </x:c>
       <x:c r="E53" s="20" t="str">
-        <x:v>https://neurips.cc/Conferences/2026/CallForPapers</x:v>
+        <x:v>https://ijcb2027.ieee-biometrics.org/call-for-papers/</x:v>
       </x:c>
       <x:c r="F53" s="22" t="n">
         <x:v>46302</x:v>
@@ -5705,39 +6177,37 @@
     </x:row>
     <x:row r="54" ht="60" hidden="0" customHeight="1">
       <x:c r="A54" s="20" t="str">
-        <x:v>NOLTA</x:v>
+        <x:v>IJCNLP</x:v>
       </x:c>
       <x:c r="B54" s="20" t="str">
-        <x:v>Signal Processing; Evolutionary Computation &amp; Optimization</x:v>
+        <x:v>Cognitive Science &amp; Computational Cognition; Explainability &amp; Interpretability; Fairness &amp; Responsible AI; Human-AI Interaction &amp; Deployment</x:v>
       </x:c>
       <x:c r="C54" s="20" t="str">
-        <x:v>Nonlinear theory and its applications, centered on chaos, bifurcations, oscillations, synchronization, nonlinear circuits, and complex networks. Neural computation, evolutionary algorithms, control, and signal processing connect to this nonlinear-systems focus. Individual application examples are not taken as additional specialist identities.</x:v>
+        <x:v>Computational linguistics and natural-language technologies in the Asia-Pacific community, including multilingual and low-resource NLP, language modeling, generation, dialogue, structured prediction, and evaluation. The 2026 edition is jointly organized as AACL-IJCNLP. Alias identity is preserved without inheriting the separate ACL conference ranking.</x:v>
       </x:c>
       <x:c r="D54" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E54" s="20" t="str">
-        <x:v>https://nolta2026.org/</x:v>
+        <x:v>https://2026.aaclnet.org/calls/main_conference_papers/</x:v>
       </x:c>
       <x:c r="F54" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="55" ht="72" hidden="0" customHeight="1">
+    <x:row r="55" ht="60" hidden="0" customHeight="1">
       <x:c r="A55" s="20" t="str">
-        <x:v>ProbML</x:v>
-      </x:c>
-      <x:c r="B55" s="20" t="str">
-        <x:v>Deep Representation Learning; Reinforcement Learning; Time Series &amp; Sequential Data; Robustness &amp; Safety</x:v>
-      </x:c>
+        <x:v>Interspeech</x:v>
+      </x:c>
+      <x:c r="B55" s="20" t="str"/>
       <x:c r="C55" s="20" t="str">
-        <x:v>Probabilistic and Bayesian machine learning, emphasizing approximate inference, variational and Monte Carlo methods, Gaussian processes, graphical and state-space models, calibration, and decisions under uncertainty. Includes Bayesian optimization and uncertainty-aware deep learning. The reviewed 2026 application focus is healthcare and climate; probabilistic reasoning remains essential to a suitable contribution.</x:v>
+        <x:v>Speech science and speech technology, linking spoken-language research with computational methods for speech recognition, speech synthesis, and speech communication. Machine learning and language models are relevant through speech and spoken-language problems. The current 2027 overview emphasizes the relationship between speech research and spoken-language technologies.</x:v>
       </x:c>
       <x:c r="D55" s="21" t="n">
-        <x:v>2026</x:v>
+        <x:v>2027</x:v>
       </x:c>
       <x:c r="E55" s="20" t="str">
-        <x:v>https://probml.cc/call/</x:v>
+        <x:v>https://interspeech2027.org/</x:v>
       </x:c>
       <x:c r="F55" s="22" t="n">
         <x:v>46302</x:v>
@@ -5745,19 +6215,19 @@
     </x:row>
     <x:row r="56" ht="60" hidden="0" customHeight="1">
       <x:c r="A56" s="20" t="str">
-        <x:v>RecSys</x:v>
+        <x:v>ISWC</x:v>
       </x:c>
       <x:c r="B56" s="20" t="str">
-        <x:v>Time Series &amp; Sequential Data; Natural Language Processing &amp; LLMs; Fairness &amp; Responsible AI; Explainability &amp; Interpretability</x:v>
+        <x:v>Machine Learning; Explainability &amp; Interpretability</x:v>
       </x:c>
       <x:c r="C56" s="20" t="str">
-        <x:v>Recommendation and personalization: user-item modeling, collaborative and content-based methods, sequential and conversational recommendation, evaluation, and deployed recommendation systems. Human and economic impacts matter alongside algorithms. Sequential data is relevant specifically through recommendation behavior; this is not a general forecasting conference.</x:v>
+        <x:v>Semantic Web and linked-data research: ontologies, knowledge graphs, representation and reasoning, semantic integration, querying, and knowledge-supported AI. Graph learning is relevant through semantic data and knowledge structures; this is not the IEEE wearable-computing symposium with the same acronym.</x:v>
       </x:c>
       <x:c r="D56" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E56" s="20" t="str">
-        <x:v>https://recsys.acm.org/recsys26/call/</x:v>
+        <x:v>https://iswc2026.semanticweb.org/calls/research</x:v>
       </x:c>
       <x:c r="F56" s="22" t="n">
         <x:v>46302</x:v>
@@ -5765,79 +6235,79 @@
     </x:row>
     <x:row r="57" ht="60" hidden="0" customHeight="1">
       <x:c r="A57" s="20" t="str">
-        <x:v>RSS</x:v>
+        <x:v>KDD</x:v>
       </x:c>
       <x:c r="B57" s="20" t="str">
-        <x:v>Planning &amp; Search; Deep Representation Learning; Probabilistic, Causal &amp; Uncertainty ML; Robustness &amp; Safety</x:v>
+        <x:v>Deep Representation Learning; Natural Language Processing &amp; LLMs; Explainability &amp; Interpretability; Privacy-preserving ML; ML Systems &amp; Infrastructure</x:v>
       </x:c>
       <x:c r="C57" s="20" t="str">
-        <x:v>Focused robotics research linking perception, learning, planning, control, manipulation, and robot-system science. Reinforcement and imitation learning, model-based behavior, and reliable autonomous systems are characteristic intersections. The 2027 review process emphasizes a scientifically developed robotic hypothesis through gated initial and invited final submissions.</x:v>
+        <x:v>Knowledge discovery and data science, centered on extracting useful structure from large, heterogeneous data. Characteristic areas include clustering, structured and relational learning, graph and text mining, recommender systems, scalable data analysis, and responsible data use. Generative AI is relevant when it advances data science, not simply because a paper uses an LLM.</x:v>
       </x:c>
       <x:c r="D57" s="21" t="n">
         <x:v>2027</x:v>
       </x:c>
       <x:c r="E57" s="20" t="str">
-        <x:v>https://roboticsconference.org/information/cfp/</x:v>
+        <x:v>https://kdd2027.kdd.org/research-track-call-for-papers/</x:v>
       </x:c>
       <x:c r="F57" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="58" ht="60" hidden="0" customHeight="1">
+    <x:row r="58" ht="84" hidden="0" customHeight="1">
       <x:c r="A58" s="20" t="str">
-        <x:v>SaTML</x:v>
+        <x:v>KR</x:v>
       </x:c>
       <x:c r="B58" s="20" t="str">
-        <x:v>Machine Learning; ML Systems &amp; Infrastructure</x:v>
+        <x:v>Machine Learning; Probabilistic, Causal &amp; Uncertainty ML; Planning &amp; Search</x:v>
       </x:c>
       <x:c r="C58" s="20" t="str">
-        <x:v>Security, safety, and trustworthiness of machine learning. Characteristic work studies attacks and defenses, privacy, verification, ML-system security, fairness, interpretability, and trustworthy data curation. Theoretical, empirical, and applied papers must engage substantively with a safety or trustworthiness question; merely using an ML model is insufficient.</x:v>
+        <x:v>Formal and symbolic AI centered on representing knowledge and drawing justified conclusions: knowledge bases, description and non-classical logics, ontologies, non-monotonic reasoning, argumentation, belief revision, and reasoning about actions. Learning, uncertainty, and explanations matter when grounded in knowledge representation or reasoning. The last published CFP includes a KR Meets Machine Learning and Explanation track; this is not a general-purpose ML conference or a confirmed promise of that 2027 track.</x:v>
       </x:c>
       <x:c r="D58" s="21" t="n">
-        <x:v>2027</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="E58" s="20" t="str">
-        <x:v>https://satml.org/call-for-papers/</x:v>
+        <x:v>https://kr.org/KR2026/call_main_track.html; https://kr.org/KR2026/</x:v>
       </x:c>
       <x:c r="F58" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="59" ht="72" hidden="0" customHeight="1">
+    <x:row r="59" ht="60" hidden="0" customHeight="1">
       <x:c r="A59" s="20" t="str">
-        <x:v>SIGIR</x:v>
+        <x:v>L4DC</x:v>
       </x:c>
       <x:c r="B59" s="20" t="str">
-        <x:v>Multimedia Learning &amp; Retrieval; Human-AI Interaction &amp; Deployment; Fairness &amp; Responsible AI; ML Systems &amp; Infrastructure</x:v>
+        <x:v>Learning Theory &amp; Statistical Foundations</x:v>
       </x:c>
       <x:c r="C59" s="20" t="str">
-        <x:v>Information access, search and ranking, query and content understanding, recommendation, conversational and multimodal retrieval, and evaluation of retrieval systems. Learning and language models are relevant through an information-retrieval contribution, including retrieval-augmented generation. The 2027 detailed track pages contain organizer placeholders; scope should be rechecked when finalized.</x:v>
+        <x:v>The interface of learning, dynamics, control, and optimization for physical and dynamical systems. Emphasizes foundations and methods for data-driven control and dynamical modeling, including theoretical, empirical, and applied contributions. Pure pattern recognition without a meaningful connection to dynamics or control is not the defining focus.</x:v>
       </x:c>
       <x:c r="D59" s="21" t="n">
         <x:v>2027</x:v>
       </x:c>
       <x:c r="E59" s="20" t="str">
-        <x:v>https://sigir2027.org/pages/submit-full.html</x:v>
+        <x:v>https://l4dc2027.control.ee.ethz.ch/home</x:v>
       </x:c>
       <x:c r="F59" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="60" ht="60" hidden="0" customHeight="1">
+    <x:row r="60" ht="72" hidden="0" customHeight="1">
       <x:c r="A60" s="20" t="str">
-        <x:v>SMC</x:v>
+        <x:v>LoG</x:v>
       </x:c>
       <x:c r="B60" s="20" t="str">
-        <x:v>Reinforcement Learning; System Identification &amp; Data-driven Dynamics; BCI &amp; Neurotechnology; Cognitive Science &amp; Computational Cognition</x:v>
+        <x:v>Complex Systems &amp; Network Science; Probabilistic, Causal &amp; Uncertainty ML; Signal Processing; Robustness &amp; Safety; ML Systems &amp; Infrastructure</x:v>
       </x:c>
       <x:c r="C60" s="20" t="str">
-        <x:v>Systems science, cybernetics, and human-machine systems. Characteristic ML-facing work includes intelligent and learning-based control, autonomous systems, adaptive decision-making, and human-AI interaction; brain-machine interfaces and cognitive systems are meaningful extensions. Its interdisciplinary remit is curated without tagging every industrial application as a core specialty.</x:v>
+        <x:v>Learning on graphs and geometry: graph neural networks, equivariant models, graph kernels, geometric and graph generative models, and statistical theory for structured data. Graph signal processing, causal graph models, robustness, and scalable graph-learning infrastructure are meaningful extensions. A graph or geometric contribution should remain central, even in an application such as language or molecular modeling.</x:v>
       </x:c>
       <x:c r="D60" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E60" s="20" t="str">
-        <x:v>https://www.ieeesmc2026.org/call-for-papers</x:v>
+        <x:v>https://logconference.org/cfp/</x:v>
       </x:c>
       <x:c r="F60" s="22" t="n">
         <x:v>46302</x:v>
@@ -5845,39 +6315,39 @@
     </x:row>
     <x:row r="61" ht="60" hidden="0" customHeight="1">
       <x:c r="A61" s="20" t="str">
-        <x:v>UAI</x:v>
+        <x:v>LREC</x:v>
       </x:c>
       <x:c r="B61" s="20" t="str">
-        <x:v>Deep Representation Learning; Reinforcement Learning; Time Series &amp; Sequential Data; Explainability &amp; Interpretability; Robustness &amp; Safety</x:v>
+        <x:v>Multimedia Learning &amp; Retrieval; Fairness &amp; Responsible AI</x:v>
       </x:c>
       <x:c r="C61" s="20" t="str">
-        <x:v>Learning and reasoning under uncertainty, centered on probabilistic and Bayesian modeling, graphical models, causal inference, approximate inference, and decision theory. Includes Monte Carlo and variational methods, uncertainty quantification, sequential models, and principled analysis of learning algorithms. Uncertainty is the organizing theme, not just another application of general-purpose AI.</x:v>
+        <x:v>Language resources, annotation, corpora and datasets, speech and multimodal resources, benchmarking, and evaluation for human-language technologies. Contributions often create or analyze reusable resources and methods for linguistic coverage and reliable assessment. The breadth of language applications is summarized without treating every domain as a defining topic.</x:v>
       </x:c>
       <x:c r="D61" s="21" t="n">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="E61" s="20" t="str">
-        <x:v>https://www.auai.org/uai2026/subject_areas; https://www.auai.org/uai2026/call_for_papers</x:v>
+        <x:v>https://lrec2026.info/third-call-for-papers/</x:v>
       </x:c>
       <x:c r="F61" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
-    <x:row r="62" ht="72" hidden="0" customHeight="1">
+    <x:row r="62" ht="60" hidden="0" customHeight="1">
       <x:c r="A62" s="20" t="str">
-        <x:v>WACV</x:v>
+        <x:v>MIDL</x:v>
       </x:c>
       <x:c r="B62" s="20" t="str">
-        <x:v>Signal Processing; Biometrics &amp; Human Sensing; Multimedia Learning &amp; Retrieval</x:v>
+        <x:v>Computer Vision &amp; Pattern Recognition; Probabilistic, Causal &amp; Uncertainty ML; Explainability &amp; Interpretability; Robustness &amp; Safety; Federated &amp; Distributed Learning</x:v>
       </x:c>
       <x:c r="C62" s="20" t="str">
-        <x:v>Applied computer vision and visual learning, with an emphasis on practical recognition, detection, segmentation, image/video analysis, 3D perception, and deployable visual systems. Human analysis and multimodal visual methods are established areas. Compared with the flagship trio, WACV particularly welcomes meaningful application-driven contributions supported by sound evaluation; its two submission rounds are routes, not different fields.</x:v>
+        <x:v>Deep learning for biomedical image analysis, especially segmentation, detection, reconstruction, registration, generative imaging, and learning from limited labels. Uncertainty, interpretability, multi-site learning, robustness, and clinical validation extend that imaging core. Multimodal foundation models are relevant when grounded in medical imaging.</x:v>
       </x:c>
       <x:c r="D62" s="21" t="n">
-        <x:v>2027</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="E62" s="20" t="str">
-        <x:v>https://wacv.thecvf.com/Conferences/2027/CallForPapers</x:v>
+        <x:v>https://2026.midl.io/call-for-papers</x:v>
       </x:c>
       <x:c r="F62" s="22" t="n">
         <x:v>46302</x:v>
@@ -5885,19 +6355,19 @@
     </x:row>
     <x:row r="63" ht="60" hidden="0" customHeight="1">
       <x:c r="A63" s="20" t="str">
-        <x:v>WSDM</x:v>
+        <x:v>MLSys</x:v>
       </x:c>
       <x:c r="B63" s="20" t="str">
-        <x:v>Information Retrieval &amp; Search; Recommender Systems; Graphs &amp; Graph Learning; LLM Agents &amp; Tool Use; Natural Language Processing &amp; LLMs</x:v>
+        <x:v>Reinforcement Learning; Privacy-preserving ML</x:v>
       </x:c>
       <x:c r="C63" s="20" t="str">
-        <x:v>Web search, ranking, recommendation and mining of web and social data. Characteristic extensions include large-scale graph analysis, conversational retrieval, foundation-model and agentic web systems, and fairness and privacy in information access. The broad emerging-applications inventory is not treated as evidence that WSDM is a specialist healthcare or climate venue.</x:v>
+        <x:v>The intersection of machine learning and computer systems, including efficient training, inference and serving, compilers and runtimes, programming abstractions, specialized hardware, distributed learning, and system monitoring. LLM and agentic workloads are considered from a systems perspective. Both systems for ML and ML methods that improve computing systems are relevant.</x:v>
       </x:c>
       <x:c r="D63" s="21" t="n">
         <x:v>2027</x:v>
       </x:c>
       <x:c r="E63" s="20" t="str">
-        <x:v>https://www.wsdm-conference.org/2027/cffp.html</x:v>
+        <x:v>https://mlsys.org/Conferences/2027/CallForResearchPapers</x:v>
       </x:c>
       <x:c r="F63" s="22" t="n">
         <x:v>46302</x:v>
@@ -5905,28 +6375,348 @@
     </x:row>
     <x:row r="64" ht="60" hidden="0" customHeight="1">
       <x:c r="A64" s="20" t="str">
-        <x:v>WWW</x:v>
+        <x:v>NAACL</x:v>
       </x:c>
       <x:c r="B64" s="20" t="str">
-        <x:v>Knowledge Representation &amp; Reasoning; Data Mining &amp; Data Science; Fairness &amp; Responsible AI; Privacy-preserving ML; Ethics &amp; Governance</x:v>
+        <x:v>Autonomous Agents &amp; Multiagent Systems; Cognitive Science &amp; Computational Cognition; Fairness &amp; Responsible AI; Robustness &amp; Safety; Human-AI Interaction &amp; Deployment</x:v>
       </x:c>
       <x:c r="C64" s="20" t="str">
-        <x:v>Research on the Web as infrastructure and a socio-technical ecosystem. Characteristic ML-facing tracks include search and recommendation, retrieval-augmented and agentic information access, graph learning, and semantic knowledge. Responsible Web and privacy research are substantive strands. Merely using a web dataset or API is explicitly insufficient topical relevance.</x:v>
+        <x:v>Language technologies and computational linguistics across the Americas community, covering multilingual and low-resource NLP, language models, dialogue, retrieval, evaluation, and linguistic analysis. The 2027 theme concerns language as a medium for agentic communication, not merely running multiple models. General application domains are not standalone specialist tags.</x:v>
       </x:c>
       <x:c r="D64" s="21" t="n">
         <x:v>2027</x:v>
       </x:c>
       <x:c r="E64" s="20" t="str">
+        <x:v>https://2027.naacl.org/calls/main_conference_papers/</x:v>
+      </x:c>
+      <x:c r="F64" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="60" hidden="0" customHeight="1">
+      <x:c r="A65" s="20" t="str">
+        <x:v>NeurIPS</x:v>
+      </x:c>
+      <x:c r="B65" s="20" t="str">
+        <x:v>Learning Theory &amp; Statistical Foundations; Probabilistic, Causal &amp; Uncertainty ML; Reinforcement Learning; Natural Language Processing &amp; LLMs; Computer Vision &amp; Pattern Recognition; ML Systems &amp; Infrastructure</x:v>
+      </x:c>
+      <x:c r="C65" s="20" t="str">
+        <x:v>Broad research in machine learning, especially deep and generative models, statistical foundations, optimization, probabilistic inference, and learning for decision-making. Language, vision, and scalable ML systems are important research communities. Interdisciplinary applications should contribute insight of wider interest to the machine-learning community.</x:v>
+      </x:c>
+      <x:c r="D65" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E65" s="20" t="str">
+        <x:v>https://neurips.cc/Conferences/2026/CallForPapers</x:v>
+      </x:c>
+      <x:c r="F65" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="60" hidden="0" customHeight="1">
+      <x:c r="A66" s="20" t="str">
+        <x:v>NICE</x:v>
+      </x:c>
+      <x:c r="B66" s="20" t="str">
+        <x:v>ML Systems &amp; Infrastructure; Deep Representation Learning; Control &amp; Robotics</x:v>
+      </x:c>
+      <x:c r="C66" s="20" t="str">
+        <x:v>Neuromorphic and brain-inspired computing at the intersection of neuroscience, algorithms and hardware. Characteristic work includes spiking neural networks, learning in neural systems, event-driven computation, neuromorphic processors and embodied applications. Research papers and late-breaking abstracts are different contribution routes.</x:v>
+      </x:c>
+      <x:c r="D66" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E66" s="20" t="str">
+        <x:v>https://easychair.org/cfp/nice2027</x:v>
+      </x:c>
+      <x:c r="F66" s="22" t="n">
+        <x:v>46303</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="60" hidden="0" customHeight="1">
+      <x:c r="A67" s="20" t="str">
+        <x:v>NODYCON</x:v>
+      </x:c>
+      <x:c r="B67" s="20" t="str">
+        <x:v>Time Series &amp; Sequential Data; Machine Learning</x:v>
+      </x:c>
+      <x:c r="C67" s="20" t="str">
+        <x:v>Nonlinear dynamics in engineering and physical systems: bifurcations, chaos, vibrations, synchronization, nonlinear control, system identification and data-driven dynamical modeling. Machine learning is relevant through discovering, forecasting or controlling dynamics. Publication is edition-specific: past Springer volumes do not imply that every later meeting has standard proceedings.</x:v>
+      </x:c>
+      <x:c r="D67" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E67" s="20" t="str">
+        <x:v>https://www.sisco-scienzadellecostruzioni.org/index.php/eventi/prossimi-eventi/conferenza/nodycon-2026</x:v>
+      </x:c>
+      <x:c r="F67" s="22" t="n">
+        <x:v>46303</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="60" hidden="0" customHeight="1">
+      <x:c r="A68" s="20" t="str">
+        <x:v>NOLTA</x:v>
+      </x:c>
+      <x:c r="B68" s="20" t="str">
+        <x:v>Signal Processing; Evolutionary Computation &amp; Optimization</x:v>
+      </x:c>
+      <x:c r="C68" s="20" t="str">
+        <x:v>Nonlinear theory and its applications, centered on chaos, bifurcations, oscillations, synchronization, nonlinear circuits, and complex networks. Neural computation, evolutionary algorithms, control, and signal processing connect to this nonlinear-systems focus. Individual application examples are not taken as additional specialist identities.</x:v>
+      </x:c>
+      <x:c r="D68" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E68" s="20" t="str">
+        <x:v>https://nolta2026.org/</x:v>
+      </x:c>
+      <x:c r="F68" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="72" hidden="0" customHeight="1">
+      <x:c r="A69" s="20" t="str">
+        <x:v>ProbML</x:v>
+      </x:c>
+      <x:c r="B69" s="20" t="str">
+        <x:v>Deep Representation Learning; Reinforcement Learning; Time Series &amp; Sequential Data; Robustness &amp; Safety</x:v>
+      </x:c>
+      <x:c r="C69" s="20" t="str">
+        <x:v>Probabilistic and Bayesian machine learning, emphasizing approximate inference, variational and Monte Carlo methods, Gaussian processes, graphical and state-space models, calibration, and decisions under uncertainty. Includes Bayesian optimization and uncertainty-aware deep learning. The reviewed 2026 application focus is healthcare and climate; probabilistic reasoning remains essential to a suitable contribution.</x:v>
+      </x:c>
+      <x:c r="D69" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E69" s="20" t="str">
+        <x:v>https://probml.cc/call/</x:v>
+      </x:c>
+      <x:c r="F69" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="60" hidden="0" customHeight="1">
+      <x:c r="A70" s="20" t="str">
+        <x:v>RecSys</x:v>
+      </x:c>
+      <x:c r="B70" s="20" t="str">
+        <x:v>Time Series &amp; Sequential Data; Natural Language Processing &amp; LLMs; Fairness &amp; Responsible AI; Explainability &amp; Interpretability</x:v>
+      </x:c>
+      <x:c r="C70" s="20" t="str">
+        <x:v>Recommendation and personalization: user-item modeling, collaborative and content-based methods, sequential and conversational recommendation, evaluation, and deployed recommendation systems. Human and economic impacts matter alongside algorithms. Sequential data is relevant specifically through recommendation behavior; this is not a general forecasting conference.</x:v>
+      </x:c>
+      <x:c r="D70" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E70" s="20" t="str">
+        <x:v>https://recsys.acm.org/recsys26/call/</x:v>
+      </x:c>
+      <x:c r="F70" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="60" hidden="0" customHeight="1">
+      <x:c r="A71" s="20" t="str">
+        <x:v>RSS</x:v>
+      </x:c>
+      <x:c r="B71" s="20" t="str">
+        <x:v>Planning &amp; Search; Deep Representation Learning; Probabilistic, Causal &amp; Uncertainty ML; Robustness &amp; Safety</x:v>
+      </x:c>
+      <x:c r="C71" s="20" t="str">
+        <x:v>Focused robotics research linking perception, learning, planning, control, manipulation, and robot-system science. Reinforcement and imitation learning, model-based behavior, and reliable autonomous systems are characteristic intersections. The 2027 review process emphasizes a scientifically developed robotic hypothesis through gated initial and invited final submissions.</x:v>
+      </x:c>
+      <x:c r="D71" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E71" s="20" t="str">
+        <x:v>https://roboticsconference.org/information/cfp/</x:v>
+      </x:c>
+      <x:c r="F71" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="48" hidden="0" customHeight="1">
+      <x:c r="A72" s="20" t="str">
+        <x:v>SAB</x:v>
+      </x:c>
+      <x:c r="B72" s="20" t="str">
+        <x:v>Machine Learning; Reinforcement Learning; Autonomous Agents &amp; Multiagent Systems</x:v>
+      </x:c>
+      <x:c r="C72" s="20" t="str">
+        <x:v>Understanding adaptive behavior through biological and artificial agents, including embodied cognition, neural and computational models, robotics, learning, evolution and collective behavior. The biennial ISAB meeting combines archival proceedings papers with deliberately non-archival contributions and poster abstracts.</x:v>
+      </x:c>
+      <x:c r="D72" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E72" s="20" t="str">
+        <x:v>https://sab-conference.org/call-for-contributions/</x:v>
+      </x:c>
+      <x:c r="F72" s="22" t="n">
+        <x:v>46303</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="60" hidden="0" customHeight="1">
+      <x:c r="A73" s="20" t="str">
+        <x:v>SaTML</x:v>
+      </x:c>
+      <x:c r="B73" s="20" t="str">
+        <x:v>Machine Learning; ML Systems &amp; Infrastructure</x:v>
+      </x:c>
+      <x:c r="C73" s="20" t="str">
+        <x:v>Security, safety, and trustworthiness of machine learning. Characteristic work studies attacks and defenses, privacy, verification, ML-system security, fairness, interpretability, and trustworthy data curation. Theoretical, empirical, and applied papers must engage substantively with a safety or trustworthiness question; merely using an ML model is insufficient.</x:v>
+      </x:c>
+      <x:c r="D73" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E73" s="20" t="str">
+        <x:v>https://satml.org/call-for-papers/</x:v>
+      </x:c>
+      <x:c r="F73" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="60" hidden="0" customHeight="1">
+      <x:c r="A74" s="20" t="str">
+        <x:v>SfN Neuroscience</x:v>
+      </x:c>
+      <x:c r="B74" s="20" t="str">
+        <x:v>EEG/MEG &amp; Neural Signals; BCI &amp; Neurotechnology</x:v>
+      </x:c>
+      <x:c r="C74" s="20" t="str">
+        <x:v>Broad neuroscience annual meeting spanning molecular and cellular neuroscience, neural circuits, systems and behavioral neuroscience, cognition, development and disease. Computational neuroscience, neuroimaging and neurotechnology are relevant parts of this broad remit, not its exclusive identity. Research abstracts are presented and archived; they are not standard full-paper conference proceedings.</x:v>
+      </x:c>
+      <x:c r="D74" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E74" s="20" t="str">
+        <x:v>https://www.sfn.org/cfa; https://www.sfn.org/meetings</x:v>
+      </x:c>
+      <x:c r="F74" s="22" t="n">
+        <x:v>46303</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="72" hidden="0" customHeight="1">
+      <x:c r="A75" s="20" t="str">
+        <x:v>SIGIR</x:v>
+      </x:c>
+      <x:c r="B75" s="20" t="str">
+        <x:v>Multimedia Learning &amp; Retrieval; Human-AI Interaction &amp; Deployment; Fairness &amp; Responsible AI; ML Systems &amp; Infrastructure</x:v>
+      </x:c>
+      <x:c r="C75" s="20" t="str">
+        <x:v>Information access, search and ranking, query and content understanding, recommendation, conversational and multimodal retrieval, and evaluation of retrieval systems. Learning and language models are relevant through an information-retrieval contribution, including retrieval-augmented generation. The 2027 detailed track pages contain organizer placeholders; scope should be rechecked when finalized.</x:v>
+      </x:c>
+      <x:c r="D75" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E75" s="20" t="str">
+        <x:v>https://sigir2027.org/pages/submit-full.html</x:v>
+      </x:c>
+      <x:c r="F75" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="60" hidden="0" customHeight="1">
+      <x:c r="A76" s="20" t="str">
+        <x:v>SMC</x:v>
+      </x:c>
+      <x:c r="B76" s="20" t="str">
+        <x:v>Reinforcement Learning; System Identification &amp; Data-driven Dynamics; BCI &amp; Neurotechnology; Cognitive Science &amp; Computational Cognition</x:v>
+      </x:c>
+      <x:c r="C76" s="20" t="str">
+        <x:v>Systems science, cybernetics, and human-machine systems. Characteristic ML-facing work includes intelligent and learning-based control, autonomous systems, adaptive decision-making, and human-AI interaction; brain-machine interfaces and cognitive systems are meaningful extensions. Its interdisciplinary remit is curated without tagging every industrial application as a core specialty.</x:v>
+      </x:c>
+      <x:c r="D76" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E76" s="20" t="str">
+        <x:v>https://www.ieeesmc2026.org/call-for-papers</x:v>
+      </x:c>
+      <x:c r="F76" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="60" hidden="0" customHeight="1">
+      <x:c r="A77" s="20" t="str">
+        <x:v>UAI</x:v>
+      </x:c>
+      <x:c r="B77" s="20" t="str">
+        <x:v>Deep Representation Learning; Reinforcement Learning; Time Series &amp; Sequential Data; Explainability &amp; Interpretability; Robustness &amp; Safety</x:v>
+      </x:c>
+      <x:c r="C77" s="20" t="str">
+        <x:v>Learning and reasoning under uncertainty, centered on probabilistic and Bayesian modeling, graphical models, causal inference, approximate inference, and decision theory. Includes Monte Carlo and variational methods, uncertainty quantification, sequential models, and principled analysis of learning algorithms. Uncertainty is the organizing theme, not just another application of general-purpose AI.</x:v>
+      </x:c>
+      <x:c r="D77" s="21" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E77" s="20" t="str">
+        <x:v>https://www.auai.org/uai2026/subject_areas; https://www.auai.org/uai2026/call_for_papers</x:v>
+      </x:c>
+      <x:c r="F77" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="72" hidden="0" customHeight="1">
+      <x:c r="A78" s="20" t="str">
+        <x:v>WACV</x:v>
+      </x:c>
+      <x:c r="B78" s="20" t="str">
+        <x:v>Signal Processing; Biometrics &amp; Human Sensing; Multimedia Learning &amp; Retrieval</x:v>
+      </x:c>
+      <x:c r="C78" s="20" t="str">
+        <x:v>Applied computer vision and visual learning, with an emphasis on practical recognition, detection, segmentation, image/video analysis, 3D perception, and deployable visual systems. Human analysis and multimodal visual methods are established areas. Compared with the flagship trio, WACV particularly welcomes meaningful application-driven contributions supported by sound evaluation; its two submission rounds are routes, not different fields.</x:v>
+      </x:c>
+      <x:c r="D78" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E78" s="20" t="str">
+        <x:v>https://wacv.thecvf.com/Conferences/2027/CallForPapers</x:v>
+      </x:c>
+      <x:c r="F78" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="60" hidden="0" customHeight="1">
+      <x:c r="A79" s="20" t="str">
+        <x:v>WSDM</x:v>
+      </x:c>
+      <x:c r="B79" s="20" t="str">
+        <x:v>Information Retrieval &amp; Search; Recommender Systems; Graphs &amp; Graph Learning; LLM Agents &amp; Tool Use; Natural Language Processing &amp; LLMs</x:v>
+      </x:c>
+      <x:c r="C79" s="20" t="str">
+        <x:v>Web search, ranking, recommendation and mining of web and social data. Characteristic extensions include large-scale graph analysis, conversational retrieval, foundation-model and agentic web systems, and fairness and privacy in information access. The broad emerging-applications inventory is not treated as evidence that WSDM is a specialist healthcare or climate venue.</x:v>
+      </x:c>
+      <x:c r="D79" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E79" s="20" t="str">
+        <x:v>https://www.wsdm-conference.org/2027/cffp.html</x:v>
+      </x:c>
+      <x:c r="F79" s="22" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="60" hidden="0" customHeight="1">
+      <x:c r="A80" s="20" t="str">
+        <x:v>WWW</x:v>
+      </x:c>
+      <x:c r="B80" s="20" t="str">
+        <x:v>Knowledge Representation &amp; Reasoning; Data Mining &amp; Data Science; Fairness &amp; Responsible AI; Privacy-preserving ML; Ethics &amp; Governance</x:v>
+      </x:c>
+      <x:c r="C80" s="20" t="str">
+        <x:v>Research on the Web as infrastructure and a socio-technical ecosystem. Characteristic ML-facing tracks include search and recommendation, retrieval-augmented and agentic information access, graph learning, and semantic knowledge. Responsible Web and privacy research are substantive strands. Merely using a web dataset or API is explicitly insufficient topical relevance.</x:v>
+      </x:c>
+      <x:c r="D80" s="21" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E80" s="20" t="str">
         <x:v>https://www2027.thewebconf.org/research-track-papers/</x:v>
       </x:c>
-      <x:c r="F64" s="22" t="n">
+      <x:c r="F80" s="22" t="n">
         <x:v>46302</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0475ca36bdfd4304"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R970268d51ee144a6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>